<commit_message>
Add Ch02 figures for model comparisons
</commit_message>
<xml_diff>
--- a/figures/figure_inventory.xlsx
+++ b/figures/figure_inventory.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Colby\Documents\GitHub\foundry-book\figures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{231F72F7-0386-44C2-B85A-C2F9FAF678EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9261BF58-3D80-4B37-8DAC-FA1E8E86CBF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="300" windowWidth="38640" windowHeight="21240" xr2:uid="{222F1F68-60B1-49B9-BFF7-2C9CF743DB25}"/>
+    <workbookView xWindow="48525" yWindow="2445" windowWidth="24405" windowHeight="14265" xr2:uid="{222F1F68-60B1-49B9-BFF7-2C9CF743DB25}"/>
   </bookViews>
   <sheets>
     <sheet name="Figure Inventory" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="70">
   <si>
     <t>Chapter</t>
   </si>
@@ -158,9 +158,6 @@
     <t>Microsoft Foundry Project Homepage</t>
   </si>
   <si>
-    <t>Figure Number</t>
-  </si>
-  <si>
     <t>Code</t>
   </si>
   <si>
@@ -183,6 +180,72 @@
   </si>
   <si>
     <t>Copying the Project Endpoint URL</t>
+  </si>
+  <si>
+    <t>ch02</t>
+  </si>
+  <si>
+    <t>Locating the Discover tab</t>
+  </si>
+  <si>
+    <t>ch02_ss_portal_001_clean.png</t>
+  </si>
+  <si>
+    <t>ch02_ss_portal_001_ann.png</t>
+  </si>
+  <si>
+    <t>ch02_ss_discover_001_clean.png</t>
+  </si>
+  <si>
+    <t>ch02_ss_discover_001_ann.png</t>
+  </si>
+  <si>
+    <t>ch02_ss_discover_002_clean.png</t>
+  </si>
+  <si>
+    <t>Exploring featured models on the Discover page</t>
+  </si>
+  <si>
+    <t>Listing all available models in Foundry</t>
+  </si>
+  <si>
+    <t>ch02_ss_compare_002_clean.png</t>
+  </si>
+  <si>
+    <t>ch02_ss_compare_001_ann.png</t>
+  </si>
+  <si>
+    <t>Locating the Compare models button</t>
+  </si>
+  <si>
+    <t>Comparing models across benchmarks and capabilities</t>
+  </si>
+  <si>
+    <t>Locating the View leaderboard button</t>
+  </si>
+  <si>
+    <t>ch02_ss_leaderboard_001_ann.png</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Exploring the model leaderboard</t>
+  </si>
+  <si>
+    <t>ch02_ss_leaderboard_002_clean.png</t>
+  </si>
+  <si>
+    <t>ch02_ss_leaderboard_003_ann.png</t>
+  </si>
+  <si>
+    <t>More details about a model's benchmark performance</t>
+  </si>
+  <si>
+    <t>ch02_ss_leaderboard_004_clean.png</t>
+  </si>
+  <si>
+    <t>Metric details across various model benchmarks</t>
   </si>
 </sst>
 </file>
@@ -565,21 +628,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B464DFF5-94DA-41E0-B03E-143380050964}">
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11" customWidth="1"/>
-    <col min="6" max="6" width="30.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="34.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="43.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="70.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="97.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>40</v>
+        <v>63</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -653,7 +716,7 @@
         <v>31</v>
       </c>
       <c r="H3" t="str">
-        <f t="shared" ref="H3:H24" si="0">IF(E3,_xlfn.CONCAT("![",G3,"](figures/",B3,"/",F3,")"),"")</f>
+        <f t="shared" ref="H3:H26" si="0">IF(E3,_xlfn.CONCAT("![",G3,"](figures/",B3,"/",F3,")"),"")</f>
         <v>![Azure Portal - Search Box](figures/ch01/ch01_ss_portal_001_ann.png)</v>
       </c>
     </row>
@@ -1100,19 +1163,19 @@
         <v>5</v>
       </c>
       <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21" t="b">
+        <v>0</v>
+      </c>
+      <c r="E21" t="b">
+        <v>1</v>
+      </c>
+      <c r="F21" t="s">
+        <v>42</v>
+      </c>
+      <c r="G21" t="s">
         <v>41</v>
-      </c>
-      <c r="D21" t="b">
-        <v>0</v>
-      </c>
-      <c r="E21" t="b">
-        <v>1</v>
-      </c>
-      <c r="F21" t="s">
-        <v>43</v>
-      </c>
-      <c r="G21" t="s">
-        <v>42</v>
       </c>
       <c r="H21" t="str">
         <f t="shared" si="0"/>
@@ -1136,10 +1199,10 @@
         <v>1</v>
       </c>
       <c r="F22" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G22" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="H22" t="str">
         <f t="shared" si="0"/>
@@ -1163,7 +1226,7 @@
         <v>0</v>
       </c>
       <c r="F23" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H23" t="str">
         <f t="shared" si="0"/>
@@ -1187,14 +1250,329 @@
         <v>1</v>
       </c>
       <c r="F24" t="s">
+        <v>46</v>
+      </c>
+      <c r="G24" t="s">
         <v>47</v>
       </c>
-      <c r="G24" t="s">
+      <c r="H24" t="str">
+        <f t="shared" si="0"/>
+        <v>![Copying the Project Endpoint URL](figures/ch01/ch01_ss_portal_012_ann.png)</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
         <v>48</v>
       </c>
-      <c r="H24" t="str">
-        <f t="shared" si="0"/>
-        <v>![Copying the Project Endpoint URL](figures/ch01/ch01_ss_portal_012_ann.png)</v>
+      <c r="C25" t="s">
+        <v>6</v>
+      </c>
+      <c r="D25" t="b">
+        <v>0</v>
+      </c>
+      <c r="E25" t="b">
+        <v>0</v>
+      </c>
+      <c r="F25" t="s">
+        <v>50</v>
+      </c>
+      <c r="H25" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>48</v>
+      </c>
+      <c r="C26" t="s">
+        <v>6</v>
+      </c>
+      <c r="D26" t="b">
+        <v>1</v>
+      </c>
+      <c r="E26" t="b">
+        <v>1</v>
+      </c>
+      <c r="F26" t="s">
+        <v>51</v>
+      </c>
+      <c r="G26" t="s">
+        <v>49</v>
+      </c>
+      <c r="H26" t="str">
+        <f>IF(E26,_xlfn.CONCAT("![",G26,"](figures/",B26,"/",F26,")"),"")</f>
+        <v>![Locating the Discover tab](figures/ch02/ch02_ss_portal_001_ann.png)</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>48</v>
+      </c>
+      <c r="C27" t="s">
+        <v>6</v>
+      </c>
+      <c r="D27" t="b">
+        <v>0</v>
+      </c>
+      <c r="E27" t="b">
+        <v>0</v>
+      </c>
+      <c r="F27" t="s">
+        <v>52</v>
+      </c>
+      <c r="H27" t="str">
+        <f t="shared" ref="H27:H36" si="1">IF(E27,_xlfn.CONCAT("![",G27,"](figures/",B27,"/",F27,")"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
+        <v>48</v>
+      </c>
+      <c r="C28" t="s">
+        <v>6</v>
+      </c>
+      <c r="D28" t="b">
+        <v>1</v>
+      </c>
+      <c r="E28" t="b">
+        <v>1</v>
+      </c>
+      <c r="F28" t="s">
+        <v>53</v>
+      </c>
+      <c r="G28" t="s">
+        <v>55</v>
+      </c>
+      <c r="H28" t="str">
+        <f t="shared" si="1"/>
+        <v>![Exploring featured models on the Discover page](figures/ch02/ch02_ss_discover_001_ann.png)</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="s">
+        <v>48</v>
+      </c>
+      <c r="C29" t="s">
+        <v>6</v>
+      </c>
+      <c r="D29" t="b">
+        <v>0</v>
+      </c>
+      <c r="E29" t="b">
+        <v>1</v>
+      </c>
+      <c r="F29" t="s">
+        <v>54</v>
+      </c>
+      <c r="G29" t="s">
+        <v>56</v>
+      </c>
+      <c r="H29" t="str">
+        <f t="shared" si="1"/>
+        <v>![Listing all available models in Foundry](figures/ch02/ch02_ss_discover_002_clean.png)</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s">
+        <v>48</v>
+      </c>
+      <c r="C30" t="s">
+        <v>6</v>
+      </c>
+      <c r="D30" t="b">
+        <v>1</v>
+      </c>
+      <c r="E30" t="b">
+        <v>1</v>
+      </c>
+      <c r="F30" t="s">
+        <v>58</v>
+      </c>
+      <c r="G30" t="s">
+        <v>59</v>
+      </c>
+      <c r="H30" t="str">
+        <f t="shared" si="1"/>
+        <v>![Locating the Compare models button](figures/ch02/ch02_ss_compare_001_ann.png)</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="s">
+        <v>48</v>
+      </c>
+      <c r="C31" t="s">
+        <v>6</v>
+      </c>
+      <c r="D31" t="b">
+        <v>0</v>
+      </c>
+      <c r="E31" t="b">
+        <v>1</v>
+      </c>
+      <c r="F31" t="s">
+        <v>57</v>
+      </c>
+      <c r="G31" t="s">
+        <v>60</v>
+      </c>
+      <c r="H31" t="str">
+        <f t="shared" si="1"/>
+        <v>![Comparing models across benchmarks and capabilities](figures/ch02/ch02_ss_compare_002_clean.png)</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="s">
+        <v>48</v>
+      </c>
+      <c r="C32" t="s">
+        <v>6</v>
+      </c>
+      <c r="D32" t="b">
+        <v>1</v>
+      </c>
+      <c r="E32" t="b">
+        <v>1</v>
+      </c>
+      <c r="F32" t="s">
+        <v>62</v>
+      </c>
+      <c r="G32" t="s">
+        <v>61</v>
+      </c>
+      <c r="H32" t="str">
+        <f t="shared" si="1"/>
+        <v>![Locating the View leaderboard button](figures/ch02/ch02_ss_leaderboard_001_ann.png)</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" t="s">
+        <v>48</v>
+      </c>
+      <c r="C33" t="s">
+        <v>6</v>
+      </c>
+      <c r="D33" t="b">
+        <v>0</v>
+      </c>
+      <c r="E33" t="b">
+        <v>1</v>
+      </c>
+      <c r="F33" t="s">
+        <v>65</v>
+      </c>
+      <c r="G33" t="s">
+        <v>64</v>
+      </c>
+      <c r="H33" t="str">
+        <f t="shared" si="1"/>
+        <v>![Exploring the model leaderboard](figures/ch02/ch02_ss_leaderboard_002_clean.png)</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" t="s">
+        <v>48</v>
+      </c>
+      <c r="C34" t="s">
+        <v>6</v>
+      </c>
+      <c r="D34" t="b">
+        <v>0</v>
+      </c>
+      <c r="E34" t="b">
+        <v>0</v>
+      </c>
+      <c r="F34" t="s">
+        <v>65</v>
+      </c>
+      <c r="H34" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" t="s">
+        <v>48</v>
+      </c>
+      <c r="C35" t="s">
+        <v>6</v>
+      </c>
+      <c r="D35" t="b">
+        <v>1</v>
+      </c>
+      <c r="E35" t="b">
+        <v>1</v>
+      </c>
+      <c r="F35" t="s">
+        <v>66</v>
+      </c>
+      <c r="G35" t="s">
+        <v>67</v>
+      </c>
+      <c r="H35" t="str">
+        <f t="shared" si="1"/>
+        <v>![More details about a model's benchmark performance](figures/ch02/ch02_ss_leaderboard_003_ann.png)</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36" t="s">
+        <v>48</v>
+      </c>
+      <c r="C36" t="s">
+        <v>6</v>
+      </c>
+      <c r="D36" t="b">
+        <v>0</v>
+      </c>
+      <c r="E36" t="b">
+        <v>1</v>
+      </c>
+      <c r="F36" t="s">
+        <v>68</v>
+      </c>
+      <c r="G36" t="s">
+        <v>69</v>
+      </c>
+      <c r="H36" t="str">
+        <f t="shared" si="1"/>
+        <v>![Metric details across various model benchmarks](figures/ch02/ch02_ss_leaderboard_004_clean.png)</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Ch02 add images for web search tool
</commit_message>
<xml_diff>
--- a/figures/figure_inventory.xlsx
+++ b/figures/figure_inventory.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Colby\Documents\GitHub\foundry-book\figures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47AED5C0-6775-49D9-AFD5-2070AE7ED01D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D09F7F3D-9C24-4FBD-836B-5A691E95B9B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="49155" yWindow="2550" windowWidth="24405" windowHeight="14265" xr2:uid="{222F1F68-60B1-49B9-BFF7-2C9CF743DB25}"/>
+    <workbookView xWindow="44715" yWindow="3780" windowWidth="24405" windowHeight="14265" xr2:uid="{222F1F68-60B1-49B9-BFF7-2C9CF743DB25}"/>
   </bookViews>
   <sheets>
     <sheet name="Figure Inventory" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="143">
   <si>
     <t>Chapter</t>
   </si>
@@ -405,6 +405,66 @@
   </si>
   <si>
     <t>ch02_ss_agent_007b_clean.png</t>
+  </si>
+  <si>
+    <t>ch02_ss_tools_001_clean.png</t>
+  </si>
+  <si>
+    <t>ch02_ss_tools_001_ann.png</t>
+  </si>
+  <si>
+    <t>Exploring Tools on the Discover page</t>
+  </si>
+  <si>
+    <t>Locating your real estate Agent</t>
+  </si>
+  <si>
+    <t>ch02_ss_tools_002_clean.png</t>
+  </si>
+  <si>
+    <t>ch02_ss_tools_002_ann.png</t>
+  </si>
+  <si>
+    <t>ch02_ss_tools_003_clean.png</t>
+  </si>
+  <si>
+    <t>ch02_ss_tools_003_ann.png</t>
+  </si>
+  <si>
+    <t>Adding a Tool to your Agent</t>
+  </si>
+  <si>
+    <t>ch02_ss_tools_004_clean.png</t>
+  </si>
+  <si>
+    <t>ch02_ss_tools_004_ann.png</t>
+  </si>
+  <si>
+    <t>Selecting the Web search Tool</t>
+  </si>
+  <si>
+    <t>ch02_ss_tools_005_clean.png</t>
+  </si>
+  <si>
+    <t>ch02_ss_tools_005_ann.png</t>
+  </si>
+  <si>
+    <t>Accepting the terms for Web Search</t>
+  </si>
+  <si>
+    <t>Saving and previewing the Agent with Web Search connected</t>
+  </si>
+  <si>
+    <t>ch02_ss_tools_006_clean.png</t>
+  </si>
+  <si>
+    <t>ch02_ss_tools_006_ann.png</t>
+  </si>
+  <si>
+    <t>ch02_ss_tools_007_clean.png</t>
+  </si>
+  <si>
+    <t>A much more function real estate Agent</t>
   </si>
 </sst>
 </file>
@@ -793,7 +853,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B464DFF5-94DA-41E0-B03E-143380050964}">
-  <dimension ref="A1:H69"/>
+  <dimension ref="A1:H82"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
@@ -1496,7 +1556,7 @@
         <v>52</v>
       </c>
       <c r="H27" t="str">
-        <f t="shared" ref="H27:H68" si="1">IF(E27,_xlfn.CONCAT("![",G27,"](figures/",B27,"/",F27,")"),"")</f>
+        <f t="shared" ref="H27:H64" si="1">IF(E27,_xlfn.CONCAT("![",G27,"](figures/",B27,"/",F27,")"),"")</f>
         <v/>
       </c>
     </row>
@@ -2593,6 +2653,339 @@
       <c r="H69" t="str">
         <f>IF(E69,_xlfn.CONCAT("![",G69,"](figures/",B69,"/",F69,")"),"")</f>
         <v>![Your Agent was published successfully](figures/ch02/ch02_ss_agent_011_clean.png)</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A70">
+        <v>69</v>
+      </c>
+      <c r="B70" t="s">
+        <v>48</v>
+      </c>
+      <c r="C70" t="s">
+        <v>6</v>
+      </c>
+      <c r="D70" t="b">
+        <v>0</v>
+      </c>
+      <c r="E70" t="b">
+        <v>0</v>
+      </c>
+      <c r="F70" t="s">
+        <v>123</v>
+      </c>
+      <c r="H70" t="str">
+        <f t="shared" ref="H70:H82" si="2">IF(E70,_xlfn.CONCAT("![",G70,"](figures/",B70,"/",F70,")"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A71">
+        <v>70</v>
+      </c>
+      <c r="B71" t="s">
+        <v>48</v>
+      </c>
+      <c r="C71" t="s">
+        <v>6</v>
+      </c>
+      <c r="D71" t="b">
+        <v>1</v>
+      </c>
+      <c r="E71" t="b">
+        <v>1</v>
+      </c>
+      <c r="F71" t="s">
+        <v>124</v>
+      </c>
+      <c r="G71" t="s">
+        <v>125</v>
+      </c>
+      <c r="H71" t="str">
+        <f t="shared" si="2"/>
+        <v>![Exploring Tools on the Discover page](figures/ch02/ch02_ss_tools_001_ann.png)</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A72">
+        <v>71</v>
+      </c>
+      <c r="B72" t="s">
+        <v>48</v>
+      </c>
+      <c r="C72" t="s">
+        <v>6</v>
+      </c>
+      <c r="D72" t="b">
+        <v>0</v>
+      </c>
+      <c r="E72" t="b">
+        <v>0</v>
+      </c>
+      <c r="F72" t="s">
+        <v>127</v>
+      </c>
+      <c r="H72" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A73">
+        <v>72</v>
+      </c>
+      <c r="B73" t="s">
+        <v>48</v>
+      </c>
+      <c r="C73" t="s">
+        <v>6</v>
+      </c>
+      <c r="D73" t="b">
+        <v>1</v>
+      </c>
+      <c r="E73" t="b">
+        <v>1</v>
+      </c>
+      <c r="F73" t="s">
+        <v>128</v>
+      </c>
+      <c r="G73" t="s">
+        <v>126</v>
+      </c>
+      <c r="H73" t="str">
+        <f t="shared" si="2"/>
+        <v>![Locating your real estate Agent](figures/ch02/ch02_ss_tools_002_ann.png)</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A74">
+        <v>73</v>
+      </c>
+      <c r="B74" t="s">
+        <v>48</v>
+      </c>
+      <c r="C74" t="s">
+        <v>6</v>
+      </c>
+      <c r="D74" t="b">
+        <v>0</v>
+      </c>
+      <c r="E74" t="b">
+        <v>0</v>
+      </c>
+      <c r="F74" t="s">
+        <v>129</v>
+      </c>
+      <c r="H74" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A75">
+        <v>74</v>
+      </c>
+      <c r="B75" t="s">
+        <v>48</v>
+      </c>
+      <c r="C75" t="s">
+        <v>6</v>
+      </c>
+      <c r="D75" t="b">
+        <v>1</v>
+      </c>
+      <c r="E75" t="b">
+        <v>1</v>
+      </c>
+      <c r="F75" t="s">
+        <v>130</v>
+      </c>
+      <c r="G75" t="s">
+        <v>131</v>
+      </c>
+      <c r="H75" t="str">
+        <f t="shared" si="2"/>
+        <v>![Adding a Tool to your Agent](figures/ch02/ch02_ss_tools_003_ann.png)</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A76">
+        <v>75</v>
+      </c>
+      <c r="B76" t="s">
+        <v>48</v>
+      </c>
+      <c r="C76" t="s">
+        <v>6</v>
+      </c>
+      <c r="D76" t="b">
+        <v>0</v>
+      </c>
+      <c r="E76" t="b">
+        <v>0</v>
+      </c>
+      <c r="F76" t="s">
+        <v>132</v>
+      </c>
+      <c r="H76" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A77">
+        <v>76</v>
+      </c>
+      <c r="B77" t="s">
+        <v>48</v>
+      </c>
+      <c r="C77" t="s">
+        <v>6</v>
+      </c>
+      <c r="D77" t="b">
+        <v>1</v>
+      </c>
+      <c r="E77" t="b">
+        <v>1</v>
+      </c>
+      <c r="F77" t="s">
+        <v>133</v>
+      </c>
+      <c r="G77" t="s">
+        <v>134</v>
+      </c>
+      <c r="H77" t="str">
+        <f t="shared" si="2"/>
+        <v>![Selecting the Web search Tool](figures/ch02/ch02_ss_tools_004_ann.png)</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A78">
+        <v>77</v>
+      </c>
+      <c r="B78" t="s">
+        <v>48</v>
+      </c>
+      <c r="C78" t="s">
+        <v>6</v>
+      </c>
+      <c r="D78" t="b">
+        <v>0</v>
+      </c>
+      <c r="E78" t="b">
+        <v>0</v>
+      </c>
+      <c r="F78" t="s">
+        <v>135</v>
+      </c>
+      <c r="H78" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A79">
+        <v>78</v>
+      </c>
+      <c r="B79" t="s">
+        <v>48</v>
+      </c>
+      <c r="C79" t="s">
+        <v>6</v>
+      </c>
+      <c r="D79" t="b">
+        <v>1</v>
+      </c>
+      <c r="E79" t="b">
+        <v>1</v>
+      </c>
+      <c r="F79" t="s">
+        <v>136</v>
+      </c>
+      <c r="G79" t="s">
+        <v>137</v>
+      </c>
+      <c r="H79" t="str">
+        <f t="shared" si="2"/>
+        <v>![Accepting the terms for Web Search](figures/ch02/ch02_ss_tools_005_ann.png)</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A80">
+        <v>79</v>
+      </c>
+      <c r="B80" t="s">
+        <v>48</v>
+      </c>
+      <c r="C80" t="s">
+        <v>6</v>
+      </c>
+      <c r="D80" t="b">
+        <v>0</v>
+      </c>
+      <c r="E80" t="b">
+        <v>0</v>
+      </c>
+      <c r="F80" t="s">
+        <v>139</v>
+      </c>
+      <c r="H80" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A81">
+        <v>80</v>
+      </c>
+      <c r="B81" t="s">
+        <v>48</v>
+      </c>
+      <c r="C81" t="s">
+        <v>6</v>
+      </c>
+      <c r="D81" t="b">
+        <v>1</v>
+      </c>
+      <c r="E81" t="b">
+        <v>1</v>
+      </c>
+      <c r="F81" t="s">
+        <v>140</v>
+      </c>
+      <c r="G81" t="s">
+        <v>138</v>
+      </c>
+      <c r="H81" t="str">
+        <f t="shared" si="2"/>
+        <v>![Saving and previewing the Agent with Web Search connected](figures/ch02/ch02_ss_tools_006_ann.png)</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A82">
+        <v>81</v>
+      </c>
+      <c r="B82" t="s">
+        <v>48</v>
+      </c>
+      <c r="C82" t="s">
+        <v>6</v>
+      </c>
+      <c r="D82" t="b">
+        <v>0</v>
+      </c>
+      <c r="E82" t="b">
+        <v>1</v>
+      </c>
+      <c r="F82" t="s">
+        <v>141</v>
+      </c>
+      <c r="G82" t="s">
+        <v>142</v>
+      </c>
+      <c r="H82" t="str">
+        <f t="shared" si="2"/>
+        <v>![A much more function real estate Agent](figures/ch02/ch02_ss_tools_007_clean.png)</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Ch02 figures for Cosmos DB
</commit_message>
<xml_diff>
--- a/figures/figure_inventory.xlsx
+++ b/figures/figure_inventory.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Colby\Documents\GitHub\foundry-book\figures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D09F7F3D-9C24-4FBD-836B-5A691E95B9B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41807B75-0B1A-49C9-B17F-6BA433DE591C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="44715" yWindow="3780" windowWidth="24405" windowHeight="14265" xr2:uid="{222F1F68-60B1-49B9-BFF7-2C9CF743DB25}"/>
+    <workbookView xWindow="43965" yWindow="3885" windowWidth="24405" windowHeight="14265" xr2:uid="{222F1F68-60B1-49B9-BFF7-2C9CF743DB25}"/>
   </bookViews>
   <sheets>
     <sheet name="Figure Inventory" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="168">
   <si>
     <t>Chapter</t>
   </si>
@@ -65,9 +65,6 @@
     <t>Illustration</t>
   </si>
   <si>
-    <t>ch01_il_001.png</t>
-  </si>
-  <si>
     <t>Used?</t>
   </si>
   <si>
@@ -465,6 +462,84 @@
   </si>
   <si>
     <t>A much more function real estate Agent</t>
+  </si>
+  <si>
+    <t>Example MCP-based architecture</t>
+  </si>
+  <si>
+    <t>ch02_il_tools_001.png</t>
+  </si>
+  <si>
+    <t>ch02_ss_tools_008_clean.png</t>
+  </si>
+  <si>
+    <t>Configuring a general MCP tool</t>
+  </si>
+  <si>
+    <t>ch01_il_portal_001.png</t>
+  </si>
+  <si>
+    <t>ch02_ss_cosmos_001_clean.png</t>
+  </si>
+  <si>
+    <t>ch02_ss_cosmos_001_ann.png</t>
+  </si>
+  <si>
+    <t>The Cosmos DB screen in the Azure Portal</t>
+  </si>
+  <si>
+    <t>Locating your Cosmos DB URI and Key</t>
+  </si>
+  <si>
+    <t>ch02_ss_cosmos_002_clean.png</t>
+  </si>
+  <si>
+    <t>ch02_ss_cosmos_002_ann.png</t>
+  </si>
+  <si>
+    <t>ch02_ss_cosmos_003_clean.png</t>
+  </si>
+  <si>
+    <t>ch02_ss_cosmos_003_ann.png</t>
+  </si>
+  <si>
+    <t>Adding another Tool to your Agent</t>
+  </si>
+  <si>
+    <t>ch02_ss_cosmos_004_clean.png</t>
+  </si>
+  <si>
+    <t>ch02_ss_cosmos_004_ann.png</t>
+  </si>
+  <si>
+    <t>Locating the Cosmos DB Tool in the Catalog</t>
+  </si>
+  <si>
+    <t>ch02_ss_cosmos_005_clean.png</t>
+  </si>
+  <si>
+    <t>ch02_ss_cosmos_005_ann.png</t>
+  </si>
+  <si>
+    <t>ch02_ss_cosmos_006_clean.png</t>
+  </si>
+  <si>
+    <t>ch02_ss_cosmos_006_ann.png</t>
+  </si>
+  <si>
+    <t>Filling in the URI and Key for the Cosmos DB Tool connection</t>
+  </si>
+  <si>
+    <t>ch02_ss_cosmos_007_clean.png</t>
+  </si>
+  <si>
+    <t>ch02_ss_cosmos_007_ann.png</t>
+  </si>
+  <si>
+    <t>Checking that your Cosmos DB Tool is connected</t>
+  </si>
+  <si>
+    <t>Information about hosting MCP servers</t>
   </si>
 </sst>
 </file>
@@ -853,10 +928,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B464DFF5-94DA-41E0-B03E-143380050964}">
-  <dimension ref="A1:H82"/>
+  <dimension ref="A1:H105"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11" customWidth="1"/>
@@ -867,7 +942,7 @@
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -879,7 +954,7 @@
         <v>7</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>2</v>
@@ -908,14 +983,14 @@
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>9</v>
+        <v>146</v>
       </c>
       <c r="G2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H2" t="str">
         <f>IF(E2,_xlfn.CONCAT("![",G2,"](figures/",B2,"/",F2,")"),"")</f>
-        <v>![Foundry Resource and Project Organization](figures/ch01/ch01_il_001.png)</v>
+        <v>![Foundry Resource and Project Organization](figures/ch01/ch01_il_portal_001.png)</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -935,10 +1010,10 @@
         <v>1</v>
       </c>
       <c r="F3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H3" t="str">
         <f t="shared" ref="H3:H25" si="0">IF(E3,_xlfn.CONCAT("![",G3,"](figures/",B3,"/",F3,")"),"")</f>
@@ -962,7 +1037,7 @@
         <v>0</v>
       </c>
       <c r="F4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H4" t="str">
         <f t="shared" si="0"/>
@@ -986,10 +1061,10 @@
         <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H5" t="str">
         <f t="shared" si="0"/>
@@ -1013,7 +1088,7 @@
         <v>0</v>
       </c>
       <c r="F6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H6" t="str">
         <f t="shared" si="0"/>
@@ -1037,10 +1112,10 @@
         <v>1</v>
       </c>
       <c r="F7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H7" t="str">
         <f t="shared" si="0"/>
@@ -1064,7 +1139,7 @@
         <v>0</v>
       </c>
       <c r="F8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H8" t="str">
         <f t="shared" si="0"/>
@@ -1088,10 +1163,10 @@
         <v>1</v>
       </c>
       <c r="F9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H9" t="str">
         <f t="shared" si="0"/>
@@ -1115,7 +1190,7 @@
         <v>0</v>
       </c>
       <c r="F10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H10" t="str">
         <f t="shared" si="0"/>
@@ -1139,10 +1214,10 @@
         <v>1</v>
       </c>
       <c r="F11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H11" t="str">
         <f t="shared" si="0"/>
@@ -1166,7 +1241,7 @@
         <v>0</v>
       </c>
       <c r="F12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H12" t="str">
         <f t="shared" si="0"/>
@@ -1190,10 +1265,10 @@
         <v>1</v>
       </c>
       <c r="F13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G13" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H13" t="str">
         <f t="shared" si="0"/>
@@ -1217,7 +1292,7 @@
         <v>0</v>
       </c>
       <c r="F14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H14" t="str">
         <f t="shared" si="0"/>
@@ -1241,10 +1316,10 @@
         <v>1</v>
       </c>
       <c r="F15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G15" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H15" t="str">
         <f t="shared" si="0"/>
@@ -1268,10 +1343,10 @@
         <v>1</v>
       </c>
       <c r="F16" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H16" t="str">
         <f t="shared" si="0"/>
@@ -1295,7 +1370,7 @@
         <v>0</v>
       </c>
       <c r="F17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H17" t="str">
         <f t="shared" si="0"/>
@@ -1319,10 +1394,10 @@
         <v>1</v>
       </c>
       <c r="F18" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G18" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H18" t="str">
         <f t="shared" si="0"/>
@@ -1346,7 +1421,7 @@
         <v>0</v>
       </c>
       <c r="F19" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H19" t="str">
         <f t="shared" si="0"/>
@@ -1370,10 +1445,10 @@
         <v>1</v>
       </c>
       <c r="F20" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G20" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H20" t="str">
         <f t="shared" si="0"/>
@@ -1388,19 +1463,19 @@
         <v>5</v>
       </c>
       <c r="C21" t="s">
+        <v>39</v>
+      </c>
+      <c r="D21" t="b">
+        <v>0</v>
+      </c>
+      <c r="E21" t="b">
+        <v>1</v>
+      </c>
+      <c r="F21" t="s">
+        <v>41</v>
+      </c>
+      <c r="G21" t="s">
         <v>40</v>
-      </c>
-      <c r="D21" t="b">
-        <v>0</v>
-      </c>
-      <c r="E21" t="b">
-        <v>1</v>
-      </c>
-      <c r="F21" t="s">
-        <v>42</v>
-      </c>
-      <c r="G21" t="s">
-        <v>41</v>
       </c>
       <c r="H21" t="str">
         <f t="shared" si="0"/>
@@ -1424,10 +1499,10 @@
         <v>1</v>
       </c>
       <c r="F22" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G22" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H22" t="str">
         <f t="shared" si="0"/>
@@ -1451,7 +1526,7 @@
         <v>0</v>
       </c>
       <c r="F23" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H23" t="str">
         <f t="shared" si="0"/>
@@ -1475,10 +1550,10 @@
         <v>1</v>
       </c>
       <c r="F24" t="s">
+        <v>45</v>
+      </c>
+      <c r="G24" t="s">
         <v>46</v>
-      </c>
-      <c r="G24" t="s">
-        <v>47</v>
       </c>
       <c r="H24" t="str">
         <f t="shared" si="0"/>
@@ -1490,7 +1565,7 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C25" t="s">
         <v>6</v>
@@ -1502,7 +1577,7 @@
         <v>0</v>
       </c>
       <c r="F25" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H25" t="str">
         <f t="shared" si="0"/>
@@ -1514,22 +1589,22 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
+        <v>47</v>
+      </c>
+      <c r="C26" t="s">
+        <v>6</v>
+      </c>
+      <c r="D26" t="b">
+        <v>1</v>
+      </c>
+      <c r="E26" t="b">
+        <v>1</v>
+      </c>
+      <c r="F26" t="s">
+        <v>50</v>
+      </c>
+      <c r="G26" t="s">
         <v>48</v>
-      </c>
-      <c r="C26" t="s">
-        <v>6</v>
-      </c>
-      <c r="D26" t="b">
-        <v>1</v>
-      </c>
-      <c r="E26" t="b">
-        <v>1</v>
-      </c>
-      <c r="F26" t="s">
-        <v>51</v>
-      </c>
-      <c r="G26" t="s">
-        <v>49</v>
       </c>
       <c r="H26" t="str">
         <f>IF(E26,_xlfn.CONCAT("![",G26,"](figures/",B26,"/",F26,")"),"")</f>
@@ -1541,7 +1616,7 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C27" t="s">
         <v>6</v>
@@ -1553,7 +1628,7 @@
         <v>0</v>
       </c>
       <c r="F27" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H27" t="str">
         <f t="shared" ref="H27:H64" si="1">IF(E27,_xlfn.CONCAT("![",G27,"](figures/",B27,"/",F27,")"),"")</f>
@@ -1565,7 +1640,7 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C28" t="s">
         <v>6</v>
@@ -1577,10 +1652,10 @@
         <v>1</v>
       </c>
       <c r="F28" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G28" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H28" t="str">
         <f t="shared" si="1"/>
@@ -1592,7 +1667,7 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C29" t="s">
         <v>6</v>
@@ -1604,10 +1679,10 @@
         <v>1</v>
       </c>
       <c r="F29" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G29" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H29" t="str">
         <f t="shared" si="1"/>
@@ -1619,7 +1694,7 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C30" t="s">
         <v>6</v>
@@ -1631,10 +1706,10 @@
         <v>1</v>
       </c>
       <c r="F30" t="s">
+        <v>57</v>
+      </c>
+      <c r="G30" t="s">
         <v>58</v>
-      </c>
-      <c r="G30" t="s">
-        <v>59</v>
       </c>
       <c r="H30" t="str">
         <f t="shared" si="1"/>
@@ -1646,7 +1721,7 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C31" t="s">
         <v>6</v>
@@ -1658,10 +1733,10 @@
         <v>1</v>
       </c>
       <c r="F31" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G31" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H31" t="str">
         <f t="shared" si="1"/>
@@ -1673,7 +1748,7 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C32" t="s">
         <v>6</v>
@@ -1685,10 +1760,10 @@
         <v>1</v>
       </c>
       <c r="F32" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G32" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="H32" t="str">
         <f t="shared" si="1"/>
@@ -1700,7 +1775,7 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C33" t="s">
         <v>6</v>
@@ -1712,10 +1787,10 @@
         <v>1</v>
       </c>
       <c r="F33" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G33" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H33" t="str">
         <f t="shared" si="1"/>
@@ -1727,7 +1802,7 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C34" t="s">
         <v>6</v>
@@ -1739,7 +1814,7 @@
         <v>0</v>
       </c>
       <c r="F34" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H34" t="str">
         <f t="shared" si="1"/>
@@ -1751,7 +1826,7 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C35" t="s">
         <v>6</v>
@@ -1763,10 +1838,10 @@
         <v>1</v>
       </c>
       <c r="F35" t="s">
+        <v>65</v>
+      </c>
+      <c r="G35" t="s">
         <v>66</v>
-      </c>
-      <c r="G35" t="s">
-        <v>67</v>
       </c>
       <c r="H35" t="str">
         <f t="shared" si="1"/>
@@ -1778,7 +1853,7 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C36" t="s">
         <v>6</v>
@@ -1790,10 +1865,10 @@
         <v>1</v>
       </c>
       <c r="F36" t="s">
+        <v>67</v>
+      </c>
+      <c r="G36" t="s">
         <v>68</v>
-      </c>
-      <c r="G36" t="s">
-        <v>69</v>
       </c>
       <c r="H36" t="str">
         <f t="shared" si="1"/>
@@ -1805,7 +1880,7 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C37" t="s">
         <v>6</v>
@@ -1817,7 +1892,7 @@
         <v>0</v>
       </c>
       <c r="F37" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H37" t="str">
         <f t="shared" si="1"/>
@@ -1829,7 +1904,7 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C38" t="s">
         <v>6</v>
@@ -1841,10 +1916,10 @@
         <v>1</v>
       </c>
       <c r="F38" t="s">
+        <v>69</v>
+      </c>
+      <c r="G38" t="s">
         <v>70</v>
-      </c>
-      <c r="G38" t="s">
-        <v>71</v>
       </c>
       <c r="H38" t="str">
         <f t="shared" si="1"/>
@@ -1856,7 +1931,7 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C39" t="s">
         <v>6</v>
@@ -1868,7 +1943,7 @@
         <v>0</v>
       </c>
       <c r="F39" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H39" t="str">
         <f t="shared" si="1"/>
@@ -1880,7 +1955,7 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C40" t="s">
         <v>6</v>
@@ -1892,10 +1967,10 @@
         <v>1</v>
       </c>
       <c r="F40" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G40" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H40" t="str">
         <f t="shared" si="1"/>
@@ -1907,7 +1982,7 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C41" t="s">
         <v>6</v>
@@ -1919,7 +1994,7 @@
         <v>0</v>
       </c>
       <c r="F41" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H41" t="str">
         <f t="shared" si="1"/>
@@ -1931,7 +2006,7 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C42" t="s">
         <v>6</v>
@@ -1943,10 +2018,10 @@
         <v>1</v>
       </c>
       <c r="F42" t="s">
+        <v>76</v>
+      </c>
+      <c r="G42" t="s">
         <v>77</v>
-      </c>
-      <c r="G42" t="s">
-        <v>78</v>
       </c>
       <c r="H42" t="str">
         <f t="shared" si="1"/>
@@ -1958,7 +2033,7 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C43" t="s">
         <v>6</v>
@@ -1970,10 +2045,10 @@
         <v>1</v>
       </c>
       <c r="F43" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G43" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H43" t="str">
         <f t="shared" si="1"/>
@@ -1985,7 +2060,7 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C44" t="s">
         <v>6</v>
@@ -1997,10 +2072,10 @@
         <v>1</v>
       </c>
       <c r="F44" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G44" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H44" t="str">
         <f t="shared" si="1"/>
@@ -2012,7 +2087,7 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C45" t="s">
         <v>6</v>
@@ -2024,7 +2099,7 @@
         <v>0</v>
       </c>
       <c r="F45" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H45" t="str">
         <f t="shared" si="1"/>
@@ -2036,7 +2111,7 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C46" t="s">
         <v>6</v>
@@ -2048,10 +2123,10 @@
         <v>1</v>
       </c>
       <c r="F46" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G46" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="H46" t="str">
         <f>IF(E46,_xlfn.CONCAT("![",G46,"](figures/",B46,"/",F46,")"),"")</f>
@@ -2063,7 +2138,7 @@
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C47" t="s">
         <v>6</v>
@@ -2075,7 +2150,7 @@
         <v>0</v>
       </c>
       <c r="F47" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H47" t="str">
         <f t="shared" si="1"/>
@@ -2087,7 +2162,7 @@
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C48" t="s">
         <v>6</v>
@@ -2099,10 +2174,10 @@
         <v>1</v>
       </c>
       <c r="F48" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G48" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H48" t="str">
         <f t="shared" si="1"/>
@@ -2114,7 +2189,7 @@
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C49" t="s">
         <v>6</v>
@@ -2126,10 +2201,10 @@
         <v>1</v>
       </c>
       <c r="F49" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G49" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H49" t="str">
         <f t="shared" si="1"/>
@@ -2141,7 +2216,7 @@
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C50" t="s">
         <v>6</v>
@@ -2153,7 +2228,7 @@
         <v>0</v>
       </c>
       <c r="F50" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H50" t="str">
         <f t="shared" si="1"/>
@@ -2165,7 +2240,7 @@
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C51" t="s">
         <v>6</v>
@@ -2177,10 +2252,10 @@
         <v>1</v>
       </c>
       <c r="F51" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G51" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H51" t="str">
         <f t="shared" si="1"/>
@@ -2192,7 +2267,7 @@
         <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C52" t="s">
         <v>6</v>
@@ -2204,7 +2279,7 @@
         <v>0</v>
       </c>
       <c r="F52" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H52" t="str">
         <f t="shared" si="1"/>
@@ -2216,7 +2291,7 @@
         <v>52</v>
       </c>
       <c r="B53" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C53" t="s">
         <v>6</v>
@@ -2228,10 +2303,10 @@
         <v>1</v>
       </c>
       <c r="F53" t="s">
+        <v>93</v>
+      </c>
+      <c r="G53" t="s">
         <v>94</v>
-      </c>
-      <c r="G53" t="s">
-        <v>95</v>
       </c>
       <c r="H53" t="str">
         <f t="shared" si="1"/>
@@ -2243,7 +2318,7 @@
         <v>53</v>
       </c>
       <c r="B54" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C54" t="s">
         <v>6</v>
@@ -2255,7 +2330,7 @@
         <v>0</v>
       </c>
       <c r="F54" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H54" t="str">
         <f t="shared" si="1"/>
@@ -2267,7 +2342,7 @@
         <v>54</v>
       </c>
       <c r="B55" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C55" t="s">
         <v>6</v>
@@ -2279,10 +2354,10 @@
         <v>1</v>
       </c>
       <c r="F55" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G55" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="H55" t="str">
         <f t="shared" si="1"/>
@@ -2294,7 +2369,7 @@
         <v>55</v>
       </c>
       <c r="B56" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C56" t="s">
         <v>6</v>
@@ -2306,10 +2381,10 @@
         <v>1</v>
       </c>
       <c r="F56" t="s">
+        <v>98</v>
+      </c>
+      <c r="G56" t="s">
         <v>99</v>
-      </c>
-      <c r="G56" t="s">
-        <v>100</v>
       </c>
       <c r="H56" t="str">
         <f t="shared" si="1"/>
@@ -2321,7 +2396,7 @@
         <v>56</v>
       </c>
       <c r="B57" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C57" t="s">
         <v>6</v>
@@ -2333,7 +2408,7 @@
         <v>0</v>
       </c>
       <c r="F57" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H57" t="str">
         <f t="shared" si="1"/>
@@ -2345,7 +2420,7 @@
         <v>57</v>
       </c>
       <c r="B58" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C58" t="s">
         <v>6</v>
@@ -2357,10 +2432,10 @@
         <v>1</v>
       </c>
       <c r="F58" t="s">
+        <v>101</v>
+      </c>
+      <c r="G58" t="s">
         <v>102</v>
-      </c>
-      <c r="G58" t="s">
-        <v>103</v>
       </c>
       <c r="H58" t="str">
         <f t="shared" si="1"/>
@@ -2372,7 +2447,7 @@
         <v>58</v>
       </c>
       <c r="B59" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C59" t="s">
         <v>6</v>
@@ -2384,7 +2459,7 @@
         <v>0</v>
       </c>
       <c r="F59" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H59" t="str">
         <f t="shared" si="1"/>
@@ -2396,7 +2471,7 @@
         <v>59</v>
       </c>
       <c r="B60" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C60" t="s">
         <v>6</v>
@@ -2408,10 +2483,10 @@
         <v>1</v>
       </c>
       <c r="F60" t="s">
+        <v>104</v>
+      </c>
+      <c r="G60" t="s">
         <v>105</v>
-      </c>
-      <c r="G60" t="s">
-        <v>106</v>
       </c>
       <c r="H60" t="str">
         <f t="shared" si="1"/>
@@ -2423,7 +2498,7 @@
         <v>60</v>
       </c>
       <c r="B61" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C61" t="s">
         <v>6</v>
@@ -2435,10 +2510,10 @@
         <v>1</v>
       </c>
       <c r="F61" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G61" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H61" t="str">
         <f t="shared" si="1"/>
@@ -2450,7 +2525,7 @@
         <v>61</v>
       </c>
       <c r="B62" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C62" t="s">
         <v>6</v>
@@ -2462,10 +2537,10 @@
         <v>1</v>
       </c>
       <c r="F62" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G62" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H62" t="str">
         <f t="shared" si="1"/>
@@ -2477,7 +2552,7 @@
         <v>62</v>
       </c>
       <c r="B63" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C63" t="s">
         <v>6</v>
@@ -2489,10 +2564,10 @@
         <v>1</v>
       </c>
       <c r="F63" t="s">
+        <v>108</v>
+      </c>
+      <c r="G63" t="s">
         <v>109</v>
-      </c>
-      <c r="G63" t="s">
-        <v>110</v>
       </c>
       <c r="H63" t="str">
         <f t="shared" si="1"/>
@@ -2504,7 +2579,7 @@
         <v>63</v>
       </c>
       <c r="B64" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C64" t="s">
         <v>6</v>
@@ -2516,10 +2591,10 @@
         <v>1</v>
       </c>
       <c r="F64" t="s">
+        <v>118</v>
+      </c>
+      <c r="G64" t="s">
         <v>119</v>
-      </c>
-      <c r="G64" t="s">
-        <v>120</v>
       </c>
       <c r="H64" t="str">
         <f t="shared" si="1"/>
@@ -2531,7 +2606,7 @@
         <v>64</v>
       </c>
       <c r="B65" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C65" t="s">
         <v>6</v>
@@ -2543,7 +2618,7 @@
         <v>0</v>
       </c>
       <c r="F65" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H65" t="str">
         <f>IF(E65,_xlfn.CONCAT("![",G65,"](figures/",B65,"/",F65,")"),"")</f>
@@ -2555,7 +2630,7 @@
         <v>65</v>
       </c>
       <c r="B66" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C66" t="s">
         <v>6</v>
@@ -2567,10 +2642,10 @@
         <v>1</v>
       </c>
       <c r="F66" t="s">
+        <v>111</v>
+      </c>
+      <c r="G66" t="s">
         <v>112</v>
-      </c>
-      <c r="G66" t="s">
-        <v>113</v>
       </c>
       <c r="H66" t="str">
         <f>IF(E66,_xlfn.CONCAT("![",G66,"](figures/",B66,"/",F66,")"),"")</f>
@@ -2582,7 +2657,7 @@
         <v>66</v>
       </c>
       <c r="B67" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C67" t="s">
         <v>6</v>
@@ -2594,7 +2669,7 @@
         <v>0</v>
       </c>
       <c r="F67" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H67" t="str">
         <f>IF(E67,_xlfn.CONCAT("![",G67,"](figures/",B67,"/",F67,")"),"")</f>
@@ -2606,7 +2681,7 @@
         <v>67</v>
       </c>
       <c r="B68" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C68" t="s">
         <v>6</v>
@@ -2618,10 +2693,10 @@
         <v>1</v>
       </c>
       <c r="F68" t="s">
+        <v>113</v>
+      </c>
+      <c r="G68" t="s">
         <v>114</v>
-      </c>
-      <c r="G68" t="s">
-        <v>115</v>
       </c>
       <c r="H68" t="str">
         <f>IF(E68,_xlfn.CONCAT("![",G68,"](figures/",B68,"/",F68,")"),"")</f>
@@ -2633,7 +2708,7 @@
         <v>68</v>
       </c>
       <c r="B69" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C69" t="s">
         <v>6</v>
@@ -2645,10 +2720,10 @@
         <v>1</v>
       </c>
       <c r="F69" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G69" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H69" t="str">
         <f>IF(E69,_xlfn.CONCAT("![",G69,"](figures/",B69,"/",F69,")"),"")</f>
@@ -2660,7 +2735,7 @@
         <v>69</v>
       </c>
       <c r="B70" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C70" t="s">
         <v>6</v>
@@ -2672,10 +2747,10 @@
         <v>0</v>
       </c>
       <c r="F70" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H70" t="str">
-        <f t="shared" ref="H70:H82" si="2">IF(E70,_xlfn.CONCAT("![",G70,"](figures/",B70,"/",F70,")"),"")</f>
+        <f t="shared" ref="H70:H105" si="2">IF(E70,_xlfn.CONCAT("![",G70,"](figures/",B70,"/",F70,")"),"")</f>
         <v/>
       </c>
     </row>
@@ -2684,7 +2759,7 @@
         <v>70</v>
       </c>
       <c r="B71" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C71" t="s">
         <v>6</v>
@@ -2696,10 +2771,10 @@
         <v>1</v>
       </c>
       <c r="F71" t="s">
+        <v>123</v>
+      </c>
+      <c r="G71" t="s">
         <v>124</v>
-      </c>
-      <c r="G71" t="s">
-        <v>125</v>
       </c>
       <c r="H71" t="str">
         <f t="shared" si="2"/>
@@ -2711,7 +2786,7 @@
         <v>71</v>
       </c>
       <c r="B72" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C72" t="s">
         <v>6</v>
@@ -2723,7 +2798,7 @@
         <v>0</v>
       </c>
       <c r="F72" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H72" t="str">
         <f t="shared" si="2"/>
@@ -2735,7 +2810,7 @@
         <v>72</v>
       </c>
       <c r="B73" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C73" t="s">
         <v>6</v>
@@ -2747,10 +2822,10 @@
         <v>1</v>
       </c>
       <c r="F73" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G73" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="H73" t="str">
         <f t="shared" si="2"/>
@@ -2762,7 +2837,7 @@
         <v>73</v>
       </c>
       <c r="B74" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C74" t="s">
         <v>6</v>
@@ -2774,7 +2849,7 @@
         <v>0</v>
       </c>
       <c r="F74" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="H74" t="str">
         <f t="shared" si="2"/>
@@ -2786,7 +2861,7 @@
         <v>74</v>
       </c>
       <c r="B75" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C75" t="s">
         <v>6</v>
@@ -2798,10 +2873,10 @@
         <v>1</v>
       </c>
       <c r="F75" t="s">
+        <v>129</v>
+      </c>
+      <c r="G75" t="s">
         <v>130</v>
-      </c>
-      <c r="G75" t="s">
-        <v>131</v>
       </c>
       <c r="H75" t="str">
         <f t="shared" si="2"/>
@@ -2813,7 +2888,7 @@
         <v>75</v>
       </c>
       <c r="B76" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C76" t="s">
         <v>6</v>
@@ -2825,7 +2900,7 @@
         <v>0</v>
       </c>
       <c r="F76" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="H76" t="str">
         <f t="shared" si="2"/>
@@ -2837,7 +2912,7 @@
         <v>76</v>
       </c>
       <c r="B77" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C77" t="s">
         <v>6</v>
@@ -2849,10 +2924,10 @@
         <v>1</v>
       </c>
       <c r="F77" t="s">
+        <v>132</v>
+      </c>
+      <c r="G77" t="s">
         <v>133</v>
-      </c>
-      <c r="G77" t="s">
-        <v>134</v>
       </c>
       <c r="H77" t="str">
         <f t="shared" si="2"/>
@@ -2864,7 +2939,7 @@
         <v>77</v>
       </c>
       <c r="B78" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C78" t="s">
         <v>6</v>
@@ -2876,7 +2951,7 @@
         <v>0</v>
       </c>
       <c r="F78" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="H78" t="str">
         <f t="shared" si="2"/>
@@ -2888,7 +2963,7 @@
         <v>78</v>
       </c>
       <c r="B79" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C79" t="s">
         <v>6</v>
@@ -2900,10 +2975,10 @@
         <v>1</v>
       </c>
       <c r="F79" t="s">
+        <v>135</v>
+      </c>
+      <c r="G79" t="s">
         <v>136</v>
-      </c>
-      <c r="G79" t="s">
-        <v>137</v>
       </c>
       <c r="H79" t="str">
         <f t="shared" si="2"/>
@@ -2915,7 +2990,7 @@
         <v>79</v>
       </c>
       <c r="B80" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C80" t="s">
         <v>6</v>
@@ -2927,7 +3002,7 @@
         <v>0</v>
       </c>
       <c r="F80" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="H80" t="str">
         <f t="shared" si="2"/>
@@ -2939,7 +3014,7 @@
         <v>80</v>
       </c>
       <c r="B81" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C81" t="s">
         <v>6</v>
@@ -2951,10 +3026,10 @@
         <v>1</v>
       </c>
       <c r="F81" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="G81" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H81" t="str">
         <f t="shared" si="2"/>
@@ -2966,7 +3041,7 @@
         <v>81</v>
       </c>
       <c r="B82" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C82" t="s">
         <v>6</v>
@@ -2978,14 +3053,488 @@
         <v>1</v>
       </c>
       <c r="F82" t="s">
+        <v>140</v>
+      </c>
+      <c r="G82" t="s">
         <v>141</v>
-      </c>
-      <c r="G82" t="s">
-        <v>142</v>
       </c>
       <c r="H82" t="str">
         <f t="shared" si="2"/>
         <v>![A much more function real estate Agent](figures/ch02/ch02_ss_tools_007_clean.png)</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A83">
+        <v>82</v>
+      </c>
+      <c r="B83" t="s">
+        <v>47</v>
+      </c>
+      <c r="C83" t="s">
+        <v>8</v>
+      </c>
+      <c r="D83" t="b">
+        <v>0</v>
+      </c>
+      <c r="E83" t="b">
+        <v>1</v>
+      </c>
+      <c r="F83" t="s">
+        <v>143</v>
+      </c>
+      <c r="G83" t="s">
+        <v>142</v>
+      </c>
+      <c r="H83" t="str">
+        <f t="shared" si="2"/>
+        <v>![Example MCP-based architecture](figures/ch02/ch02_il_tools_001.png)</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A84">
+        <v>83</v>
+      </c>
+      <c r="B84" t="s">
+        <v>47</v>
+      </c>
+      <c r="C84" t="s">
+        <v>6</v>
+      </c>
+      <c r="D84" t="b">
+        <v>0</v>
+      </c>
+      <c r="E84" t="b">
+        <v>1</v>
+      </c>
+      <c r="F84" t="s">
+        <v>144</v>
+      </c>
+      <c r="G84" t="s">
+        <v>145</v>
+      </c>
+      <c r="H84" t="str">
+        <f t="shared" si="2"/>
+        <v>![Configuring a general MCP tool](figures/ch02/ch02_ss_tools_008_clean.png)</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A85">
+        <v>84</v>
+      </c>
+      <c r="B85" t="s">
+        <v>47</v>
+      </c>
+      <c r="C85" t="s">
+        <v>6</v>
+      </c>
+      <c r="D85" t="b">
+        <v>0</v>
+      </c>
+      <c r="E85" t="b">
+        <v>0</v>
+      </c>
+      <c r="F85" t="s">
+        <v>147</v>
+      </c>
+      <c r="H85" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A86">
+        <v>85</v>
+      </c>
+      <c r="B86" t="s">
+        <v>47</v>
+      </c>
+      <c r="C86" t="s">
+        <v>6</v>
+      </c>
+      <c r="D86" t="b">
+        <v>1</v>
+      </c>
+      <c r="E86" t="b">
+        <v>1</v>
+      </c>
+      <c r="F86" t="s">
+        <v>148</v>
+      </c>
+      <c r="G86" t="s">
+        <v>149</v>
+      </c>
+      <c r="H86" t="str">
+        <f t="shared" si="2"/>
+        <v>![The Cosmos DB screen in the Azure Portal](figures/ch02/ch02_ss_cosmos_001_ann.png)</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A87">
+        <v>86</v>
+      </c>
+      <c r="B87" t="s">
+        <v>47</v>
+      </c>
+      <c r="C87" t="s">
+        <v>6</v>
+      </c>
+      <c r="D87" t="b">
+        <v>0</v>
+      </c>
+      <c r="E87" t="b">
+        <v>0</v>
+      </c>
+      <c r="F87" t="s">
+        <v>151</v>
+      </c>
+      <c r="H87" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A88">
+        <v>87</v>
+      </c>
+      <c r="B88" t="s">
+        <v>47</v>
+      </c>
+      <c r="C88" t="s">
+        <v>6</v>
+      </c>
+      <c r="D88" t="b">
+        <v>1</v>
+      </c>
+      <c r="E88" t="b">
+        <v>1</v>
+      </c>
+      <c r="F88" t="s">
+        <v>152</v>
+      </c>
+      <c r="G88" t="s">
+        <v>150</v>
+      </c>
+      <c r="H88" t="str">
+        <f t="shared" si="2"/>
+        <v>![Locating your Cosmos DB URI and Key](figures/ch02/ch02_ss_cosmos_002_ann.png)</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A89">
+        <v>88</v>
+      </c>
+      <c r="B89" t="s">
+        <v>47</v>
+      </c>
+      <c r="C89" t="s">
+        <v>6</v>
+      </c>
+      <c r="D89" t="b">
+        <v>0</v>
+      </c>
+      <c r="E89" t="b">
+        <v>0</v>
+      </c>
+      <c r="F89" t="s">
+        <v>153</v>
+      </c>
+      <c r="H89" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A90">
+        <v>89</v>
+      </c>
+      <c r="B90" t="s">
+        <v>47</v>
+      </c>
+      <c r="C90" t="s">
+        <v>6</v>
+      </c>
+      <c r="D90" t="b">
+        <v>1</v>
+      </c>
+      <c r="E90" t="b">
+        <v>1</v>
+      </c>
+      <c r="F90" t="s">
+        <v>154</v>
+      </c>
+      <c r="G90" t="s">
+        <v>155</v>
+      </c>
+      <c r="H90" t="str">
+        <f t="shared" si="2"/>
+        <v>![Adding another Tool to your Agent](figures/ch02/ch02_ss_cosmos_003_ann.png)</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A91">
+        <v>90</v>
+      </c>
+      <c r="B91" t="s">
+        <v>47</v>
+      </c>
+      <c r="C91" t="s">
+        <v>6</v>
+      </c>
+      <c r="D91" t="b">
+        <v>0</v>
+      </c>
+      <c r="E91" t="b">
+        <v>0</v>
+      </c>
+      <c r="F91" t="s">
+        <v>156</v>
+      </c>
+      <c r="H91" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A92">
+        <v>91</v>
+      </c>
+      <c r="B92" t="s">
+        <v>47</v>
+      </c>
+      <c r="C92" t="s">
+        <v>6</v>
+      </c>
+      <c r="D92" t="b">
+        <v>1</v>
+      </c>
+      <c r="E92" t="b">
+        <v>1</v>
+      </c>
+      <c r="F92" t="s">
+        <v>157</v>
+      </c>
+      <c r="G92" t="s">
+        <v>158</v>
+      </c>
+      <c r="H92" t="str">
+        <f t="shared" si="2"/>
+        <v>![Locating the Cosmos DB Tool in the Catalog](figures/ch02/ch02_ss_cosmos_004_ann.png)</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A93">
+        <v>92</v>
+      </c>
+      <c r="B93" t="s">
+        <v>47</v>
+      </c>
+      <c r="C93" t="s">
+        <v>6</v>
+      </c>
+      <c r="D93" t="b">
+        <v>0</v>
+      </c>
+      <c r="E93" t="b">
+        <v>0</v>
+      </c>
+      <c r="F93" t="s">
+        <v>159</v>
+      </c>
+      <c r="H93" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A94">
+        <v>93</v>
+      </c>
+      <c r="B94" t="s">
+        <v>47</v>
+      </c>
+      <c r="C94" t="s">
+        <v>6</v>
+      </c>
+      <c r="D94" t="b">
+        <v>1</v>
+      </c>
+      <c r="E94" t="b">
+        <v>1</v>
+      </c>
+      <c r="F94" t="s">
+        <v>160</v>
+      </c>
+      <c r="G94" t="s">
+        <v>167</v>
+      </c>
+      <c r="H94" t="str">
+        <f t="shared" si="2"/>
+        <v>![Information about hosting MCP servers](figures/ch02/ch02_ss_cosmos_005_ann.png)</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A95">
+        <v>94</v>
+      </c>
+      <c r="B95" t="s">
+        <v>47</v>
+      </c>
+      <c r="C95" t="s">
+        <v>6</v>
+      </c>
+      <c r="D95" t="b">
+        <v>0</v>
+      </c>
+      <c r="E95" t="b">
+        <v>0</v>
+      </c>
+      <c r="F95" t="s">
+        <v>161</v>
+      </c>
+      <c r="H95" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A96">
+        <v>95</v>
+      </c>
+      <c r="B96" t="s">
+        <v>47</v>
+      </c>
+      <c r="C96" t="s">
+        <v>6</v>
+      </c>
+      <c r="D96" t="b">
+        <v>1</v>
+      </c>
+      <c r="E96" t="b">
+        <v>1</v>
+      </c>
+      <c r="F96" t="s">
+        <v>162</v>
+      </c>
+      <c r="G96" t="s">
+        <v>163</v>
+      </c>
+      <c r="H96" t="str">
+        <f t="shared" si="2"/>
+        <v>![Filling in the URI and Key for the Cosmos DB Tool connection](figures/ch02/ch02_ss_cosmos_006_ann.png)</v>
+      </c>
+    </row>
+    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A97">
+        <v>96</v>
+      </c>
+      <c r="B97" t="s">
+        <v>47</v>
+      </c>
+      <c r="C97" t="s">
+        <v>6</v>
+      </c>
+      <c r="D97" t="b">
+        <v>0</v>
+      </c>
+      <c r="E97" t="b">
+        <v>0</v>
+      </c>
+      <c r="F97" t="s">
+        <v>164</v>
+      </c>
+      <c r="H97" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A98">
+        <v>97</v>
+      </c>
+      <c r="B98" t="s">
+        <v>47</v>
+      </c>
+      <c r="C98" t="s">
+        <v>6</v>
+      </c>
+      <c r="D98" t="b">
+        <v>1</v>
+      </c>
+      <c r="E98" t="b">
+        <v>1</v>
+      </c>
+      <c r="F98" t="s">
+        <v>165</v>
+      </c>
+      <c r="G98" t="s">
+        <v>166</v>
+      </c>
+      <c r="H98" t="str">
+        <f t="shared" si="2"/>
+        <v>![Checking that your Cosmos DB Tool is connected](figures/ch02/ch02_ss_cosmos_007_ann.png)</v>
+      </c>
+    </row>
+    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A99">
+        <v>98</v>
+      </c>
+      <c r="H99" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A100">
+        <v>99</v>
+      </c>
+      <c r="H100" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A101">
+        <v>100</v>
+      </c>
+      <c r="H101" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A102">
+        <v>101</v>
+      </c>
+      <c r="H102" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A103">
+        <v>102</v>
+      </c>
+      <c r="H103" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A104">
+        <v>103</v>
+      </c>
+      <c r="H104" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A105">
+        <v>104</v>
+      </c>
+      <c r="H105" t="str">
+        <f t="shared" si="2"/>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Ch02 Cosmos DB database creation figures
</commit_message>
<xml_diff>
--- a/figures/figure_inventory.xlsx
+++ b/figures/figure_inventory.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Colby\Documents\GitHub\foundry-book\figures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41807B75-0B1A-49C9-B17F-6BA433DE591C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E97F12B-A2E6-43DD-A21B-00429D59F5BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43965" yWindow="3885" windowWidth="24405" windowHeight="14265" xr2:uid="{222F1F68-60B1-49B9-BFF7-2C9CF743DB25}"/>
+    <workbookView xWindow="44955" yWindow="5895" windowWidth="24405" windowHeight="14265" xr2:uid="{222F1F68-60B1-49B9-BFF7-2C9CF743DB25}"/>
   </bookViews>
   <sheets>
     <sheet name="Figure Inventory" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="179">
   <si>
     <t>Chapter</t>
   </si>
@@ -540,6 +540,39 @@
   </si>
   <si>
     <t>Information about hosting MCP servers</t>
+  </si>
+  <si>
+    <t>ch02_ss_database_001_clean.png</t>
+  </si>
+  <si>
+    <t>ch02_ss_database_001_ann.png</t>
+  </si>
+  <si>
+    <t>Creating a new Cosmos DB container</t>
+  </si>
+  <si>
+    <t>ch02_ss_database_002_clean.png</t>
+  </si>
+  <si>
+    <t>ch02_ss_database_002_ann.png</t>
+  </si>
+  <si>
+    <t>Uploading property records to your database</t>
+  </si>
+  <si>
+    <t>Listing your property records</t>
+  </si>
+  <si>
+    <t>ch02_ss_database_003_clean.png</t>
+  </si>
+  <si>
+    <t>ch02_ss_database_003_ann.png</t>
+  </si>
+  <si>
+    <t>ch02_ss_database_004_clean.png</t>
+  </si>
+  <si>
+    <t>Creating a new Cosmos DB database</t>
   </si>
 </sst>
 </file>
@@ -3478,6 +3511,21 @@
       <c r="A99">
         <v>98</v>
       </c>
+      <c r="B99" t="s">
+        <v>47</v>
+      </c>
+      <c r="C99" t="s">
+        <v>6</v>
+      </c>
+      <c r="D99" t="b">
+        <v>0</v>
+      </c>
+      <c r="E99" t="b">
+        <v>0</v>
+      </c>
+      <c r="F99" t="s">
+        <v>168</v>
+      </c>
       <c r="H99" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -3487,15 +3535,48 @@
       <c r="A100">
         <v>99</v>
       </c>
+      <c r="B100" t="s">
+        <v>47</v>
+      </c>
+      <c r="C100" t="s">
+        <v>6</v>
+      </c>
+      <c r="D100" t="b">
+        <v>1</v>
+      </c>
+      <c r="E100" t="b">
+        <v>1</v>
+      </c>
+      <c r="F100" t="s">
+        <v>169</v>
+      </c>
+      <c r="G100" t="s">
+        <v>170</v>
+      </c>
       <c r="H100" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>![Creating a new Cosmos DB container](figures/ch02/ch02_ss_database_001_ann.png)</v>
       </c>
     </row>
     <row r="101" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>100</v>
       </c>
+      <c r="B101" t="s">
+        <v>47</v>
+      </c>
+      <c r="C101" t="s">
+        <v>6</v>
+      </c>
+      <c r="D101" t="b">
+        <v>0</v>
+      </c>
+      <c r="E101" t="b">
+        <v>0</v>
+      </c>
+      <c r="F101" t="s">
+        <v>171</v>
+      </c>
       <c r="H101" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -3505,15 +3586,48 @@
       <c r="A102">
         <v>101</v>
       </c>
+      <c r="B102" t="s">
+        <v>47</v>
+      </c>
+      <c r="C102" t="s">
+        <v>6</v>
+      </c>
+      <c r="D102" t="b">
+        <v>1</v>
+      </c>
+      <c r="E102" t="b">
+        <v>1</v>
+      </c>
+      <c r="F102" t="s">
+        <v>172</v>
+      </c>
+      <c r="G102" t="s">
+        <v>178</v>
+      </c>
       <c r="H102" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>![Creating a new Cosmos DB database](figures/ch02/ch02_ss_database_002_ann.png)</v>
       </c>
     </row>
     <row r="103" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>102</v>
       </c>
+      <c r="B103" t="s">
+        <v>47</v>
+      </c>
+      <c r="C103" t="s">
+        <v>6</v>
+      </c>
+      <c r="D103" t="b">
+        <v>0</v>
+      </c>
+      <c r="E103" t="b">
+        <v>0</v>
+      </c>
+      <c r="F103" t="s">
+        <v>175</v>
+      </c>
       <c r="H103" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -3523,18 +3637,54 @@
       <c r="A104">
         <v>103</v>
       </c>
+      <c r="B104" t="s">
+        <v>47</v>
+      </c>
+      <c r="C104" t="s">
+        <v>6</v>
+      </c>
+      <c r="D104" t="b">
+        <v>1</v>
+      </c>
+      <c r="E104" t="b">
+        <v>1</v>
+      </c>
+      <c r="F104" t="s">
+        <v>176</v>
+      </c>
+      <c r="G104" t="s">
+        <v>173</v>
+      </c>
       <c r="H104" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>![Uploading property records to your database](figures/ch02/ch02_ss_database_003_ann.png)</v>
       </c>
     </row>
     <row r="105" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>104</v>
       </c>
+      <c r="B105" t="s">
+        <v>47</v>
+      </c>
+      <c r="C105" t="s">
+        <v>6</v>
+      </c>
+      <c r="D105" t="b">
+        <v>0</v>
+      </c>
+      <c r="E105" t="b">
+        <v>1</v>
+      </c>
+      <c r="F105" t="s">
+        <v>177</v>
+      </c>
+      <c r="G105" t="s">
+        <v>174</v>
+      </c>
       <c r="H105" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>![Listing your property records](figures/ch02/ch02_ss_database_004_clean.png)</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add MCP server deployment figures to Ch02
</commit_message>
<xml_diff>
--- a/figures/figure_inventory.xlsx
+++ b/figures/figure_inventory.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Colby\Documents\GitHub\foundry-book\figures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E97F12B-A2E6-43DD-A21B-00429D59F5BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D02A8C30-02DE-4B87-87C6-56029AED7B8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="44955" yWindow="5895" windowWidth="24405" windowHeight="14265" xr2:uid="{222F1F68-60B1-49B9-BFF7-2C9CF743DB25}"/>
+    <workbookView xWindow="42180" yWindow="6435" windowWidth="27645" windowHeight="14265" xr2:uid="{222F1F68-60B1-49B9-BFF7-2C9CF743DB25}"/>
   </bookViews>
   <sheets>
     <sheet name="Figure Inventory" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="424" uniqueCount="197">
   <si>
     <t>Chapter</t>
   </si>
@@ -527,9 +527,6 @@
     <t>ch02_ss_cosmos_006_ann.png</t>
   </si>
   <si>
-    <t>Filling in the URI and Key for the Cosmos DB Tool connection</t>
-  </si>
-  <si>
     <t>ch02_ss_cosmos_007_clean.png</t>
   </si>
   <si>
@@ -573,6 +570,63 @@
   </si>
   <si>
     <t>Creating a new Cosmos DB database</t>
+  </si>
+  <si>
+    <t>ch02_ss_mcp_001_clean.png</t>
+  </si>
+  <si>
+    <t>ch02_ss_mcp_002_clean.png</t>
+  </si>
+  <si>
+    <t>Selecting your Subscription and Resource Group in the azd prompt</t>
+  </si>
+  <si>
+    <t>azd has successfully deployed the resources</t>
+  </si>
+  <si>
+    <t>Successful deployment of the MCP Toolkit</t>
+  </si>
+  <si>
+    <t>ch02_ss_mcp_003_clean.png</t>
+  </si>
+  <si>
+    <t>ch02_ss_mcp_003_ann.png</t>
+  </si>
+  <si>
+    <t>ch02_ss_mcp_004_clean.png</t>
+  </si>
+  <si>
+    <t>ch02_ss_mcp_004_ann.png</t>
+  </si>
+  <si>
+    <t>Authenticating the MCP Toolkit with your Tenant and Entra App IDs</t>
+  </si>
+  <si>
+    <t>ch02_ss_mcp_005_clean.png</t>
+  </si>
+  <si>
+    <t>ch02_ss_mcp_005_ann.png</t>
+  </si>
+  <si>
+    <t>Granting permissions to the MCP Toolkit app</t>
+  </si>
+  <si>
+    <t>ch02_ss_mcp_006_clean.png</t>
+  </si>
+  <si>
+    <t>ch02_ss_mcp_006_ann.png</t>
+  </si>
+  <si>
+    <t>Successful authentication to the MCP Toolkit app</t>
+  </si>
+  <si>
+    <t>Filling in the URI and authentication for the Cosmos DB Tool connection</t>
+  </si>
+  <si>
+    <t>ch02_ss_cosmos_008_clean.png</t>
+  </si>
+  <si>
+    <t>Checking the Cosmos DB Tool usage in the Agent response</t>
   </si>
 </sst>
 </file>
@@ -961,16 +1015,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B464DFF5-94DA-41E0-B03E-143380050964}">
-  <dimension ref="A1:H105"/>
+  <dimension ref="A1:H116"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11" customWidth="1"/>
+    <col min="5" max="5" width="6.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="34.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="43.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="97.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="51.5703125" customWidth="1"/>
+    <col min="8" max="8" width="108.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -2783,7 +2838,7 @@
         <v>122</v>
       </c>
       <c r="H70" t="str">
-        <f t="shared" ref="H70:H105" si="2">IF(E70,_xlfn.CONCAT("![",G70,"](figures/",B70,"/",F70,")"),"")</f>
+        <f t="shared" ref="H70:H116" si="2">IF(E70,_xlfn.CONCAT("![",G70,"](figures/",B70,"/",F70,")"),"")</f>
         <v/>
       </c>
     </row>
@@ -3164,14 +3219,17 @@
         <v>0</v>
       </c>
       <c r="E85" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F85" t="s">
-        <v>147</v>
+        <v>178</v>
+      </c>
+      <c r="G85" t="s">
+        <v>180</v>
       </c>
       <c r="H85" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>![Selecting your Subscription and Resource Group in the azd prompt](figures/ch02/ch02_ss_mcp_001_clean.png)</v>
       </c>
     </row>
     <row r="86" spans="1:8" x14ac:dyDescent="0.25">
@@ -3185,20 +3243,20 @@
         <v>6</v>
       </c>
       <c r="D86" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E86" t="b">
         <v>1</v>
       </c>
       <c r="F86" t="s">
-        <v>148</v>
+        <v>179</v>
       </c>
       <c r="G86" t="s">
-        <v>149</v>
+        <v>181</v>
       </c>
       <c r="H86" t="str">
-        <f t="shared" si="2"/>
-        <v>![The Cosmos DB screen in the Azure Portal](figures/ch02/ch02_ss_cosmos_001_ann.png)</v>
+        <f>IF(E86,_xlfn.CONCAT("![",G86,"](figures/",B86,"/",F86,")"),"")</f>
+        <v>![azd has successfully deployed the resources](figures/ch02/ch02_ss_mcp_002_clean.png)</v>
       </c>
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.25">
@@ -3218,10 +3276,10 @@
         <v>0</v>
       </c>
       <c r="F87" t="s">
-        <v>151</v>
+        <v>183</v>
       </c>
       <c r="H87" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="H87:H95" si="3">IF(E87,_xlfn.CONCAT("![",G87,"](figures/",B87,"/",F87,")"),"")</f>
         <v/>
       </c>
     </row>
@@ -3242,14 +3300,14 @@
         <v>1</v>
       </c>
       <c r="F88" t="s">
-        <v>152</v>
+        <v>184</v>
       </c>
       <c r="G88" t="s">
-        <v>150</v>
+        <v>182</v>
       </c>
       <c r="H88" t="str">
-        <f t="shared" si="2"/>
-        <v>![Locating your Cosmos DB URI and Key](figures/ch02/ch02_ss_cosmos_002_ann.png)</v>
+        <f t="shared" si="3"/>
+        <v>![Successful deployment of the MCP Toolkit](figures/ch02/ch02_ss_mcp_003_ann.png)</v>
       </c>
     </row>
     <row r="89" spans="1:8" x14ac:dyDescent="0.25">
@@ -3269,10 +3327,10 @@
         <v>0</v>
       </c>
       <c r="F89" t="s">
-        <v>153</v>
+        <v>185</v>
       </c>
       <c r="H89" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -3293,14 +3351,14 @@
         <v>1</v>
       </c>
       <c r="F90" t="s">
-        <v>154</v>
+        <v>186</v>
       </c>
       <c r="G90" t="s">
-        <v>155</v>
+        <v>187</v>
       </c>
       <c r="H90" t="str">
-        <f t="shared" si="2"/>
-        <v>![Adding another Tool to your Agent](figures/ch02/ch02_ss_cosmos_003_ann.png)</v>
+        <f t="shared" si="3"/>
+        <v>![Authenticating the MCP Toolkit with your Tenant and Entra App IDs](figures/ch02/ch02_ss_mcp_004_ann.png)</v>
       </c>
     </row>
     <row r="91" spans="1:8" x14ac:dyDescent="0.25">
@@ -3320,10 +3378,10 @@
         <v>0</v>
       </c>
       <c r="F91" t="s">
-        <v>156</v>
+        <v>188</v>
       </c>
       <c r="H91" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -3344,14 +3402,14 @@
         <v>1</v>
       </c>
       <c r="F92" t="s">
-        <v>157</v>
+        <v>189</v>
       </c>
       <c r="G92" t="s">
-        <v>158</v>
+        <v>190</v>
       </c>
       <c r="H92" t="str">
-        <f t="shared" si="2"/>
-        <v>![Locating the Cosmos DB Tool in the Catalog](figures/ch02/ch02_ss_cosmos_004_ann.png)</v>
+        <f t="shared" si="3"/>
+        <v>![Granting permissions to the MCP Toolkit app](figures/ch02/ch02_ss_mcp_005_ann.png)</v>
       </c>
     </row>
     <row r="93" spans="1:8" x14ac:dyDescent="0.25">
@@ -3371,10 +3429,10 @@
         <v>0</v>
       </c>
       <c r="F93" t="s">
-        <v>159</v>
+        <v>191</v>
       </c>
       <c r="H93" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -3395,14 +3453,14 @@
         <v>1</v>
       </c>
       <c r="F94" t="s">
-        <v>160</v>
+        <v>192</v>
       </c>
       <c r="G94" t="s">
-        <v>167</v>
+        <v>193</v>
       </c>
       <c r="H94" t="str">
-        <f t="shared" si="2"/>
-        <v>![Information about hosting MCP servers](figures/ch02/ch02_ss_cosmos_005_ann.png)</v>
+        <f t="shared" si="3"/>
+        <v>![Successful authentication to the MCP Toolkit app](figures/ch02/ch02_ss_mcp_006_ann.png)</v>
       </c>
     </row>
     <row r="95" spans="1:8" x14ac:dyDescent="0.25">
@@ -3422,10 +3480,10 @@
         <v>0</v>
       </c>
       <c r="F95" t="s">
-        <v>161</v>
+        <v>147</v>
       </c>
       <c r="H95" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -3446,14 +3504,14 @@
         <v>1</v>
       </c>
       <c r="F96" t="s">
-        <v>162</v>
+        <v>148</v>
       </c>
       <c r="G96" t="s">
-        <v>163</v>
+        <v>149</v>
       </c>
       <c r="H96" t="str">
         <f t="shared" si="2"/>
-        <v>![Filling in the URI and Key for the Cosmos DB Tool connection](figures/ch02/ch02_ss_cosmos_006_ann.png)</v>
+        <v>![The Cosmos DB screen in the Azure Portal](figures/ch02/ch02_ss_cosmos_001_ann.png)</v>
       </c>
     </row>
     <row r="97" spans="1:8" x14ac:dyDescent="0.25">
@@ -3473,7 +3531,7 @@
         <v>0</v>
       </c>
       <c r="F97" t="s">
-        <v>164</v>
+        <v>151</v>
       </c>
       <c r="H97" t="str">
         <f t="shared" si="2"/>
@@ -3497,14 +3555,14 @@
         <v>1</v>
       </c>
       <c r="F98" t="s">
-        <v>165</v>
+        <v>152</v>
       </c>
       <c r="G98" t="s">
-        <v>166</v>
+        <v>150</v>
       </c>
       <c r="H98" t="str">
         <f t="shared" si="2"/>
-        <v>![Checking that your Cosmos DB Tool is connected](figures/ch02/ch02_ss_cosmos_007_ann.png)</v>
+        <v>![Locating your Cosmos DB URI and Key](figures/ch02/ch02_ss_cosmos_002_ann.png)</v>
       </c>
     </row>
     <row r="99" spans="1:8" x14ac:dyDescent="0.25">
@@ -3524,7 +3582,7 @@
         <v>0</v>
       </c>
       <c r="F99" t="s">
-        <v>168</v>
+        <v>153</v>
       </c>
       <c r="H99" t="str">
         <f t="shared" si="2"/>
@@ -3548,14 +3606,14 @@
         <v>1</v>
       </c>
       <c r="F100" t="s">
-        <v>169</v>
+        <v>154</v>
       </c>
       <c r="G100" t="s">
-        <v>170</v>
+        <v>155</v>
       </c>
       <c r="H100" t="str">
         <f t="shared" si="2"/>
-        <v>![Creating a new Cosmos DB container](figures/ch02/ch02_ss_database_001_ann.png)</v>
+        <v>![Adding another Tool to your Agent](figures/ch02/ch02_ss_cosmos_003_ann.png)</v>
       </c>
     </row>
     <row r="101" spans="1:8" x14ac:dyDescent="0.25">
@@ -3575,7 +3633,7 @@
         <v>0</v>
       </c>
       <c r="F101" t="s">
-        <v>171</v>
+        <v>156</v>
       </c>
       <c r="H101" t="str">
         <f t="shared" si="2"/>
@@ -3599,14 +3657,14 @@
         <v>1</v>
       </c>
       <c r="F102" t="s">
-        <v>172</v>
+        <v>157</v>
       </c>
       <c r="G102" t="s">
-        <v>178</v>
+        <v>158</v>
       </c>
       <c r="H102" t="str">
         <f t="shared" si="2"/>
-        <v>![Creating a new Cosmos DB database](figures/ch02/ch02_ss_database_002_ann.png)</v>
+        <v>![Locating the Cosmos DB Tool in the Catalog](figures/ch02/ch02_ss_cosmos_004_ann.png)</v>
       </c>
     </row>
     <row r="103" spans="1:8" x14ac:dyDescent="0.25">
@@ -3626,7 +3684,7 @@
         <v>0</v>
       </c>
       <c r="F103" t="s">
-        <v>175</v>
+        <v>159</v>
       </c>
       <c r="H103" t="str">
         <f t="shared" si="2"/>
@@ -3650,14 +3708,14 @@
         <v>1</v>
       </c>
       <c r="F104" t="s">
-        <v>176</v>
+        <v>160</v>
       </c>
       <c r="G104" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="H104" t="str">
         <f t="shared" si="2"/>
-        <v>![Uploading property records to your database](figures/ch02/ch02_ss_database_003_ann.png)</v>
+        <v>![Information about hosting MCP servers](figures/ch02/ch02_ss_cosmos_005_ann.png)</v>
       </c>
     </row>
     <row r="105" spans="1:8" x14ac:dyDescent="0.25">
@@ -3674,15 +3732,297 @@
         <v>0</v>
       </c>
       <c r="E105" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F105" t="s">
+        <v>161</v>
+      </c>
+      <c r="H105" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A106">
+        <v>105</v>
+      </c>
+      <c r="B106" t="s">
+        <v>47</v>
+      </c>
+      <c r="C106" t="s">
+        <v>6</v>
+      </c>
+      <c r="D106" t="b">
+        <v>1</v>
+      </c>
+      <c r="E106" t="b">
+        <v>1</v>
+      </c>
+      <c r="F106" t="s">
+        <v>162</v>
+      </c>
+      <c r="G106" t="s">
+        <v>194</v>
+      </c>
+      <c r="H106" t="str">
+        <f t="shared" si="2"/>
+        <v>![Filling in the URI and authentication for the Cosmos DB Tool connection](figures/ch02/ch02_ss_cosmos_006_ann.png)</v>
+      </c>
+    </row>
+    <row r="107" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A107">
+        <v>106</v>
+      </c>
+      <c r="B107" t="s">
+        <v>47</v>
+      </c>
+      <c r="C107" t="s">
+        <v>6</v>
+      </c>
+      <c r="D107" t="b">
+        <v>0</v>
+      </c>
+      <c r="E107" t="b">
+        <v>0</v>
+      </c>
+      <c r="F107" t="s">
+        <v>163</v>
+      </c>
+      <c r="H107" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="108" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A108">
+        <v>107</v>
+      </c>
+      <c r="B108" t="s">
+        <v>47</v>
+      </c>
+      <c r="C108" t="s">
+        <v>6</v>
+      </c>
+      <c r="D108" t="b">
+        <v>1</v>
+      </c>
+      <c r="E108" t="b">
+        <v>1</v>
+      </c>
+      <c r="F108" t="s">
+        <v>164</v>
+      </c>
+      <c r="G108" t="s">
+        <v>165</v>
+      </c>
+      <c r="H108" t="str">
+        <f t="shared" si="2"/>
+        <v>![Checking that your Cosmos DB Tool is connected](figures/ch02/ch02_ss_cosmos_007_ann.png)</v>
+      </c>
+    </row>
+    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A109">
+        <v>108</v>
+      </c>
+      <c r="B109" t="s">
+        <v>47</v>
+      </c>
+      <c r="C109" t="s">
+        <v>6</v>
+      </c>
+      <c r="D109" t="b">
+        <v>0</v>
+      </c>
+      <c r="E109" t="b">
+        <v>1</v>
+      </c>
+      <c r="F109" t="s">
+        <v>195</v>
+      </c>
+      <c r="G109" t="s">
+        <v>196</v>
+      </c>
+      <c r="H109" t="str">
+        <f t="shared" si="2"/>
+        <v>![Checking the Cosmos DB Tool usage in the Agent response](figures/ch02/ch02_ss_cosmos_008_clean.png)</v>
+      </c>
+    </row>
+    <row r="110" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A110">
+        <v>109</v>
+      </c>
+      <c r="B110" t="s">
+        <v>47</v>
+      </c>
+      <c r="C110" t="s">
+        <v>6</v>
+      </c>
+      <c r="D110" t="b">
+        <v>0</v>
+      </c>
+      <c r="E110" t="b">
+        <v>0</v>
+      </c>
+      <c r="F110" t="s">
+        <v>167</v>
+      </c>
+      <c r="H110" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="111" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A111">
+        <v>110</v>
+      </c>
+      <c r="B111" t="s">
+        <v>47</v>
+      </c>
+      <c r="C111" t="s">
+        <v>6</v>
+      </c>
+      <c r="D111" t="b">
+        <v>1</v>
+      </c>
+      <c r="E111" t="b">
+        <v>1</v>
+      </c>
+      <c r="F111" t="s">
+        <v>168</v>
+      </c>
+      <c r="G111" t="s">
+        <v>169</v>
+      </c>
+      <c r="H111" t="str">
+        <f t="shared" si="2"/>
+        <v>![Creating a new Cosmos DB container](figures/ch02/ch02_ss_database_001_ann.png)</v>
+      </c>
+    </row>
+    <row r="112" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A112">
+        <v>111</v>
+      </c>
+      <c r="B112" t="s">
+        <v>47</v>
+      </c>
+      <c r="C112" t="s">
+        <v>6</v>
+      </c>
+      <c r="D112" t="b">
+        <v>0</v>
+      </c>
+      <c r="E112" t="b">
+        <v>0</v>
+      </c>
+      <c r="F112" t="s">
+        <v>170</v>
+      </c>
+      <c r="H112" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="113" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A113">
+        <v>112</v>
+      </c>
+      <c r="B113" t="s">
+        <v>47</v>
+      </c>
+      <c r="C113" t="s">
+        <v>6</v>
+      </c>
+      <c r="D113" t="b">
+        <v>1</v>
+      </c>
+      <c r="E113" t="b">
+        <v>1</v>
+      </c>
+      <c r="F113" t="s">
+        <v>171</v>
+      </c>
+      <c r="G113" t="s">
         <v>177</v>
       </c>
-      <c r="G105" t="s">
+      <c r="H113" t="str">
+        <f t="shared" si="2"/>
+        <v>![Creating a new Cosmos DB database](figures/ch02/ch02_ss_database_002_ann.png)</v>
+      </c>
+    </row>
+    <row r="114" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A114">
+        <v>113</v>
+      </c>
+      <c r="B114" t="s">
+        <v>47</v>
+      </c>
+      <c r="C114" t="s">
+        <v>6</v>
+      </c>
+      <c r="D114" t="b">
+        <v>0</v>
+      </c>
+      <c r="E114" t="b">
+        <v>0</v>
+      </c>
+      <c r="F114" t="s">
         <v>174</v>
       </c>
-      <c r="H105" t="str">
+      <c r="H114" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="115" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A115">
+        <v>114</v>
+      </c>
+      <c r="B115" t="s">
+        <v>47</v>
+      </c>
+      <c r="C115" t="s">
+        <v>6</v>
+      </c>
+      <c r="D115" t="b">
+        <v>1</v>
+      </c>
+      <c r="E115" t="b">
+        <v>1</v>
+      </c>
+      <c r="F115" t="s">
+        <v>175</v>
+      </c>
+      <c r="G115" t="s">
+        <v>172</v>
+      </c>
+      <c r="H115" t="str">
+        <f t="shared" si="2"/>
+        <v>![Uploading property records to your database](figures/ch02/ch02_ss_database_003_ann.png)</v>
+      </c>
+    </row>
+    <row r="116" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A116">
+        <v>115</v>
+      </c>
+      <c r="B116" t="s">
+        <v>47</v>
+      </c>
+      <c r="C116" t="s">
+        <v>6</v>
+      </c>
+      <c r="D116" t="b">
+        <v>0</v>
+      </c>
+      <c r="E116" t="b">
+        <v>1</v>
+      </c>
+      <c r="F116" t="s">
+        <v>176</v>
+      </c>
+      <c r="G116" t="s">
+        <v>173</v>
+      </c>
+      <c r="H116" t="str">
         <f t="shared" si="2"/>
         <v>![Listing your property records](figures/ch02/ch02_ss_database_004_clean.png)</v>
       </c>

</xml_diff>

<commit_message>
Migrate model deployment figures from Ch02 folder to Ch01
</commit_message>
<xml_diff>
--- a/figures/figure_inventory.xlsx
+++ b/figures/figure_inventory.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Colby\Documents\GitHub\foundry-book\figures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D02A8C30-02DE-4B87-87C6-56029AED7B8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BD3A053-2DFB-416A-9066-2159A569004E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="42180" yWindow="6435" windowWidth="27645" windowHeight="14265" xr2:uid="{222F1F68-60B1-49B9-BFF7-2C9CF743DB25}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{222F1F68-60B1-49B9-BFF7-2C9CF743DB25}"/>
   </bookViews>
   <sheets>
     <sheet name="Figure Inventory" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="424" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="200">
   <si>
     <t>Chapter</t>
   </si>
@@ -185,33 +185,12 @@
     <t>Locating the Discover tab</t>
   </si>
   <si>
-    <t>ch02_ss_portal_001_clean.png</t>
-  </si>
-  <si>
-    <t>ch02_ss_portal_001_ann.png</t>
-  </si>
-  <si>
-    <t>ch02_ss_discover_001_clean.png</t>
-  </si>
-  <si>
-    <t>ch02_ss_discover_001_ann.png</t>
-  </si>
-  <si>
-    <t>ch02_ss_discover_002_clean.png</t>
-  </si>
-  <si>
     <t>Exploring featured models on the Discover page</t>
   </si>
   <si>
     <t>Listing all available models in Foundry</t>
   </si>
   <si>
-    <t>ch02_ss_compare_002_clean.png</t>
-  </si>
-  <si>
-    <t>ch02_ss_compare_001_ann.png</t>
-  </si>
-  <si>
     <t>Locating the Compare models button</t>
   </si>
   <si>
@@ -221,84 +200,36 @@
     <t>Locating the View leaderboard button</t>
   </si>
   <si>
-    <t>ch02_ss_leaderboard_001_ann.png</t>
-  </si>
-  <si>
     <t>ID</t>
   </si>
   <si>
     <t>Exploring the model leaderboard</t>
   </si>
   <si>
-    <t>ch02_ss_leaderboard_002_clean.png</t>
-  </si>
-  <si>
-    <t>ch02_ss_leaderboard_003_ann.png</t>
-  </si>
-  <si>
     <t>More details about a model's benchmark performance</t>
   </si>
   <si>
-    <t>ch02_ss_leaderboard_004_clean.png</t>
-  </si>
-  <si>
     <t>Metric details across various model benchmarks</t>
   </si>
   <si>
-    <t>ch02_ss_deploy_001_ann.png</t>
-  </si>
-  <si>
     <t>Searching for the Phi-4 model</t>
   </si>
   <si>
-    <t>ch02_ss_deploy_001_clean.png</t>
-  </si>
-  <si>
     <t>Deploying Phi-4 with Default settings</t>
   </si>
   <si>
-    <t>ch02_ss_deploy_002_clean.png</t>
-  </si>
-  <si>
-    <t>ch02_ss_deploy_002_ann.png</t>
-  </si>
-  <si>
-    <t>ch02_ss_deploy_003_clean.png</t>
-  </si>
-  <si>
-    <t>ch02_ss_deploy_003_ann.png</t>
-  </si>
-  <si>
     <t>Agreeing to the terms for deploying Phi-4</t>
   </si>
   <si>
     <t>Playground UI for experimenting with a Phi-4 deployment</t>
   </si>
   <si>
-    <t>ch02_ss_deploy_004_clean.png</t>
-  </si>
-  <si>
     <t>Learning to make intergalactic pizza</t>
   </si>
   <si>
-    <t>ch02_ss_deploy_005_clean.png</t>
-  </si>
-  <si>
     <t>Deployment endpoint and key on the Details tab</t>
   </si>
   <si>
-    <t>ch02_ss_deploy_006_ann.png</t>
-  </si>
-  <si>
-    <t>ch02_ss_deploy_006_clean.png</t>
-  </si>
-  <si>
-    <t>ch02_ss_deploy_007_ann.png</t>
-  </si>
-  <si>
-    <t>ch02_ss_deploy_007_clean.png</t>
-  </si>
-  <si>
     <t>Modifying model parameters</t>
   </si>
   <si>
@@ -627,6 +558,84 @@
   </si>
   <si>
     <t>Checking the Cosmos DB Tool usage in the Agent response</t>
+  </si>
+  <si>
+    <t>ch02_ss_cosmos_008_ann.png</t>
+  </si>
+  <si>
+    <t>ch02_ss_cosmos_009_clean.png</t>
+  </si>
+  <si>
+    <t>A successful Cosmos DB Tool call and augmented Agent response</t>
+  </si>
+  <si>
+    <t>ch01_ss_portal_013_clean.png</t>
+  </si>
+  <si>
+    <t>ch01_ss_portal_013_ann.png</t>
+  </si>
+  <si>
+    <t>ch01_ss_discover_001_clean.png</t>
+  </si>
+  <si>
+    <t>ch01_ss_discover_001_ann.png</t>
+  </si>
+  <si>
+    <t>ch01_ss_discover_002_clean.png</t>
+  </si>
+  <si>
+    <t>ch01_ss_compare_001_ann.png</t>
+  </si>
+  <si>
+    <t>ch01_ss_compare_002_clean.png</t>
+  </si>
+  <si>
+    <t>ch01_ss_leaderboard_001_ann.png</t>
+  </si>
+  <si>
+    <t>ch01_ss_leaderboard_002_clean.png</t>
+  </si>
+  <si>
+    <t>ch01_ss_leaderboard_003_ann.png</t>
+  </si>
+  <si>
+    <t>ch01_ss_leaderboard_004_clean.png</t>
+  </si>
+  <si>
+    <t>ch01_ss_deploy_001_clean.png</t>
+  </si>
+  <si>
+    <t>ch01_ss_deploy_001_ann.png</t>
+  </si>
+  <si>
+    <t>ch01_ss_deploy_002_clean.png</t>
+  </si>
+  <si>
+    <t>ch01_ss_deploy_002_ann.png</t>
+  </si>
+  <si>
+    <t>ch01_ss_deploy_003_clean.png</t>
+  </si>
+  <si>
+    <t>ch01_ss_deploy_003_ann.png</t>
+  </si>
+  <si>
+    <t>ch01_ss_deploy_004_clean.png</t>
+  </si>
+  <si>
+    <t>ch01_ss_deploy_005_clean.png</t>
+  </si>
+  <si>
+    <t>ch01_ss_deploy_006_clean.png</t>
+  </si>
+  <si>
+    <t>ch01_ss_deploy_006_ann.png</t>
+  </si>
+  <si>
+    <t>ch01_ss_deploy_007_clean.png</t>
+  </si>
+  <si>
+    <t>ch01_ss_deploy_007_ann.png</t>
   </si>
 </sst>
 </file>
@@ -1015,7 +1024,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B464DFF5-94DA-41E0-B03E-143380050964}">
-  <dimension ref="A1:H116"/>
+  <dimension ref="A1:H118"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1030,7 +1039,7 @@
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -1071,7 +1080,7 @@
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>146</v>
+        <v>123</v>
       </c>
       <c r="G2" t="s">
         <v>31</v>
@@ -1653,7 +1662,7 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="C25" t="s">
         <v>6</v>
@@ -1665,7 +1674,7 @@
         <v>0</v>
       </c>
       <c r="F25" t="s">
-        <v>49</v>
+        <v>177</v>
       </c>
       <c r="H25" t="str">
         <f t="shared" si="0"/>
@@ -1677,7 +1686,7 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="C26" t="s">
         <v>6</v>
@@ -1689,14 +1698,14 @@
         <v>1</v>
       </c>
       <c r="F26" t="s">
-        <v>50</v>
+        <v>178</v>
       </c>
       <c r="G26" t="s">
         <v>48</v>
       </c>
       <c r="H26" t="str">
         <f>IF(E26,_xlfn.CONCAT("![",G26,"](figures/",B26,"/",F26,")"),"")</f>
-        <v>![Locating the Discover tab](figures/ch02/ch02_ss_portal_001_ann.png)</v>
+        <v>![Locating the Discover tab](figures/ch01/ch01_ss_portal_013_ann.png)</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
@@ -1704,7 +1713,7 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="C27" t="s">
         <v>6</v>
@@ -1716,7 +1725,7 @@
         <v>0</v>
       </c>
       <c r="F27" t="s">
-        <v>51</v>
+        <v>179</v>
       </c>
       <c r="H27" t="str">
         <f t="shared" ref="H27:H64" si="1">IF(E27,_xlfn.CONCAT("![",G27,"](figures/",B27,"/",F27,")"),"")</f>
@@ -1728,7 +1737,7 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="C28" t="s">
         <v>6</v>
@@ -1740,14 +1749,14 @@
         <v>1</v>
       </c>
       <c r="F28" t="s">
-        <v>52</v>
+        <v>180</v>
       </c>
       <c r="G28" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="H28" t="str">
         <f t="shared" si="1"/>
-        <v>![Exploring featured models on the Discover page](figures/ch02/ch02_ss_discover_001_ann.png)</v>
+        <v>![Exploring featured models on the Discover page](figures/ch01/ch01_ss_discover_001_ann.png)</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
@@ -1755,7 +1764,7 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="C29" t="s">
         <v>6</v>
@@ -1767,14 +1776,14 @@
         <v>1</v>
       </c>
       <c r="F29" t="s">
-        <v>53</v>
+        <v>181</v>
       </c>
       <c r="G29" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="H29" t="str">
         <f t="shared" si="1"/>
-        <v>![Listing all available models in Foundry](figures/ch02/ch02_ss_discover_002_clean.png)</v>
+        <v>![Listing all available models in Foundry](figures/ch01/ch01_ss_discover_002_clean.png)</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
@@ -1782,7 +1791,7 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="C30" t="s">
         <v>6</v>
@@ -1794,14 +1803,14 @@
         <v>1</v>
       </c>
       <c r="F30" t="s">
-        <v>57</v>
+        <v>182</v>
       </c>
       <c r="G30" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="H30" t="str">
         <f t="shared" si="1"/>
-        <v>![Locating the Compare models button](figures/ch02/ch02_ss_compare_001_ann.png)</v>
+        <v>![Locating the Compare models button](figures/ch01/ch01_ss_compare_001_ann.png)</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
@@ -1809,7 +1818,7 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="C31" t="s">
         <v>6</v>
@@ -1821,14 +1830,14 @@
         <v>1</v>
       </c>
       <c r="F31" t="s">
-        <v>56</v>
+        <v>183</v>
       </c>
       <c r="G31" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="H31" t="str">
         <f t="shared" si="1"/>
-        <v>![Comparing models across benchmarks and capabilities](figures/ch02/ch02_ss_compare_002_clean.png)</v>
+        <v>![Comparing models across benchmarks and capabilities](figures/ch01/ch01_ss_compare_002_clean.png)</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
@@ -1836,7 +1845,7 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="C32" t="s">
         <v>6</v>
@@ -1848,14 +1857,14 @@
         <v>1</v>
       </c>
       <c r="F32" t="s">
-        <v>61</v>
+        <v>184</v>
       </c>
       <c r="G32" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="H32" t="str">
         <f t="shared" si="1"/>
-        <v>![Locating the View leaderboard button](figures/ch02/ch02_ss_leaderboard_001_ann.png)</v>
+        <v>![Locating the View leaderboard button](figures/ch01/ch01_ss_leaderboard_001_ann.png)</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
@@ -1863,7 +1872,7 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="C33" t="s">
         <v>6</v>
@@ -1875,14 +1884,14 @@
         <v>1</v>
       </c>
       <c r="F33" t="s">
-        <v>64</v>
+        <v>185</v>
       </c>
       <c r="G33" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="H33" t="str">
         <f t="shared" si="1"/>
-        <v>![Exploring the model leaderboard](figures/ch02/ch02_ss_leaderboard_002_clean.png)</v>
+        <v>![Exploring the model leaderboard](figures/ch01/ch01_ss_leaderboard_002_clean.png)</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
@@ -1890,7 +1899,7 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="C34" t="s">
         <v>6</v>
@@ -1902,7 +1911,7 @@
         <v>0</v>
       </c>
       <c r="F34" t="s">
-        <v>64</v>
+        <v>185</v>
       </c>
       <c r="H34" t="str">
         <f t="shared" si="1"/>
@@ -1914,7 +1923,7 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="C35" t="s">
         <v>6</v>
@@ -1926,14 +1935,14 @@
         <v>1</v>
       </c>
       <c r="F35" t="s">
-        <v>65</v>
+        <v>186</v>
       </c>
       <c r="G35" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="H35" t="str">
         <f t="shared" si="1"/>
-        <v>![More details about a model's benchmark performance](figures/ch02/ch02_ss_leaderboard_003_ann.png)</v>
+        <v>![More details about a model's benchmark performance](figures/ch01/ch01_ss_leaderboard_003_ann.png)</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
@@ -1941,7 +1950,7 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="C36" t="s">
         <v>6</v>
@@ -1953,14 +1962,14 @@
         <v>1</v>
       </c>
       <c r="F36" t="s">
-        <v>67</v>
+        <v>187</v>
       </c>
       <c r="G36" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="H36" t="str">
         <f t="shared" si="1"/>
-        <v>![Metric details across various model benchmarks](figures/ch02/ch02_ss_leaderboard_004_clean.png)</v>
+        <v>![Metric details across various model benchmarks](figures/ch01/ch01_ss_leaderboard_004_clean.png)</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
@@ -1968,7 +1977,7 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="C37" t="s">
         <v>6</v>
@@ -1980,7 +1989,7 @@
         <v>0</v>
       </c>
       <c r="F37" t="s">
-        <v>71</v>
+        <v>188</v>
       </c>
       <c r="H37" t="str">
         <f t="shared" si="1"/>
@@ -1992,7 +2001,7 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="C38" t="s">
         <v>6</v>
@@ -2004,14 +2013,14 @@
         <v>1</v>
       </c>
       <c r="F38" t="s">
-        <v>69</v>
+        <v>189</v>
       </c>
       <c r="G38" t="s">
-        <v>70</v>
+        <v>58</v>
       </c>
       <c r="H38" t="str">
         <f t="shared" si="1"/>
-        <v>![Searching for the Phi-4 model](figures/ch02/ch02_ss_deploy_001_ann.png)</v>
+        <v>![Searching for the Phi-4 model](figures/ch01/ch01_ss_deploy_001_ann.png)</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
@@ -2019,7 +2028,7 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="C39" t="s">
         <v>6</v>
@@ -2031,7 +2040,7 @@
         <v>0</v>
       </c>
       <c r="F39" t="s">
-        <v>73</v>
+        <v>190</v>
       </c>
       <c r="H39" t="str">
         <f t="shared" si="1"/>
@@ -2043,7 +2052,7 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="C40" t="s">
         <v>6</v>
@@ -2055,14 +2064,14 @@
         <v>1</v>
       </c>
       <c r="F40" t="s">
-        <v>74</v>
+        <v>191</v>
       </c>
       <c r="G40" t="s">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="H40" t="str">
         <f t="shared" si="1"/>
-        <v>![Deploying Phi-4 with Default settings](figures/ch02/ch02_ss_deploy_002_ann.png)</v>
+        <v>![Deploying Phi-4 with Default settings](figures/ch01/ch01_ss_deploy_002_ann.png)</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
@@ -2070,7 +2079,7 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="C41" t="s">
         <v>6</v>
@@ -2082,7 +2091,7 @@
         <v>0</v>
       </c>
       <c r="F41" t="s">
-        <v>75</v>
+        <v>192</v>
       </c>
       <c r="H41" t="str">
         <f t="shared" si="1"/>
@@ -2094,7 +2103,7 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="C42" t="s">
         <v>6</v>
@@ -2106,14 +2115,14 @@
         <v>1</v>
       </c>
       <c r="F42" t="s">
-        <v>76</v>
+        <v>193</v>
       </c>
       <c r="G42" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="H42" t="str">
         <f t="shared" si="1"/>
-        <v>![Agreeing to the terms for deploying Phi-4](figures/ch02/ch02_ss_deploy_003_ann.png)</v>
+        <v>![Agreeing to the terms for deploying Phi-4](figures/ch01/ch01_ss_deploy_003_ann.png)</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
@@ -2121,7 +2130,7 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="C43" t="s">
         <v>6</v>
@@ -2133,14 +2142,14 @@
         <v>1</v>
       </c>
       <c r="F43" t="s">
-        <v>79</v>
+        <v>194</v>
       </c>
       <c r="G43" t="s">
-        <v>78</v>
+        <v>61</v>
       </c>
       <c r="H43" t="str">
         <f t="shared" si="1"/>
-        <v>![Playground UI for experimenting with a Phi-4 deployment](figures/ch02/ch02_ss_deploy_004_clean.png)</v>
+        <v>![Playground UI for experimenting with a Phi-4 deployment](figures/ch01/ch01_ss_deploy_004_clean.png)</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
@@ -2148,7 +2157,7 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="C44" t="s">
         <v>6</v>
@@ -2160,14 +2169,14 @@
         <v>1</v>
       </c>
       <c r="F44" t="s">
-        <v>81</v>
+        <v>195</v>
       </c>
       <c r="G44" t="s">
-        <v>80</v>
+        <v>62</v>
       </c>
       <c r="H44" t="str">
         <f t="shared" si="1"/>
-        <v>![Learning to make intergalactic pizza](figures/ch02/ch02_ss_deploy_005_clean.png)</v>
+        <v>![Learning to make intergalactic pizza](figures/ch01/ch01_ss_deploy_005_clean.png)</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
@@ -2175,7 +2184,7 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="C45" t="s">
         <v>6</v>
@@ -2187,7 +2196,7 @@
         <v>0</v>
       </c>
       <c r="F45" t="s">
-        <v>84</v>
+        <v>196</v>
       </c>
       <c r="H45" t="str">
         <f t="shared" si="1"/>
@@ -2199,7 +2208,7 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="C46" t="s">
         <v>6</v>
@@ -2211,14 +2220,14 @@
         <v>1</v>
       </c>
       <c r="F46" t="s">
-        <v>83</v>
+        <v>197</v>
       </c>
       <c r="G46" t="s">
-        <v>87</v>
+        <v>64</v>
       </c>
       <c r="H46" t="str">
         <f>IF(E46,_xlfn.CONCAT("![",G46,"](figures/",B46,"/",F46,")"),"")</f>
-        <v>![Modifying model parameters](figures/ch02/ch02_ss_deploy_006_ann.png)</v>
+        <v>![Modifying model parameters](figures/ch01/ch01_ss_deploy_006_ann.png)</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
@@ -2226,7 +2235,7 @@
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="C47" t="s">
         <v>6</v>
@@ -2238,7 +2247,7 @@
         <v>0</v>
       </c>
       <c r="F47" t="s">
-        <v>86</v>
+        <v>198</v>
       </c>
       <c r="H47" t="str">
         <f t="shared" si="1"/>
@@ -2250,7 +2259,7 @@
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="C48" t="s">
         <v>6</v>
@@ -2262,14 +2271,14 @@
         <v>1</v>
       </c>
       <c r="F48" t="s">
-        <v>85</v>
+        <v>199</v>
       </c>
       <c r="G48" t="s">
-        <v>82</v>
+        <v>63</v>
       </c>
       <c r="H48" t="str">
         <f t="shared" si="1"/>
-        <v>![Deployment endpoint and key on the Details tab](figures/ch02/ch02_ss_deploy_007_ann.png)</v>
+        <v>![Deployment endpoint and key on the Details tab](figures/ch01/ch01_ss_deploy_007_ann.png)</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
@@ -2277,7 +2286,7 @@
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="C49" t="s">
         <v>6</v>
@@ -2289,14 +2298,14 @@
         <v>1</v>
       </c>
       <c r="F49" t="s">
-        <v>86</v>
+        <v>198</v>
       </c>
       <c r="G49" t="s">
-        <v>88</v>
+        <v>65</v>
       </c>
       <c r="H49" t="str">
         <f t="shared" si="1"/>
-        <v>![A slightly more martian pizza recipe](figures/ch02/ch02_ss_deploy_007_clean.png)</v>
+        <v>![A slightly more martian pizza recipe](figures/ch01/ch01_ss_deploy_007_clean.png)</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
@@ -2316,7 +2325,7 @@
         <v>0</v>
       </c>
       <c r="F50" t="s">
-        <v>90</v>
+        <v>67</v>
       </c>
       <c r="H50" t="str">
         <f t="shared" si="1"/>
@@ -2340,10 +2349,10 @@
         <v>1</v>
       </c>
       <c r="F51" t="s">
-        <v>89</v>
+        <v>66</v>
       </c>
       <c r="G51" t="s">
-        <v>91</v>
+        <v>68</v>
       </c>
       <c r="H51" t="str">
         <f t="shared" si="1"/>
@@ -2367,7 +2376,7 @@
         <v>0</v>
       </c>
       <c r="F52" t="s">
-        <v>92</v>
+        <v>69</v>
       </c>
       <c r="H52" t="str">
         <f t="shared" si="1"/>
@@ -2391,10 +2400,10 @@
         <v>1</v>
       </c>
       <c r="F53" t="s">
-        <v>93</v>
+        <v>70</v>
       </c>
       <c r="G53" t="s">
-        <v>94</v>
+        <v>71</v>
       </c>
       <c r="H53" t="str">
         <f t="shared" si="1"/>
@@ -2418,7 +2427,7 @@
         <v>0</v>
       </c>
       <c r="F54" t="s">
-        <v>95</v>
+        <v>72</v>
       </c>
       <c r="H54" t="str">
         <f t="shared" si="1"/>
@@ -2442,10 +2451,10 @@
         <v>1</v>
       </c>
       <c r="F55" t="s">
-        <v>97</v>
+        <v>74</v>
       </c>
       <c r="G55" t="s">
-        <v>96</v>
+        <v>73</v>
       </c>
       <c r="H55" t="str">
         <f t="shared" si="1"/>
@@ -2469,10 +2478,10 @@
         <v>1</v>
       </c>
       <c r="F56" t="s">
-        <v>98</v>
+        <v>75</v>
       </c>
       <c r="G56" t="s">
-        <v>99</v>
+        <v>76</v>
       </c>
       <c r="H56" t="str">
         <f t="shared" si="1"/>
@@ -2496,7 +2505,7 @@
         <v>0</v>
       </c>
       <c r="F57" t="s">
-        <v>100</v>
+        <v>77</v>
       </c>
       <c r="H57" t="str">
         <f t="shared" si="1"/>
@@ -2520,10 +2529,10 @@
         <v>1</v>
       </c>
       <c r="F58" t="s">
-        <v>101</v>
+        <v>78</v>
       </c>
       <c r="G58" t="s">
-        <v>102</v>
+        <v>79</v>
       </c>
       <c r="H58" t="str">
         <f t="shared" si="1"/>
@@ -2547,7 +2556,7 @@
         <v>0</v>
       </c>
       <c r="F59" t="s">
-        <v>103</v>
+        <v>80</v>
       </c>
       <c r="H59" t="str">
         <f t="shared" si="1"/>
@@ -2571,10 +2580,10 @@
         <v>1</v>
       </c>
       <c r="F60" t="s">
-        <v>104</v>
+        <v>81</v>
       </c>
       <c r="G60" t="s">
-        <v>105</v>
+        <v>82</v>
       </c>
       <c r="H60" t="str">
         <f t="shared" si="1"/>
@@ -2598,10 +2607,10 @@
         <v>1</v>
       </c>
       <c r="F61" t="s">
-        <v>107</v>
+        <v>84</v>
       </c>
       <c r="G61" t="s">
-        <v>106</v>
+        <v>83</v>
       </c>
       <c r="H61" t="str">
         <f t="shared" si="1"/>
@@ -2625,10 +2634,10 @@
         <v>1</v>
       </c>
       <c r="F62" t="s">
-        <v>121</v>
+        <v>98</v>
       </c>
       <c r="G62" t="s">
-        <v>120</v>
+        <v>97</v>
       </c>
       <c r="H62" t="str">
         <f t="shared" si="1"/>
@@ -2652,10 +2661,10 @@
         <v>1</v>
       </c>
       <c r="F63" t="s">
-        <v>108</v>
+        <v>85</v>
       </c>
       <c r="G63" t="s">
-        <v>109</v>
+        <v>86</v>
       </c>
       <c r="H63" t="str">
         <f t="shared" si="1"/>
@@ -2679,10 +2688,10 @@
         <v>1</v>
       </c>
       <c r="F64" t="s">
-        <v>118</v>
+        <v>95</v>
       </c>
       <c r="G64" t="s">
-        <v>119</v>
+        <v>96</v>
       </c>
       <c r="H64" t="str">
         <f t="shared" si="1"/>
@@ -2706,7 +2715,7 @@
         <v>0</v>
       </c>
       <c r="F65" t="s">
-        <v>110</v>
+        <v>87</v>
       </c>
       <c r="H65" t="str">
         <f>IF(E65,_xlfn.CONCAT("![",G65,"](figures/",B65,"/",F65,")"),"")</f>
@@ -2730,10 +2739,10 @@
         <v>1</v>
       </c>
       <c r="F66" t="s">
-        <v>111</v>
+        <v>88</v>
       </c>
       <c r="G66" t="s">
-        <v>112</v>
+        <v>89</v>
       </c>
       <c r="H66" t="str">
         <f>IF(E66,_xlfn.CONCAT("![",G66,"](figures/",B66,"/",F66,")"),"")</f>
@@ -2757,7 +2766,7 @@
         <v>0</v>
       </c>
       <c r="F67" t="s">
-        <v>115</v>
+        <v>92</v>
       </c>
       <c r="H67" t="str">
         <f>IF(E67,_xlfn.CONCAT("![",G67,"](figures/",B67,"/",F67,")"),"")</f>
@@ -2781,10 +2790,10 @@
         <v>1</v>
       </c>
       <c r="F68" t="s">
-        <v>113</v>
+        <v>90</v>
       </c>
       <c r="G68" t="s">
-        <v>114</v>
+        <v>91</v>
       </c>
       <c r="H68" t="str">
         <f>IF(E68,_xlfn.CONCAT("![",G68,"](figures/",B68,"/",F68,")"),"")</f>
@@ -2808,10 +2817,10 @@
         <v>1</v>
       </c>
       <c r="F69" t="s">
-        <v>117</v>
+        <v>94</v>
       </c>
       <c r="G69" t="s">
-        <v>116</v>
+        <v>93</v>
       </c>
       <c r="H69" t="str">
         <f>IF(E69,_xlfn.CONCAT("![",G69,"](figures/",B69,"/",F69,")"),"")</f>
@@ -2835,10 +2844,10 @@
         <v>0</v>
       </c>
       <c r="F70" t="s">
-        <v>122</v>
+        <v>99</v>
       </c>
       <c r="H70" t="str">
-        <f t="shared" ref="H70:H116" si="2">IF(E70,_xlfn.CONCAT("![",G70,"](figures/",B70,"/",F70,")"),"")</f>
+        <f t="shared" ref="H70:H118" si="2">IF(E70,_xlfn.CONCAT("![",G70,"](figures/",B70,"/",F70,")"),"")</f>
         <v/>
       </c>
     </row>
@@ -2859,10 +2868,10 @@
         <v>1</v>
       </c>
       <c r="F71" t="s">
-        <v>123</v>
+        <v>100</v>
       </c>
       <c r="G71" t="s">
-        <v>124</v>
+        <v>101</v>
       </c>
       <c r="H71" t="str">
         <f t="shared" si="2"/>
@@ -2886,7 +2895,7 @@
         <v>0</v>
       </c>
       <c r="F72" t="s">
-        <v>126</v>
+        <v>103</v>
       </c>
       <c r="H72" t="str">
         <f t="shared" si="2"/>
@@ -2910,10 +2919,10 @@
         <v>1</v>
       </c>
       <c r="F73" t="s">
-        <v>127</v>
+        <v>104</v>
       </c>
       <c r="G73" t="s">
-        <v>125</v>
+        <v>102</v>
       </c>
       <c r="H73" t="str">
         <f t="shared" si="2"/>
@@ -2937,7 +2946,7 @@
         <v>0</v>
       </c>
       <c r="F74" t="s">
-        <v>128</v>
+        <v>105</v>
       </c>
       <c r="H74" t="str">
         <f t="shared" si="2"/>
@@ -2961,10 +2970,10 @@
         <v>1</v>
       </c>
       <c r="F75" t="s">
-        <v>129</v>
+        <v>106</v>
       </c>
       <c r="G75" t="s">
-        <v>130</v>
+        <v>107</v>
       </c>
       <c r="H75" t="str">
         <f t="shared" si="2"/>
@@ -2988,7 +2997,7 @@
         <v>0</v>
       </c>
       <c r="F76" t="s">
-        <v>131</v>
+        <v>108</v>
       </c>
       <c r="H76" t="str">
         <f t="shared" si="2"/>
@@ -3012,10 +3021,10 @@
         <v>1</v>
       </c>
       <c r="F77" t="s">
-        <v>132</v>
+        <v>109</v>
       </c>
       <c r="G77" t="s">
-        <v>133</v>
+        <v>110</v>
       </c>
       <c r="H77" t="str">
         <f t="shared" si="2"/>
@@ -3039,7 +3048,7 @@
         <v>0</v>
       </c>
       <c r="F78" t="s">
-        <v>134</v>
+        <v>111</v>
       </c>
       <c r="H78" t="str">
         <f t="shared" si="2"/>
@@ -3063,10 +3072,10 @@
         <v>1</v>
       </c>
       <c r="F79" t="s">
-        <v>135</v>
+        <v>112</v>
       </c>
       <c r="G79" t="s">
-        <v>136</v>
+        <v>113</v>
       </c>
       <c r="H79" t="str">
         <f t="shared" si="2"/>
@@ -3090,7 +3099,7 @@
         <v>0</v>
       </c>
       <c r="F80" t="s">
-        <v>138</v>
+        <v>115</v>
       </c>
       <c r="H80" t="str">
         <f t="shared" si="2"/>
@@ -3114,10 +3123,10 @@
         <v>1</v>
       </c>
       <c r="F81" t="s">
-        <v>139</v>
+        <v>116</v>
       </c>
       <c r="G81" t="s">
-        <v>137</v>
+        <v>114</v>
       </c>
       <c r="H81" t="str">
         <f t="shared" si="2"/>
@@ -3141,10 +3150,10 @@
         <v>1</v>
       </c>
       <c r="F82" t="s">
-        <v>140</v>
+        <v>117</v>
       </c>
       <c r="G82" t="s">
-        <v>141</v>
+        <v>118</v>
       </c>
       <c r="H82" t="str">
         <f t="shared" si="2"/>
@@ -3168,10 +3177,10 @@
         <v>1</v>
       </c>
       <c r="F83" t="s">
-        <v>143</v>
+        <v>120</v>
       </c>
       <c r="G83" t="s">
-        <v>142</v>
+        <v>119</v>
       </c>
       <c r="H83" t="str">
         <f t="shared" si="2"/>
@@ -3195,10 +3204,10 @@
         <v>1</v>
       </c>
       <c r="F84" t="s">
-        <v>144</v>
+        <v>121</v>
       </c>
       <c r="G84" t="s">
-        <v>145</v>
+        <v>122</v>
       </c>
       <c r="H84" t="str">
         <f t="shared" si="2"/>
@@ -3222,10 +3231,10 @@
         <v>1</v>
       </c>
       <c r="F85" t="s">
-        <v>178</v>
+        <v>155</v>
       </c>
       <c r="G85" t="s">
-        <v>180</v>
+        <v>157</v>
       </c>
       <c r="H85" t="str">
         <f t="shared" si="2"/>
@@ -3249,10 +3258,10 @@
         <v>1</v>
       </c>
       <c r="F86" t="s">
-        <v>179</v>
+        <v>156</v>
       </c>
       <c r="G86" t="s">
-        <v>181</v>
+        <v>158</v>
       </c>
       <c r="H86" t="str">
         <f>IF(E86,_xlfn.CONCAT("![",G86,"](figures/",B86,"/",F86,")"),"")</f>
@@ -3276,7 +3285,7 @@
         <v>0</v>
       </c>
       <c r="F87" t="s">
-        <v>183</v>
+        <v>160</v>
       </c>
       <c r="H87" t="str">
         <f t="shared" ref="H87:H95" si="3">IF(E87,_xlfn.CONCAT("![",G87,"](figures/",B87,"/",F87,")"),"")</f>
@@ -3300,10 +3309,10 @@
         <v>1</v>
       </c>
       <c r="F88" t="s">
-        <v>184</v>
+        <v>161</v>
       </c>
       <c r="G88" t="s">
-        <v>182</v>
+        <v>159</v>
       </c>
       <c r="H88" t="str">
         <f t="shared" si="3"/>
@@ -3327,7 +3336,7 @@
         <v>0</v>
       </c>
       <c r="F89" t="s">
-        <v>185</v>
+        <v>162</v>
       </c>
       <c r="H89" t="str">
         <f t="shared" si="3"/>
@@ -3351,10 +3360,10 @@
         <v>1</v>
       </c>
       <c r="F90" t="s">
-        <v>186</v>
+        <v>163</v>
       </c>
       <c r="G90" t="s">
-        <v>187</v>
+        <v>164</v>
       </c>
       <c r="H90" t="str">
         <f t="shared" si="3"/>
@@ -3378,7 +3387,7 @@
         <v>0</v>
       </c>
       <c r="F91" t="s">
-        <v>188</v>
+        <v>165</v>
       </c>
       <c r="H91" t="str">
         <f t="shared" si="3"/>
@@ -3402,10 +3411,10 @@
         <v>1</v>
       </c>
       <c r="F92" t="s">
-        <v>189</v>
+        <v>166</v>
       </c>
       <c r="G92" t="s">
-        <v>190</v>
+        <v>167</v>
       </c>
       <c r="H92" t="str">
         <f t="shared" si="3"/>
@@ -3429,7 +3438,7 @@
         <v>0</v>
       </c>
       <c r="F93" t="s">
-        <v>191</v>
+        <v>168</v>
       </c>
       <c r="H93" t="str">
         <f t="shared" si="3"/>
@@ -3453,10 +3462,10 @@
         <v>1</v>
       </c>
       <c r="F94" t="s">
-        <v>192</v>
+        <v>169</v>
       </c>
       <c r="G94" t="s">
-        <v>193</v>
+        <v>170</v>
       </c>
       <c r="H94" t="str">
         <f t="shared" si="3"/>
@@ -3480,7 +3489,7 @@
         <v>0</v>
       </c>
       <c r="F95" t="s">
-        <v>147</v>
+        <v>124</v>
       </c>
       <c r="H95" t="str">
         <f t="shared" si="3"/>
@@ -3504,10 +3513,10 @@
         <v>1</v>
       </c>
       <c r="F96" t="s">
-        <v>148</v>
+        <v>125</v>
       </c>
       <c r="G96" t="s">
-        <v>149</v>
+        <v>126</v>
       </c>
       <c r="H96" t="str">
         <f t="shared" si="2"/>
@@ -3531,7 +3540,7 @@
         <v>0</v>
       </c>
       <c r="F97" t="s">
-        <v>151</v>
+        <v>128</v>
       </c>
       <c r="H97" t="str">
         <f t="shared" si="2"/>
@@ -3555,10 +3564,10 @@
         <v>1</v>
       </c>
       <c r="F98" t="s">
-        <v>152</v>
+        <v>129</v>
       </c>
       <c r="G98" t="s">
-        <v>150</v>
+        <v>127</v>
       </c>
       <c r="H98" t="str">
         <f t="shared" si="2"/>
@@ -3582,7 +3591,7 @@
         <v>0</v>
       </c>
       <c r="F99" t="s">
-        <v>153</v>
+        <v>130</v>
       </c>
       <c r="H99" t="str">
         <f t="shared" si="2"/>
@@ -3606,10 +3615,10 @@
         <v>1</v>
       </c>
       <c r="F100" t="s">
-        <v>154</v>
+        <v>131</v>
       </c>
       <c r="G100" t="s">
-        <v>155</v>
+        <v>132</v>
       </c>
       <c r="H100" t="str">
         <f t="shared" si="2"/>
@@ -3633,7 +3642,7 @@
         <v>0</v>
       </c>
       <c r="F101" t="s">
-        <v>156</v>
+        <v>133</v>
       </c>
       <c r="H101" t="str">
         <f t="shared" si="2"/>
@@ -3657,10 +3666,10 @@
         <v>1</v>
       </c>
       <c r="F102" t="s">
-        <v>157</v>
+        <v>134</v>
       </c>
       <c r="G102" t="s">
-        <v>158</v>
+        <v>135</v>
       </c>
       <c r="H102" t="str">
         <f t="shared" si="2"/>
@@ -3684,7 +3693,7 @@
         <v>0</v>
       </c>
       <c r="F103" t="s">
-        <v>159</v>
+        <v>136</v>
       </c>
       <c r="H103" t="str">
         <f t="shared" si="2"/>
@@ -3708,10 +3717,10 @@
         <v>1</v>
       </c>
       <c r="F104" t="s">
-        <v>160</v>
+        <v>137</v>
       </c>
       <c r="G104" t="s">
-        <v>166</v>
+        <v>143</v>
       </c>
       <c r="H104" t="str">
         <f t="shared" si="2"/>
@@ -3735,7 +3744,7 @@
         <v>0</v>
       </c>
       <c r="F105" t="s">
-        <v>161</v>
+        <v>138</v>
       </c>
       <c r="H105" t="str">
         <f t="shared" si="2"/>
@@ -3759,10 +3768,10 @@
         <v>1</v>
       </c>
       <c r="F106" t="s">
-        <v>162</v>
+        <v>139</v>
       </c>
       <c r="G106" t="s">
-        <v>194</v>
+        <v>171</v>
       </c>
       <c r="H106" t="str">
         <f t="shared" si="2"/>
@@ -3786,7 +3795,7 @@
         <v>0</v>
       </c>
       <c r="F107" t="s">
-        <v>163</v>
+        <v>140</v>
       </c>
       <c r="H107" t="str">
         <f t="shared" si="2"/>
@@ -3810,10 +3819,10 @@
         <v>1</v>
       </c>
       <c r="F108" t="s">
-        <v>164</v>
+        <v>141</v>
       </c>
       <c r="G108" t="s">
-        <v>165</v>
+        <v>142</v>
       </c>
       <c r="H108" t="str">
         <f t="shared" si="2"/>
@@ -3834,17 +3843,14 @@
         <v>0</v>
       </c>
       <c r="E109" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F109" t="s">
-        <v>195</v>
-      </c>
-      <c r="G109" t="s">
-        <v>196</v>
+        <v>172</v>
       </c>
       <c r="H109" t="str">
         <f t="shared" si="2"/>
-        <v>![Checking the Cosmos DB Tool usage in the Agent response](figures/ch02/ch02_ss_cosmos_008_clean.png)</v>
+        <v/>
       </c>
     </row>
     <row r="110" spans="1:8" x14ac:dyDescent="0.25">
@@ -3858,17 +3864,20 @@
         <v>6</v>
       </c>
       <c r="D110" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E110" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F110" t="s">
-        <v>167</v>
+        <v>174</v>
+      </c>
+      <c r="G110" t="s">
+        <v>173</v>
       </c>
       <c r="H110" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>![Checking the Cosmos DB Tool usage in the Agent response](figures/ch02/ch02_ss_cosmos_008_ann.png)</v>
       </c>
     </row>
     <row r="111" spans="1:8" x14ac:dyDescent="0.25">
@@ -3882,20 +3891,20 @@
         <v>6</v>
       </c>
       <c r="D111" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E111" t="b">
         <v>1</v>
       </c>
       <c r="F111" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="G111" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="H111" t="str">
         <f t="shared" si="2"/>
-        <v>![Creating a new Cosmos DB container](figures/ch02/ch02_ss_database_001_ann.png)</v>
+        <v>![A successful Cosmos DB Tool call and augmented Agent response](figures/ch02/ch02_ss_cosmos_009_clean.png)</v>
       </c>
     </row>
     <row r="112" spans="1:8" x14ac:dyDescent="0.25">
@@ -3915,7 +3924,7 @@
         <v>0</v>
       </c>
       <c r="F112" t="s">
-        <v>170</v>
+        <v>144</v>
       </c>
       <c r="H112" t="str">
         <f t="shared" si="2"/>
@@ -3939,14 +3948,14 @@
         <v>1</v>
       </c>
       <c r="F113" t="s">
-        <v>171</v>
+        <v>145</v>
       </c>
       <c r="G113" t="s">
-        <v>177</v>
+        <v>146</v>
       </c>
       <c r="H113" t="str">
         <f t="shared" si="2"/>
-        <v>![Creating a new Cosmos DB database](figures/ch02/ch02_ss_database_002_ann.png)</v>
+        <v>![Creating a new Cosmos DB container](figures/ch02/ch02_ss_database_001_ann.png)</v>
       </c>
     </row>
     <row r="114" spans="1:8" x14ac:dyDescent="0.25">
@@ -3966,7 +3975,7 @@
         <v>0</v>
       </c>
       <c r="F114" t="s">
-        <v>174</v>
+        <v>147</v>
       </c>
       <c r="H114" t="str">
         <f t="shared" si="2"/>
@@ -3990,14 +3999,14 @@
         <v>1</v>
       </c>
       <c r="F115" t="s">
-        <v>175</v>
+        <v>148</v>
       </c>
       <c r="G115" t="s">
-        <v>172</v>
+        <v>154</v>
       </c>
       <c r="H115" t="str">
         <f t="shared" si="2"/>
-        <v>![Uploading property records to your database](figures/ch02/ch02_ss_database_003_ann.png)</v>
+        <v>![Creating a new Cosmos DB database](figures/ch02/ch02_ss_database_002_ann.png)</v>
       </c>
     </row>
     <row r="116" spans="1:8" x14ac:dyDescent="0.25">
@@ -4014,15 +4023,66 @@
         <v>0</v>
       </c>
       <c r="E116" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F116" t="s">
-        <v>176</v>
-      </c>
-      <c r="G116" t="s">
-        <v>173</v>
+        <v>151</v>
       </c>
       <c r="H116" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="117" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A117">
+        <v>116</v>
+      </c>
+      <c r="B117" t="s">
+        <v>47</v>
+      </c>
+      <c r="C117" t="s">
+        <v>6</v>
+      </c>
+      <c r="D117" t="b">
+        <v>1</v>
+      </c>
+      <c r="E117" t="b">
+        <v>1</v>
+      </c>
+      <c r="F117" t="s">
+        <v>152</v>
+      </c>
+      <c r="G117" t="s">
+        <v>149</v>
+      </c>
+      <c r="H117" t="str">
+        <f t="shared" si="2"/>
+        <v>![Uploading property records to your database](figures/ch02/ch02_ss_database_003_ann.png)</v>
+      </c>
+    </row>
+    <row r="118" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A118">
+        <v>117</v>
+      </c>
+      <c r="B118" t="s">
+        <v>47</v>
+      </c>
+      <c r="C118" t="s">
+        <v>6</v>
+      </c>
+      <c r="D118" t="b">
+        <v>0</v>
+      </c>
+      <c r="E118" t="b">
+        <v>1</v>
+      </c>
+      <c r="F118" t="s">
+        <v>153</v>
+      </c>
+      <c r="G118" t="s">
+        <v>150</v>
+      </c>
+      <c r="H118" t="str">
         <f t="shared" si="2"/>
         <v>![Listing your property records](figures/ch02/ch02_ss_database_004_clean.png)</v>
       </c>

</xml_diff>

<commit_message>
Add knowledge base figures for Ch04
</commit_message>
<xml_diff>
--- a/figures/figure_inventory.xlsx
+++ b/figures/figure_inventory.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Colby\Documents\GitHub\foundry-book\figures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3376D93-EFEC-430B-B8A2-11F99EA6A026}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C6BE426-13B2-4F67-B78D-75D95314A64E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{222F1F68-60B1-49B9-BFF7-2C9CF743DB25}"/>
+    <workbookView xWindow="44535" yWindow="2445" windowWidth="27645" windowHeight="14040" xr2:uid="{222F1F68-60B1-49B9-BFF7-2C9CF743DB25}"/>
   </bookViews>
   <sheets>
     <sheet name="Figure Inventory" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="457" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="231">
   <si>
     <t>Type</t>
   </si>
@@ -731,6 +731,30 @@
   </si>
   <si>
     <t>A much more functional real estate Agent</t>
+  </si>
+  <si>
+    <t>ss_knowledge_001_clean.png</t>
+  </si>
+  <si>
+    <t>ss_knowledge_001_ann.png</t>
+  </si>
+  <si>
+    <t>Connecting to an Azure AI Search resource</t>
+  </si>
+  <si>
+    <t>ss_knowledge_002_clean.png</t>
+  </si>
+  <si>
+    <t>ss_knowledge_002_ann.png</t>
+  </si>
+  <si>
+    <t>Creating a new Knowledge Base</t>
+  </si>
+  <si>
+    <t>Building a multi-source Agent for financial insights</t>
+  </si>
+  <si>
+    <t>il_multisource_001.png</t>
   </si>
 </sst>
 </file>
@@ -1123,7 +1147,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B464DFF5-94DA-41E0-B03E-143380050964}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:J119"/>
+  <dimension ref="A1:J124"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1232,11 +1256,11 @@
         <v>3498</v>
       </c>
       <c r="I3" t="str">
-        <f t="shared" ref="I3:I62" si="0">_xlfn.CONCAT("{#fig-",H3,"}")</f>
+        <f t="shared" ref="I3:I47" si="0">_xlfn.CONCAT("{#fig-",H3,"}")</f>
         <v>{#fig-3498}</v>
       </c>
       <c r="J3" t="str">
-        <f t="shared" ref="J3:J64" si="1">IF(E3,_xlfn.CONCAT("![",G3,"](figures/",B3,"/",F3,")",I3),"")</f>
+        <f t="shared" ref="J3:J47" si="1">IF(E3,_xlfn.CONCAT("![",G3,"](figures/",B3,"/",F3,")",I3),"")</f>
         <v>![Foundry Resource and Project Organization](figures/in/il_portal_001.png){#fig-3498}</v>
       </c>
     </row>
@@ -4956,11 +4980,11 @@
         <v>5117</v>
       </c>
       <c r="I113" t="str">
-        <f t="shared" ref="I113:I119" si="4">_xlfn.CONCAT("{#fig-",H113,"}")</f>
+        <f t="shared" ref="I113:I124" si="4">_xlfn.CONCAT("{#fig-",H113,"}")</f>
         <v>{#fig-5117}</v>
       </c>
       <c r="J113" t="str">
-        <f t="shared" ref="J113:J119" si="5">IF(E113,_xlfn.CONCAT("![",G113,"](figures/",B113,"/",F113,")",I113),"")</f>
+        <f t="shared" ref="J113:J124" si="5">IF(E113,_xlfn.CONCAT("![",G113,"](figures/",B113,"/",F113,")",I113),"")</f>
         <v>![Creating a new Cosmos DB container](figures/ad/ss_database_001_ann.png){#fig-5117}</v>
       </c>
     </row>
@@ -5166,6 +5190,175 @@
       <c r="J119" t="str">
         <f t="shared" si="5"/>
         <v>![Orchestrating multi-source, complex RAG pipelines](figures/kb/il_layers_001.png){#fig-2B5B}</v>
+      </c>
+    </row>
+    <row r="120" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A120">
+        <v>121</v>
+      </c>
+      <c r="B120" t="s">
+        <v>100</v>
+      </c>
+      <c r="C120" t="s">
+        <v>6</v>
+      </c>
+      <c r="D120" t="b">
+        <v>0</v>
+      </c>
+      <c r="E120" t="b">
+        <v>1</v>
+      </c>
+      <c r="F120" t="s">
+        <v>230</v>
+      </c>
+      <c r="G120" t="s">
+        <v>229</v>
+      </c>
+      <c r="H120" s="1" t="str" cm="1">
+        <f t="array" ref="H120">CRC16HASH(F120)</f>
+        <v>E787</v>
+      </c>
+      <c r="I120" t="str">
+        <f t="shared" si="4"/>
+        <v>{#fig-E787}</v>
+      </c>
+      <c r="J120" t="str">
+        <f t="shared" si="5"/>
+        <v>![Building a multi-source Agent for financial insights](figures/kb/il_multisource_001.png){#fig-E787}</v>
+      </c>
+    </row>
+    <row r="121" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A121">
+        <v>122</v>
+      </c>
+      <c r="B121" t="s">
+        <v>100</v>
+      </c>
+      <c r="C121" t="s">
+        <v>4</v>
+      </c>
+      <c r="D121" t="b">
+        <v>0</v>
+      </c>
+      <c r="E121" t="b">
+        <v>0</v>
+      </c>
+      <c r="F121" t="s">
+        <v>223</v>
+      </c>
+      <c r="H121" s="1" t="str" cm="1">
+        <f t="array" ref="H121">CRC16HASH(F121)</f>
+        <v>6B1C</v>
+      </c>
+      <c r="I121" t="str">
+        <f t="shared" si="4"/>
+        <v>{#fig-6B1C}</v>
+      </c>
+      <c r="J121" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="122" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A122">
+        <v>123</v>
+      </c>
+      <c r="B122" t="s">
+        <v>100</v>
+      </c>
+      <c r="C122" t="s">
+        <v>4</v>
+      </c>
+      <c r="D122" t="b">
+        <v>1</v>
+      </c>
+      <c r="E122" t="b">
+        <v>1</v>
+      </c>
+      <c r="F122" t="s">
+        <v>224</v>
+      </c>
+      <c r="G122" t="s">
+        <v>225</v>
+      </c>
+      <c r="H122" s="1" t="str" cm="1">
+        <f t="array" ref="H122">CRC16HASH(F122)</f>
+        <v>33E</v>
+      </c>
+      <c r="I122" t="str">
+        <f t="shared" si="4"/>
+        <v>{#fig-33E}</v>
+      </c>
+      <c r="J122" t="str">
+        <f t="shared" si="5"/>
+        <v>![Connecting to an Azure AI Search resource](figures/kb/ss_knowledge_001_ann.png){#fig-33E}</v>
+      </c>
+    </row>
+    <row r="123" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A123">
+        <v>124</v>
+      </c>
+      <c r="B123" t="s">
+        <v>100</v>
+      </c>
+      <c r="C123" t="s">
+        <v>4</v>
+      </c>
+      <c r="D123" t="b">
+        <v>0</v>
+      </c>
+      <c r="E123" t="b">
+        <v>0</v>
+      </c>
+      <c r="F123" t="s">
+        <v>226</v>
+      </c>
+      <c r="H123" s="1" t="str" cm="1">
+        <f t="array" ref="H123">CRC16HASH(F123)</f>
+        <v>2F13</v>
+      </c>
+      <c r="I123" t="str">
+        <f t="shared" si="4"/>
+        <v>{#fig-2F13}</v>
+      </c>
+      <c r="J123" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="124" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A124">
+        <v>125</v>
+      </c>
+      <c r="B124" t="s">
+        <v>100</v>
+      </c>
+      <c r="C124" t="s">
+        <v>4</v>
+      </c>
+      <c r="D124" t="b">
+        <v>1</v>
+      </c>
+      <c r="E124" t="b">
+        <v>1</v>
+      </c>
+      <c r="F124" t="s">
+        <v>227</v>
+      </c>
+      <c r="G124" t="s">
+        <v>228</v>
+      </c>
+      <c r="H124" s="1" t="str" cm="1">
+        <f t="array" ref="H124">CRC16HASH(F124)</f>
+        <v>F32A</v>
+      </c>
+      <c r="I124" t="str">
+        <f t="shared" si="4"/>
+        <v>{#fig-F32A}</v>
+      </c>
+      <c r="J124" t="str">
+        <f t="shared" si="5"/>
+        <v>![Creating a new Knowledge Base](figures/kb/ss_knowledge_002_ann.png){#fig-F32A}</v>
       </c>
     </row>
   </sheetData>
@@ -5178,6 +5371,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F9AFBD1-7D36-4720-9798-1D6F918A5E59}">
+  <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>

<commit_message>
Add enrichment illustration for Ch04
</commit_message>
<xml_diff>
--- a/figures/figure_inventory.xlsx
+++ b/figures/figure_inventory.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Colby\Documents\GitHub\foundry-book\figures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE584073-5F04-404F-B673-A2B5EA6DBED1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDA3D290-E316-4829-A6B0-45DFDE5F8FAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{222F1F68-60B1-49B9-BFF7-2C9CF743DB25}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Chapters" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Figure Inventory'!$A$1:$J$193</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Figure Inventory'!$A$1:$J$194</definedName>
   </definedNames>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="720" uniqueCount="331">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="724" uniqueCount="333">
   <si>
     <t>Type</t>
   </si>
@@ -1055,6 +1055,12 @@
   </si>
   <si>
     <t>Asking about Microsoft's 2026 outlook</t>
+  </si>
+  <si>
+    <t>il_enrichment_001.png</t>
+  </si>
+  <si>
+    <t>Enrichment tasks for documents</t>
   </si>
 </sst>
 </file>
@@ -1142,11 +1148,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1631,11 +1647,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B464DFF5-94DA-41E0-B03E-143380050964}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:J193"/>
+  <dimension ref="A1:J194"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.28515625" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="6.5703125" bestFit="1" customWidth="1"/>
@@ -2495,7 +2511,7 @@
       <c r="A26">
         <v>26</v>
       </c>
-      <c r="B26" s="7" t="s">
+      <c r="B26" s="4" t="s">
         <v>98</v>
       </c>
       <c r="C26" t="s">
@@ -2527,7 +2543,7 @@
       <c r="A27">
         <v>27</v>
       </c>
-      <c r="B27" s="7" t="s">
+      <c r="B27" s="4" t="s">
         <v>98</v>
       </c>
       <c r="C27" t="s">
@@ -2562,7 +2578,7 @@
       <c r="A28">
         <v>28</v>
       </c>
-      <c r="B28" s="7" t="s">
+      <c r="B28" s="4" t="s">
         <v>98</v>
       </c>
       <c r="C28" t="s">
@@ -2594,7 +2610,7 @@
       <c r="A29">
         <v>29</v>
       </c>
-      <c r="B29" s="7" t="s">
+      <c r="B29" s="4" t="s">
         <v>98</v>
       </c>
       <c r="C29" t="s">
@@ -2629,7 +2645,7 @@
       <c r="A30">
         <v>30</v>
       </c>
-      <c r="B30" s="7" t="s">
+      <c r="B30" s="4" t="s">
         <v>98</v>
       </c>
       <c r="C30" t="s">
@@ -2664,7 +2680,7 @@
       <c r="A31">
         <v>31</v>
       </c>
-      <c r="B31" s="7" t="s">
+      <c r="B31" s="4" t="s">
         <v>98</v>
       </c>
       <c r="C31" t="s">
@@ -2699,7 +2715,7 @@
       <c r="A32">
         <v>32</v>
       </c>
-      <c r="B32" s="7" t="s">
+      <c r="B32" s="4" t="s">
         <v>98</v>
       </c>
       <c r="C32" t="s">
@@ -2734,7 +2750,7 @@
       <c r="A33">
         <v>33</v>
       </c>
-      <c r="B33" s="7" t="s">
+      <c r="B33" s="4" t="s">
         <v>98</v>
       </c>
       <c r="C33" t="s">
@@ -2769,7 +2785,7 @@
       <c r="A34">
         <v>34</v>
       </c>
-      <c r="B34" s="7" t="s">
+      <c r="B34" s="4" t="s">
         <v>98</v>
       </c>
       <c r="C34" t="s">
@@ -2804,7 +2820,7 @@
       <c r="A35">
         <v>36</v>
       </c>
-      <c r="B35" s="7" t="s">
+      <c r="B35" s="4" t="s">
         <v>98</v>
       </c>
       <c r="C35" t="s">
@@ -2839,7 +2855,7 @@
       <c r="A36">
         <v>37</v>
       </c>
-      <c r="B36" s="7" t="s">
+      <c r="B36" s="4" t="s">
         <v>98</v>
       </c>
       <c r="C36" t="s">
@@ -2874,7 +2890,7 @@
       <c r="A37">
         <v>38</v>
       </c>
-      <c r="B37" s="7" t="s">
+      <c r="B37" s="4" t="s">
         <v>98</v>
       </c>
       <c r="C37" t="s">
@@ -2906,7 +2922,7 @@
       <c r="A38">
         <v>39</v>
       </c>
-      <c r="B38" s="7" t="s">
+      <c r="B38" s="4" t="s">
         <v>98</v>
       </c>
       <c r="C38" t="s">
@@ -2941,7 +2957,7 @@
       <c r="A39">
         <v>40</v>
       </c>
-      <c r="B39" s="7" t="s">
+      <c r="B39" s="4" t="s">
         <v>98</v>
       </c>
       <c r="C39" t="s">
@@ -2973,7 +2989,7 @@
       <c r="A40">
         <v>41</v>
       </c>
-      <c r="B40" s="7" t="s">
+      <c r="B40" s="4" t="s">
         <v>98</v>
       </c>
       <c r="C40" t="s">
@@ -3008,7 +3024,7 @@
       <c r="A41">
         <v>42</v>
       </c>
-      <c r="B41" s="7" t="s">
+      <c r="B41" s="4" t="s">
         <v>98</v>
       </c>
       <c r="C41" t="s">
@@ -3040,7 +3056,7 @@
       <c r="A42">
         <v>43</v>
       </c>
-      <c r="B42" s="7" t="s">
+      <c r="B42" s="4" t="s">
         <v>98</v>
       </c>
       <c r="C42" t="s">
@@ -3075,7 +3091,7 @@
       <c r="A43">
         <v>44</v>
       </c>
-      <c r="B43" s="7" t="s">
+      <c r="B43" s="4" t="s">
         <v>98</v>
       </c>
       <c r="C43" t="s">
@@ -3110,7 +3126,7 @@
       <c r="A44">
         <v>45</v>
       </c>
-      <c r="B44" s="7" t="s">
+      <c r="B44" s="4" t="s">
         <v>98</v>
       </c>
       <c r="C44" t="s">
@@ -3145,7 +3161,7 @@
       <c r="A45">
         <v>46</v>
       </c>
-      <c r="B45" s="7" t="s">
+      <c r="B45" s="4" t="s">
         <v>98</v>
       </c>
       <c r="C45" t="s">
@@ -3177,7 +3193,7 @@
       <c r="A46">
         <v>47</v>
       </c>
-      <c r="B46" s="7" t="s">
+      <c r="B46" s="4" t="s">
         <v>98</v>
       </c>
       <c r="C46" t="s">
@@ -3212,7 +3228,7 @@
       <c r="A47">
         <v>48</v>
       </c>
-      <c r="B47" s="7" t="s">
+      <c r="B47" s="4" t="s">
         <v>98</v>
       </c>
       <c r="C47" t="s">
@@ -3244,7 +3260,7 @@
       <c r="A48">
         <v>49</v>
       </c>
-      <c r="B48" s="7" t="s">
+      <c r="B48" s="4" t="s">
         <v>98</v>
       </c>
       <c r="C48" t="s">
@@ -3279,7 +3295,7 @@
       <c r="A49">
         <v>50</v>
       </c>
-      <c r="B49" s="7" t="s">
+      <c r="B49" s="4" t="s">
         <v>98</v>
       </c>
       <c r="C49" t="s">
@@ -3314,7 +3330,7 @@
       <c r="A50">
         <v>51</v>
       </c>
-      <c r="B50" s="4" t="s">
+      <c r="B50" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C50" t="s">
@@ -3349,7 +3365,7 @@
       <c r="A51">
         <v>52</v>
       </c>
-      <c r="B51" s="4" t="s">
+      <c r="B51" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C51" t="s">
@@ -3381,7 +3397,7 @@
       <c r="A52">
         <v>53</v>
       </c>
-      <c r="B52" s="4" t="s">
+      <c r="B52" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C52" t="s">
@@ -3416,7 +3432,7 @@
       <c r="A53">
         <v>54</v>
       </c>
-      <c r="B53" s="4" t="s">
+      <c r="B53" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C53" t="s">
@@ -3448,7 +3464,7 @@
       <c r="A54">
         <v>55</v>
       </c>
-      <c r="B54" s="4" t="s">
+      <c r="B54" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C54" t="s">
@@ -3483,7 +3499,7 @@
       <c r="A55">
         <v>56</v>
       </c>
-      <c r="B55" s="4" t="s">
+      <c r="B55" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C55" t="s">
@@ -3515,7 +3531,7 @@
       <c r="A56">
         <v>57</v>
       </c>
-      <c r="B56" s="4" t="s">
+      <c r="B56" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C56" t="s">
@@ -3550,7 +3566,7 @@
       <c r="A57">
         <v>58</v>
       </c>
-      <c r="B57" s="4" t="s">
+      <c r="B57" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C57" t="s">
@@ -3585,7 +3601,7 @@
       <c r="A58">
         <v>59</v>
       </c>
-      <c r="B58" s="4" t="s">
+      <c r="B58" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C58" t="s">
@@ -3617,7 +3633,7 @@
       <c r="A59">
         <v>60</v>
       </c>
-      <c r="B59" s="4" t="s">
+      <c r="B59" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C59" t="s">
@@ -3652,7 +3668,7 @@
       <c r="A60">
         <v>61</v>
       </c>
-      <c r="B60" s="4" t="s">
+      <c r="B60" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C60" t="s">
@@ -3684,7 +3700,7 @@
       <c r="A61">
         <v>62</v>
       </c>
-      <c r="B61" s="4" t="s">
+      <c r="B61" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C61" t="s">
@@ -3719,7 +3735,7 @@
       <c r="A62">
         <v>63</v>
       </c>
-      <c r="B62" s="4" t="s">
+      <c r="B62" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C62" t="s">
@@ -3754,7 +3770,7 @@
       <c r="A63">
         <v>64</v>
       </c>
-      <c r="B63" s="4" t="s">
+      <c r="B63" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C63" t="s">
@@ -3786,7 +3802,7 @@
       <c r="A64">
         <v>65</v>
       </c>
-      <c r="B64" s="4" t="s">
+      <c r="B64" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C64" t="s">
@@ -3821,7 +3837,7 @@
       <c r="A65">
         <v>66</v>
       </c>
-      <c r="B65" s="4" t="s">
+      <c r="B65" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C65" t="s">
@@ -3853,7 +3869,7 @@
       <c r="A66">
         <v>67</v>
       </c>
-      <c r="B66" s="4" t="s">
+      <c r="B66" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C66" t="s">
@@ -3888,7 +3904,7 @@
       <c r="A67">
         <v>68</v>
       </c>
-      <c r="B67" s="4" t="s">
+      <c r="B67" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C67" t="s">
@@ -3920,7 +3936,7 @@
       <c r="A68">
         <v>69</v>
       </c>
-      <c r="B68" s="4" t="s">
+      <c r="B68" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C68" t="s">
@@ -3955,7 +3971,7 @@
       <c r="A69">
         <v>70</v>
       </c>
-      <c r="B69" s="4" t="s">
+      <c r="B69" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C69" t="s">
@@ -3987,7 +4003,7 @@
       <c r="A70">
         <v>71</v>
       </c>
-      <c r="B70" s="4" t="s">
+      <c r="B70" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C70" t="s">
@@ -4022,7 +4038,7 @@
       <c r="A71">
         <v>72</v>
       </c>
-      <c r="B71" s="4" t="s">
+      <c r="B71" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C71" t="s">
@@ -4054,7 +4070,7 @@
       <c r="A72">
         <v>73</v>
       </c>
-      <c r="B72" s="4" t="s">
+      <c r="B72" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C72" t="s">
@@ -4089,7 +4105,7 @@
       <c r="A73">
         <v>74</v>
       </c>
-      <c r="B73" s="4" t="s">
+      <c r="B73" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C73" t="s">
@@ -4124,7 +4140,7 @@
       <c r="A74">
         <v>75</v>
       </c>
-      <c r="B74" s="4" t="s">
+      <c r="B74" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C74" t="s">
@@ -4156,7 +4172,7 @@
       <c r="A75">
         <v>76</v>
       </c>
-      <c r="B75" s="4" t="s">
+      <c r="B75" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C75" t="s">
@@ -4191,7 +4207,7 @@
       <c r="A76">
         <v>77</v>
       </c>
-      <c r="B76" s="4" t="s">
+      <c r="B76" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C76" t="s">
@@ -4223,7 +4239,7 @@
       <c r="A77">
         <v>78</v>
       </c>
-      <c r="B77" s="4" t="s">
+      <c r="B77" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C77" t="s">
@@ -4258,7 +4274,7 @@
       <c r="A78">
         <v>79</v>
       </c>
-      <c r="B78" s="4" t="s">
+      <c r="B78" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C78" t="s">
@@ -4290,7 +4306,7 @@
       <c r="A79">
         <v>80</v>
       </c>
-      <c r="B79" s="4" t="s">
+      <c r="B79" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C79" t="s">
@@ -4325,7 +4341,7 @@
       <c r="A80">
         <v>81</v>
       </c>
-      <c r="B80" s="4" t="s">
+      <c r="B80" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C80" t="s">
@@ -4357,7 +4373,7 @@
       <c r="A81">
         <v>82</v>
       </c>
-      <c r="B81" s="4" t="s">
+      <c r="B81" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C81" t="s">
@@ -4392,7 +4408,7 @@
       <c r="A82">
         <v>83</v>
       </c>
-      <c r="B82" s="4" t="s">
+      <c r="B82" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C82" t="s">
@@ -4424,7 +4440,7 @@
       <c r="A83">
         <v>84</v>
       </c>
-      <c r="B83" s="4" t="s">
+      <c r="B83" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C83" t="s">
@@ -4459,7 +4475,7 @@
       <c r="A84">
         <v>85</v>
       </c>
-      <c r="B84" s="4" t="s">
+      <c r="B84" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C84" t="s">
@@ -4491,7 +4507,7 @@
       <c r="A85">
         <v>86</v>
       </c>
-      <c r="B85" s="4" t="s">
+      <c r="B85" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C85" t="s">
@@ -4526,7 +4542,7 @@
       <c r="A86">
         <v>87</v>
       </c>
-      <c r="B86" s="4" t="s">
+      <c r="B86" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C86" t="s">
@@ -4558,7 +4574,7 @@
       <c r="A87">
         <v>88</v>
       </c>
-      <c r="B87" s="4" t="s">
+      <c r="B87" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C87" t="s">
@@ -4593,7 +4609,7 @@
       <c r="A88">
         <v>89</v>
       </c>
-      <c r="B88" s="4" t="s">
+      <c r="B88" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C88" t="s">
@@ -4628,7 +4644,7 @@
       <c r="A89">
         <v>90</v>
       </c>
-      <c r="B89" s="4" t="s">
+      <c r="B89" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C89" t="s">
@@ -4663,7 +4679,7 @@
       <c r="A90">
         <v>91</v>
       </c>
-      <c r="B90" s="4" t="s">
+      <c r="B90" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C90" t="s">
@@ -4698,7 +4714,7 @@
       <c r="A91">
         <v>92</v>
       </c>
-      <c r="B91" s="4" t="s">
+      <c r="B91" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C91" t="s">
@@ -4733,7 +4749,7 @@
       <c r="A92">
         <v>93</v>
       </c>
-      <c r="B92" s="4" t="s">
+      <c r="B92" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C92" t="s">
@@ -4768,7 +4784,7 @@
       <c r="A93">
         <v>94</v>
       </c>
-      <c r="B93" s="4" t="s">
+      <c r="B93" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C93" t="s">
@@ -4800,7 +4816,7 @@
       <c r="A94">
         <v>95</v>
       </c>
-      <c r="B94" s="4" t="s">
+      <c r="B94" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C94" t="s">
@@ -4835,7 +4851,7 @@
       <c r="A95">
         <v>96</v>
       </c>
-      <c r="B95" s="4" t="s">
+      <c r="B95" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C95" t="s">
@@ -4867,7 +4883,7 @@
       <c r="A96">
         <v>97</v>
       </c>
-      <c r="B96" s="4" t="s">
+      <c r="B96" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C96" t="s">
@@ -4902,7 +4918,7 @@
       <c r="A97">
         <v>98</v>
       </c>
-      <c r="B97" s="4" t="s">
+      <c r="B97" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C97" t="s">
@@ -4934,7 +4950,7 @@
       <c r="A98">
         <v>99</v>
       </c>
-      <c r="B98" s="4" t="s">
+      <c r="B98" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C98" t="s">
@@ -4969,7 +4985,7 @@
       <c r="A99">
         <v>100</v>
       </c>
-      <c r="B99" s="4" t="s">
+      <c r="B99" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C99" t="s">
@@ -5001,7 +5017,7 @@
       <c r="A100">
         <v>101</v>
       </c>
-      <c r="B100" s="4" t="s">
+      <c r="B100" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C100" t="s">
@@ -5036,7 +5052,7 @@
       <c r="A101">
         <v>102</v>
       </c>
-      <c r="B101" s="4" t="s">
+      <c r="B101" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C101" t="s">
@@ -5068,7 +5084,7 @@
       <c r="A102">
         <v>103</v>
       </c>
-      <c r="B102" s="4" t="s">
+      <c r="B102" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C102" t="s">
@@ -5103,7 +5119,7 @@
       <c r="A103">
         <v>104</v>
       </c>
-      <c r="B103" s="4" t="s">
+      <c r="B103" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C103" t="s">
@@ -5135,7 +5151,7 @@
       <c r="A104">
         <v>105</v>
       </c>
-      <c r="B104" s="4" t="s">
+      <c r="B104" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C104" t="s">
@@ -5170,7 +5186,7 @@
       <c r="A105">
         <v>106</v>
       </c>
-      <c r="B105" s="4" t="s">
+      <c r="B105" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C105" t="s">
@@ -5202,7 +5218,7 @@
       <c r="A106">
         <v>107</v>
       </c>
-      <c r="B106" s="4" t="s">
+      <c r="B106" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C106" t="s">
@@ -5237,7 +5253,7 @@
       <c r="A107">
         <v>108</v>
       </c>
-      <c r="B107" s="4" t="s">
+      <c r="B107" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C107" t="s">
@@ -5269,7 +5285,7 @@
       <c r="A108">
         <v>109</v>
       </c>
-      <c r="B108" s="4" t="s">
+      <c r="B108" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C108" t="s">
@@ -5304,7 +5320,7 @@
       <c r="A109">
         <v>110</v>
       </c>
-      <c r="B109" s="4" t="s">
+      <c r="B109" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C109" t="s">
@@ -5336,7 +5352,7 @@
       <c r="A110">
         <v>111</v>
       </c>
-      <c r="B110" s="4" t="s">
+      <c r="B110" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C110" t="s">
@@ -5371,7 +5387,7 @@
       <c r="A111">
         <v>112</v>
       </c>
-      <c r="B111" s="4" t="s">
+      <c r="B111" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C111" t="s">
@@ -5403,7 +5419,7 @@
       <c r="A112">
         <v>113</v>
       </c>
-      <c r="B112" s="4" t="s">
+      <c r="B112" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C112" t="s">
@@ -5438,7 +5454,7 @@
       <c r="A113">
         <v>114</v>
       </c>
-      <c r="B113" s="4" t="s">
+      <c r="B113" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C113" t="s">
@@ -5470,7 +5486,7 @@
       <c r="A114">
         <v>115</v>
       </c>
-      <c r="B114" s="4" t="s">
+      <c r="B114" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C114" t="s">
@@ -5505,7 +5521,7 @@
       <c r="A115">
         <v>116</v>
       </c>
-      <c r="B115" s="4" t="s">
+      <c r="B115" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C115" t="s">
@@ -5537,7 +5553,7 @@
       <c r="A116">
         <v>117</v>
       </c>
-      <c r="B116" s="4" t="s">
+      <c r="B116" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C116" t="s">
@@ -5572,7 +5588,7 @@
       <c r="A117">
         <v>118</v>
       </c>
-      <c r="B117" s="4" t="s">
+      <c r="B117" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C117" t="s">
@@ -5607,7 +5623,7 @@
       <c r="A118">
         <v>119</v>
       </c>
-      <c r="B118" s="4" t="s">
+      <c r="B118" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C118" t="s">
@@ -5639,7 +5655,7 @@
       <c r="A119">
         <v>120</v>
       </c>
-      <c r="B119" s="4" t="s">
+      <c r="B119" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C119" t="s">
@@ -5662,11 +5678,11 @@
         <v>5117</v>
       </c>
       <c r="I119" t="str">
-        <f t="shared" ref="I119:I193" si="4">_xlfn.CONCAT("{#fig-",H119,"}")</f>
+        <f t="shared" ref="I119:I194" si="4">_xlfn.CONCAT("{#fig-",H119,"}")</f>
         <v>{#fig-5117}</v>
       </c>
       <c r="J119" t="str">
-        <f t="shared" ref="J119:J181" si="5">IF(E119,_xlfn.CONCAT("![",G119,"](figures/",B119,"/",F119,")",I119),"")</f>
+        <f t="shared" ref="J119:J182" si="5">IF(E119,_xlfn.CONCAT("![",G119,"](figures/",B119,"/",F119,")",I119),"")</f>
         <v>![Creating a new Cosmos DB container](figures/ad/ss_database_001_ann.png){#fig-5117}</v>
       </c>
     </row>
@@ -5674,7 +5690,7 @@
       <c r="A120">
         <v>121</v>
       </c>
-      <c r="B120" s="4" t="s">
+      <c r="B120" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C120" t="s">
@@ -5706,7 +5722,7 @@
       <c r="A121">
         <v>122</v>
       </c>
-      <c r="B121" s="4" t="s">
+      <c r="B121" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C121" t="s">
@@ -5741,7 +5757,7 @@
       <c r="A122">
         <v>123</v>
       </c>
-      <c r="B122" s="4" t="s">
+      <c r="B122" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C122" t="s">
@@ -5773,7 +5789,7 @@
       <c r="A123">
         <v>124</v>
       </c>
-      <c r="B123" s="4" t="s">
+      <c r="B123" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C123" t="s">
@@ -5808,7 +5824,7 @@
       <c r="A124">
         <v>125</v>
       </c>
-      <c r="B124" s="4" t="s">
+      <c r="B124" s="5" t="s">
         <v>99</v>
       </c>
       <c r="C124" t="s">
@@ -5843,7 +5859,7 @@
       <c r="A125">
         <v>126</v>
       </c>
-      <c r="B125" s="5" t="s">
+      <c r="B125" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C125" t="s">
@@ -5878,7 +5894,7 @@
       <c r="A126">
         <v>127</v>
       </c>
-      <c r="B126" s="5" t="s">
+      <c r="B126" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C126" t="s">
@@ -5913,11 +5929,11 @@
       <c r="A127">
         <v>128</v>
       </c>
-      <c r="B127" s="5" t="s">
+      <c r="B127" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C127" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D127" t="b">
         <v>0</v>
@@ -5926,29 +5942,29 @@
         <v>1</v>
       </c>
       <c r="F127" t="s">
-        <v>292</v>
+        <v>331</v>
       </c>
       <c r="G127" t="s">
-        <v>296</v>
+        <v>332</v>
       </c>
       <c r="H127" s="1" t="str" cm="1">
         <f t="array" ref="H127">CRC16HASH(F127)</f>
-        <v>CB8E</v>
+        <v>3399</v>
       </c>
       <c r="I127" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-CB8E}</v>
+        <v>{#fig-3399}</v>
       </c>
       <c r="J127" t="str">
         <f t="shared" si="5"/>
-        <v>![Microsoft's public earnings release page](figures/kb/ss_storage_001_clean.png){#fig-CB8E}</v>
+        <v>![Enrichment tasks for documents](figures/kb/il_enrichment_001.png){#fig-3399}</v>
       </c>
     </row>
     <row r="128" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>129</v>
       </c>
-      <c r="B128" s="5" t="s">
+      <c r="B128" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C128" t="s">
@@ -5958,367 +5974,367 @@
         <v>0</v>
       </c>
       <c r="E128" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F128" t="s">
-        <v>106</v>
+        <v>292</v>
+      </c>
+      <c r="G128" t="s">
+        <v>296</v>
       </c>
       <c r="H128" s="1" t="str" cm="1">
         <f t="array" ref="H128">CRC16HASH(F128)</f>
-        <v>449C</v>
+        <v>CB8E</v>
       </c>
       <c r="I128" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-449C}</v>
+        <v>{#fig-CB8E}</v>
       </c>
       <c r="J128" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>![Microsoft's public earnings release page](figures/kb/ss_storage_001_clean.png){#fig-CB8E}</v>
       </c>
     </row>
     <row r="129" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>130</v>
       </c>
-      <c r="B129" s="5" t="s">
+      <c r="B129" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C129" t="s">
         <v>4</v>
       </c>
       <c r="D129" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E129" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F129" t="s">
-        <v>105</v>
-      </c>
-      <c r="G129" t="s">
-        <v>297</v>
+        <v>106</v>
       </c>
       <c r="H129" s="1" t="str" cm="1">
         <f t="array" ref="H129">CRC16HASH(F129)</f>
-        <v>693E</v>
+        <v>449C</v>
       </c>
       <c r="I129" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-693E}</v>
+        <v>{#fig-449C}</v>
       </c>
       <c r="J129" t="str">
         <f t="shared" si="5"/>
-        <v>![Creating a new Container in Azure Storage](figures/kb/ss_portal_001_ann.png){#fig-693E}</v>
+        <v/>
       </c>
     </row>
     <row r="130" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>131</v>
       </c>
-      <c r="B130" s="5" t="s">
+      <c r="B130" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C130" t="s">
         <v>4</v>
       </c>
       <c r="D130" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E130" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F130" t="s">
-        <v>294</v>
+        <v>105</v>
+      </c>
+      <c r="G130" t="s">
+        <v>297</v>
       </c>
       <c r="H130" s="1" t="str" cm="1">
         <f t="array" ref="H130">CRC16HASH(F130)</f>
-        <v>8F81</v>
+        <v>693E</v>
       </c>
       <c r="I130" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-8F81}</v>
+        <v>{#fig-693E}</v>
       </c>
       <c r="J130" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>![Creating a new Container in Azure Storage](figures/kb/ss_portal_001_ann.png){#fig-693E}</v>
       </c>
     </row>
     <row r="131" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A131">
         <v>132</v>
       </c>
-      <c r="B131" s="5" t="s">
+      <c r="B131" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C131" t="s">
         <v>4</v>
       </c>
       <c r="D131" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E131" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F131" t="s">
-        <v>295</v>
-      </c>
-      <c r="G131" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="H131" s="1" t="str" cm="1">
         <f t="array" ref="H131">CRC16HASH(F131)</f>
-        <v>72EE</v>
+        <v>8F81</v>
       </c>
       <c r="I131" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-72EE}</v>
+        <v>{#fig-8F81}</v>
       </c>
       <c r="J131" t="str">
         <f t="shared" si="5"/>
-        <v>![Uploading the financial reports to Azure Storage](figures/kb/ss_storage_002_ann.png){#fig-72EE}</v>
+        <v/>
       </c>
     </row>
     <row r="132" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A132">
         <v>133</v>
       </c>
-      <c r="B132" s="5" t="s">
+      <c r="B132" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C132" t="s">
         <v>4</v>
       </c>
       <c r="D132" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E132" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F132" t="s">
-        <v>283</v>
+        <v>295</v>
+      </c>
+      <c r="G132" t="s">
+        <v>293</v>
       </c>
       <c r="H132" s="1" t="str" cm="1">
         <f t="array" ref="H132">CRC16HASH(F132)</f>
-        <v>ECD1</v>
+        <v>72EE</v>
       </c>
       <c r="I132" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-ECD1}</v>
+        <v>{#fig-72EE}</v>
       </c>
       <c r="J132" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>![Uploading the financial reports to Azure Storage](figures/kb/ss_storage_002_ann.png){#fig-72EE}</v>
       </c>
     </row>
     <row r="133" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A133">
         <v>134</v>
       </c>
-      <c r="B133" s="5" t="s">
+      <c r="B133" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C133" t="s">
         <v>4</v>
       </c>
       <c r="D133" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E133" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F133" t="s">
-        <v>284</v>
-      </c>
-      <c r="G133" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="H133" s="1" t="str" cm="1">
         <f t="array" ref="H133">CRC16HASH(F133)</f>
-        <v>F62E</v>
+        <v>ECD1</v>
       </c>
       <c r="I133" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-F62E}</v>
+        <v>{#fig-ECD1}</v>
       </c>
       <c r="J133" t="str">
         <f t="shared" si="5"/>
-        <v>![Importing data into Azure AI Search](figures/kb/ss_search_001_ann.png){#fig-F62E}</v>
+        <v/>
       </c>
     </row>
     <row r="134" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A134">
         <v>135</v>
       </c>
-      <c r="B134" s="5" t="s">
+      <c r="B134" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C134" t="s">
         <v>4</v>
       </c>
       <c r="D134" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E134" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F134" t="s">
-        <v>287</v>
+        <v>284</v>
+      </c>
+      <c r="G134" t="s">
+        <v>285</v>
       </c>
       <c r="H134" s="1" t="str" cm="1">
         <f t="array" ref="H134">CRC16HASH(F134)</f>
-        <v>A8DE</v>
+        <v>F62E</v>
       </c>
       <c r="I134" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-A8DE}</v>
+        <v>{#fig-F62E}</v>
       </c>
       <c r="J134" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>![Importing data into Azure AI Search](figures/kb/ss_search_001_ann.png){#fig-F62E}</v>
       </c>
     </row>
     <row r="135" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A135">
         <v>136</v>
       </c>
-      <c r="B135" s="5" t="s">
+      <c r="B135" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C135" t="s">
         <v>4</v>
       </c>
       <c r="D135" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E135" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F135" t="s">
-        <v>288</v>
-      </c>
-      <c r="G135" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="H135" s="1" t="str" cm="1">
         <f t="array" ref="H135">CRC16HASH(F135)</f>
-        <v>63A</v>
+        <v>A8DE</v>
       </c>
       <c r="I135" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-63A}</v>
+        <v>{#fig-A8DE}</v>
       </c>
       <c r="J135" t="str">
         <f t="shared" si="5"/>
-        <v>![Selecting the Azure Blob Storage built-in indexer](figures/kb/ss_search_002_ann.png){#fig-63A}</v>
+        <v/>
       </c>
     </row>
     <row r="136" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A136">
         <v>137</v>
       </c>
-      <c r="B136" s="5" t="s">
+      <c r="B136" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C136" t="s">
         <v>4</v>
       </c>
       <c r="D136" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E136" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F136" t="s">
-        <v>291</v>
+        <v>288</v>
+      </c>
+      <c r="G136" t="s">
+        <v>286</v>
       </c>
       <c r="H136" s="1" t="str" cm="1">
         <f t="array" ref="H136">CRC16HASH(F136)</f>
-        <v>54DA</v>
+        <v>63A</v>
       </c>
       <c r="I136" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-54DA}</v>
+        <v>{#fig-63A}</v>
       </c>
       <c r="J136" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>![Selecting the Azure Blob Storage built-in indexer](figures/kb/ss_search_002_ann.png){#fig-63A}</v>
       </c>
     </row>
     <row r="137" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A137">
         <v>138</v>
       </c>
-      <c r="B137" s="5" t="s">
+      <c r="B137" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C137" t="s">
         <v>4</v>
       </c>
       <c r="D137" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E137" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F137" t="s">
-        <v>290</v>
-      </c>
-      <c r="G137" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="H137" s="1" t="str" cm="1">
         <f t="array" ref="H137">CRC16HASH(F137)</f>
-        <v>9637</v>
+        <v>54DA</v>
       </c>
       <c r="I137" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-9637}</v>
+        <v>{#fig-54DA}</v>
       </c>
       <c r="J137" t="str">
         <f t="shared" si="5"/>
-        <v>![Selecting the Keyword search scenario](figures/kb/ss_search_003_ann.png){#fig-9637}</v>
+        <v/>
       </c>
     </row>
     <row r="138" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A138">
         <v>139</v>
       </c>
-      <c r="B138" s="5" t="s">
+      <c r="B138" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C138" t="s">
         <v>4</v>
       </c>
       <c r="D138" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E138" t="b">
         <v>1</v>
       </c>
       <c r="F138" t="s">
-        <v>298</v>
+        <v>290</v>
       </c>
       <c r="G138" t="s">
-        <v>299</v>
+        <v>289</v>
       </c>
       <c r="H138" s="1" t="str" cm="1">
         <f t="array" ref="H138">CRC16HASH(F138)</f>
-        <v>20C0</v>
+        <v>9637</v>
       </c>
       <c r="I138" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-20C0}</v>
+        <v>{#fig-9637}</v>
       </c>
       <c r="J138" t="str">
-        <f>IF(E138,_xlfn.CONCAT("![",G138,"](figures/",B138,"/",F138,")",I138),"")</f>
-        <v>![Connecting to data for the Keyword search](figures/kb/ss_search_004_clean.png){#fig-20C0}</v>
+        <f t="shared" si="5"/>
+        <v>![Selecting the Keyword search scenario](figures/kb/ss_search_003_ann.png){#fig-9637}</v>
       </c>
     </row>
     <row r="139" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A139">
         <v>140</v>
       </c>
-      <c r="B139" s="5" t="s">
+      <c r="B139" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C139" t="s">
@@ -6328,233 +6344,233 @@
         <v>0</v>
       </c>
       <c r="E139" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F139" t="s">
-        <v>305</v>
+        <v>298</v>
+      </c>
+      <c r="G139" t="s">
+        <v>299</v>
       </c>
       <c r="H139" s="1" t="str" cm="1">
         <f t="array" ref="H139">CRC16HASH(F139)</f>
-        <v>258D</v>
+        <v>20C0</v>
       </c>
       <c r="I139" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-258D}</v>
+        <v>{#fig-20C0}</v>
       </c>
       <c r="J139" t="str">
-        <f t="shared" si="5"/>
-        <v/>
+        <f>IF(E139,_xlfn.CONCAT("![",G139,"](figures/",B139,"/",F139,")",I139),"")</f>
+        <v>![Connecting to data for the Keyword search](figures/kb/ss_search_004_clean.png){#fig-20C0}</v>
       </c>
     </row>
     <row r="140" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A140">
         <v>141</v>
       </c>
-      <c r="B140" s="5" t="s">
+      <c r="B140" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C140" t="s">
         <v>4</v>
       </c>
       <c r="D140" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E140" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F140" t="s">
-        <v>306</v>
-      </c>
-      <c r="G140" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H140" s="1" t="str" cm="1">
         <f t="array" ref="H140">CRC16HASH(F140)</f>
-        <v>6AFC</v>
+        <v>258D</v>
       </c>
       <c r="I140" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-6AFC}</v>
+        <v>{#fig-258D}</v>
       </c>
       <c r="J140" t="str">
         <f t="shared" si="5"/>
-        <v>![Enrichments options for Keyword search](figures/kb/ss_enrichments_001_ann.png){#fig-6AFC}</v>
+        <v/>
       </c>
     </row>
     <row r="141" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A141">
         <v>142</v>
       </c>
-      <c r="B141" s="5" t="s">
+      <c r="B141" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C141" t="s">
         <v>4</v>
       </c>
       <c r="D141" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E141" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F141" t="s">
-        <v>300</v>
+        <v>306</v>
+      </c>
+      <c r="G141" t="s">
+        <v>308</v>
       </c>
       <c r="H141" s="1" t="str" cm="1">
         <f t="array" ref="H141">CRC16HASH(F141)</f>
-        <v>6182</v>
+        <v>6AFC</v>
       </c>
       <c r="I141" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-6182}</v>
+        <v>{#fig-6AFC}</v>
       </c>
       <c r="J141" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>![Enrichments options for Keyword search](figures/kb/ss_enrichments_001_ann.png){#fig-6AFC}</v>
       </c>
     </row>
     <row r="142" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A142">
         <v>143</v>
       </c>
-      <c r="B142" s="5" t="s">
+      <c r="B142" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C142" t="s">
         <v>4</v>
       </c>
       <c r="D142" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E142" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F142" t="s">
-        <v>301</v>
-      </c>
-      <c r="G142" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="H142" s="1" t="str" cm="1">
         <f t="array" ref="H142">CRC16HASH(F142)</f>
-        <v>9AE8</v>
+        <v>6182</v>
       </c>
       <c r="I142" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-9AE8}</v>
+        <v>{#fig-6182}</v>
       </c>
       <c r="J142" t="str">
         <f t="shared" si="5"/>
-        <v>![Extract entities selection](figures/kb/ss_enrichments_002_ann.png){#fig-9AE8}</v>
+        <v/>
       </c>
     </row>
     <row r="143" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A143">
         <v>144</v>
       </c>
-      <c r="B143" s="5" t="s">
+      <c r="B143" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C143" t="s">
         <v>4</v>
       </c>
       <c r="D143" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E143" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F143" t="s">
-        <v>304</v>
+        <v>301</v>
+      </c>
+      <c r="G143" t="s">
+        <v>302</v>
       </c>
       <c r="H143" s="1" t="str" cm="1">
         <f t="array" ref="H143">CRC16HASH(F143)</f>
-        <v>9D86</v>
+        <v>9AE8</v>
       </c>
       <c r="I143" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-9D86}</v>
+        <v>{#fig-9AE8}</v>
       </c>
       <c r="J143" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>![Extract entities selection](figures/kb/ss_enrichments_002_ann.png){#fig-9AE8}</v>
       </c>
     </row>
     <row r="144" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A144">
         <v>145</v>
       </c>
-      <c r="B144" s="5" t="s">
+      <c r="B144" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C144" t="s">
         <v>4</v>
       </c>
       <c r="D144" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E144" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F144" t="s">
-        <v>303</v>
-      </c>
-      <c r="G144" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="H144" s="1" t="str" cm="1">
         <f t="array" ref="H144">CRC16HASH(F144)</f>
-        <v>AE5</v>
+        <v>9D86</v>
       </c>
       <c r="I144" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-AE5}</v>
+        <v>{#fig-9D86}</v>
       </c>
       <c r="J144" t="str">
         <f t="shared" si="5"/>
-        <v>![Extract text from images selection](figures/kb/ss_enrichments_003_ann.png){#fig-AE5}</v>
+        <v/>
       </c>
     </row>
     <row r="145" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A145">
         <v>146</v>
       </c>
-      <c r="B145" s="5" t="s">
+      <c r="B145" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C145" t="s">
         <v>4</v>
       </c>
       <c r="D145" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E145" t="b">
         <v>1</v>
       </c>
       <c r="F145" t="s">
-        <v>310</v>
+        <v>303</v>
       </c>
       <c r="G145" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="H145" s="1" t="str" cm="1">
         <f t="array" ref="H145">CRC16HASH(F145)</f>
-        <v>E99C</v>
+        <v>AE5</v>
       </c>
       <c r="I145" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-E99C}</v>
+        <v>{#fig-AE5}</v>
       </c>
       <c r="J145" t="str">
         <f t="shared" si="5"/>
-        <v>![Previewing the field mappings](figures/kb/ss_enrichments_004_clean.png){#fig-E99C}</v>
+        <v>![Extract text from images selection](figures/kb/ss_enrichments_003_ann.png){#fig-AE5}</v>
       </c>
     </row>
     <row r="146" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A146">
         <v>147</v>
       </c>
-      <c r="B146" s="5" t="s">
+      <c r="B146" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C146" t="s">
@@ -6564,635 +6580,635 @@
         <v>0</v>
       </c>
       <c r="E146" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F146" t="s">
-        <v>311</v>
+        <v>310</v>
+      </c>
+      <c r="G146" t="s">
+        <v>309</v>
       </c>
       <c r="H146" s="1" t="str" cm="1">
         <f t="array" ref="H146">CRC16HASH(F146)</f>
-        <v>1598</v>
+        <v>E99C</v>
       </c>
       <c r="I146" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-1598}</v>
+        <v>{#fig-E99C}</v>
       </c>
       <c r="J146" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>![Previewing the field mappings](figures/kb/ss_enrichments_004_clean.png){#fig-E99C}</v>
       </c>
     </row>
     <row r="147" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A147">
         <v>148</v>
       </c>
-      <c r="B147" s="5" t="s">
+      <c r="B147" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C147" t="s">
         <v>4</v>
       </c>
       <c r="D147" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E147" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F147" t="s">
-        <v>312</v>
-      </c>
-      <c r="G147" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="H147" s="1" t="str" cm="1">
         <f t="array" ref="H147">CRC16HASH(F147)</f>
-        <v>AACE</v>
+        <v>1598</v>
       </c>
       <c r="I147" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-AACE}</v>
+        <v>{#fig-1598}</v>
       </c>
       <c r="J147" t="str">
         <f t="shared" si="5"/>
-        <v>![Advanced settings for semantic search and re-indexing on a schedule](figures/kb/ss_enrichments_005_ann.png){#fig-AACE}</v>
+        <v/>
       </c>
     </row>
     <row r="148" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A148">
         <v>149</v>
       </c>
-      <c r="B148" s="5" t="s">
+      <c r="B148" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C148" t="s">
         <v>4</v>
       </c>
       <c r="D148" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E148" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F148" t="s">
-        <v>313</v>
+        <v>312</v>
+      </c>
+      <c r="G148" t="s">
+        <v>315</v>
       </c>
       <c r="H148" s="1" t="str" cm="1">
         <f t="array" ref="H148">CRC16HASH(F148)</f>
-        <v>5197</v>
+        <v>AACE</v>
       </c>
       <c r="I148" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-5197}</v>
+        <v>{#fig-AACE}</v>
       </c>
       <c r="J148" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>![Advanced settings for semantic search and re-indexing on a schedule](figures/kb/ss_enrichments_005_ann.png){#fig-AACE}</v>
       </c>
     </row>
     <row r="149" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A149">
         <v>150</v>
       </c>
-      <c r="B149" s="5" t="s">
+      <c r="B149" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C149" t="s">
         <v>4</v>
       </c>
       <c r="D149" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E149" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F149" t="s">
-        <v>314</v>
-      </c>
-      <c r="G149" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="H149" s="1" t="str" cm="1">
         <f t="array" ref="H149">CRC16HASH(F149)</f>
-        <v>5ADA</v>
+        <v>5197</v>
       </c>
       <c r="I149" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-5ADA}</v>
+        <v>{#fig-5197}</v>
       </c>
       <c r="J149" t="str">
         <f t="shared" si="5"/>
-        <v>![Reviewing the selections for Keyword search](figures/kb/ss_enrichments_006_ann.png){#fig-5ADA}</v>
+        <v/>
       </c>
     </row>
     <row r="150" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A150">
         <v>151</v>
       </c>
-      <c r="B150" s="5" t="s">
+      <c r="B150" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C150" t="s">
         <v>4</v>
       </c>
       <c r="D150" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E150" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F150" t="s">
-        <v>317</v>
+        <v>314</v>
+      </c>
+      <c r="G150" t="s">
+        <v>316</v>
       </c>
       <c r="H150" s="1" t="str" cm="1">
         <f t="array" ref="H150">CRC16HASH(F150)</f>
-        <v>DCC4</v>
+        <v>5ADA</v>
       </c>
       <c r="I150" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-DCC4}</v>
+        <v>{#fig-5ADA}</v>
       </c>
       <c r="J150" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>![Reviewing the selections for Keyword search](figures/kb/ss_enrichments_006_ann.png){#fig-5ADA}</v>
       </c>
     </row>
     <row r="151" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A151">
         <v>152</v>
       </c>
-      <c r="B151" s="5" t="s">
+      <c r="B151" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C151" t="s">
         <v>4</v>
       </c>
       <c r="D151" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E151" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F151" t="s">
-        <v>318</v>
-      </c>
-      <c r="G151" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="H151" s="1" t="str" cm="1">
         <f t="array" ref="H151">CRC16HASH(F151)</f>
-        <v>361C</v>
+        <v>DCC4</v>
       </c>
       <c r="I151" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-361C}</v>
+        <v>{#fig-DCC4}</v>
       </c>
       <c r="J151" t="str">
         <f t="shared" si="5"/>
-        <v>![A successful indexing of the Microsoft financial documents from Azure Storage](figures/kb/ss_search_005_ann.png){#fig-361C}</v>
+        <v/>
       </c>
     </row>
     <row r="152" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A152">
         <v>153</v>
       </c>
-      <c r="B152" s="5" t="s">
+      <c r="B152" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C152" t="s">
         <v>4</v>
       </c>
       <c r="D152" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E152" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F152" t="s">
-        <v>223</v>
+        <v>318</v>
+      </c>
+      <c r="G152" t="s">
+        <v>319</v>
       </c>
       <c r="H152" s="1" t="str" cm="1">
         <f t="array" ref="H152">CRC16HASH(F152)</f>
-        <v>6B1C</v>
+        <v>361C</v>
       </c>
       <c r="I152" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-6B1C}</v>
+        <v>{#fig-361C}</v>
       </c>
       <c r="J152" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>![A successful indexing of the Microsoft financial documents from Azure Storage](figures/kb/ss_search_005_ann.png){#fig-361C}</v>
       </c>
     </row>
     <row r="153" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A153">
         <v>154</v>
       </c>
-      <c r="B153" s="5" t="s">
+      <c r="B153" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C153" t="s">
         <v>4</v>
       </c>
       <c r="D153" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E153" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F153" t="s">
-        <v>224</v>
-      </c>
-      <c r="G153" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="H153" s="1" t="str" cm="1">
         <f t="array" ref="H153">CRC16HASH(F153)</f>
-        <v>33E</v>
+        <v>6B1C</v>
       </c>
       <c r="I153" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-33E}</v>
+        <v>{#fig-6B1C}</v>
       </c>
       <c r="J153" t="str">
         <f t="shared" si="5"/>
-        <v>![Connecting to an Azure AI Search resource](figures/kb/ss_knowledge_001_ann.png){#fig-33E}</v>
+        <v/>
       </c>
     </row>
     <row r="154" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A154">
         <v>155</v>
       </c>
-      <c r="B154" s="5" t="s">
+      <c r="B154" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C154" t="s">
         <v>4</v>
       </c>
       <c r="D154" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E154" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F154" t="s">
-        <v>226</v>
+        <v>224</v>
+      </c>
+      <c r="G154" t="s">
+        <v>225</v>
       </c>
       <c r="H154" s="1" t="str" cm="1">
         <f t="array" ref="H154">CRC16HASH(F154)</f>
-        <v>2F13</v>
+        <v>33E</v>
       </c>
       <c r="I154" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-2F13}</v>
+        <v>{#fig-33E}</v>
       </c>
       <c r="J154" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>![Connecting to an Azure AI Search resource](figures/kb/ss_knowledge_001_ann.png){#fig-33E}</v>
       </c>
     </row>
     <row r="155" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A155">
         <v>156</v>
       </c>
-      <c r="B155" s="5" t="s">
+      <c r="B155" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C155" t="s">
         <v>4</v>
       </c>
       <c r="D155" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E155" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F155" t="s">
-        <v>227</v>
-      </c>
-      <c r="G155" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="H155" s="1" t="str" cm="1">
         <f t="array" ref="H155">CRC16HASH(F155)</f>
-        <v>F32A</v>
+        <v>2F13</v>
       </c>
       <c r="I155" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-F32A}</v>
+        <v>{#fig-2F13}</v>
       </c>
       <c r="J155" t="str">
         <f t="shared" si="5"/>
-        <v>![Creating a new Knowledge Base](figures/kb/ss_knowledge_002_ann.png){#fig-F32A}</v>
+        <v/>
       </c>
     </row>
     <row r="156" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A156">
         <v>157</v>
       </c>
-      <c r="B156" s="5" t="s">
+      <c r="B156" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C156" t="s">
         <v>4</v>
       </c>
       <c r="D156" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E156" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F156" t="s">
-        <v>231</v>
+        <v>227</v>
+      </c>
+      <c r="G156" t="s">
+        <v>228</v>
       </c>
       <c r="H156" s="1" t="str" cm="1">
         <f t="array" ref="H156">CRC16HASH(F156)</f>
-        <v>D317</v>
+        <v>F32A</v>
       </c>
       <c r="I156" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-D317}</v>
+        <v>{#fig-F32A}</v>
       </c>
       <c r="J156" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>![Creating a new Knowledge Base](figures/kb/ss_knowledge_002_ann.png){#fig-F32A}</v>
       </c>
     </row>
     <row r="157" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A157">
         <v>158</v>
       </c>
-      <c r="B157" s="5" t="s">
+      <c r="B157" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C157" t="s">
         <v>4</v>
       </c>
       <c r="D157" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E157" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F157" t="s">
-        <v>320</v>
-      </c>
-      <c r="G157" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="H157" s="1" t="str" cm="1">
         <f t="array" ref="H157">CRC16HASH(F157)</f>
-        <v>6327</v>
+        <v>D317</v>
       </c>
       <c r="I157" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-6327}</v>
+        <v>{#fig-D317}</v>
       </c>
       <c r="J157" t="str">
         <f t="shared" si="5"/>
-        <v>![Selecting a Knowledge Base type](figures/kb/ss_knowledge_003_ann.png){#fig-6327}</v>
+        <v/>
       </c>
     </row>
     <row r="158" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A158">
         <v>159</v>
       </c>
-      <c r="B158" s="5" t="s">
+      <c r="B158" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C158" t="s">
         <v>4</v>
       </c>
       <c r="D158" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E158" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F158" t="s">
-        <v>322</v>
+        <v>320</v>
+      </c>
+      <c r="G158" t="s">
+        <v>232</v>
       </c>
       <c r="H158" s="1" t="str" cm="1">
         <f t="array" ref="H158">CRC16HASH(F158)</f>
-        <v>A70D</v>
+        <v>6327</v>
       </c>
       <c r="I158" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-A70D}</v>
+        <v>{#fig-6327}</v>
       </c>
       <c r="J158" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>![Selecting a Knowledge Base type](figures/kb/ss_knowledge_003_ann.png){#fig-6327}</v>
       </c>
     </row>
     <row r="159" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A159">
         <v>160</v>
       </c>
-      <c r="B159" s="5" t="s">
+      <c r="B159" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C159" t="s">
         <v>4</v>
       </c>
       <c r="D159" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E159" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F159" t="s">
-        <v>323</v>
-      </c>
-      <c r="G159" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="H159" s="1" t="str" cm="1">
         <f t="array" ref="H159">CRC16HASH(F159)</f>
-        <v>5301</v>
+        <v>A70D</v>
       </c>
       <c r="I159" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-5301}</v>
+        <v>{#fig-A70D}</v>
       </c>
       <c r="J159" t="str">
         <f t="shared" si="5"/>
-        <v>![Connecting to the Search Index](figures/kb/ss_knowledge_004_ann.png){#fig-5301}</v>
+        <v/>
       </c>
     </row>
     <row r="160" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A160">
         <v>161</v>
       </c>
-      <c r="B160" s="5" t="s">
+      <c r="B160" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C160" t="s">
         <v>4</v>
       </c>
       <c r="D160" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E160" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F160" t="s">
-        <v>324</v>
+        <v>323</v>
+      </c>
+      <c r="G160" t="s">
+        <v>321</v>
       </c>
       <c r="H160" s="1" t="str" cm="1">
         <f t="array" ref="H160">CRC16HASH(F160)</f>
-        <v>5B09</v>
+        <v>5301</v>
       </c>
       <c r="I160" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-5B09}</v>
+        <v>{#fig-5301}</v>
       </c>
       <c r="J160" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>![Connecting to the Search Index](figures/kb/ss_knowledge_004_ann.png){#fig-5301}</v>
       </c>
     </row>
     <row r="161" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A161">
         <v>162</v>
       </c>
-      <c r="B161" s="5" t="s">
+      <c r="B161" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C161" t="s">
         <v>4</v>
       </c>
       <c r="D161" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E161" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F161" t="s">
-        <v>325</v>
-      </c>
-      <c r="G161" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="H161" s="1" t="str" cm="1">
         <f t="array" ref="H161">CRC16HASH(F161)</f>
-        <v>C30C</v>
+        <v>5B09</v>
       </c>
       <c r="I161" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-C30C}</v>
+        <v>{#fig-5B09}</v>
       </c>
       <c r="J161" t="str">
         <f t="shared" si="5"/>
-        <v>![Final steps in creating the knowledge base](figures/kb/ss_knowledge_005_ann.png){#fig-C30C}</v>
+        <v/>
       </c>
     </row>
     <row r="162" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A162">
         <v>163</v>
       </c>
-      <c r="B162" s="5" t="s">
+      <c r="B162" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C162" t="s">
         <v>4</v>
       </c>
       <c r="D162" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E162" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F162" t="s">
-        <v>151</v>
+        <v>325</v>
+      </c>
+      <c r="G162" t="s">
+        <v>326</v>
       </c>
       <c r="H162" s="1" t="str" cm="1">
         <f t="array" ref="H162">CRC16HASH(F162)</f>
-        <v>AFD</v>
+        <v>C30C</v>
       </c>
       <c r="I162" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-AFD}</v>
+        <v>{#fig-C30C}</v>
       </c>
       <c r="J162" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>![Final steps in creating the knowledge base](figures/kb/ss_knowledge_005_ann.png){#fig-C30C}</v>
       </c>
     </row>
     <row r="163" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A163">
         <v>164</v>
       </c>
-      <c r="B163" s="5" t="s">
+      <c r="B163" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C163" t="s">
         <v>4</v>
       </c>
       <c r="D163" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E163" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F163" t="s">
-        <v>152</v>
-      </c>
-      <c r="G163" t="s">
-        <v>328</v>
+        <v>151</v>
       </c>
       <c r="H163" s="1" t="str" cm="1">
         <f t="array" ref="H163">CRC16HASH(F163)</f>
-        <v>1BC</v>
+        <v>AFD</v>
       </c>
       <c r="I163" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-1BC}</v>
+        <v>{#fig-AFD}</v>
       </c>
       <c r="J163" t="str">
         <f t="shared" si="5"/>
-        <v>![Connecting the Agent to the knowledge base](figures/kb/ss_agent_001_ann.png){#fig-1BC}</v>
+        <v/>
       </c>
     </row>
     <row r="164" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A164">
         <v>165</v>
       </c>
-      <c r="B164" s="5" t="s">
+      <c r="B164" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C164" t="s">
         <v>4</v>
       </c>
       <c r="D164" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E164" t="b">
         <v>1</v>
       </c>
       <c r="F164" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G164" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="H164" s="1" t="str" cm="1">
         <f t="array" ref="H164">CRC16HASH(F164)</f>
-        <v>4EF2</v>
+        <v>1BC</v>
       </c>
       <c r="I164" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-4EF2}</v>
+        <v>{#fig-1BC}</v>
       </c>
       <c r="J164" t="str">
         <f t="shared" si="5"/>
-        <v>![Asking the Robo CFO Agent about year over year revenue](figures/kb/ss_agent_002_clean.png){#fig-4EF2}</v>
+        <v>![Connecting the Agent to the knowledge base](figures/kb/ss_agent_001_ann.png){#fig-1BC}</v>
       </c>
     </row>
     <row r="165" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A165">
         <v>166</v>
       </c>
-      <c r="B165" s="5" t="s">
+      <c r="B165" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C165" t="s">
@@ -7205,29 +7221,29 @@
         <v>1</v>
       </c>
       <c r="F165" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="G165" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="H165" s="1" t="str" cm="1">
         <f t="array" ref="H165">CRC16HASH(F165)</f>
-        <v>B2F6</v>
+        <v>4EF2</v>
       </c>
       <c r="I165" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-B2F6}</v>
+        <v>{#fig-4EF2}</v>
       </c>
       <c r="J165" t="str">
         <f t="shared" si="5"/>
-        <v>![Asking about Microsoft's 2026 outlook](figures/kb/ss_agent_003_clean.png){#fig-B2F6}</v>
+        <v>![Asking the Robo CFO Agent about year over year revenue](figures/kb/ss_agent_002_clean.png){#fig-4EF2}</v>
       </c>
     </row>
     <row r="166" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A166">
         <v>167</v>
       </c>
-      <c r="B166" s="5" t="s">
+      <c r="B166" s="6" t="s">
         <v>100</v>
       </c>
       <c r="C166" t="s">
@@ -7240,22 +7256,22 @@
         <v>1</v>
       </c>
       <c r="F166" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="G166" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="H166" s="1" t="str" cm="1">
         <f t="array" ref="H166">CRC16HASH(F166)</f>
-        <v>C6EC</v>
+        <v>B2F6</v>
       </c>
       <c r="I166" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-C6EC}</v>
+        <v>{#fig-B2F6}</v>
       </c>
       <c r="J166" t="str">
         <f t="shared" si="5"/>
-        <v>![The "Microsoft FY26 Q2 Outlook" PowerPoint slide](figures/kb/ss_agent_004_clean.png){#fig-C6EC}</v>
+        <v>![Asking about Microsoft's 2026 outlook](figures/kb/ss_agent_003_clean.png){#fig-B2F6}</v>
       </c>
     </row>
     <row r="167" spans="1:10" x14ac:dyDescent="0.25">
@@ -7263,7 +7279,7 @@
         <v>168</v>
       </c>
       <c r="B167" s="6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C167" t="s">
         <v>4</v>
@@ -7272,163 +7288,166 @@
         <v>0</v>
       </c>
       <c r="E167" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F167" t="s">
-        <v>233</v>
+        <v>157</v>
+      </c>
+      <c r="G167" t="s">
+        <v>329</v>
       </c>
       <c r="H167" s="1" t="str" cm="1">
         <f t="array" ref="H167">CRC16HASH(F167)</f>
-        <v>8E61</v>
+        <v>C6EC</v>
       </c>
       <c r="I167" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-8E61}</v>
+        <v>{#fig-C6EC}</v>
       </c>
       <c r="J167" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>![The "Microsoft FY26 Q2 Outlook" PowerPoint slide](figures/kb/ss_agent_004_clean.png){#fig-C6EC}</v>
       </c>
     </row>
     <row r="168" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A168">
         <v>169</v>
       </c>
-      <c r="B168" s="6" t="s">
+      <c r="B168" s="7" t="s">
         <v>101</v>
       </c>
       <c r="C168" t="s">
         <v>4</v>
       </c>
       <c r="D168" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E168" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F168" t="s">
-        <v>234</v>
-      </c>
-      <c r="G168" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="H168" s="1" t="str" cm="1">
         <f t="array" ref="H168">CRC16HASH(F168)</f>
-        <v>706E</v>
+        <v>8E61</v>
       </c>
       <c r="I168" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-706E}</v>
+        <v>{#fig-8E61}</v>
       </c>
       <c r="J168" t="str">
         <f t="shared" si="5"/>
-        <v>![Creating a new fine-tuning job](figures/ft/ss_finetune_001_ann.png){#fig-706E}</v>
+        <v/>
       </c>
     </row>
     <row r="169" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A169">
         <v>170</v>
       </c>
-      <c r="B169" s="6" t="s">
+      <c r="B169" s="7" t="s">
         <v>101</v>
       </c>
       <c r="C169" t="s">
         <v>4</v>
       </c>
       <c r="D169" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E169" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F169" t="s">
-        <v>235</v>
+        <v>234</v>
+      </c>
+      <c r="G169" t="s">
+        <v>238</v>
       </c>
       <c r="H169" s="1" t="str" cm="1">
         <f t="array" ref="H169">CRC16HASH(F169)</f>
-        <v>CA6E</v>
+        <v>706E</v>
       </c>
       <c r="I169" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-CA6E}</v>
+        <v>{#fig-706E}</v>
       </c>
       <c r="J169" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>![Creating a new fine-tuning job](figures/ft/ss_finetune_001_ann.png){#fig-706E}</v>
       </c>
     </row>
     <row r="170" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A170">
         <v>171</v>
       </c>
-      <c r="B170" s="6" t="s">
+      <c r="B170" s="7" t="s">
         <v>101</v>
       </c>
       <c r="C170" t="s">
         <v>4</v>
       </c>
       <c r="D170" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E170" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F170" t="s">
-        <v>236</v>
-      </c>
-      <c r="G170" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="H170" s="1" t="str" cm="1">
         <f t="array" ref="H170">CRC16HASH(F170)</f>
-        <v>807A</v>
+        <v>CA6E</v>
       </c>
       <c r="I170" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-807A}</v>
+        <v>{#fig-CA6E}</v>
       </c>
       <c r="J170" t="str">
         <f t="shared" si="5"/>
-        <v>![Defining the fine-tuning job setting](figures/ft/ss_finetune_002_ann.png){#fig-807A}</v>
+        <v/>
       </c>
     </row>
     <row r="171" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A171">
         <v>172</v>
       </c>
-      <c r="B171" s="6" t="s">
+      <c r="B171" s="7" t="s">
         <v>101</v>
       </c>
       <c r="C171" t="s">
         <v>4</v>
       </c>
       <c r="D171" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E171" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F171" t="s">
-        <v>239</v>
+        <v>236</v>
+      </c>
+      <c r="G171" t="s">
+        <v>237</v>
       </c>
       <c r="H171" s="1" t="str" cm="1">
         <f t="array" ref="H171">CRC16HASH(F171)</f>
-        <v>366A</v>
+        <v>807A</v>
       </c>
       <c r="I171" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-366A}</v>
+        <v>{#fig-807A}</v>
       </c>
       <c r="J171" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>![Defining the fine-tuning job setting](figures/ft/ss_finetune_002_ann.png){#fig-807A}</v>
       </c>
     </row>
     <row r="172" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A172">
         <v>173</v>
       </c>
-      <c r="B172" s="6" t="s">
+      <c r="B172" s="7" t="s">
         <v>101</v>
       </c>
       <c r="C172" t="s">
@@ -7441,15 +7460,15 @@
         <v>0</v>
       </c>
       <c r="F172" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="H172" s="1" t="str" cm="1">
         <f t="array" ref="H172">CRC16HASH(F172)</f>
-        <v>394C</v>
+        <v>366A</v>
       </c>
       <c r="I172" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-394C}</v>
+        <v>{#fig-366A}</v>
       </c>
       <c r="J172" t="str">
         <f t="shared" si="5"/>
@@ -7460,74 +7479,74 @@
       <c r="A173">
         <v>174</v>
       </c>
-      <c r="B173" s="6" t="s">
+      <c r="B173" s="7" t="s">
         <v>101</v>
       </c>
       <c r="C173" t="s">
         <v>4</v>
       </c>
       <c r="D173" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E173" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F173" t="s">
-        <v>241</v>
-      </c>
-      <c r="G173" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="H173" s="1" t="str" cm="1">
         <f t="array" ref="H173">CRC16HASH(F173)</f>
-        <v>1077</v>
+        <v>394C</v>
       </c>
       <c r="I173" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-1077}</v>
+        <v>{#fig-394C}</v>
       </c>
       <c r="J173" t="str">
         <f t="shared" si="5"/>
-        <v>![Viewing the status of your new tuning job](figures/ft/ss_finetune_003_ann.png){#fig-1077}</v>
+        <v/>
       </c>
     </row>
     <row r="174" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A174">
         <v>175</v>
       </c>
-      <c r="B174" s="6" t="s">
+      <c r="B174" s="7" t="s">
         <v>101</v>
       </c>
       <c r="C174" t="s">
         <v>4</v>
       </c>
       <c r="D174" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E174" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F174" t="s">
-        <v>243</v>
+        <v>241</v>
+      </c>
+      <c r="G174" t="s">
+        <v>242</v>
       </c>
       <c r="H174" s="1" t="str" cm="1">
         <f t="array" ref="H174">CRC16HASH(F174)</f>
-        <v>4270</v>
+        <v>1077</v>
       </c>
       <c r="I174" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-4270}</v>
+        <v>{#fig-1077}</v>
       </c>
       <c r="J174" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>![Viewing the status of your new tuning job](figures/ft/ss_finetune_003_ann.png){#fig-1077}</v>
       </c>
     </row>
     <row r="175" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A175">
         <v>176</v>
       </c>
-      <c r="B175" s="6" t="s">
+      <c r="B175" s="7" t="s">
         <v>101</v>
       </c>
       <c r="C175" t="s">
@@ -7540,15 +7559,15 @@
         <v>0</v>
       </c>
       <c r="F175" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="H175" s="1" t="str" cm="1">
         <f t="array" ref="H175">CRC16HASH(F175)</f>
-        <v>BE74</v>
+        <v>4270</v>
       </c>
       <c r="I175" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-BE74}</v>
+        <v>{#fig-4270}</v>
       </c>
       <c r="J175" t="str">
         <f t="shared" si="5"/>
@@ -7559,211 +7578,208 @@
       <c r="A176">
         <v>177</v>
       </c>
-      <c r="B176" s="6" t="s">
+      <c r="B176" s="7" t="s">
         <v>101</v>
       </c>
       <c r="C176" t="s">
         <v>4</v>
       </c>
       <c r="D176" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E176" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F176" t="s">
-        <v>251</v>
-      </c>
-      <c r="G176" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="H176" s="1" t="str" cm="1">
         <f t="array" ref="H176">CRC16HASH(F176)</f>
-        <v>B05C</v>
+        <v>BE74</v>
       </c>
       <c r="I176" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-B05C}</v>
+        <v>{#fig-BE74}</v>
       </c>
       <c r="J176" t="str">
         <f t="shared" si="5"/>
-        <v>![The Monitor tab, showing fine-tuning metrics](figures/ft/ss_finetune_005_ann.png){#fig-B05C}</v>
+        <v/>
       </c>
     </row>
     <row r="177" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A177">
         <v>178</v>
       </c>
-      <c r="B177" s="6" t="s">
+      <c r="B177" s="7" t="s">
         <v>101</v>
       </c>
       <c r="C177" t="s">
         <v>4</v>
       </c>
       <c r="D177" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E177" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F177" t="s">
-        <v>253</v>
+        <v>251</v>
+      </c>
+      <c r="G177" t="s">
+        <v>252</v>
       </c>
       <c r="H177" s="1" t="str" cm="1">
         <f t="array" ref="H177">CRC16HASH(F177)</f>
-        <v>FA7B</v>
+        <v>B05C</v>
       </c>
       <c r="I177" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-FA7B}</v>
+        <v>{#fig-B05C}</v>
       </c>
       <c r="J177" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>![The Monitor tab, showing fine-tuning metrics](figures/ft/ss_finetune_005_ann.png){#fig-B05C}</v>
       </c>
     </row>
     <row r="178" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A178">
         <v>179</v>
       </c>
-      <c r="B178" s="6" t="s">
+      <c r="B178" s="7" t="s">
         <v>101</v>
       </c>
       <c r="C178" t="s">
         <v>4</v>
       </c>
       <c r="D178" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E178" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F178" t="s">
-        <v>254</v>
-      </c>
-      <c r="G178" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="H178" s="1" t="str" cm="1">
         <f t="array" ref="H178">CRC16HASH(F178)</f>
-        <v>4048</v>
+        <v>FA7B</v>
       </c>
       <c r="I178" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-4048}</v>
+        <v>{#fig-FA7B}</v>
       </c>
       <c r="J178" t="str">
         <f t="shared" si="5"/>
-        <v>![A completed fine-tuning status and metrics](figures/ft/ss_finetune_006_ann.png){#fig-4048}</v>
+        <v/>
       </c>
     </row>
     <row r="179" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A179">
         <v>180</v>
       </c>
-      <c r="B179" s="6" t="s">
+      <c r="B179" s="7" t="s">
         <v>101</v>
       </c>
       <c r="C179" t="s">
         <v>4</v>
       </c>
       <c r="D179" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E179" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F179" t="s">
-        <v>257</v>
+        <v>254</v>
+      </c>
+      <c r="G179" t="s">
+        <v>255</v>
       </c>
       <c r="H179" s="1" t="str" cm="1">
         <f t="array" ref="H179">CRC16HASH(F179)</f>
-        <v>67F</v>
+        <v>4048</v>
       </c>
       <c r="I179" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-67F}</v>
+        <v>{#fig-4048}</v>
       </c>
       <c r="J179" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>![A completed fine-tuning status and metrics](figures/ft/ss_finetune_006_ann.png){#fig-4048}</v>
       </c>
     </row>
     <row r="180" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A180">
         <v>181</v>
       </c>
-      <c r="B180" s="6" t="s">
+      <c r="B180" s="7" t="s">
         <v>101</v>
       </c>
       <c r="C180" t="s">
         <v>4</v>
       </c>
       <c r="D180" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E180" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F180" t="s">
-        <v>258</v>
-      </c>
-      <c r="G180" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="H180" s="1" t="str" cm="1">
         <f t="array" ref="H180">CRC16HASH(F180)</f>
-        <v>D045</v>
+        <v>67F</v>
       </c>
       <c r="I180" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-D045}</v>
+        <v>{#fig-67F}</v>
       </c>
       <c r="J180" t="str">
         <f t="shared" si="5"/>
-        <v>![Customizing the fine-tuned model deployment](figures/ft/ss_finetune_007_ann.png){#fig-D045}</v>
+        <v/>
       </c>
     </row>
     <row r="181" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A181">
         <v>182</v>
       </c>
-      <c r="B181" s="6" t="s">
+      <c r="B181" s="7" t="s">
         <v>101</v>
       </c>
       <c r="C181" t="s">
         <v>4</v>
       </c>
       <c r="D181" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E181" t="b">
         <v>1</v>
       </c>
       <c r="F181" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="G181" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="H181" s="1" t="str" cm="1">
         <f t="array" ref="H181">CRC16HASH(F181)</f>
-        <v>124F</v>
+        <v>D045</v>
       </c>
       <c r="I181" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-124F}</v>
+        <v>{#fig-D045}</v>
       </c>
       <c r="J181" t="str">
         <f t="shared" si="5"/>
-        <v>![Adding instructions and playing with your new medical assistant model](figures/ft/ss_finetune_008_clean.png){#fig-124F}</v>
+        <v>![Customizing the fine-tuned model deployment](figures/ft/ss_finetune_007_ann.png){#fig-D045}</v>
       </c>
     </row>
     <row r="182" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A182">
         <v>183</v>
       </c>
-      <c r="B182" s="6" t="s">
+      <c r="B182" s="7" t="s">
         <v>101</v>
       </c>
       <c r="C182" t="s">
@@ -7773,163 +7789,166 @@
         <v>0</v>
       </c>
       <c r="E182" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F182" t="s">
-        <v>244</v>
+        <v>260</v>
+      </c>
+      <c r="G182" t="s">
+        <v>259</v>
       </c>
       <c r="H182" s="1" t="str" cm="1">
         <f t="array" ref="H182">CRC16HASH(F182)</f>
-        <v>174F</v>
+        <v>124F</v>
       </c>
       <c r="I182" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-174F}</v>
+        <v>{#fig-124F}</v>
       </c>
       <c r="J182" t="str">
-        <f t="shared" ref="J182:J193" si="6">IF(E182,_xlfn.CONCAT("![",G182,"](figures/",B182,"/",F182,")",I182),"")</f>
-        <v/>
+        <f t="shared" si="5"/>
+        <v>![Adding instructions and playing with your new medical assistant model](figures/ft/ss_finetune_008_clean.png){#fig-124F}</v>
       </c>
     </row>
     <row r="183" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A183">
         <v>184</v>
       </c>
-      <c r="B183" s="6" t="s">
+      <c r="B183" s="7" t="s">
         <v>101</v>
       </c>
       <c r="C183" t="s">
         <v>4</v>
       </c>
       <c r="D183" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E183" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F183" t="s">
-        <v>245</v>
-      </c>
-      <c r="G183" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="H183" s="1" t="str" cm="1">
         <f t="array" ref="H183">CRC16HASH(F183)</f>
-        <v>2C04</v>
+        <v>174F</v>
       </c>
       <c r="I183" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-2C04}</v>
+        <v>{#fig-174F}</v>
       </c>
       <c r="J183" t="str">
-        <f t="shared" si="6"/>
-        <v>![Navigating to the Synthetic generation tab](figures/ft/ss_syntheticdata_001_ann.png){#fig-2C04}</v>
+        <f t="shared" ref="J183:J194" si="6">IF(E183,_xlfn.CONCAT("![",G183,"](figures/",B183,"/",F183,")",I183),"")</f>
+        <v/>
       </c>
     </row>
     <row r="184" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A184">
         <v>185</v>
       </c>
-      <c r="B184" s="6" t="s">
+      <c r="B184" s="7" t="s">
         <v>101</v>
       </c>
       <c r="C184" t="s">
         <v>4</v>
       </c>
       <c r="D184" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E184" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F184" t="s">
-        <v>246</v>
+        <v>245</v>
+      </c>
+      <c r="G184" t="s">
+        <v>249</v>
       </c>
       <c r="H184" s="1" t="str" cm="1">
         <f t="array" ref="H184">CRC16HASH(F184)</f>
-        <v>5340</v>
+        <v>2C04</v>
       </c>
       <c r="I184" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-5340}</v>
+        <v>{#fig-2C04}</v>
       </c>
       <c r="J184" t="str">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-    </row>
-    <row r="185" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>![Navigating to the Synthetic generation tab](figures/ft/ss_syntheticdata_001_ann.png){#fig-2C04}</v>
+      </c>
+    </row>
+    <row r="185" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A185">
         <v>186</v>
       </c>
-      <c r="B185" s="6" t="s">
+      <c r="B185" s="7" t="s">
         <v>101</v>
       </c>
       <c r="C185" t="s">
         <v>4</v>
       </c>
       <c r="D185" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E185" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F185" t="s">
-        <v>247</v>
-      </c>
-      <c r="G185" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="H185" s="1" t="str" cm="1">
         <f t="array" ref="H185">CRC16HASH(F185)</f>
-        <v>DC10</v>
+        <v>5340</v>
       </c>
       <c r="I185" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-DC10}</v>
+        <v>{#fig-5340}</v>
       </c>
       <c r="J185" t="str">
         <f t="shared" si="6"/>
-        <v>![Adding cardiology documents for synthetic data generation](figures/ft/ss_syntheticdata_002_ann.png){#fig-DC10}</v>
-      </c>
-    </row>
-    <row r="186" spans="1:10" x14ac:dyDescent="0.25">
+        <v/>
+      </c>
+    </row>
+    <row r="186" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A186">
         <v>187</v>
       </c>
-      <c r="B186" s="6" t="s">
+      <c r="B186" s="7" t="s">
         <v>101</v>
       </c>
       <c r="C186" t="s">
         <v>4</v>
       </c>
       <c r="D186" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E186" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F186" t="s">
-        <v>261</v>
+        <v>247</v>
+      </c>
+      <c r="G186" t="s">
+        <v>248</v>
       </c>
       <c r="H186" s="1" t="str" cm="1">
         <f t="array" ref="H186">CRC16HASH(F186)</f>
-        <v>AF44</v>
+        <v>DC10</v>
       </c>
       <c r="I186" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-AF44}</v>
+        <v>{#fig-DC10}</v>
       </c>
       <c r="J186" t="str">
         <f t="shared" si="6"/>
-        <v/>
+        <v>![Adding cardiology documents for synthetic data generation](figures/ft/ss_syntheticdata_002_ann.png){#fig-DC10}</v>
       </c>
     </row>
     <row r="187" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A187">
         <v>188</v>
       </c>
-      <c r="B187" s="6" t="s">
+      <c r="B187" s="7" t="s">
         <v>101</v>
       </c>
       <c r="C187" t="s">
@@ -7939,169 +7958,166 @@
         <v>0</v>
       </c>
       <c r="E187" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F187" t="s">
-        <v>262</v>
-      </c>
-      <c r="G187" t="s">
-        <v>268</v>
+        <v>261</v>
       </c>
       <c r="H187" s="1" t="str" cm="1">
         <f t="array" ref="H187">CRC16HASH(F187)</f>
-        <v>2555</v>
+        <v>AF44</v>
       </c>
       <c r="I187" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-2555}</v>
+        <v>{#fig-AF44}</v>
       </c>
       <c r="J187" t="str">
         <f t="shared" si="6"/>
-        <v>![Monitoring the queued synthetic data job](figures/ft/ss_syntheticdata_003a_clean.png){#fig-2555}</v>
+        <v/>
       </c>
     </row>
     <row r="188" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A188">
         <v>189</v>
       </c>
-      <c r="B188" s="6" t="s">
+      <c r="B188" s="7" t="s">
         <v>101</v>
       </c>
       <c r="C188" t="s">
         <v>4</v>
       </c>
       <c r="D188" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E188" t="b">
         <v>1</v>
       </c>
       <c r="F188" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="G188" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="H188" s="1" t="str" cm="1">
         <f t="array" ref="H188">CRC16HASH(F188)</f>
-        <v>4C1D</v>
+        <v>2555</v>
       </c>
       <c r="I188" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-4C1D}</v>
+        <v>{#fig-2555}</v>
       </c>
       <c r="J188" t="str">
         <f t="shared" si="6"/>
-        <v>![Viewing the synthetic data job results](figures/ft/ss_syntheticdata_003_ann.png){#fig-4C1D}</v>
+        <v>![Monitoring the queued synthetic data job](figures/ft/ss_syntheticdata_003a_clean.png){#fig-2555}</v>
       </c>
     </row>
     <row r="189" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A189">
         <v>190</v>
       </c>
-      <c r="B189" s="6" t="s">
+      <c r="B189" s="7" t="s">
         <v>101</v>
       </c>
       <c r="C189" t="s">
         <v>4</v>
       </c>
       <c r="D189" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E189" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F189" t="s">
-        <v>265</v>
+        <v>263</v>
+      </c>
+      <c r="G189" t="s">
+        <v>264</v>
       </c>
       <c r="H189" s="1" t="str" cm="1">
         <f t="array" ref="H189">CRC16HASH(F189)</f>
-        <v>DB5E</v>
+        <v>4C1D</v>
       </c>
       <c r="I189" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-DB5E}</v>
+        <v>{#fig-4C1D}</v>
       </c>
       <c r="J189" t="str">
         <f t="shared" si="6"/>
-        <v/>
+        <v>![Viewing the synthetic data job results](figures/ft/ss_syntheticdata_003_ann.png){#fig-4C1D}</v>
       </c>
     </row>
     <row r="190" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A190">
         <v>191</v>
       </c>
-      <c r="B190" s="6" t="s">
+      <c r="B190" s="7" t="s">
         <v>101</v>
       </c>
       <c r="C190" t="s">
         <v>4</v>
       </c>
       <c r="D190" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E190" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F190" t="s">
-        <v>266</v>
-      </c>
-      <c r="G190" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="H190" s="1" t="str" cm="1">
         <f t="array" ref="H190">CRC16HASH(F190)</f>
-        <v>7C3B</v>
+        <v>DB5E</v>
       </c>
       <c r="I190" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-7C3B}</v>
+        <v>{#fig-DB5E}</v>
       </c>
       <c r="J190" t="str">
         <f t="shared" si="6"/>
-        <v>![Continuing to fine-tune with the new cardiology synthetic data](figures/ft/ss_syntheticdata_004_ann.png){#fig-7C3B}</v>
+        <v/>
       </c>
     </row>
     <row r="191" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A191">
         <v>192</v>
       </c>
-      <c r="B191" s="6" t="s">
+      <c r="B191" s="7" t="s">
         <v>101</v>
       </c>
       <c r="C191" t="s">
         <v>4</v>
       </c>
       <c r="D191" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E191" t="b">
         <v>1</v>
       </c>
       <c r="F191" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="G191" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="H191" s="1" t="str" cm="1">
         <f t="array" ref="H191">CRC16HASH(F191)</f>
-        <v>5DD6</v>
+        <v>7C3B</v>
       </c>
       <c r="I191" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-5DD6}</v>
+        <v>{#fig-7C3B}</v>
       </c>
       <c r="J191" t="str">
         <f t="shared" si="6"/>
-        <v>![Initializing a fine-tuning job from the CLI](figures/ft/ss_cli_001_clean.png){#fig-5DD6}</v>
+        <v>![Continuing to fine-tune with the new cardiology synthetic data](figures/ft/ss_syntheticdata_004_ann.png){#fig-7C3B}</v>
       </c>
     </row>
     <row r="192" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A192">
         <v>193</v>
       </c>
-      <c r="B192" s="6" t="s">
+      <c r="B192" s="7" t="s">
         <v>101</v>
       </c>
       <c r="C192" t="s">
@@ -8114,29 +8130,29 @@
         <v>1</v>
       </c>
       <c r="F192" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="G192" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="H192" s="1" t="str" cm="1">
         <f t="array" ref="H192">CRC16HASH(F192)</f>
-        <v>19D9</v>
+        <v>5DD6</v>
       </c>
       <c r="I192" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-19D9}</v>
+        <v>{#fig-5DD6}</v>
       </c>
       <c r="J192" t="str">
         <f t="shared" si="6"/>
-        <v>![Uploading training data and starting the fine-tuning job](figures/ft/ss_cli_002_clean.png){#fig-19D9}</v>
+        <v>![Initializing a fine-tuning job from the CLI](figures/ft/ss_cli_001_clean.png){#fig-5DD6}</v>
       </c>
     </row>
     <row r="193" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A193">
         <v>194</v>
       </c>
-      <c r="B193" s="6" t="s">
+      <c r="B193" s="7" t="s">
         <v>101</v>
       </c>
       <c r="C193" t="s">
@@ -8149,26 +8165,61 @@
         <v>1</v>
       </c>
       <c r="F193" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="G193" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="H193" s="1" t="str" cm="1">
         <f t="array" ref="H193">CRC16HASH(F193)</f>
-        <v>E5DD</v>
+        <v>19D9</v>
       </c>
       <c r="I193" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-E5DD}</v>
+        <v>{#fig-19D9}</v>
       </c>
       <c r="J193" t="str">
         <f t="shared" si="6"/>
+        <v>![Uploading training data and starting the fine-tuning job](figures/ft/ss_cli_002_clean.png){#fig-19D9}</v>
+      </c>
+    </row>
+    <row r="194" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A194">
+        <v>195</v>
+      </c>
+      <c r="B194" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C194" t="s">
+        <v>4</v>
+      </c>
+      <c r="D194" t="b">
+        <v>0</v>
+      </c>
+      <c r="E194" t="b">
+        <v>1</v>
+      </c>
+      <c r="F194" t="s">
+        <v>272</v>
+      </c>
+      <c r="G194" t="s">
+        <v>274</v>
+      </c>
+      <c r="H194" s="1" t="str" cm="1">
+        <f t="array" ref="H194">CRC16HASH(F194)</f>
+        <v>E5DD</v>
+      </c>
+      <c r="I194" t="str">
+        <f t="shared" si="4"/>
+        <v>{#fig-E5DD}</v>
+      </c>
+      <c r="J194" t="str">
+        <f t="shared" si="6"/>
         <v>![Listing fine-tuning jobs and showing job details](figures/ft/ss_cli_003_clean.png){#fig-E5DD}</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J193" xr:uid="{B464DFF5-94DA-41E0-B03E-143380050964}"/>
+  <autoFilter ref="A1:J194" xr:uid="{B464DFF5-94DA-41E0-B03E-143380050964}"/>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Rename Foundry Local macOS screenshot (Ch 08) and add to inventory
</commit_message>
<xml_diff>
--- a/figures/figure_inventory.xlsx
+++ b/figures/figure_inventory.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Colby\Documents\GitHub\foundry-book\figures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30B7A6CC-6189-4943-86A0-8081CECC66D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3FAC243-A45E-4158-B6C7-C2816B337D7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{222F1F68-60B1-49B9-BFF7-2C9CF743DB25}"/>
   </bookViews>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="741" uniqueCount="340">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="757" uniqueCount="349">
   <si>
     <t>Type</t>
   </si>
@@ -1082,6 +1082,33 @@
   </si>
   <si>
     <t>Knowledge sources as part of the AI Search data retreival</t>
+  </si>
+  <si>
+    <t>ed</t>
+  </si>
+  <si>
+    <t>ss_local_001_clean.png</t>
+  </si>
+  <si>
+    <t>ss_local_002_clean.png</t>
+  </si>
+  <si>
+    <t>ss_local_003_clean.png</t>
+  </si>
+  <si>
+    <t>ss_local_004_clean.png</t>
+  </si>
+  <si>
+    <t>Chatting with an LLM using the Foundry Local Python SDK</t>
+  </si>
+  <si>
+    <t>Audio transcription with a Whisper model using the Foundry Local Javascript app</t>
+  </si>
+  <si>
+    <t>Chatting with a Phi-4 model with reasoning using the Foundry Local CLI</t>
+  </si>
+  <si>
+    <t>Chatting with a small Qwen 2.5 model using the Foundry Local CLI</t>
   </si>
 </sst>
 </file>
@@ -1111,7 +1138,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1148,6 +1175,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF66CCFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -1161,7 +1194,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1184,6 +1217,9 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1192,6 +1228,7 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FF66CCFF"/>
       <color rgb="FFCCCCFF"/>
       <color rgb="FFFFCCFF"/>
     </mruColors>
@@ -1668,7 +1705,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B464DFF5-94DA-41E0-B03E-143380050964}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:J199"/>
+  <dimension ref="A1:J203"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.5703125" bestFit="1" customWidth="1"/>
@@ -1677,7 +1714,7 @@
     <col min="4" max="4" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="6.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="34.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="51.5703125" customWidth="1"/>
+    <col min="7" max="7" width="73.85546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="8.28515625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="13.140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="51.28515625" customWidth="1"/>
@@ -8403,6 +8440,146 @@
       <c r="J199" t="str">
         <f t="shared" si="6"/>
         <v>![Listing fine-tuning jobs and showing job details](figures/ft/ss_cli_003_clean_neg.png){#fig-7077}</v>
+      </c>
+    </row>
+    <row r="200" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A200">
+        <v>201</v>
+      </c>
+      <c r="B200" s="8" t="s">
+        <v>340</v>
+      </c>
+      <c r="C200" t="s">
+        <v>4</v>
+      </c>
+      <c r="D200" t="b">
+        <v>0</v>
+      </c>
+      <c r="E200" t="b">
+        <v>1</v>
+      </c>
+      <c r="F200" t="s">
+        <v>341</v>
+      </c>
+      <c r="G200" t="s">
+        <v>348</v>
+      </c>
+      <c r="H200" s="1" t="str" cm="1">
+        <f t="array" ref="H200">CRC16HASH(F200)</f>
+        <v>9AEF</v>
+      </c>
+      <c r="I200" t="str">
+        <f t="shared" ref="I200:I203" si="8">_xlfn.CONCAT("{#fig-",H200,"}")</f>
+        <v>{#fig-9AEF}</v>
+      </c>
+      <c r="J200" t="str">
+        <f t="shared" ref="J200:J203" si="9">IF(E200,_xlfn.CONCAT("![",G200,"](figures/",B200,"/",F200,")",I200),"")</f>
+        <v>![Chatting with a small Qwen 2.5 model using the Foundry Local CLI](figures/ed/ss_local_001_clean.png){#fig-9AEF}</v>
+      </c>
+    </row>
+    <row r="201" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A201">
+        <v>202</v>
+      </c>
+      <c r="B201" s="8" t="s">
+        <v>340</v>
+      </c>
+      <c r="C201" t="s">
+        <v>4</v>
+      </c>
+      <c r="D201" t="b">
+        <v>0</v>
+      </c>
+      <c r="E201" t="b">
+        <v>1</v>
+      </c>
+      <c r="F201" t="s">
+        <v>342</v>
+      </c>
+      <c r="G201" t="s">
+        <v>347</v>
+      </c>
+      <c r="H201" s="1" t="str" cm="1">
+        <f t="array" ref="H201">CRC16HASH(F201)</f>
+        <v>DEE0</v>
+      </c>
+      <c r="I201" t="str">
+        <f t="shared" si="8"/>
+        <v>{#fig-DEE0}</v>
+      </c>
+      <c r="J201" t="str">
+        <f t="shared" si="9"/>
+        <v>![Chatting with a Phi-4 model with reasoning using the Foundry Local CLI](figures/ed/ss_local_002_clean.png){#fig-DEE0}</v>
+      </c>
+    </row>
+    <row r="202" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A202">
+        <v>203</v>
+      </c>
+      <c r="B202" s="8" t="s">
+        <v>340</v>
+      </c>
+      <c r="C202" t="s">
+        <v>4</v>
+      </c>
+      <c r="D202" t="b">
+        <v>0</v>
+      </c>
+      <c r="E202" t="b">
+        <v>1</v>
+      </c>
+      <c r="F202" t="s">
+        <v>343</v>
+      </c>
+      <c r="G202" t="s">
+        <v>345</v>
+      </c>
+      <c r="H202" s="1" t="str" cm="1">
+        <f t="array" ref="H202">CRC16HASH(F202)</f>
+        <v>22E4</v>
+      </c>
+      <c r="I202" t="str">
+        <f t="shared" si="8"/>
+        <v>{#fig-22E4}</v>
+      </c>
+      <c r="J202" t="str">
+        <f t="shared" si="9"/>
+        <v>![Chatting with an LLM using the Foundry Local Python SDK](figures/ed/ss_local_003_clean.png){#fig-22E4}</v>
+      </c>
+    </row>
+    <row r="203" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A203">
+        <v>204</v>
+      </c>
+      <c r="B203" s="8" t="s">
+        <v>340</v>
+      </c>
+      <c r="C203" t="s">
+        <v>4</v>
+      </c>
+      <c r="D203" t="b">
+        <v>0</v>
+      </c>
+      <c r="E203" t="b">
+        <v>1</v>
+      </c>
+      <c r="F203" t="s">
+        <v>344</v>
+      </c>
+      <c r="G203" t="s">
+        <v>346</v>
+      </c>
+      <c r="H203" s="1" t="str" cm="1">
+        <f t="array" ref="H203">CRC16HASH(F203)</f>
+        <v>56FE</v>
+      </c>
+      <c r="I203" t="str">
+        <f t="shared" si="8"/>
+        <v>{#fig-56FE}</v>
+      </c>
+      <c r="J203" t="str">
+        <f t="shared" si="9"/>
+        <v>![Audio transcription with a Whisper model using the Foundry Local Javascript app](figures/ed/ss_local_004_clean.png){#fig-56FE}</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update figure inventory for Ch08
</commit_message>
<xml_diff>
--- a/figures/figure_inventory.xlsx
+++ b/figures/figure_inventory.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Colby\Documents\GitHub\foundry-book\figures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3FAC243-A45E-4158-B6C7-C2816B337D7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6CF7972-36F1-4E06-A0A2-57519246D043}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{222F1F68-60B1-49B9-BFF7-2C9CF743DB25}"/>
   </bookViews>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="757" uniqueCount="349">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="777" uniqueCount="359">
   <si>
     <t>Type</t>
   </si>
@@ -1109,6 +1109,36 @@
   </si>
   <si>
     <t>Chatting with a small Qwen 2.5 model using the Foundry Local CLI</t>
+  </si>
+  <si>
+    <t>il_local_001_clean.png</t>
+  </si>
+  <si>
+    <t>il_local_002_clean.png</t>
+  </si>
+  <si>
+    <t>Key features of Foundry Local</t>
+  </si>
+  <si>
+    <t>Architecture components of Foundry Local</t>
+  </si>
+  <si>
+    <t>ss_localsite_001_clean.png</t>
+  </si>
+  <si>
+    <t>The Foundry Local website homepage</t>
+  </si>
+  <si>
+    <t>Quantization example walkthrough from FP32 to INT4</t>
+  </si>
+  <si>
+    <t>il_quant_001_clean.png</t>
+  </si>
+  <si>
+    <t>ss_olive_001_clean.png</t>
+  </si>
+  <si>
+    <t>Quantization of Qwen 2.5 0.5B for CPU inference using Olive</t>
   </si>
 </sst>
 </file>
@@ -1705,7 +1735,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B464DFF5-94DA-41E0-B03E-143380050964}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:J203"/>
+  <dimension ref="A1:J208"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.5703125" bestFit="1" customWidth="1"/>
@@ -8450,7 +8480,7 @@
         <v>340</v>
       </c>
       <c r="C200" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D200" t="b">
         <v>0</v>
@@ -8459,22 +8489,22 @@
         <v>1</v>
       </c>
       <c r="F200" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="G200" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="H200" s="1" t="str" cm="1">
         <f t="array" ref="H200">CRC16HASH(F200)</f>
-        <v>9AEF</v>
+        <v>8639</v>
       </c>
       <c r="I200" t="str">
-        <f t="shared" ref="I200:I203" si="8">_xlfn.CONCAT("{#fig-",H200,"}")</f>
-        <v>{#fig-9AEF}</v>
+        <f t="shared" ref="I200:I202" si="8">_xlfn.CONCAT("{#fig-",H200,"}")</f>
+        <v>{#fig-8639}</v>
       </c>
       <c r="J200" t="str">
-        <f t="shared" ref="J200:J203" si="9">IF(E200,_xlfn.CONCAT("![",G200,"](figures/",B200,"/",F200,")",I200),"")</f>
-        <v>![Chatting with a small Qwen 2.5 model using the Foundry Local CLI](figures/ed/ss_local_001_clean.png){#fig-9AEF}</v>
+        <f t="shared" ref="J200:J202" si="9">IF(E200,_xlfn.CONCAT("![",G200,"](figures/",B200,"/",F200,")",I200),"")</f>
+        <v>![Key features of Foundry Local](figures/ed/il_local_001_clean.png){#fig-8639}</v>
       </c>
     </row>
     <row r="201" spans="1:10" x14ac:dyDescent="0.25">
@@ -8485,7 +8515,7 @@
         <v>340</v>
       </c>
       <c r="C201" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D201" t="b">
         <v>0</v>
@@ -8494,22 +8524,22 @@
         <v>1</v>
       </c>
       <c r="F201" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="G201" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="H201" s="1" t="str" cm="1">
         <f t="array" ref="H201">CRC16HASH(F201)</f>
-        <v>DEE0</v>
+        <v>C236</v>
       </c>
       <c r="I201" t="str">
         <f t="shared" si="8"/>
-        <v>{#fig-DEE0}</v>
+        <v>{#fig-C236}</v>
       </c>
       <c r="J201" t="str">
         <f t="shared" si="9"/>
-        <v>![Chatting with a Phi-4 model with reasoning using the Foundry Local CLI](figures/ed/ss_local_002_clean.png){#fig-DEE0}</v>
+        <v>![Architecture components of Foundry Local](figures/ed/il_local_002_clean.png){#fig-C236}</v>
       </c>
     </row>
     <row r="202" spans="1:10" x14ac:dyDescent="0.25">
@@ -8529,22 +8559,22 @@
         <v>1</v>
       </c>
       <c r="F202" t="s">
-        <v>343</v>
+        <v>353</v>
       </c>
       <c r="G202" t="s">
-        <v>345</v>
+        <v>354</v>
       </c>
       <c r="H202" s="1" t="str" cm="1">
         <f t="array" ref="H202">CRC16HASH(F202)</f>
-        <v>22E4</v>
+        <v>6A11</v>
       </c>
       <c r="I202" t="str">
         <f t="shared" si="8"/>
-        <v>{#fig-22E4}</v>
+        <v>{#fig-6A11}</v>
       </c>
       <c r="J202" t="str">
         <f t="shared" si="9"/>
-        <v>![Chatting with an LLM using the Foundry Local Python SDK](figures/ed/ss_local_003_clean.png){#fig-22E4}</v>
+        <v>![The Foundry Local website homepage](figures/ed/ss_localsite_001_clean.png){#fig-6A11}</v>
       </c>
     </row>
     <row r="203" spans="1:10" x14ac:dyDescent="0.25">
@@ -8564,22 +8594,197 @@
         <v>1</v>
       </c>
       <c r="F203" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="G203" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="H203" s="1" t="str" cm="1">
         <f t="array" ref="H203">CRC16HASH(F203)</f>
+        <v>9AEF</v>
+      </c>
+      <c r="I203" t="str">
+        <f t="shared" ref="I203:I207" si="10">_xlfn.CONCAT("{#fig-",H203,"}")</f>
+        <v>{#fig-9AEF}</v>
+      </c>
+      <c r="J203" t="str">
+        <f t="shared" ref="J203:J206" si="11">IF(E203,_xlfn.CONCAT("![",G203,"](figures/",B203,"/",F203,")",I203),"")</f>
+        <v>![Chatting with a small Qwen 2.5 model using the Foundry Local CLI](figures/ed/ss_local_001_clean.png){#fig-9AEF}</v>
+      </c>
+    </row>
+    <row r="204" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A204">
+        <v>205</v>
+      </c>
+      <c r="B204" s="8" t="s">
+        <v>340</v>
+      </c>
+      <c r="C204" t="s">
+        <v>4</v>
+      </c>
+      <c r="D204" t="b">
+        <v>0</v>
+      </c>
+      <c r="E204" t="b">
+        <v>1</v>
+      </c>
+      <c r="F204" t="s">
+        <v>342</v>
+      </c>
+      <c r="G204" t="s">
+        <v>347</v>
+      </c>
+      <c r="H204" s="1" t="str" cm="1">
+        <f t="array" ref="H204">CRC16HASH(F204)</f>
+        <v>DEE0</v>
+      </c>
+      <c r="I204" t="str">
+        <f t="shared" si="10"/>
+        <v>{#fig-DEE0}</v>
+      </c>
+      <c r="J204" t="str">
+        <f t="shared" si="11"/>
+        <v>![Chatting with a Phi-4 model with reasoning using the Foundry Local CLI](figures/ed/ss_local_002_clean.png){#fig-DEE0}</v>
+      </c>
+    </row>
+    <row r="205" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A205">
+        <v>206</v>
+      </c>
+      <c r="B205" s="8" t="s">
+        <v>340</v>
+      </c>
+      <c r="C205" t="s">
+        <v>4</v>
+      </c>
+      <c r="D205" t="b">
+        <v>0</v>
+      </c>
+      <c r="E205" t="b">
+        <v>1</v>
+      </c>
+      <c r="F205" t="s">
+        <v>343</v>
+      </c>
+      <c r="G205" t="s">
+        <v>345</v>
+      </c>
+      <c r="H205" s="1" t="str" cm="1">
+        <f t="array" ref="H205">CRC16HASH(F205)</f>
+        <v>22E4</v>
+      </c>
+      <c r="I205" t="str">
+        <f t="shared" si="10"/>
+        <v>{#fig-22E4}</v>
+      </c>
+      <c r="J205" t="str">
+        <f t="shared" si="11"/>
+        <v>![Chatting with an LLM using the Foundry Local Python SDK](figures/ed/ss_local_003_clean.png){#fig-22E4}</v>
+      </c>
+    </row>
+    <row r="206" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A206">
+        <v>207</v>
+      </c>
+      <c r="B206" s="8" t="s">
+        <v>340</v>
+      </c>
+      <c r="C206" t="s">
+        <v>4</v>
+      </c>
+      <c r="D206" t="b">
+        <v>0</v>
+      </c>
+      <c r="E206" t="b">
+        <v>1</v>
+      </c>
+      <c r="F206" t="s">
+        <v>344</v>
+      </c>
+      <c r="G206" t="s">
+        <v>346</v>
+      </c>
+      <c r="H206" s="1" t="str" cm="1">
+        <f t="array" ref="H206">CRC16HASH(F206)</f>
         <v>56FE</v>
       </c>
-      <c r="I203" t="str">
-        <f t="shared" si="8"/>
+      <c r="I206" t="str">
+        <f t="shared" si="10"/>
         <v>{#fig-56FE}</v>
       </c>
-      <c r="J203" t="str">
-        <f t="shared" si="9"/>
+      <c r="J206" t="str">
+        <f t="shared" si="11"/>
         <v>![Audio transcription with a Whisper model using the Foundry Local Javascript app](figures/ed/ss_local_004_clean.png){#fig-56FE}</v>
+      </c>
+    </row>
+    <row r="207" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A207">
+        <v>208</v>
+      </c>
+      <c r="B207" s="8" t="s">
+        <v>340</v>
+      </c>
+      <c r="C207" t="s">
+        <v>6</v>
+      </c>
+      <c r="D207" t="b">
+        <v>0</v>
+      </c>
+      <c r="E207" t="b">
+        <v>1</v>
+      </c>
+      <c r="F207" t="s">
+        <v>356</v>
+      </c>
+      <c r="G207" t="s">
+        <v>355</v>
+      </c>
+      <c r="H207" s="1" t="str" cm="1">
+        <f t="array" ref="H207">CRC16HASH(F207)</f>
+        <v>6908</v>
+      </c>
+      <c r="I207" t="str">
+        <f t="shared" si="10"/>
+        <v>{#fig-6908}</v>
+      </c>
+      <c r="J207" t="str">
+        <f t="shared" ref="J207" si="12">IF(E207,_xlfn.CONCAT("![",G207,"](figures/",B207,"/",F207,")",I207),"")</f>
+        <v>![Quantization example walkthrough from FP32 to INT4](figures/ed/il_quant_001_clean.png){#fig-6908}</v>
+      </c>
+    </row>
+    <row r="208" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A208">
+        <v>209</v>
+      </c>
+      <c r="B208" s="8" t="s">
+        <v>340</v>
+      </c>
+      <c r="C208" t="s">
+        <v>4</v>
+      </c>
+      <c r="D208" t="b">
+        <v>0</v>
+      </c>
+      <c r="E208" t="b">
+        <v>1</v>
+      </c>
+      <c r="F208" t="s">
+        <v>357</v>
+      </c>
+      <c r="G208" t="s">
+        <v>358</v>
+      </c>
+      <c r="H208" s="1" t="str" cm="1">
+        <f t="array" ref="H208">CRC16HASH(F208)</f>
+        <v>C0FB</v>
+      </c>
+      <c r="I208" t="str">
+        <f t="shared" ref="I208" si="13">_xlfn.CONCAT("{#fig-",H208,"}")</f>
+        <v>{#fig-C0FB}</v>
+      </c>
+      <c r="J208" t="str">
+        <f t="shared" ref="J208" si="14">IF(E208,_xlfn.CONCAT("![",G208,"](figures/",B208,"/",F208,")",I208),"")</f>
+        <v>![Quantization of Qwen 2.5 0.5B for CPU inference using Olive](figures/ed/ss_olive_001_clean.png){#fig-C0FB}</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Ch07 per MC's recommendations
</commit_message>
<xml_diff>
--- a/figures/figure_inventory.xlsx
+++ b/figures/figure_inventory.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Colby\Documents\GitHub\foundry-book\figures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F5695AC-96E4-47AA-85DC-3C7D47AB2CFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D276D82F-1C8E-4A94-B4B1-2D7CE9F7069F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{222F1F68-60B1-49B9-BFF7-2C9CF743DB25}"/>
   </bookViews>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1044" uniqueCount="472">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1048" uniqueCount="474">
   <si>
     <t>Type</t>
   </si>
@@ -1478,6 +1478,12 @@
   </si>
   <si>
     <t>Orchestrating Agents with Workflows</t>
+  </si>
+  <si>
+    <t>il_controls_001_clean.png</t>
+  </si>
+  <si>
+    <t>Control intervention points in an Agent response flow</t>
   </si>
 </sst>
 </file>
@@ -2093,7 +2099,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B464DFF5-94DA-41E0-B03E-143380050964}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:J282"/>
+  <dimension ref="A1:J283"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.5703125" bestFit="1" customWidth="1"/>
@@ -10337,11 +10343,11 @@
         <v>8453</v>
       </c>
       <c r="I244" t="str">
-        <f t="shared" ref="I244:I251" si="16">_xlfn.CONCAT("{#fig-",H244,"}")</f>
+        <f t="shared" ref="I244:I252" si="16">_xlfn.CONCAT("{#fig-",H244,"}")</f>
         <v>{#fig-8453}</v>
       </c>
       <c r="J244" t="str">
-        <f t="shared" ref="J244:J251" si="17">IF(E244,_xlfn.CONCAT("![",G244,"](figures/",B244,"/",F244,")",I244),"")</f>
+        <f t="shared" ref="J244:J252" si="17">IF(E244,_xlfn.CONCAT("![",G244,"](figures/",B244,"/",F244,")",I244),"")</f>
         <v/>
       </c>
     </row>
@@ -10455,28 +10461,31 @@
         <v>417</v>
       </c>
       <c r="C248" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D248" t="b">
         <v>0</v>
       </c>
       <c r="E248" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F248" t="s">
-        <v>427</v>
+        <v>472</v>
+      </c>
+      <c r="G248" t="s">
+        <v>473</v>
       </c>
       <c r="H248" s="1" t="str" cm="1">
         <f t="array" ref="H248">CRC16HASH(F248)</f>
-        <v>C4D</v>
+        <v>515E</v>
       </c>
       <c r="I248" t="str">
         <f t="shared" si="16"/>
-        <v>{#fig-C4D}</v>
+        <v>{#fig-515E}</v>
       </c>
       <c r="J248" t="str">
         <f t="shared" si="17"/>
-        <v/>
+        <v>![Control intervention points in an Agent response flow](figures/am/il_controls_001_clean.png){#fig-515E}</v>
       </c>
     </row>
     <row r="249" spans="1:10" x14ac:dyDescent="0.25">
@@ -10490,28 +10499,25 @@
         <v>4</v>
       </c>
       <c r="D249" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E249" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F249" t="s">
-        <v>428</v>
-      </c>
-      <c r="G249" t="s">
-        <v>431</v>
+        <v>427</v>
       </c>
       <c r="H249" s="1" t="str" cm="1">
         <f t="array" ref="H249">CRC16HASH(F249)</f>
-        <v>8802</v>
+        <v>C4D</v>
       </c>
       <c r="I249" t="str">
         <f t="shared" si="16"/>
-        <v>{#fig-8802}</v>
+        <v>{#fig-C4D}</v>
       </c>
       <c r="J249" t="str">
         <f t="shared" si="17"/>
-        <v>![Reviewing the Controls added to the Guardrail](figures/am/ss_guardrails_004_ann.png){#fig-8802}</v>
+        <v/>
       </c>
     </row>
     <row r="250" spans="1:10" x14ac:dyDescent="0.25">
@@ -10525,25 +10531,28 @@
         <v>4</v>
       </c>
       <c r="D250" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E250" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F250" t="s">
-        <v>429</v>
+        <v>428</v>
+      </c>
+      <c r="G250" t="s">
+        <v>431</v>
       </c>
       <c r="H250" s="1" t="str" cm="1">
         <f t="array" ref="H250">CRC16HASH(F250)</f>
-        <v>F049</v>
+        <v>8802</v>
       </c>
       <c r="I250" t="str">
         <f t="shared" si="16"/>
-        <v>{#fig-F049}</v>
+        <v>{#fig-8802}</v>
       </c>
       <c r="J250" t="str">
         <f t="shared" si="17"/>
-        <v/>
+        <v>![Reviewing the Controls added to the Guardrail](figures/am/ss_guardrails_004_ann.png){#fig-8802}</v>
       </c>
     </row>
     <row r="251" spans="1:10" x14ac:dyDescent="0.25">
@@ -10557,28 +10566,25 @@
         <v>4</v>
       </c>
       <c r="D251" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E251" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F251" t="s">
-        <v>430</v>
-      </c>
-      <c r="G251" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
       <c r="H251" s="1" t="str" cm="1">
         <f t="array" ref="H251">CRC16HASH(F251)</f>
-        <v>180F</v>
+        <v>F049</v>
       </c>
       <c r="I251" t="str">
         <f t="shared" si="16"/>
-        <v>{#fig-180F}</v>
+        <v>{#fig-F049}</v>
       </c>
       <c r="J251" t="str">
         <f t="shared" si="17"/>
-        <v>![Applying the Guardrail to Models and Agents](figures/am/ss_guardrails_005_ann.png){#fig-180F}</v>
+        <v/>
       </c>
     </row>
     <row r="252" spans="1:10" x14ac:dyDescent="0.25">
@@ -10592,28 +10598,28 @@
         <v>4</v>
       </c>
       <c r="D252" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E252" t="b">
         <v>1</v>
       </c>
       <c r="F252" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
       <c r="G252" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="H252" s="1" t="str" cm="1">
         <f t="array" ref="H252">CRC16HASH(F252)</f>
-        <v>B446</v>
+        <v>180F</v>
       </c>
       <c r="I252" t="str">
-        <f t="shared" ref="I252:I260" si="18">_xlfn.CONCAT("{#fig-",H252,"}")</f>
-        <v>{#fig-B446}</v>
+        <f t="shared" si="16"/>
+        <v>{#fig-180F}</v>
       </c>
       <c r="J252" t="str">
-        <f t="shared" ref="J252:J260" si="19">IF(E252,_xlfn.CONCAT("![",G252,"](figures/",B252,"/",F252,")",I252),"")</f>
-        <v>![Reviewing the Guardrail selections before saving](figures/am/ss_guardrails_006_clean.png){#fig-B446}</v>
+        <f t="shared" si="17"/>
+        <v>![Applying the Guardrail to Models and Agents](figures/am/ss_guardrails_005_ann.png){#fig-180F}</v>
       </c>
     </row>
     <row r="253" spans="1:10" x14ac:dyDescent="0.25">
@@ -10630,22 +10636,25 @@
         <v>0</v>
       </c>
       <c r="E253" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F253" t="s">
-        <v>436</v>
+        <v>433</v>
+      </c>
+      <c r="G253" t="s">
+        <v>434</v>
       </c>
       <c r="H253" s="1" t="str" cm="1">
         <f t="array" ref="H253">CRC16HASH(F253)</f>
-        <v>A120</v>
+        <v>B446</v>
       </c>
       <c r="I253" t="str">
-        <f t="shared" si="18"/>
-        <v>{#fig-A120}</v>
+        <f t="shared" ref="I253:I261" si="18">_xlfn.CONCAT("{#fig-",H253,"}")</f>
+        <v>{#fig-B446}</v>
       </c>
       <c r="J253" t="str">
-        <f t="shared" si="19"/>
-        <v/>
+        <f t="shared" ref="J253:J261" si="19">IF(E253,_xlfn.CONCAT("![",G253,"](figures/",B253,"/",F253,")",I253),"")</f>
+        <v>![Reviewing the Guardrail selections before saving](figures/am/ss_guardrails_006_clean.png){#fig-B446}</v>
       </c>
     </row>
     <row r="254" spans="1:10" x14ac:dyDescent="0.25">
@@ -10659,28 +10668,25 @@
         <v>4</v>
       </c>
       <c r="D254" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E254" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F254" t="s">
-        <v>437</v>
-      </c>
-      <c r="G254" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="H254" s="1" t="str" cm="1">
         <f t="array" ref="H254">CRC16HASH(F254)</f>
-        <v>9B6C</v>
+        <v>A120</v>
       </c>
       <c r="I254" t="str">
         <f t="shared" si="18"/>
-        <v>{#fig-9B6C}</v>
+        <v>{#fig-A120}</v>
       </c>
       <c r="J254" t="str">
         <f t="shared" si="19"/>
-        <v>![Locating Blocklists from the Foundry UI](figures/am/ss_blocklists_001_ann.png){#fig-9B6C}</v>
+        <v/>
       </c>
     </row>
     <row r="255" spans="1:10" x14ac:dyDescent="0.25">
@@ -10694,25 +10700,28 @@
         <v>4</v>
       </c>
       <c r="D255" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E255" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F255" t="s">
-        <v>440</v>
+        <v>437</v>
+      </c>
+      <c r="G255" t="s">
+        <v>435</v>
       </c>
       <c r="H255" s="1" t="str" cm="1">
         <f t="array" ref="H255">CRC16HASH(F255)</f>
-        <v>E52F</v>
+        <v>9B6C</v>
       </c>
       <c r="I255" t="str">
         <f t="shared" si="18"/>
-        <v>{#fig-E52F}</v>
+        <v>{#fig-9B6C}</v>
       </c>
       <c r="J255" t="str">
         <f t="shared" si="19"/>
-        <v/>
+        <v>![Locating Blocklists from the Foundry UI](figures/am/ss_blocklists_001_ann.png){#fig-9B6C}</v>
       </c>
     </row>
     <row r="256" spans="1:10" x14ac:dyDescent="0.25">
@@ -10726,28 +10735,25 @@
         <v>4</v>
       </c>
       <c r="D256" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E256" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F256" t="s">
-        <v>439</v>
-      </c>
-      <c r="G256" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="H256" s="1" t="str" cm="1">
         <f t="array" ref="H256">CRC16HASH(F256)</f>
-        <v>6B78</v>
+        <v>E52F</v>
       </c>
       <c r="I256" t="str">
         <f t="shared" si="18"/>
-        <v>{#fig-6B78}</v>
+        <v>{#fig-E52F}</v>
       </c>
       <c r="J256" t="str">
         <f t="shared" si="19"/>
-        <v>![Making a new Blocklist of competitor AI products](figures/am/ss_blocklists_002_ann.png){#fig-6B78}</v>
+        <v/>
       </c>
     </row>
     <row r="257" spans="1:10" x14ac:dyDescent="0.25">
@@ -10761,28 +10767,28 @@
         <v>4</v>
       </c>
       <c r="D257" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E257" t="b">
         <v>1</v>
       </c>
       <c r="F257" t="s">
-        <v>442</v>
+        <v>439</v>
       </c>
       <c r="G257" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="H257" s="1" t="str" cm="1">
         <f t="array" ref="H257">CRC16HASH(F257)</f>
-        <v>192B</v>
+        <v>6B78</v>
       </c>
       <c r="I257" t="str">
         <f t="shared" si="18"/>
-        <v>{#fig-192B}</v>
+        <v>{#fig-6B78}</v>
       </c>
       <c r="J257" t="str">
         <f t="shared" si="19"/>
-        <v>![Adding the Blocklist in a Guardrail](figures/am/ss_blocklists_003_clean.png){#fig-192B}</v>
+        <v>![Making a new Blocklist of competitor AI products](figures/am/ss_blocklists_002_ann.png){#fig-6B78}</v>
       </c>
     </row>
     <row r="258" spans="1:10" x14ac:dyDescent="0.25">
@@ -10802,22 +10808,22 @@
         <v>1</v>
       </c>
       <c r="F258" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="G258" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
       <c r="H258" s="1" t="str" cm="1">
         <f t="array" ref="H258">CRC16HASH(F258)</f>
-        <v>8807</v>
+        <v>192B</v>
       </c>
       <c r="I258" t="str">
         <f t="shared" si="18"/>
-        <v>{#fig-8807}</v>
+        <v>{#fig-192B}</v>
       </c>
       <c r="J258" t="str">
         <f t="shared" si="19"/>
-        <v>![Exploring the available third-party integrations](figures/am/ss_integrations_001_clean.png){#fig-8807}</v>
+        <v>![Adding the Blocklist in a Guardrail](figures/am/ss_blocklists_003_clean.png){#fig-192B}</v>
       </c>
     </row>
     <row r="259" spans="1:10" x14ac:dyDescent="0.25">
@@ -10834,22 +10840,25 @@
         <v>0</v>
       </c>
       <c r="E259" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F259" t="s">
-        <v>445</v>
+        <v>443</v>
+      </c>
+      <c r="G259" t="s">
+        <v>444</v>
       </c>
       <c r="H259" s="1" t="str" cm="1">
         <f t="array" ref="H259">CRC16HASH(F259)</f>
-        <v>68D</v>
+        <v>8807</v>
       </c>
       <c r="I259" t="str">
         <f t="shared" si="18"/>
-        <v>{#fig-68D}</v>
+        <v>{#fig-8807}</v>
       </c>
       <c r="J259" t="str">
         <f t="shared" si="19"/>
-        <v/>
+        <v>![Exploring the available third-party integrations](figures/am/ss_integrations_001_clean.png){#fig-8807}</v>
       </c>
     </row>
     <row r="260" spans="1:10" x14ac:dyDescent="0.25">
@@ -10863,28 +10872,25 @@
         <v>4</v>
       </c>
       <c r="D260" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E260" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F260" t="s">
-        <v>446</v>
-      </c>
-      <c r="G260" t="s">
-        <v>450</v>
+        <v>445</v>
       </c>
       <c r="H260" s="1" t="str" cm="1">
         <f t="array" ref="H260">CRC16HASH(F260)</f>
-        <v>5103</v>
+        <v>68D</v>
       </c>
       <c r="I260" t="str">
         <f t="shared" si="18"/>
-        <v>{#fig-5103}</v>
+        <v>{#fig-68D}</v>
       </c>
       <c r="J260" t="str">
         <f t="shared" si="19"/>
-        <v>![The Conrol Plane's Operate page of the Foundry UI](figures/am/ss_controlplane_001_ann.png){#fig-5103}</v>
+        <v/>
       </c>
     </row>
     <row r="261" spans="1:10" x14ac:dyDescent="0.25">
@@ -10898,25 +10904,28 @@
         <v>4</v>
       </c>
       <c r="D261" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E261" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F261" t="s">
-        <v>447</v>
+        <v>446</v>
+      </c>
+      <c r="G261" t="s">
+        <v>450</v>
       </c>
       <c r="H261" s="1" t="str" cm="1">
         <f t="array" ref="H261">CRC16HASH(F261)</f>
-        <v>4282</v>
+        <v>5103</v>
       </c>
       <c r="I261" t="str">
-        <f t="shared" ref="I261:I270" si="20">_xlfn.CONCAT("{#fig-",H261,"}")</f>
-        <v>{#fig-4282}</v>
+        <f t="shared" si="18"/>
+        <v>{#fig-5103}</v>
       </c>
       <c r="J261" t="str">
-        <f t="shared" ref="J261:J271" si="21">IF(E261,_xlfn.CONCAT("![",G261,"](figures/",B261,"/",F261,")",I261),"")</f>
-        <v/>
+        <f t="shared" si="19"/>
+        <v>![The Conrol Plane's Operate page of the Foundry UI](figures/am/ss_controlplane_001_ann.png){#fig-5103}</v>
       </c>
     </row>
     <row r="262" spans="1:10" x14ac:dyDescent="0.25">
@@ -10930,28 +10939,25 @@
         <v>4</v>
       </c>
       <c r="D262" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E262" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F262" t="s">
-        <v>448</v>
-      </c>
-      <c r="G262" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="H262" s="1" t="str" cm="1">
         <f t="array" ref="H262">CRC16HASH(F262)</f>
-        <v>A117</v>
+        <v>4282</v>
       </c>
       <c r="I262" t="str">
-        <f t="shared" si="20"/>
-        <v>{#fig-A117}</v>
+        <f t="shared" ref="I262:I271" si="20">_xlfn.CONCAT("{#fig-",H262,"}")</f>
+        <v>{#fig-4282}</v>
       </c>
       <c r="J262" t="str">
-        <f t="shared" si="21"/>
-        <v>![Viewing all your assets in the Control Plane](figures/am/ss_controlplane_002_ann.png){#fig-A117}</v>
+        <f t="shared" ref="J262:J272" si="21">IF(E262,_xlfn.CONCAT("![",G262,"](figures/",B262,"/",F262,")",I262),"")</f>
+        <v/>
       </c>
     </row>
     <row r="263" spans="1:10" x14ac:dyDescent="0.25">
@@ -10965,28 +10971,28 @@
         <v>4</v>
       </c>
       <c r="D263" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E263" t="b">
         <v>1</v>
       </c>
       <c r="F263" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="G263" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="H263" s="1" t="str" cm="1">
         <f t="array" ref="H263">CRC16HASH(F263)</f>
-        <v>4282</v>
+        <v>A117</v>
       </c>
       <c r="I263" t="str">
         <f t="shared" si="20"/>
-        <v>{#fig-4282}</v>
+        <v>{#fig-A117}</v>
       </c>
       <c r="J263" t="str">
         <f t="shared" si="21"/>
-        <v>![Viewing the Monitor tab of an Agent](figures/am/ss_controlplane_002_clean.png){#fig-4282}</v>
+        <v>![Viewing all your assets in the Control Plane](figures/am/ss_controlplane_002_ann.png){#fig-A117}</v>
       </c>
     </row>
     <row r="264" spans="1:10" x14ac:dyDescent="0.25">
@@ -11003,22 +11009,25 @@
         <v>0</v>
       </c>
       <c r="E264" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F264" t="s">
-        <v>453</v>
+        <v>447</v>
+      </c>
+      <c r="G264" t="s">
+        <v>451</v>
       </c>
       <c r="H264" s="1" t="str" cm="1">
         <f t="array" ref="H264">CRC16HASH(F264)</f>
-        <v>ED37</v>
+        <v>4282</v>
       </c>
       <c r="I264" t="str">
         <f t="shared" si="20"/>
-        <v>{#fig-ED37}</v>
+        <v>{#fig-4282}</v>
       </c>
       <c r="J264" t="str">
         <f t="shared" si="21"/>
-        <v/>
+        <v>![Viewing the Monitor tab of an Agent](figures/am/ss_controlplane_002_clean.png){#fig-4282}</v>
       </c>
     </row>
     <row r="265" spans="1:10" x14ac:dyDescent="0.25">
@@ -11032,28 +11041,25 @@
         <v>4</v>
       </c>
       <c r="D265" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E265" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F265" t="s">
-        <v>454</v>
-      </c>
-      <c r="G265" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="H265" s="1" t="str" cm="1">
         <f t="array" ref="H265">CRC16HASH(F265)</f>
-        <v>34A7</v>
+        <v>ED37</v>
       </c>
       <c r="I265" t="str">
         <f t="shared" si="20"/>
-        <v>{#fig-34A7}</v>
+        <v>{#fig-ED37}</v>
       </c>
       <c r="J265" t="str">
         <f t="shared" si="21"/>
-        <v>![Viewing the Quotas table in the Control Plane](figures/am/ss_quotas_001_ann.png){#fig-34A7}</v>
+        <v/>
       </c>
     </row>
     <row r="266" spans="1:10" x14ac:dyDescent="0.25">
@@ -11067,25 +11073,28 @@
         <v>4</v>
       </c>
       <c r="D266" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E266" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F266" t="s">
-        <v>457</v>
+        <v>454</v>
+      </c>
+      <c r="G266" t="s">
+        <v>452</v>
       </c>
       <c r="H266" s="1" t="str" cm="1">
         <f t="array" ref="H266">CRC16HASH(F266)</f>
-        <v>A938</v>
+        <v>34A7</v>
       </c>
       <c r="I266" t="str">
         <f t="shared" si="20"/>
-        <v>{#fig-A938}</v>
+        <v>{#fig-34A7}</v>
       </c>
       <c r="J266" t="str">
         <f t="shared" si="21"/>
-        <v/>
+        <v>![Viewing the Quotas table in the Control Plane](figures/am/ss_quotas_001_ann.png){#fig-34A7}</v>
       </c>
     </row>
     <row r="267" spans="1:10" x14ac:dyDescent="0.25">
@@ -11099,28 +11108,25 @@
         <v>4</v>
       </c>
       <c r="D267" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E267" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F267" t="s">
-        <v>458</v>
-      </c>
-      <c r="G267" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="H267" s="1" t="str" cm="1">
         <f t="array" ref="H267">CRC16HASH(F267)</f>
-        <v>C4B3</v>
+        <v>A938</v>
       </c>
       <c r="I267" t="str">
         <f t="shared" si="20"/>
-        <v>{#fig-C4B3}</v>
+        <v>{#fig-A938}</v>
       </c>
       <c r="J267" t="str">
         <f t="shared" si="21"/>
-        <v>![Editing the quota for a model](figures/am/ss_quotas_002_ann.png){#fig-C4B3}</v>
+        <v/>
       </c>
     </row>
     <row r="268" spans="1:10" x14ac:dyDescent="0.25">
@@ -11134,25 +11140,28 @@
         <v>4</v>
       </c>
       <c r="D268" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E268" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F268" t="s">
-        <v>460</v>
+        <v>458</v>
+      </c>
+      <c r="G268" t="s">
+        <v>459</v>
       </c>
       <c r="H268" s="1" t="str" cm="1">
         <f t="array" ref="H268">CRC16HASH(F268)</f>
-        <v>1510</v>
+        <v>C4B3</v>
       </c>
       <c r="I268" t="str">
         <f t="shared" si="20"/>
-        <v>{#fig-1510}</v>
+        <v>{#fig-C4B3}</v>
       </c>
       <c r="J268" t="str">
         <f t="shared" si="21"/>
-        <v/>
+        <v>![Editing the quota for a model](figures/am/ss_quotas_002_ann.png){#fig-C4B3}</v>
       </c>
     </row>
     <row r="269" spans="1:10" x14ac:dyDescent="0.25">
@@ -11166,28 +11175,25 @@
         <v>4</v>
       </c>
       <c r="D269" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E269" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F269" t="s">
-        <v>461</v>
-      </c>
-      <c r="G269" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="H269" s="1" t="str" cm="1">
         <f t="array" ref="H269">CRC16HASH(F269)</f>
-        <v>AB2E</v>
+        <v>1510</v>
       </c>
       <c r="I269" t="str">
         <f t="shared" si="20"/>
-        <v>{#fig-AB2E}</v>
+        <v>{#fig-1510}</v>
       </c>
       <c r="J269" t="str">
         <f t="shared" si="21"/>
-        <v>![Enabling Microsoft Purview monitoring of your Foundry Project](figures/am/ss_compliance_001_ann.png){#fig-AB2E}</v>
+        <v/>
       </c>
     </row>
     <row r="270" spans="1:10" x14ac:dyDescent="0.25">
@@ -11201,28 +11207,28 @@
         <v>4</v>
       </c>
       <c r="D270" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E270" t="b">
         <v>1</v>
       </c>
       <c r="F270" t="s">
-        <v>468</v>
+        <v>461</v>
       </c>
       <c r="G270" t="s">
-        <v>469</v>
+        <v>462</v>
       </c>
       <c r="H270" s="1" t="str" cm="1">
         <f t="array" ref="H270">CRC16HASH(F270)</f>
-        <v>A73E</v>
+        <v>AB2E</v>
       </c>
       <c r="I270" t="str">
         <f t="shared" si="20"/>
-        <v>{#fig-A73E}</v>
+        <v>{#fig-AB2E}</v>
       </c>
       <c r="J270" t="str">
         <f t="shared" si="21"/>
-        <v>![The Agent ID dashboard from the Azure Portal](figures/am/ss_agentid_001_clean.png){#fig-A73E}</v>
+        <v>![Enabling Microsoft Purview monitoring of your Foundry Project](figures/am/ss_compliance_001_ann.png){#fig-AB2E}</v>
       </c>
     </row>
     <row r="271" spans="1:10" x14ac:dyDescent="0.25">
@@ -11239,22 +11245,25 @@
         <v>0</v>
       </c>
       <c r="E271" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F271" t="s">
-        <v>465</v>
+        <v>468</v>
+      </c>
+      <c r="G271" t="s">
+        <v>469</v>
       </c>
       <c r="H271" s="1" t="str" cm="1">
         <f t="array" ref="H271">CRC16HASH(F271)</f>
-        <v>375E</v>
+        <v>A73E</v>
       </c>
       <c r="I271" t="str">
-        <f t="shared" ref="I271:I274" si="22">_xlfn.CONCAT("{#fig-",H271,"}")</f>
-        <v>{#fig-375E}</v>
+        <f t="shared" si="20"/>
+        <v>{#fig-A73E}</v>
       </c>
       <c r="J271" t="str">
         <f t="shared" si="21"/>
-        <v/>
+        <v>![The Agent ID dashboard from the Azure Portal](figures/am/ss_agentid_001_clean.png){#fig-A73E}</v>
       </c>
     </row>
     <row r="272" spans="1:10" x14ac:dyDescent="0.25">
@@ -11268,28 +11277,25 @@
         <v>4</v>
       </c>
       <c r="D272" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E272" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F272" t="s">
-        <v>463</v>
-      </c>
-      <c r="G272" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="H272" s="1" t="str" cm="1">
         <f t="array" ref="H272">CRC16HASH(F272)</f>
-        <v>D3C6</v>
+        <v>375E</v>
       </c>
       <c r="I272" t="str">
-        <f t="shared" si="22"/>
-        <v>{#fig-D3C6}</v>
+        <f t="shared" ref="I272:I275" si="22">_xlfn.CONCAT("{#fig-",H272,"}")</f>
+        <v>{#fig-375E}</v>
       </c>
       <c r="J272" t="str">
-        <f t="shared" ref="J272:J274" si="23">IF(E272,_xlfn.CONCAT("![",G272,"](figures/",B272,"/",F272,")",I272),"")</f>
-        <v>![Publishing an Agent to retrieve its Principal ID](figures/am/ss_entra_001_ann.png){#fig-D3C6}</v>
+        <f t="shared" si="21"/>
+        <v/>
       </c>
     </row>
     <row r="273" spans="1:10" x14ac:dyDescent="0.25">
@@ -11303,39 +11309,39 @@
         <v>4</v>
       </c>
       <c r="D273" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E273" t="b">
         <v>1</v>
       </c>
       <c r="F273" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="G273" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="H273" s="1" t="str" cm="1">
         <f t="array" ref="H273">CRC16HASH(F273)</f>
-        <v>7351</v>
+        <v>D3C6</v>
       </c>
       <c r="I273" t="str">
         <f t="shared" si="22"/>
-        <v>{#fig-7351}</v>
+        <v>{#fig-D3C6}</v>
       </c>
       <c r="J273" t="str">
-        <f t="shared" si="23"/>
-        <v>![The general Application ID for the Foundry Project in Entra ID](figures/am/ss_entra_002_clean.png){#fig-7351}</v>
+        <f t="shared" ref="J273:J275" si="23">IF(E273,_xlfn.CONCAT("![",G273,"](figures/",B273,"/",F273,")",I273),"")</f>
+        <v>![Publishing an Agent to retrieve its Principal ID](figures/am/ss_entra_001_ann.png){#fig-D3C6}</v>
       </c>
     </row>
     <row r="274" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A274">
         <v>275</v>
       </c>
-      <c r="B274" s="8" t="s">
-        <v>335</v>
+      <c r="B274" s="10" t="s">
+        <v>417</v>
       </c>
       <c r="C274" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D274" t="b">
         <v>0</v>
@@ -11344,22 +11350,22 @@
         <v>1</v>
       </c>
       <c r="F274" t="s">
-        <v>344</v>
+        <v>464</v>
       </c>
       <c r="G274" t="s">
-        <v>346</v>
+        <v>466</v>
       </c>
       <c r="H274" s="1" t="str" cm="1">
         <f t="array" ref="H274">CRC16HASH(F274)</f>
-        <v>8639</v>
+        <v>7351</v>
       </c>
       <c r="I274" t="str">
         <f t="shared" si="22"/>
-        <v>{#fig-8639}</v>
+        <v>{#fig-7351}</v>
       </c>
       <c r="J274" t="str">
         <f t="shared" si="23"/>
-        <v>![Key features of Foundry Local](figures/ed/il_local_001_clean.png){#fig-8639}</v>
+        <v>![The general Application ID for the Foundry Project in Entra ID](figures/am/ss_entra_002_clean.png){#fig-7351}</v>
       </c>
     </row>
     <row r="275" spans="1:10" x14ac:dyDescent="0.25">
@@ -11379,22 +11385,22 @@
         <v>1</v>
       </c>
       <c r="F275" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="G275" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="H275" s="1" t="str" cm="1">
         <f t="array" ref="H275">CRC16HASH(F275)</f>
-        <v>C236</v>
+        <v>8639</v>
       </c>
       <c r="I275" t="str">
-        <f t="shared" ref="I275:I276" si="24">_xlfn.CONCAT("{#fig-",H275,"}")</f>
-        <v>{#fig-C236}</v>
+        <f t="shared" si="22"/>
+        <v>{#fig-8639}</v>
       </c>
       <c r="J275" t="str">
-        <f t="shared" ref="J275:J276" si="25">IF(E275,_xlfn.CONCAT("![",G275,"](figures/",B275,"/",F275,")",I275),"")</f>
-        <v>![Architecture components of Foundry Local](figures/ed/il_local_002_clean.png){#fig-C236}</v>
+        <f t="shared" si="23"/>
+        <v>![Key features of Foundry Local](figures/ed/il_local_001_clean.png){#fig-8639}</v>
       </c>
     </row>
     <row r="276" spans="1:10" x14ac:dyDescent="0.25">
@@ -11405,7 +11411,7 @@
         <v>335</v>
       </c>
       <c r="C276" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D276" t="b">
         <v>0</v>
@@ -11414,22 +11420,22 @@
         <v>1</v>
       </c>
       <c r="F276" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="G276" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="H276" s="1" t="str" cm="1">
         <f t="array" ref="H276">CRC16HASH(F276)</f>
-        <v>6A11</v>
+        <v>C236</v>
       </c>
       <c r="I276" t="str">
-        <f t="shared" si="24"/>
-        <v>{#fig-6A11}</v>
+        <f t="shared" ref="I276:I277" si="24">_xlfn.CONCAT("{#fig-",H276,"}")</f>
+        <v>{#fig-C236}</v>
       </c>
       <c r="J276" t="str">
-        <f t="shared" si="25"/>
-        <v>![The Foundry Local website homepage](figures/ed/ss_localsite_001_clean.png){#fig-6A11}</v>
+        <f t="shared" ref="J276:J277" si="25">IF(E276,_xlfn.CONCAT("![",G276,"](figures/",B276,"/",F276,")",I276),"")</f>
+        <v>![Architecture components of Foundry Local](figures/ed/il_local_002_clean.png){#fig-C236}</v>
       </c>
     </row>
     <row r="277" spans="1:10" x14ac:dyDescent="0.25">
@@ -11449,22 +11455,22 @@
         <v>1</v>
       </c>
       <c r="F277" t="s">
-        <v>336</v>
+        <v>348</v>
       </c>
       <c r="G277" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
       <c r="H277" s="1" t="str" cm="1">
         <f t="array" ref="H277">CRC16HASH(F277)</f>
-        <v>9AEF</v>
+        <v>6A11</v>
       </c>
       <c r="I277" t="str">
-        <f t="shared" ref="I277:I281" si="26">_xlfn.CONCAT("{#fig-",H277,"}")</f>
-        <v>{#fig-9AEF}</v>
+        <f t="shared" si="24"/>
+        <v>{#fig-6A11}</v>
       </c>
       <c r="J277" t="str">
-        <f t="shared" ref="J277:J280" si="27">IF(E277,_xlfn.CONCAT("![",G277,"](figures/",B277,"/",F277,")",I277),"")</f>
-        <v>![Chatting with a small Qwen 2.5 model using the Foundry Local CLI](figures/ed/ss_local_001_clean.png){#fig-9AEF}</v>
+        <f t="shared" si="25"/>
+        <v>![The Foundry Local website homepage](figures/ed/ss_localsite_001_clean.png){#fig-6A11}</v>
       </c>
     </row>
     <row r="278" spans="1:10" x14ac:dyDescent="0.25">
@@ -11484,22 +11490,22 @@
         <v>1</v>
       </c>
       <c r="F278" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="G278" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="H278" s="1" t="str" cm="1">
         <f t="array" ref="H278">CRC16HASH(F278)</f>
-        <v>DEE0</v>
+        <v>9AEF</v>
       </c>
       <c r="I278" t="str">
-        <f t="shared" si="26"/>
-        <v>{#fig-DEE0}</v>
+        <f t="shared" ref="I278:I282" si="26">_xlfn.CONCAT("{#fig-",H278,"}")</f>
+        <v>{#fig-9AEF}</v>
       </c>
       <c r="J278" t="str">
-        <f t="shared" si="27"/>
-        <v>![Chatting with a Phi-4 model with reasoning using the Foundry Local CLI](figures/ed/ss_local_002_clean.png){#fig-DEE0}</v>
+        <f t="shared" ref="J278:J281" si="27">IF(E278,_xlfn.CONCAT("![",G278,"](figures/",B278,"/",F278,")",I278),"")</f>
+        <v>![Chatting with a small Qwen 2.5 model using the Foundry Local CLI](figures/ed/ss_local_001_clean.png){#fig-9AEF}</v>
       </c>
     </row>
     <row r="279" spans="1:10" x14ac:dyDescent="0.25">
@@ -11519,22 +11525,22 @@
         <v>1</v>
       </c>
       <c r="F279" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="G279" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="H279" s="1" t="str" cm="1">
         <f t="array" ref="H279">CRC16HASH(F279)</f>
-        <v>22E4</v>
+        <v>DEE0</v>
       </c>
       <c r="I279" t="str">
         <f t="shared" si="26"/>
-        <v>{#fig-22E4}</v>
+        <v>{#fig-DEE0}</v>
       </c>
       <c r="J279" t="str">
         <f t="shared" si="27"/>
-        <v>![Chatting with an LLM using the Foundry Local Python SDK](figures/ed/ss_local_003_clean.png){#fig-22E4}</v>
+        <v>![Chatting with a Phi-4 model with reasoning using the Foundry Local CLI](figures/ed/ss_local_002_clean.png){#fig-DEE0}</v>
       </c>
     </row>
     <row r="280" spans="1:10" x14ac:dyDescent="0.25">
@@ -11554,22 +11560,22 @@
         <v>1</v>
       </c>
       <c r="F280" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="G280" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="H280" s="1" t="str" cm="1">
         <f t="array" ref="H280">CRC16HASH(F280)</f>
-        <v>56FE</v>
+        <v>22E4</v>
       </c>
       <c r="I280" t="str">
         <f t="shared" si="26"/>
-        <v>{#fig-56FE}</v>
+        <v>{#fig-22E4}</v>
       </c>
       <c r="J280" t="str">
         <f t="shared" si="27"/>
-        <v>![Audio transcription with a Whisper model using the Foundry Local Javascript app](figures/ed/ss_local_004_clean.png){#fig-56FE}</v>
+        <v>![Chatting with an LLM using the Foundry Local Python SDK](figures/ed/ss_local_003_clean.png){#fig-22E4}</v>
       </c>
     </row>
     <row r="281" spans="1:10" x14ac:dyDescent="0.25">
@@ -11580,7 +11586,7 @@
         <v>335</v>
       </c>
       <c r="C281" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D281" t="b">
         <v>0</v>
@@ -11589,22 +11595,22 @@
         <v>1</v>
       </c>
       <c r="F281" t="s">
-        <v>351</v>
+        <v>339</v>
       </c>
       <c r="G281" t="s">
-        <v>350</v>
+        <v>341</v>
       </c>
       <c r="H281" s="1" t="str" cm="1">
         <f t="array" ref="H281">CRC16HASH(F281)</f>
-        <v>6908</v>
+        <v>56FE</v>
       </c>
       <c r="I281" t="str">
         <f t="shared" si="26"/>
-        <v>{#fig-6908}</v>
+        <v>{#fig-56FE}</v>
       </c>
       <c r="J281" t="str">
-        <f t="shared" ref="J281" si="28">IF(E281,_xlfn.CONCAT("![",G281,"](figures/",B281,"/",F281,")",I281),"")</f>
-        <v>![Quantization example walkthrough from FP32 to INT4](figures/ed/il_quant_001_clean.png){#fig-6908}</v>
+        <f t="shared" si="27"/>
+        <v>![Audio transcription with a Whisper model using the Foundry Local Javascript app](figures/ed/ss_local_004_clean.png){#fig-56FE}</v>
       </c>
     </row>
     <row r="282" spans="1:10" x14ac:dyDescent="0.25">
@@ -11615,7 +11621,7 @@
         <v>335</v>
       </c>
       <c r="C282" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D282" t="b">
         <v>0</v>
@@ -11624,21 +11630,56 @@
         <v>1</v>
       </c>
       <c r="F282" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="G282" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="H282" s="1" t="str" cm="1">
         <f t="array" ref="H282">CRC16HASH(F282)</f>
+        <v>6908</v>
+      </c>
+      <c r="I282" t="str">
+        <f t="shared" si="26"/>
+        <v>{#fig-6908}</v>
+      </c>
+      <c r="J282" t="str">
+        <f t="shared" ref="J282" si="28">IF(E282,_xlfn.CONCAT("![",G282,"](figures/",B282,"/",F282,")",I282),"")</f>
+        <v>![Quantization example walkthrough from FP32 to INT4](figures/ed/il_quant_001_clean.png){#fig-6908}</v>
+      </c>
+    </row>
+    <row r="283" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A283">
+        <v>284</v>
+      </c>
+      <c r="B283" s="8" t="s">
+        <v>335</v>
+      </c>
+      <c r="C283" t="s">
+        <v>4</v>
+      </c>
+      <c r="D283" t="b">
+        <v>0</v>
+      </c>
+      <c r="E283" t="b">
+        <v>1</v>
+      </c>
+      <c r="F283" t="s">
+        <v>352</v>
+      </c>
+      <c r="G283" t="s">
+        <v>353</v>
+      </c>
+      <c r="H283" s="1" t="str" cm="1">
+        <f t="array" ref="H283">CRC16HASH(F283)</f>
         <v>C0FB</v>
       </c>
-      <c r="I282" t="str">
-        <f t="shared" ref="I282" si="29">_xlfn.CONCAT("{#fig-",H282,"}")</f>
+      <c r="I283" t="str">
+        <f t="shared" ref="I283" si="29">_xlfn.CONCAT("{#fig-",H283,"}")</f>
         <v>{#fig-C0FB}</v>
       </c>
-      <c r="J282" t="str">
-        <f t="shared" ref="J282" si="30">IF(E282,_xlfn.CONCAT("![",G282,"](figures/",B282,"/",F282,")",I282),"")</f>
+      <c r="J283" t="str">
+        <f t="shared" ref="J283" si="30">IF(E283,_xlfn.CONCAT("![",G283,"](figures/",B283,"/",F283,")",I283),"")</f>
         <v>![Quantization of Qwen 2.5 0.5B for CPU inference using Olive](figures/ed/ss_olive_001_clean.png){#fig-C0FB}</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add figures for Ch09
</commit_message>
<xml_diff>
--- a/figures/figure_inventory.xlsx
+++ b/figures/figure_inventory.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Colby\Documents\GitHub\foundry-book\figures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D276D82F-1C8E-4A94-B4B1-2D7CE9F7069F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D0D187A-F98F-4698-9569-4F03DC36A207}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{222F1F68-60B1-49B9-BFF7-2C9CF743DB25}"/>
   </bookViews>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1048" uniqueCount="474">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1111" uniqueCount="503">
   <si>
     <t>Type</t>
   </si>
@@ -1484,13 +1484,100 @@
   </si>
   <si>
     <t>Control intervention points in an Agent response flow</t>
+  </si>
+  <si>
+    <t>il_govframework_001_clean.png</t>
+  </si>
+  <si>
+    <t>Governance workflow of the Microsoft Agent Governance Toolkit</t>
+  </si>
+  <si>
+    <t>il_govframework_002_clean.png</t>
+  </si>
+  <si>
+    <t>The 4 privilege rings of zero-trust Agent identity</t>
+  </si>
+  <si>
+    <t>Locating the memory capability on an Agent</t>
+  </si>
+  <si>
+    <t>ss_memory_001_clean.png</t>
+  </si>
+  <si>
+    <t>ss_memory_002_clean.png</t>
+  </si>
+  <si>
+    <t>ss_memory_001_ann.png</t>
+  </si>
+  <si>
+    <t>Editing the memory store</t>
+  </si>
+  <si>
+    <t>il_memory_001_clean.png</t>
+  </si>
+  <si>
+    <t>How a memory store recalls previous context</t>
+  </si>
+  <si>
+    <t>ss_evaluations_001_clean.png</t>
+  </si>
+  <si>
+    <t>ss_evaluations_001_ann.png</t>
+  </si>
+  <si>
+    <t>Locating the Evaluations screen</t>
+  </si>
+  <si>
+    <t>ss_evaluations_002_clean.png</t>
+  </si>
+  <si>
+    <t>Configuring the evaluation process for an agent using synthetic data</t>
+  </si>
+  <si>
+    <t>ss_evaluations_003_clean.png</t>
+  </si>
+  <si>
+    <t>ss_evaluations_003_ann.png</t>
+  </si>
+  <si>
+    <t>The Evaluator catalog show the details of a built-in evaluator</t>
+  </si>
+  <si>
+    <t>ss_batchjobs_001_clean.png</t>
+  </si>
+  <si>
+    <t>ss_batchjobs_001_ann.png</t>
+  </si>
+  <si>
+    <t>Locating the Batch jobs feature under Models</t>
+  </si>
+  <si>
+    <t>ss_batchjobs_002_clean.png</t>
+  </si>
+  <si>
+    <t>Uploading .jsonl data to create a batch job</t>
+  </si>
+  <si>
+    <t>Locating the AI Services options under Models</t>
+  </si>
+  <si>
+    <t>ss_aiservices_001_clean.png</t>
+  </si>
+  <si>
+    <t>ss_aiservices_001_ann.png</t>
+  </si>
+  <si>
+    <t>Testing out the Voice Live AI service in a Playground</t>
+  </si>
+  <si>
+    <t>ss_aiservices_002_clean.png</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1512,8 +1599,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1568,6 +1662,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -1581,7 +1681,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1611,6 +1711,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -2099,7 +2202,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B464DFF5-94DA-41E0-B03E-143380050964}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:J283"/>
+  <dimension ref="A1:J300"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.5703125" bestFit="1" customWidth="1"/>
@@ -11675,12 +11778,592 @@
         <v>C0FB</v>
       </c>
       <c r="I283" t="str">
-        <f t="shared" ref="I283" si="29">_xlfn.CONCAT("{#fig-",H283,"}")</f>
+        <f t="shared" ref="I283:I300" si="29">_xlfn.CONCAT("{#fig-",H283,"}")</f>
         <v>{#fig-C0FB}</v>
       </c>
       <c r="J283" t="str">
-        <f t="shared" ref="J283" si="30">IF(E283,_xlfn.CONCAT("![",G283,"](figures/",B283,"/",F283,")",I283),"")</f>
+        <f t="shared" ref="J283:J300" si="30">IF(E283,_xlfn.CONCAT("![",G283,"](figures/",B283,"/",F283,")",I283),"")</f>
         <v>![Quantization of Qwen 2.5 0.5B for CPU inference using Olive](figures/ed/ss_olive_001_clean.png){#fig-C0FB}</v>
+      </c>
+    </row>
+    <row r="284" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A284">
+        <v>285</v>
+      </c>
+      <c r="B284" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="C284" t="s">
+        <v>6</v>
+      </c>
+      <c r="D284" t="b">
+        <v>0</v>
+      </c>
+      <c r="E284" t="b">
+        <v>1</v>
+      </c>
+      <c r="F284" t="s">
+        <v>483</v>
+      </c>
+      <c r="G284" t="s">
+        <v>484</v>
+      </c>
+      <c r="H284" s="1" t="str" cm="1">
+        <f t="array" ref="H284">CRC16HASH(F284)</f>
+        <v>9BA0</v>
+      </c>
+      <c r="I284" t="str">
+        <f t="shared" si="29"/>
+        <v>{#fig-9BA0}</v>
+      </c>
+      <c r="J284" t="str">
+        <f t="shared" si="30"/>
+        <v>![How a memory store recalls previous context](figures/co/il_memory_001_clean.png){#fig-9BA0}</v>
+      </c>
+    </row>
+    <row r="285" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A285">
+        <v>286</v>
+      </c>
+      <c r="B285" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="C285" t="s">
+        <v>4</v>
+      </c>
+      <c r="D285" t="b">
+        <v>0</v>
+      </c>
+      <c r="E285" t="b">
+        <v>0</v>
+      </c>
+      <c r="F285" t="s">
+        <v>479</v>
+      </c>
+      <c r="H285" s="1" t="str" cm="1">
+        <f t="array" ref="H285">CRC16HASH(F285)</f>
+        <v>53D</v>
+      </c>
+      <c r="I285" t="str">
+        <f t="shared" si="29"/>
+        <v>{#fig-53D}</v>
+      </c>
+      <c r="J285" t="str">
+        <f t="shared" si="30"/>
+        <v/>
+      </c>
+    </row>
+    <row r="286" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A286">
+        <v>287</v>
+      </c>
+      <c r="B286" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="C286" t="s">
+        <v>4</v>
+      </c>
+      <c r="D286" t="b">
+        <v>1</v>
+      </c>
+      <c r="E286" t="b">
+        <v>1</v>
+      </c>
+      <c r="F286" t="s">
+        <v>481</v>
+      </c>
+      <c r="G286" t="s">
+        <v>478</v>
+      </c>
+      <c r="H286" s="1" t="str" cm="1">
+        <f t="array" ref="H286">CRC16HASH(F286)</f>
+        <v>D4BD</v>
+      </c>
+      <c r="I286" t="str">
+        <f t="shared" si="29"/>
+        <v>{#fig-D4BD}</v>
+      </c>
+      <c r="J286" t="str">
+        <f t="shared" si="30"/>
+        <v>![Locating the memory capability on an Agent](figures/co/ss_memory_001_ann.png){#fig-D4BD}</v>
+      </c>
+    </row>
+    <row r="287" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A287">
+        <v>288</v>
+      </c>
+      <c r="B287" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="C287" t="s">
+        <v>4</v>
+      </c>
+      <c r="D287" t="b">
+        <v>0</v>
+      </c>
+      <c r="E287" t="b">
+        <v>1</v>
+      </c>
+      <c r="F287" t="s">
+        <v>480</v>
+      </c>
+      <c r="G287" t="s">
+        <v>482</v>
+      </c>
+      <c r="H287" s="1" t="str" cm="1">
+        <f t="array" ref="H287">CRC16HASH(F287)</f>
+        <v>4132</v>
+      </c>
+      <c r="I287" t="str">
+        <f t="shared" si="29"/>
+        <v>{#fig-4132}</v>
+      </c>
+      <c r="J287" t="str">
+        <f t="shared" si="30"/>
+        <v>![Editing the memory store](figures/co/ss_memory_002_clean.png){#fig-4132}</v>
+      </c>
+    </row>
+    <row r="288" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A288">
+        <v>289</v>
+      </c>
+      <c r="B288" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="C288" t="s">
+        <v>4</v>
+      </c>
+      <c r="D288" t="b">
+        <v>0</v>
+      </c>
+      <c r="E288" t="b">
+        <v>0</v>
+      </c>
+      <c r="F288" t="s">
+        <v>485</v>
+      </c>
+      <c r="H288" s="1" t="str" cm="1">
+        <f t="array" ref="H288">CRC16HASH(F288)</f>
+        <v>1501</v>
+      </c>
+      <c r="I288" t="str">
+        <f t="shared" si="29"/>
+        <v>{#fig-1501}</v>
+      </c>
+      <c r="J288" t="str">
+        <f t="shared" si="30"/>
+        <v/>
+      </c>
+    </row>
+    <row r="289" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A289">
+        <v>290</v>
+      </c>
+      <c r="B289" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="C289" t="s">
+        <v>4</v>
+      </c>
+      <c r="D289" t="b">
+        <v>1</v>
+      </c>
+      <c r="E289" t="b">
+        <v>1</v>
+      </c>
+      <c r="F289" t="s">
+        <v>486</v>
+      </c>
+      <c r="G289" t="s">
+        <v>487</v>
+      </c>
+      <c r="H289" s="1" t="str" cm="1">
+        <f t="array" ref="H289">CRC16HASH(F289)</f>
+        <v>AB12</v>
+      </c>
+      <c r="I289" t="str">
+        <f t="shared" si="29"/>
+        <v>{#fig-AB12}</v>
+      </c>
+      <c r="J289" t="str">
+        <f t="shared" si="30"/>
+        <v>![Locating the Evaluations screen](figures/co/ss_evaluations_001_ann.png){#fig-AB12}</v>
+      </c>
+    </row>
+    <row r="290" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A290">
+        <v>291</v>
+      </c>
+      <c r="B290" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="C290" t="s">
+        <v>4</v>
+      </c>
+      <c r="D290" t="b">
+        <v>0</v>
+      </c>
+      <c r="E290" t="b">
+        <v>1</v>
+      </c>
+      <c r="F290" t="s">
+        <v>488</v>
+      </c>
+      <c r="G290" t="s">
+        <v>489</v>
+      </c>
+      <c r="H290" s="1" t="str" cm="1">
+        <f t="array" ref="H290">CRC16HASH(F290)</f>
+        <v>510E</v>
+      </c>
+      <c r="I290" t="str">
+        <f t="shared" si="29"/>
+        <v>{#fig-510E}</v>
+      </c>
+      <c r="J290" t="str">
+        <f t="shared" si="30"/>
+        <v>![Configuring the evaluation process for an agent using synthetic data](figures/co/ss_evaluations_002_clean.png){#fig-510E}</v>
+      </c>
+    </row>
+    <row r="291" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A291">
+        <v>292</v>
+      </c>
+      <c r="B291" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="C291" t="s">
+        <v>4</v>
+      </c>
+      <c r="D291" t="b">
+        <v>0</v>
+      </c>
+      <c r="E291" t="b">
+        <v>0</v>
+      </c>
+      <c r="F291" t="s">
+        <v>490</v>
+      </c>
+      <c r="H291" s="1" t="str" cm="1">
+        <f t="array" ref="H291">CRC16HASH(F291)</f>
+        <v>AD0A</v>
+      </c>
+      <c r="I291" t="str">
+        <f t="shared" si="29"/>
+        <v>{#fig-AD0A}</v>
+      </c>
+      <c r="J291" t="str">
+        <f t="shared" si="30"/>
+        <v/>
+      </c>
+    </row>
+    <row r="292" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A292">
+        <v>293</v>
+      </c>
+      <c r="B292" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="C292" t="s">
+        <v>4</v>
+      </c>
+      <c r="D292" t="b">
+        <v>1</v>
+      </c>
+      <c r="E292" t="b">
+        <v>1</v>
+      </c>
+      <c r="F292" t="s">
+        <v>491</v>
+      </c>
+      <c r="G292" t="s">
+        <v>492</v>
+      </c>
+      <c r="H292" s="1" t="str" cm="1">
+        <f t="array" ref="H292">CRC16HASH(F292)</f>
+        <v>CB0B</v>
+      </c>
+      <c r="I292" t="str">
+        <f t="shared" si="29"/>
+        <v>{#fig-CB0B}</v>
+      </c>
+      <c r="J292" t="str">
+        <f t="shared" si="30"/>
+        <v>![The Evaluator catalog show the details of a built-in evaluator](figures/co/ss_evaluations_003_ann.png){#fig-CB0B}</v>
+      </c>
+    </row>
+    <row r="293" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A293">
+        <v>294</v>
+      </c>
+      <c r="B293" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="C293" t="s">
+        <v>4</v>
+      </c>
+      <c r="D293" t="b">
+        <v>0</v>
+      </c>
+      <c r="E293" t="b">
+        <v>0</v>
+      </c>
+      <c r="F293" t="s">
+        <v>493</v>
+      </c>
+      <c r="H293" s="1" t="str" cm="1">
+        <f t="array" ref="H293">CRC16HASH(F293)</f>
+        <v>A472</v>
+      </c>
+      <c r="I293" t="str">
+        <f t="shared" si="29"/>
+        <v>{#fig-A472}</v>
+      </c>
+      <c r="J293" t="str">
+        <f t="shared" si="30"/>
+        <v/>
+      </c>
+    </row>
+    <row r="294" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A294">
+        <v>295</v>
+      </c>
+      <c r="B294" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="C294" t="s">
+        <v>4</v>
+      </c>
+      <c r="D294" t="b">
+        <v>1</v>
+      </c>
+      <c r="E294" t="b">
+        <v>1</v>
+      </c>
+      <c r="F294" t="s">
+        <v>494</v>
+      </c>
+      <c r="G294" t="s">
+        <v>495</v>
+      </c>
+      <c r="H294" s="1" t="str" cm="1">
+        <f t="array" ref="H294">CRC16HASH(F294)</f>
+        <v>17AA</v>
+      </c>
+      <c r="I294" t="str">
+        <f t="shared" si="29"/>
+        <v>{#fig-17AA}</v>
+      </c>
+      <c r="J294" t="str">
+        <f t="shared" si="30"/>
+        <v>![Locating the Batch jobs feature under Models](figures/co/ss_batchjobs_001_ann.png){#fig-17AA}</v>
+      </c>
+    </row>
+    <row r="295" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A295">
+        <v>296</v>
+      </c>
+      <c r="B295" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="C295" t="s">
+        <v>4</v>
+      </c>
+      <c r="D295" t="b">
+        <v>0</v>
+      </c>
+      <c r="E295" t="b">
+        <v>1</v>
+      </c>
+      <c r="F295" t="s">
+        <v>496</v>
+      </c>
+      <c r="G295" t="s">
+        <v>497</v>
+      </c>
+      <c r="H295" s="1" t="str" cm="1">
+        <f t="array" ref="H295">CRC16HASH(F295)</f>
+        <v>E07D</v>
+      </c>
+      <c r="I295" t="str">
+        <f t="shared" si="29"/>
+        <v>{#fig-E07D}</v>
+      </c>
+      <c r="J295" t="str">
+        <f t="shared" si="30"/>
+        <v>![Uploading .jsonl data to create a batch job](figures/co/ss_batchjobs_002_clean.png){#fig-E07D}</v>
+      </c>
+    </row>
+    <row r="296" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A296">
+        <v>297</v>
+      </c>
+      <c r="B296" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="C296" t="s">
+        <v>4</v>
+      </c>
+      <c r="D296" t="b">
+        <v>0</v>
+      </c>
+      <c r="E296" t="b">
+        <v>0</v>
+      </c>
+      <c r="F296" t="s">
+        <v>499</v>
+      </c>
+      <c r="H296" s="1" t="str" cm="1">
+        <f t="array" ref="H296">CRC16HASH(F296)</f>
+        <v>8700</v>
+      </c>
+      <c r="I296" t="str">
+        <f t="shared" si="29"/>
+        <v>{#fig-8700}</v>
+      </c>
+      <c r="J296" t="str">
+        <f t="shared" si="30"/>
+        <v/>
+      </c>
+    </row>
+    <row r="297" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A297">
+        <v>298</v>
+      </c>
+      <c r="B297" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="C297" t="s">
+        <v>4</v>
+      </c>
+      <c r="D297" t="b">
+        <v>1</v>
+      </c>
+      <c r="E297" t="b">
+        <v>1</v>
+      </c>
+      <c r="F297" t="s">
+        <v>500</v>
+      </c>
+      <c r="G297" t="s">
+        <v>498</v>
+      </c>
+      <c r="H297" s="1" t="str" cm="1">
+        <f t="array" ref="H297">CRC16HASH(F297)</f>
+        <v>2CED</v>
+      </c>
+      <c r="I297" t="str">
+        <f t="shared" si="29"/>
+        <v>{#fig-2CED}</v>
+      </c>
+      <c r="J297" t="str">
+        <f t="shared" si="30"/>
+        <v>![Locating the AI Services options under Models](figures/co/ss_aiservices_001_ann.png){#fig-2CED}</v>
+      </c>
+    </row>
+    <row r="298" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A298">
+        <v>299</v>
+      </c>
+      <c r="B298" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="C298" t="s">
+        <v>4</v>
+      </c>
+      <c r="D298" t="b">
+        <v>0</v>
+      </c>
+      <c r="E298" t="b">
+        <v>1</v>
+      </c>
+      <c r="F298" t="s">
+        <v>502</v>
+      </c>
+      <c r="G298" t="s">
+        <v>501</v>
+      </c>
+      <c r="H298" s="1" t="str" cm="1">
+        <f t="array" ref="H298">CRC16HASH(F298)</f>
+        <v>C30F</v>
+      </c>
+      <c r="I298" t="str">
+        <f t="shared" si="29"/>
+        <v>{#fig-C30F}</v>
+      </c>
+      <c r="J298" t="str">
+        <f t="shared" si="30"/>
+        <v>![Testing out the Voice Live AI service in a Playground](figures/co/ss_aiservices_002_clean.png){#fig-C30F}</v>
+      </c>
+    </row>
+    <row r="299" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A299">
+        <v>303</v>
+      </c>
+      <c r="B299" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="C299" t="s">
+        <v>6</v>
+      </c>
+      <c r="D299" t="b">
+        <v>0</v>
+      </c>
+      <c r="E299" t="b">
+        <v>1</v>
+      </c>
+      <c r="F299" t="s">
+        <v>474</v>
+      </c>
+      <c r="G299" t="s">
+        <v>475</v>
+      </c>
+      <c r="H299" s="1" t="str" cm="1">
+        <f t="array" ref="H299">CRC16HASH(F299)</f>
+        <v>1FED</v>
+      </c>
+      <c r="I299" t="str">
+        <f t="shared" si="29"/>
+        <v>{#fig-1FED}</v>
+      </c>
+      <c r="J299" t="str">
+        <f t="shared" si="30"/>
+        <v>![Governance workflow of the Microsoft Agent Governance Toolkit](figures/co/il_govframework_001_clean.png){#fig-1FED}</v>
+      </c>
+    </row>
+    <row r="300" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A300">
+        <v>304</v>
+      </c>
+      <c r="B300" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="C300" t="s">
+        <v>6</v>
+      </c>
+      <c r="D300" t="b">
+        <v>0</v>
+      </c>
+      <c r="E300" t="b">
+        <v>1</v>
+      </c>
+      <c r="F300" t="s">
+        <v>476</v>
+      </c>
+      <c r="G300" t="s">
+        <v>477</v>
+      </c>
+      <c r="H300" s="1" t="str" cm="1">
+        <f t="array" ref="H300">CRC16HASH(F300)</f>
+        <v>5BE2</v>
+      </c>
+      <c r="I300" t="str">
+        <f t="shared" si="29"/>
+        <v>{#fig-5BE2}</v>
+      </c>
+      <c r="J300" t="str">
+        <f t="shared" si="30"/>
+        <v>![The 4 privilege rings of zero-trust Agent identity](figures/co/il_govframework_002_clean.png){#fig-5BE2}</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Best Practices figures to Ch09
</commit_message>
<xml_diff>
--- a/figures/figure_inventory.xlsx
+++ b/figures/figure_inventory.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Colby\Documents\GitHub\foundry-book\figures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD19EDAF-EF00-4754-A4E2-5F4F0F315775}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE438F32-BF06-49D6-B4D7-1EA635D7BF87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{222F1F68-60B1-49B9-BFF7-2C9CF743DB25}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{222F1F68-60B1-49B9-BFF7-2C9CF743DB25}"/>
   </bookViews>
   <sheets>
     <sheet name="Figure Inventory" sheetId="1" r:id="rId1"/>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1115" uniqueCount="505">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1138" uniqueCount="515">
   <si>
     <t>Type</t>
   </si>
@@ -1577,6 +1577,36 @@
   </si>
   <si>
     <t>Potpourri and Conclusion</t>
+  </si>
+  <si>
+    <t>A more sophisticated architecture with private networking</t>
+  </si>
+  <si>
+    <t>il_architecture_002_clean.png</t>
+  </si>
+  <si>
+    <t>Viewing the Cost Management screen for the Foundry-related resources</t>
+  </si>
+  <si>
+    <t>ss_costs_001_clean.png</t>
+  </si>
+  <si>
+    <t>Viewing the Application Insights service for the Foundry Project</t>
+  </si>
+  <si>
+    <t>Role-based access controls for Foundry resources</t>
+  </si>
+  <si>
+    <t>ss_identity_001_clean.png</t>
+  </si>
+  <si>
+    <t>ss_monitor_001_clean.png</t>
+  </si>
+  <si>
+    <t>ss_monitor_001_ann.png</t>
+  </si>
+  <si>
+    <t>ss_monitor_002_clean.png</t>
   </si>
 </sst>
 </file>
@@ -2211,7 +2241,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B464DFF5-94DA-41E0-B03E-143380050964}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:J301"/>
+  <dimension ref="A1:J307"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.5703125" bestFit="1" customWidth="1"/>
@@ -11787,11 +11817,11 @@
         <v>C0FB</v>
       </c>
       <c r="I283" t="str">
-        <f t="shared" ref="I283:I300" si="29">_xlfn.CONCAT("{#fig-",H283,"}")</f>
+        <f t="shared" ref="I283:I303" si="29">_xlfn.CONCAT("{#fig-",H283,"}")</f>
         <v>{#fig-C0FB}</v>
       </c>
       <c r="J283" t="str">
-        <f t="shared" ref="J283:J300" si="30">IF(E283,_xlfn.CONCAT("![",G283,"](figures/",B283,"/",F283,")",I283),"")</f>
+        <f t="shared" ref="J283:J303" si="30">IF(E283,_xlfn.CONCAT("![",G283,"](figures/",B283,"/",F283,")",I283),"")</f>
         <v>![Quantization of Qwen 2.5 0.5B for CPU inference using Olive](figures/ed/ss_olive_001_clean.png){#fig-C0FB}</v>
       </c>
     </row>
@@ -12307,7 +12337,7 @@
     </row>
     <row r="299" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A299">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="B299" s="11" t="s">
         <v>92</v>
@@ -12342,7 +12372,7 @@
     </row>
     <row r="300" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A300">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="B300" s="11" t="s">
         <v>92</v>
@@ -12377,13 +12407,13 @@
     </row>
     <row r="301" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A301">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="B301" s="11" t="s">
         <v>92</v>
       </c>
       <c r="C301" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D301" t="b">
         <v>0</v>
@@ -12392,22 +12422,229 @@
         <v>1</v>
       </c>
       <c r="F301" t="s">
-        <v>502</v>
+        <v>511</v>
       </c>
       <c r="G301" t="s">
-        <v>503</v>
+        <v>510</v>
       </c>
       <c r="H301" s="1" t="str" cm="1">
         <f t="array" ref="H301">CRC16HASH(F301)</f>
+        <v>285E</v>
+      </c>
+      <c r="I301" t="str">
+        <f t="shared" si="29"/>
+        <v>{#fig-285E}</v>
+      </c>
+      <c r="J301" t="str">
+        <f t="shared" si="30"/>
+        <v>![Role-based access controls for Foundry resources](figures/co/ss_identity_001_clean.png){#fig-285E}</v>
+      </c>
+    </row>
+    <row r="302" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A302">
+        <v>303</v>
+      </c>
+      <c r="B302" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="C302" t="s">
+        <v>4</v>
+      </c>
+      <c r="D302" t="b">
+        <v>0</v>
+      </c>
+      <c r="E302" t="b">
+        <v>0</v>
+      </c>
+      <c r="F302" t="s">
+        <v>512</v>
+      </c>
+      <c r="H302" s="1" t="str" cm="1">
+        <f t="array" ref="H302">CRC16HASH(F302)</f>
+        <v>DE11</v>
+      </c>
+      <c r="I302" t="str">
+        <f t="shared" si="29"/>
+        <v>{#fig-DE11}</v>
+      </c>
+      <c r="J302" t="str">
+        <f t="shared" si="30"/>
+        <v/>
+      </c>
+    </row>
+    <row r="303" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A303">
+        <v>304</v>
+      </c>
+      <c r="B303" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="C303" t="s">
+        <v>4</v>
+      </c>
+      <c r="D303" t="b">
+        <v>0</v>
+      </c>
+      <c r="E303" t="b">
+        <v>1</v>
+      </c>
+      <c r="F303" t="s">
+        <v>513</v>
+      </c>
+      <c r="G303" t="s">
+        <v>450</v>
+      </c>
+      <c r="H303" s="1" t="str" cm="1">
+        <f t="array" ref="H303">CRC16HASH(F303)</f>
+        <v>30D0</v>
+      </c>
+      <c r="I303" t="str">
+        <f t="shared" si="29"/>
+        <v>{#fig-30D0}</v>
+      </c>
+      <c r="J303" t="str">
+        <f t="shared" si="30"/>
+        <v>![Viewing the Monitor tab of an Agent](figures/co/ss_monitor_001_ann.png){#fig-30D0}</v>
+      </c>
+    </row>
+    <row r="304" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A304">
+        <v>305</v>
+      </c>
+      <c r="B304" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="C304" t="s">
+        <v>4</v>
+      </c>
+      <c r="D304" t="b">
+        <v>0</v>
+      </c>
+      <c r="E304" t="b">
+        <v>1</v>
+      </c>
+      <c r="F304" t="s">
+        <v>514</v>
+      </c>
+      <c r="G304" t="s">
+        <v>509</v>
+      </c>
+      <c r="H304" s="1" t="str" cm="1">
+        <f t="array" ref="H304">CRC16HASH(F304)</f>
+        <v>9A1E</v>
+      </c>
+      <c r="I304" t="str">
+        <f t="shared" ref="I304" si="31">_xlfn.CONCAT("{#fig-",H304,"}")</f>
+        <v>{#fig-9A1E}</v>
+      </c>
+      <c r="J304" t="str">
+        <f t="shared" ref="J304" si="32">IF(E304,_xlfn.CONCAT("![",G304,"](figures/",B304,"/",F304,")",I304),"")</f>
+        <v>![Viewing the Application Insights service for the Foundry Project](figures/co/ss_monitor_002_clean.png){#fig-9A1E}</v>
+      </c>
+    </row>
+    <row r="305" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A305">
+        <v>306</v>
+      </c>
+      <c r="B305" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="C305" t="s">
+        <v>4</v>
+      </c>
+      <c r="D305" t="b">
+        <v>0</v>
+      </c>
+      <c r="E305" t="b">
+        <v>1</v>
+      </c>
+      <c r="F305" t="s">
+        <v>508</v>
+      </c>
+      <c r="G305" t="s">
+        <v>507</v>
+      </c>
+      <c r="H305" s="1" t="str" cm="1">
+        <f t="array" ref="H305">CRC16HASH(F305)</f>
+        <v>DD24</v>
+      </c>
+      <c r="I305" t="str">
+        <f t="shared" ref="I305" si="33">_xlfn.CONCAT("{#fig-",H305,"}")</f>
+        <v>{#fig-DD24}</v>
+      </c>
+      <c r="J305" t="str">
+        <f t="shared" ref="J305" si="34">IF(E305,_xlfn.CONCAT("![",G305,"](figures/",B305,"/",F305,")",I305),"")</f>
+        <v>![Viewing the Cost Management screen for the Foundry-related resources](figures/co/ss_costs_001_clean.png){#fig-DD24}</v>
+      </c>
+    </row>
+    <row r="306" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A306">
+        <v>307</v>
+      </c>
+      <c r="B306" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="C306" t="s">
+        <v>6</v>
+      </c>
+      <c r="D306" t="b">
+        <v>0</v>
+      </c>
+      <c r="E306" t="b">
+        <v>1</v>
+      </c>
+      <c r="F306" t="s">
+        <v>502</v>
+      </c>
+      <c r="G306" t="s">
+        <v>503</v>
+      </c>
+      <c r="H306" s="1" t="str" cm="1">
+        <f t="array" ref="H306">CRC16HASH(F306)</f>
         <v>F9BA</v>
       </c>
-      <c r="I301" t="str">
-        <f t="shared" ref="I301" si="31">_xlfn.CONCAT("{#fig-",H301,"}")</f>
+      <c r="I306" t="str">
+        <f t="shared" ref="I306" si="35">_xlfn.CONCAT("{#fig-",H306,"}")</f>
         <v>{#fig-F9BA}</v>
       </c>
-      <c r="J301" t="str">
-        <f t="shared" ref="J301" si="32">IF(E301,_xlfn.CONCAT("![",G301,"](figures/",B301,"/",F301,")",I301),"")</f>
+      <c r="J306" t="str">
+        <f t="shared" ref="J306" si="36">IF(E306,_xlfn.CONCAT("![",G306,"](figures/",B306,"/",F306,")",I306),"")</f>
         <v>![A basic, mostly serverless architecture for AI](figures/co/il_architecture_001_clean.png){#fig-F9BA}</v>
+      </c>
+    </row>
+    <row r="307" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A307">
+        <v>308</v>
+      </c>
+      <c r="B307" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="C307" t="s">
+        <v>6</v>
+      </c>
+      <c r="D307" t="b">
+        <v>0</v>
+      </c>
+      <c r="E307" t="b">
+        <v>1</v>
+      </c>
+      <c r="F307" t="s">
+        <v>506</v>
+      </c>
+      <c r="G307" t="s">
+        <v>505</v>
+      </c>
+      <c r="H307" s="1" t="str" cm="1">
+        <f t="array" ref="H307">CRC16HASH(F307)</f>
+        <v>BDB5</v>
+      </c>
+      <c r="I307" t="str">
+        <f t="shared" ref="I307" si="37">_xlfn.CONCAT("{#fig-",H307,"}")</f>
+        <v>{#fig-BDB5}</v>
+      </c>
+      <c r="J307" t="str">
+        <f t="shared" ref="J307" si="38">IF(E307,_xlfn.CONCAT("![",G307,"](figures/",B307,"/",F307,")",I307),"")</f>
+        <v>![A more sophisticated architecture with private networking](figures/co/il_architecture_002_clean.png){#fig-BDB5}</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Workflow portal figure names in Ch06
(To avoid conflicting hash codes with Ch01
</commit_message>
<xml_diff>
--- a/figures/figure_inventory.xlsx
+++ b/figures/figure_inventory.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Colby\Documents\GitHub\foundry-book\figures\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/colbyford/Documents/GitHub/foundry-book/figures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9714A1D4-DB82-4C27-BBC1-CCEE8DED436E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{917815D1-3703-9D46-AA37-55F05A8E38C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{222F1F68-60B1-49B9-BFF7-2C9CF743DB25}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="44800" windowHeight="22520" xr2:uid="{222F1F68-60B1-49B9-BFF7-2C9CF743DB25}"/>
   </bookViews>
   <sheets>
     <sheet name="Figure Inventory" sheetId="1" r:id="rId1"/>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1142" uniqueCount="517">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1142" uniqueCount="521">
   <si>
     <t>Type</t>
   </si>
@@ -1613,6 +1613,18 @@
   </si>
   <si>
     <t>How GraphRAG forms an entity knowledge graph of communities</t>
+  </si>
+  <si>
+    <t>ss_wfportal_001_clean.png</t>
+  </si>
+  <si>
+    <t>ss_wfportal_001_ann.png</t>
+  </si>
+  <si>
+    <t>ss_wfportal_002_clean.png</t>
+  </si>
+  <si>
+    <t>ss_wfportal_002_ann.png</t>
   </si>
 </sst>
 </file>
@@ -2248,21 +2260,21 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B464DFF5-94DA-41E0-B03E-143380050964}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:J308"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="34.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="73.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="34.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="73.83203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.1640625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="118" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>29</v>
       </c>
@@ -2294,7 +2306,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2329,7 +2341,7 @@
         <v>![Parts of the Microsoft Foundry platform](figures/in/il_foundryplatform_001.png){#fig-4C72}</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>3</v>
       </c>
@@ -2364,7 +2376,7 @@
         <v>![Foundry Resource and Project Organization](figures/in/il_portal_001.png){#fig-3498}</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>4</v>
       </c>
@@ -2399,7 +2411,7 @@
         <v>![Azure Portal - Search Box](figures/in/ss_portal_001_ann.png){#fig-693E}</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>5</v>
       </c>
@@ -2431,7 +2443,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>6</v>
       </c>
@@ -2466,7 +2478,7 @@
         <v>![Azure Portal - Searching for "Microsoft Foundry"](figures/in/ss_portal_002_ann.png){#fig-992A}</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>7</v>
       </c>
@@ -2498,7 +2510,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>8</v>
       </c>
@@ -2533,7 +2545,7 @@
         <v>![Azure Portal - Creating a Foundry Resource](figures/in/ss_portal_003_ann.png){#fig-927}</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>9</v>
       </c>
@@ -2565,7 +2577,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>10</v>
       </c>
@@ -2600,7 +2612,7 @@
         <v>![Create a Foundry Resource - Basics tab](figures/in/ss_portal_004_ann.png){#fig-3901}</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>11</v>
       </c>
@@ -2632,7 +2644,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>12</v>
       </c>
@@ -2667,7 +2679,7 @@
         <v>![Create a Foundry Resource - Storage tab](figures/in/ss_portal_005_ann.png){#fig-A90C}</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>13</v>
       </c>
@@ -2699,7 +2711,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>14</v>
       </c>
@@ -2734,7 +2746,7 @@
         <v>![Create a Foundry Resource - Review + Create tab](figures/in/ss_portal_006_ann.png){#fig-5918}</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>15</v>
       </c>
@@ -2766,7 +2778,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>16</v>
       </c>
@@ -2801,7 +2813,7 @@
         <v>![Azure Portal - Deployment Overview](figures/in/ss_portal_007_clean.png){#fig-CC82}</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>17</v>
       </c>
@@ -2836,7 +2848,7 @@
         <v>![Azure Portal - Resource Group of Foundry-related Resources](figures/in/ss_portal_008_ann.png){#fig-3954}</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>18</v>
       </c>
@@ -2868,7 +2880,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>19</v>
       </c>
@@ -2903,7 +2915,7 @@
         <v>![Azure Portal - Foundry Resource](figures/in/ss_portal_009_ann.png){#fig-A959}</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>20</v>
       </c>
@@ -2935,7 +2947,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>21</v>
       </c>
@@ -2970,7 +2982,7 @@
         <v>![Microsoft Foundry Project Homepage](figures/in/ss_portal_010_clean.png){#fig-7B65}</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>22</v>
       </c>
@@ -3005,7 +3017,7 @@
         <v>![Example Azure CLI Login Subscription Selection](figures/in/cd_cli_001.png){#fig-360B}</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>23</v>
       </c>
@@ -3040,7 +3052,7 @@
         <v>![Foundry Portal Header](figures/in/ss_portalheader_011_clean.png){#fig-B78E}</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>24</v>
       </c>
@@ -3072,7 +3084,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>25</v>
       </c>
@@ -3107,7 +3119,7 @@
         <v>![Copying the Project Endpoint URL](figures/in/ss_portal_012_ann.png){#fig-5C7B}</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>26</v>
       </c>
@@ -3139,7 +3151,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>27</v>
       </c>
@@ -3174,7 +3186,7 @@
         <v>![Locating the Discover tab](figures/md/ss_portal_013_ann.png){#fig-CC76}</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>28</v>
       </c>
@@ -3206,7 +3218,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>29</v>
       </c>
@@ -3241,7 +3253,7 @@
         <v>![Exploring featured models on the Discover page](figures/md/ss_discover_001_ann.png){#fig-BF54}</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>30</v>
       </c>
@@ -3276,7 +3288,7 @@
         <v>![Listing all available models in Foundry](figures/md/ss_discover_002_clean.png){#fig-3E3C}</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>31</v>
       </c>
@@ -3311,7 +3323,7 @@
         <v>![Locating the Compare models button](figures/md/ss_compare_001_ann.png){#fig-767C}</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>32</v>
       </c>
@@ -3346,7 +3358,7 @@
         <v>![Comparing models across benchmarks and capabilities](figures/md/ss_compare_002_clean.png){#fig-68E2}</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>33</v>
       </c>
@@ -3381,7 +3393,7 @@
         <v>![Locating the View leaderboard button](figures/md/ss_leaderboard_001_ann.png){#fig-4BC0}</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>34</v>
       </c>
@@ -3416,7 +3428,7 @@
         <v>![Exploring the model leaderboard](figures/md/ss_leaderboard_002_clean.png){#fig-7953}</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>36</v>
       </c>
@@ -3451,7 +3463,7 @@
         <v>![More details about a model's benchmark performance](figures/md/ss_leaderboard_003_ann.png){#fig-2BD9}</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>37</v>
       </c>
@@ -3486,7 +3498,7 @@
         <v>![Metric details across various model benchmarks](figures/md/ss_leaderboard_004_clean.png){#fig-F14D}</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>38</v>
       </c>
@@ -3518,7 +3530,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>39</v>
       </c>
@@ -3553,7 +3565,7 @@
         <v>![Searching for the Phi-4 model](figures/md/ss_deploy_001_ann.png){#fig-FF9}</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>40</v>
       </c>
@@ -3585,7 +3597,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>41</v>
       </c>
@@ -3620,7 +3632,7 @@
         <v>![Deploying Phi-4 with Default settings](figures/md/ss_deploy_002_ann.png){#fig-FFED}</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>42</v>
       </c>
@@ -3652,7 +3664,7 @@
         <v/>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>43</v>
       </c>
@@ -3687,7 +3699,7 @@
         <v>![Agreeing to the terms for deploying Phi-4](figures/md/ss_deploy_003_ann.png){#fig-6FE0}</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>44</v>
       </c>
@@ -3722,7 +3734,7 @@
         <v>![Playground UI for experimenting with a Phi-4 deployment](figures/md/ss_deploy_004_clean.png){#fig-925F}</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>45</v>
       </c>
@@ -3757,7 +3769,7 @@
         <v>![Learning to make intergalactic pizza](figures/md/ss_deploy_005_clean.png){#fig-6E5B}</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>46</v>
       </c>
@@ -3789,7 +3801,7 @@
         <v/>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>47</v>
       </c>
@@ -3824,7 +3836,7 @@
         <v>![Modifying model parameters](figures/md/ss_deploy_006_ann.png){#fig-3FDF}</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>48</v>
       </c>
@@ -3856,7 +3868,7 @@
         <v/>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>49</v>
       </c>
@@ -3891,7 +3903,7 @@
         <v>![A slightly more martian pizza recipe](figures/md/ss_deploy_008_clean.png){#fig-C260}</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>50</v>
       </c>
@@ -3926,7 +3938,7 @@
         <v>![Deployment endpoint and key on the Details tab](figures/md/ss_deploy_007_ann.png){#fig-AFD2}</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>51</v>
       </c>
@@ -3961,7 +3973,7 @@
         <v>![The agentic flow between inputs, the model, tools, and outputs](figures/ad/il_agent_001.png){#fig-2027}</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>52</v>
       </c>
@@ -3993,7 +4005,7 @@
         <v/>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>53</v>
       </c>
@@ -4028,7 +4040,7 @@
         <v>![Creating an agent from the Agents tab](figures/ad/ss_agent_001_ann.png){#fig-1BC}</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>54</v>
       </c>
@@ -4060,7 +4072,7 @@
         <v/>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>55</v>
       </c>
@@ -4095,7 +4107,7 @@
         <v>![Giving your new agent a name](figures/ad/ss_agent_002_ann.png){#fig-F1A8}</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>56</v>
       </c>
@@ -4127,7 +4139,7 @@
         <v/>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>57</v>
       </c>
@@ -4162,7 +4174,7 @@
         <v>![Listing all Agents in your Project](figures/ad/ss_agent_003_ann.png){#fig-61A5}</v>
       </c>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>58</v>
       </c>
@@ -4197,7 +4209,7 @@
         <v>![Your real estate Agent's Playground](figures/ad/ss_agent_004_clean.png){#fig-C6EC}</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>59</v>
       </c>
@@ -4229,7 +4241,7 @@
         <v/>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A59">
         <v>60</v>
       </c>
@@ -4264,7 +4276,7 @@
         <v>![Giving the real estate Agent instructions](figures/ad/ss_agent_005_ann.png){#fig-C18E}</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A60">
         <v>61</v>
       </c>
@@ -4296,7 +4308,7 @@
         <v/>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A61">
         <v>62</v>
       </c>
@@ -4331,7 +4343,7 @@
         <v>![Previewing an Agent app](figures/ad/ss_agent_006_ann.png){#fig-319A}</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A62">
         <v>63</v>
       </c>
@@ -4366,7 +4378,7 @@
         <v>![Your demo Agent app](figures/ad/ss_agent_007_clean.png){#fig-82E3}</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A63">
         <v>64</v>
       </c>
@@ -4398,7 +4410,7 @@
         <v/>
       </c>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A64">
         <v>65</v>
       </c>
@@ -4433,7 +4445,7 @@
         <v>![An example, yet beautiful home on Zillow](figures/ad/ss_agent_007b_cens_clean.png){#fig-AC5A}</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A65">
         <v>66</v>
       </c>
@@ -4465,7 +4477,7 @@
         <v/>
       </c>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A66">
         <v>67</v>
       </c>
@@ -4500,7 +4512,7 @@
         <v>![The Agent's Instagram post](figures/ad/ss_agent_008_cens_clean.png){#fig-1600}</v>
       </c>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A67">
         <v>68</v>
       </c>
@@ -4532,7 +4544,7 @@
         <v/>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A68">
         <v>69</v>
       </c>
@@ -4567,7 +4579,7 @@
         <v>![The Agent failing to read from the web](figures/ad/ss_agent_008b_cens_clean.png){#fig-5F6F}</v>
       </c>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A69">
         <v>70</v>
       </c>
@@ -4599,7 +4611,7 @@
         <v/>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A70">
         <v>71</v>
       </c>
@@ -4634,7 +4646,7 @@
         <v>![Publishing your Agent](figures/ad/ss_agent_009_ann.png){#fig-C1DB}</v>
       </c>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A71">
         <v>72</v>
       </c>
@@ -4666,7 +4678,7 @@
         <v/>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A72">
         <v>73</v>
       </c>
@@ -4701,7 +4713,7 @@
         <v>![Making your Agent production-ready](figures/ad/ss_agent_010_ann.png){#fig-54E0}</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A73">
         <v>74</v>
       </c>
@@ -4736,7 +4748,7 @@
         <v>![Your Agent was published successfully](figures/ad/ss_agent_011_clean.png){#fig-C900}</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A74">
         <v>75</v>
       </c>
@@ -4768,7 +4780,7 @@
         <v/>
       </c>
     </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A75">
         <v>76</v>
       </c>
@@ -4803,7 +4815,7 @@
         <v>![Exploring Tools on the Discover page](figures/ad/ss_tools_001_ann.png){#fig-D127}</v>
       </c>
     </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A76">
         <v>77</v>
       </c>
@@ -4835,7 +4847,7 @@
         <v/>
       </c>
     </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A77">
         <v>78</v>
       </c>
@@ -4870,7 +4882,7 @@
         <v>![Locating your real estate Agent](figures/ad/ss_tools_002_ann.png){#fig-2133}</v>
       </c>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A78">
         <v>79</v>
       </c>
@@ -4902,7 +4914,7 @@
         <v/>
       </c>
     </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A79">
         <v>80</v>
       </c>
@@ -4937,7 +4949,7 @@
         <v>![Adding a Tool to your Agent](figures/ad/ss_tools_003_ann.png){#fig-B13E}</v>
       </c>
     </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A80">
         <v>81</v>
       </c>
@@ -4969,7 +4981,7 @@
         <v/>
       </c>
     </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A81">
         <v>82</v>
       </c>
@@ -5004,7 +5016,7 @@
         <v>![Selecting the Web search Tool](figures/ad/ss_tools_004_ann.png){#fig-8118}</v>
       </c>
     </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A82">
         <v>83</v>
       </c>
@@ -5036,7 +5048,7 @@
         <v/>
       </c>
     </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A83">
         <v>84</v>
       </c>
@@ -5071,7 +5083,7 @@
         <v>![Accepting the terms for Web Search](figures/ad/ss_tools_005_ann.png){#fig-1115}</v>
       </c>
     </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A84">
         <v>85</v>
       </c>
@@ -5103,7 +5115,7 @@
         <v/>
       </c>
     </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A85">
         <v>86</v>
       </c>
@@ -5138,7 +5150,7 @@
         <v>![Saving and previewing the Agent with Web Search connected](figures/ad/ss_tools_006_ann.png){#fig-E101}</v>
       </c>
     </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A86">
         <v>87</v>
       </c>
@@ -5170,7 +5182,7 @@
         <v/>
       </c>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A87">
         <v>88</v>
       </c>
@@ -5205,7 +5217,7 @@
         <v>![A much more functional real estate Agent](figures/ad/ss_tools_007_cens_clean.png){#fig-BB7C}</v>
       </c>
     </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A88">
         <v>89</v>
       </c>
@@ -5240,7 +5252,7 @@
         <v>![Example MCP-based architecture](figures/ad/il_tools_001.png){#fig-4852}</v>
       </c>
     </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A89">
         <v>90</v>
       </c>
@@ -5275,7 +5287,7 @@
         <v>![Foundry MCP client-server flow](figures/ad/il_mcp_001.png){#fig-3CBD}</v>
       </c>
     </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A90">
         <v>91</v>
       </c>
@@ -5310,7 +5322,7 @@
         <v>![Configuring a general MCP tool](figures/ad/ss_tools_008_clean.png){#fig-3AB9}</v>
       </c>
     </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A91">
         <v>92</v>
       </c>
@@ -5345,7 +5357,7 @@
         <v>![Selecting your Subscription and Resource Group in the azd prompt](figures/ad/ss_mcp_001_clean.png){#fig-C02E}</v>
       </c>
     </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A92">
         <v>93</v>
       </c>
@@ -5380,7 +5392,7 @@
         <v>![azd has successfully deployed the resources](figures/ad/ss_mcp_002_clean.png){#fig-8421}</v>
       </c>
     </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A93">
         <v>94</v>
       </c>
@@ -5412,7 +5424,7 @@
         <v/>
       </c>
     </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A94">
         <v>95</v>
       </c>
@@ -5447,7 +5459,7 @@
         <v>![Successful deployment of the MCP Toolkit](figures/ad/ss_mcp_003_ann.png){#fig-B89C}</v>
       </c>
     </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A95">
         <v>96</v>
       </c>
@@ -5479,7 +5491,7 @@
         <v/>
       </c>
     </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A96">
         <v>97</v>
       </c>
@@ -5514,7 +5526,7 @@
         <v>![Authenticating the MCP Toolkit with your Tenant and Entra App IDs](figures/ad/ss_mcp_004_ann.png){#fig-88BA}</v>
       </c>
     </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A97">
         <v>98</v>
       </c>
@@ -5546,7 +5558,7 @@
         <v/>
       </c>
     </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A98">
         <v>99</v>
       </c>
@@ -5581,7 +5593,7 @@
         <v>![Granting permissions to the MCP Toolkit app](figures/ad/ss_mcp_005_ann.png){#fig-18B7}</v>
       </c>
     </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A99">
         <v>100</v>
       </c>
@@ -5613,7 +5625,7 @@
         <v/>
       </c>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A100">
         <v>101</v>
       </c>
@@ -5648,7 +5660,7 @@
         <v>![Successful authentication to the MCP Toolkit app](figures/ad/ss_mcp_006_ann.png){#fig-E8A3}</v>
       </c>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A101">
         <v>102</v>
       </c>
@@ -5680,7 +5692,7 @@
         <v/>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A102">
         <v>103</v>
       </c>
@@ -5715,7 +5727,7 @@
         <v>![The Cosmos DB screen in the Azure Portal](figures/ad/ss_cosmos_001_ann.png){#fig-23F7}</v>
       </c>
     </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A103">
         <v>104</v>
       </c>
@@ -5747,7 +5759,7 @@
         <v/>
       </c>
     </row>
-    <row r="104" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A104">
         <v>105</v>
       </c>
@@ -5782,7 +5794,7 @@
         <v>![Locating your Cosmos DB URI and Key](figures/ad/ss_cosmos_002_ann.png){#fig-D3E3}</v>
       </c>
     </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A105">
         <v>106</v>
       </c>
@@ -5814,7 +5826,7 @@
         <v/>
       </c>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A106">
         <v>107</v>
       </c>
@@ -5849,7 +5861,7 @@
         <v>![Adding another Tool to your Agent](figures/ad/ss_cosmos_003_ann.png){#fig-43EE}</v>
       </c>
     </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A107">
         <v>108</v>
       </c>
@@ -5881,7 +5893,7 @@
         <v/>
       </c>
     </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A108">
         <v>109</v>
       </c>
@@ -5916,7 +5928,7 @@
         <v>![Locating the Cosmos DB Tool in the Catalog](figures/ad/ss_cosmos_004_ann.png){#fig-73C8}</v>
       </c>
     </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A109">
         <v>110</v>
       </c>
@@ -5948,7 +5960,7 @@
         <v/>
       </c>
     </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A110">
         <v>111</v>
       </c>
@@ -5983,7 +5995,7 @@
         <v>![Information about hosting MCP servers](figures/ad/ss_cosmos_005_ann.png){#fig-E3C5}</v>
       </c>
     </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A111">
         <v>112</v>
       </c>
@@ -6015,7 +6027,7 @@
         <v/>
       </c>
     </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A112">
         <v>113</v>
       </c>
@@ -6050,7 +6062,7 @@
         <v>![Filling in the URI and authentication for the Cosmos DB Tool connection](figures/ad/ss_cosmos_006_ann.png){#fig-13D1}</v>
       </c>
     </row>
-    <row r="113" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A113">
         <v>114</v>
       </c>
@@ -6082,7 +6094,7 @@
         <v/>
       </c>
     </row>
-    <row r="114" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A114">
         <v>115</v>
       </c>
@@ -6117,7 +6129,7 @@
         <v>![Checking that your Cosmos DB Tool is connected](figures/ad/ss_cosmos_007_ann.png){#fig-83DC}</v>
       </c>
     </row>
-    <row r="115" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A115">
         <v>116</v>
       </c>
@@ -6149,7 +6161,7 @@
         <v/>
       </c>
     </row>
-    <row r="116" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A116">
         <v>117</v>
       </c>
@@ -6184,7 +6196,7 @@
         <v>![Checking the Cosmos DB Tool usage in the Agent response](figures/ad/ss_cosmos_008_ann.png){#fig-739D}</v>
       </c>
     </row>
-    <row r="117" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A117">
         <v>118</v>
       </c>
@@ -6219,7 +6231,7 @@
         <v>![A successful Cosmos DB Tool call and augmented Agent response](figures/ad/ss_cosmos_009_clean.png){#fig-8361}</v>
       </c>
     </row>
-    <row r="118" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A118">
         <v>119</v>
       </c>
@@ -6251,7 +6263,7 @@
         <v/>
       </c>
     </row>
-    <row r="119" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A119">
         <v>120</v>
       </c>
@@ -6286,7 +6298,7 @@
         <v>![Creating a new Cosmos DB container](figures/ad/ss_database_001_ann.png){#fig-5117}</v>
       </c>
     </row>
-    <row r="120" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A120">
         <v>121</v>
       </c>
@@ -6318,7 +6330,7 @@
         <v/>
       </c>
     </row>
-    <row r="121" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A121">
         <v>122</v>
       </c>
@@ -6353,7 +6365,7 @@
         <v>![Creating a new Cosmos DB database](figures/ad/ss_database_002_ann.png){#fig-A103}</v>
       </c>
     </row>
-    <row r="122" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A122">
         <v>123</v>
       </c>
@@ -6385,7 +6397,7 @@
         <v/>
       </c>
     </row>
-    <row r="123" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A123">
         <v>124</v>
       </c>
@@ -6420,7 +6432,7 @@
         <v>![Uploading property records to your database](figures/ad/ss_database_003_ann.png){#fig-310E}</v>
       </c>
     </row>
-    <row r="124" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A124">
         <v>125</v>
       </c>
@@ -6455,7 +6467,7 @@
         <v>![Listing your property records](figures/ad/ss_database_004_clean.png){#fig-CA93}</v>
       </c>
     </row>
-    <row r="125" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A125">
         <v>126</v>
       </c>
@@ -6490,7 +6502,7 @@
         <v>![Orchestrating multi-source, complex RAG pipelines](figures/kb/il_layers_001.png){#fig-2B5B}</v>
       </c>
     </row>
-    <row r="126" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A126">
         <v>127</v>
       </c>
@@ -6525,7 +6537,7 @@
         <v>![Building a multi-source Agent for financial insights](figures/kb/il_multisource_001.png){#fig-E787}</v>
       </c>
     </row>
-    <row r="127" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A127">
         <v>128</v>
       </c>
@@ -6560,7 +6572,7 @@
         <v>![The basic RAG pattern](figures/kb/il_rag_001.png){#fig-D293}</v>
       </c>
     </row>
-    <row r="128" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A128">
         <v>129</v>
       </c>
@@ -6595,7 +6607,7 @@
         <v>![Knowledge sources as part of the AI Search data retreival](figures/kb/il_knowledgesources_001.png){#fig-E63}</v>
       </c>
     </row>
-    <row r="129" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A129">
         <v>130</v>
       </c>
@@ -6630,7 +6642,7 @@
         <v>![Enrichment tasks for documents](figures/kb/il_enrichment_001.png){#fig-3399}</v>
       </c>
     </row>
-    <row r="130" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A130">
         <v>131</v>
       </c>
@@ -6665,7 +6677,7 @@
         <v>![Microsoft's public earnings release page](figures/kb/ss_storage_001_clean.png){#fig-CB8E}</v>
       </c>
     </row>
-    <row r="131" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A131">
         <v>132</v>
       </c>
@@ -6697,7 +6709,7 @@
         <v/>
       </c>
     </row>
-    <row r="132" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A132">
         <v>133</v>
       </c>
@@ -6732,7 +6744,7 @@
         <v>![Creating a new Container in Azure Storage](figures/kb/ss_portal_001_ann.png){#fig-693E}</v>
       </c>
     </row>
-    <row r="133" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A133">
         <v>134</v>
       </c>
@@ -6764,7 +6776,7 @@
         <v/>
       </c>
     </row>
-    <row r="134" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A134">
         <v>135</v>
       </c>
@@ -6799,7 +6811,7 @@
         <v>![Uploading the financial reports to Azure Storage](figures/kb/ss_storage_002_ann.png){#fig-72EE}</v>
       </c>
     </row>
-    <row r="135" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A135">
         <v>136</v>
       </c>
@@ -6831,7 +6843,7 @@
         <v/>
       </c>
     </row>
-    <row r="136" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A136">
         <v>137</v>
       </c>
@@ -6866,7 +6878,7 @@
         <v>![Importing data into Azure AI Search](figures/kb/ss_search_001_ann.png){#fig-F62E}</v>
       </c>
     </row>
-    <row r="137" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A137">
         <v>138</v>
       </c>
@@ -6898,7 +6910,7 @@
         <v/>
       </c>
     </row>
-    <row r="138" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A138">
         <v>139</v>
       </c>
@@ -6933,7 +6945,7 @@
         <v>![Selecting the Azure Blob Storage built-in indexer](figures/kb/ss_search_002_ann.png){#fig-63A}</v>
       </c>
     </row>
-    <row r="139" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A139">
         <v>140</v>
       </c>
@@ -6965,7 +6977,7 @@
         <v/>
       </c>
     </row>
-    <row r="140" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A140">
         <v>141</v>
       </c>
@@ -7000,7 +7012,7 @@
         <v>![Selecting the Keyword search scenario](figures/kb/ss_search_003_ann.png){#fig-9637}</v>
       </c>
     </row>
-    <row r="141" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A141">
         <v>142</v>
       </c>
@@ -7035,7 +7047,7 @@
         <v>![Connecting to data for the Keyword search](figures/kb/ss_search_004_clean.png){#fig-20C0}</v>
       </c>
     </row>
-    <row r="142" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A142">
         <v>143</v>
       </c>
@@ -7067,7 +7079,7 @@
         <v/>
       </c>
     </row>
-    <row r="143" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A143">
         <v>144</v>
       </c>
@@ -7102,7 +7114,7 @@
         <v>![Enrichments options for Keyword search](figures/kb/ss_enrichments_001_ann.png){#fig-6AFC}</v>
       </c>
     </row>
-    <row r="144" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A144">
         <v>145</v>
       </c>
@@ -7134,7 +7146,7 @@
         <v/>
       </c>
     </row>
-    <row r="145" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A145">
         <v>146</v>
       </c>
@@ -7169,7 +7181,7 @@
         <v>![Extract entities selection](figures/kb/ss_enrichments_002_ann.png){#fig-9AE8}</v>
       </c>
     </row>
-    <row r="146" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A146">
         <v>147</v>
       </c>
@@ -7201,7 +7213,7 @@
         <v/>
       </c>
     </row>
-    <row r="147" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A147">
         <v>148</v>
       </c>
@@ -7236,7 +7248,7 @@
         <v>![Extract text from images selection](figures/kb/ss_enrichments_003_ann.png){#fig-AE5}</v>
       </c>
     </row>
-    <row r="148" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A148">
         <v>149</v>
       </c>
@@ -7271,7 +7283,7 @@
         <v>![Previewing the field mappings](figures/kb/ss_enrichments_004_clean.png){#fig-E99C}</v>
       </c>
     </row>
-    <row r="149" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A149">
         <v>150</v>
       </c>
@@ -7303,7 +7315,7 @@
         <v/>
       </c>
     </row>
-    <row r="150" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A150">
         <v>151</v>
       </c>
@@ -7338,7 +7350,7 @@
         <v>![Advanced settings for semantic search and re-indexing on a schedule](figures/kb/ss_enrichments_005_ann.png){#fig-AACE}</v>
       </c>
     </row>
-    <row r="151" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A151">
         <v>152</v>
       </c>
@@ -7370,7 +7382,7 @@
         <v/>
       </c>
     </row>
-    <row r="152" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A152">
         <v>153</v>
       </c>
@@ -7405,7 +7417,7 @@
         <v>![Reviewing the selections for Keyword search](figures/kb/ss_enrichments_006_ann.png){#fig-5ADA}</v>
       </c>
     </row>
-    <row r="153" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A153">
         <v>154</v>
       </c>
@@ -7437,7 +7449,7 @@
         <v/>
       </c>
     </row>
-    <row r="154" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A154">
         <v>155</v>
       </c>
@@ -7472,7 +7484,7 @@
         <v>![A successful indexing of the Microsoft financial documents from Azure Storage](figures/kb/ss_search_005_ann.png){#fig-361C}</v>
       </c>
     </row>
-    <row r="155" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A155">
         <v>156</v>
       </c>
@@ -7504,7 +7516,7 @@
         <v/>
       </c>
     </row>
-    <row r="156" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A156">
         <v>157</v>
       </c>
@@ -7539,7 +7551,7 @@
         <v>![Connecting to an Azure AI Search resource](figures/kb/ss_knowledge_001_ann.png){#fig-33E}</v>
       </c>
     </row>
-    <row r="157" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A157">
         <v>158</v>
       </c>
@@ -7571,7 +7583,7 @@
         <v/>
       </c>
     </row>
-    <row r="158" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A158">
         <v>159</v>
       </c>
@@ -7606,7 +7618,7 @@
         <v>![Creating a new Knowledge Base](figures/kb/ss_knowledge_002_ann.png){#fig-F32A}</v>
       </c>
     </row>
-    <row r="159" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A159">
         <v>160</v>
       </c>
@@ -7638,7 +7650,7 @@
         <v/>
       </c>
     </row>
-    <row r="160" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A160">
         <v>161</v>
       </c>
@@ -7673,7 +7685,7 @@
         <v>![Selecting a Knowledge Base type](figures/kb/ss_knowledge_003_ann.png){#fig-6327}</v>
       </c>
     </row>
-    <row r="161" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A161">
         <v>162</v>
       </c>
@@ -7705,7 +7717,7 @@
         <v/>
       </c>
     </row>
-    <row r="162" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A162">
         <v>163</v>
       </c>
@@ -7740,7 +7752,7 @@
         <v>![Connecting to the Search Index](figures/kb/ss_knowledge_004_ann.png){#fig-5301}</v>
       </c>
     </row>
-    <row r="163" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A163">
         <v>164</v>
       </c>
@@ -7772,7 +7784,7 @@
         <v/>
       </c>
     </row>
-    <row r="164" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A164">
         <v>165</v>
       </c>
@@ -7807,7 +7819,7 @@
         <v>![Final steps in creating the knowledge base](figures/kb/ss_knowledge_005_ann.png){#fig-C30C}</v>
       </c>
     </row>
-    <row r="165" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A165">
         <v>166</v>
       </c>
@@ -7839,7 +7851,7 @@
         <v/>
       </c>
     </row>
-    <row r="166" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A166">
         <v>167</v>
       </c>
@@ -7874,7 +7886,7 @@
         <v>![Connecting the Agent to the knowledge base](figures/kb/ss_agent_001_ann.png){#fig-1BC}</v>
       </c>
     </row>
-    <row r="167" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A167">
         <v>168</v>
       </c>
@@ -7909,7 +7921,7 @@
         <v>![Asking the Robo CFO Agent about year over year revenue](figures/kb/ss_agent_002_clean.png){#fig-4EF2}</v>
       </c>
     </row>
-    <row r="168" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A168">
         <v>169</v>
       </c>
@@ -7944,7 +7956,7 @@
         <v>![Asking about Microsoft's 2026 outlook](figures/kb/ss_agent_003_clean.png){#fig-B2F6}</v>
       </c>
     </row>
-    <row r="169" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A169">
         <v>170</v>
       </c>
@@ -7979,7 +7991,7 @@
         <v>![The "Microsoft FY26 Q2 Outlook" PowerPoint slide](figures/kb/ss_agent_004_clean.png){#fig-C6EC}</v>
       </c>
     </row>
-    <row r="170" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A170">
         <v>171</v>
       </c>
@@ -8011,7 +8023,7 @@
         <v/>
       </c>
     </row>
-    <row r="171" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A171">
         <v>172</v>
       </c>
@@ -8046,7 +8058,7 @@
         <v>![Creating a new fine-tuning job](figures/ft/ss_finetune_001_ann.png){#fig-706E}</v>
       </c>
     </row>
-    <row r="172" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A172">
         <v>173</v>
       </c>
@@ -8078,7 +8090,7 @@
         <v/>
       </c>
     </row>
-    <row r="173" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A173">
         <v>174</v>
       </c>
@@ -8113,7 +8125,7 @@
         <v>![Defining the fine-tuning job setting](figures/ft/ss_finetune_002_ann.png){#fig-807A}</v>
       </c>
     </row>
-    <row r="174" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A174">
         <v>175</v>
       </c>
@@ -8145,7 +8157,7 @@
         <v/>
       </c>
     </row>
-    <row r="175" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A175">
         <v>176</v>
       </c>
@@ -8177,7 +8189,7 @@
         <v/>
       </c>
     </row>
-    <row r="176" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A176">
         <v>177</v>
       </c>
@@ -8212,7 +8224,7 @@
         <v>![Viewing the status of your new tuning job](figures/ft/ss_finetune_003_ann.png){#fig-1077}</v>
       </c>
     </row>
-    <row r="177" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A177">
         <v>178</v>
       </c>
@@ -8244,7 +8256,7 @@
         <v/>
       </c>
     </row>
-    <row r="178" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A178">
         <v>179</v>
       </c>
@@ -8276,7 +8288,7 @@
         <v/>
       </c>
     </row>
-    <row r="179" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A179">
         <v>180</v>
       </c>
@@ -8311,7 +8323,7 @@
         <v>![The Monitor tab, showing fine-tuning metrics](figures/ft/ss_finetune_005_ann.png){#fig-B05C}</v>
       </c>
     </row>
-    <row r="180" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A180">
         <v>181</v>
       </c>
@@ -8343,7 +8355,7 @@
         <v/>
       </c>
     </row>
-    <row r="181" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A181">
         <v>182</v>
       </c>
@@ -8378,7 +8390,7 @@
         <v>![A completed fine-tuning status and metrics](figures/ft/ss_finetune_006_ann.png){#fig-4048}</v>
       </c>
     </row>
-    <row r="182" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A182">
         <v>183</v>
       </c>
@@ -8410,7 +8422,7 @@
         <v/>
       </c>
     </row>
-    <row r="183" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A183">
         <v>184</v>
       </c>
@@ -8445,7 +8457,7 @@
         <v>![Customizing the fine-tuned model deployment](figures/ft/ss_finetune_007_ann.png){#fig-D045}</v>
       </c>
     </row>
-    <row r="184" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A184">
         <v>185</v>
       </c>
@@ -8480,7 +8492,7 @@
         <v>![Adding instructions and playing with your new medical assistant model](figures/ft/ss_finetune_008_clean.png){#fig-124F}</v>
       </c>
     </row>
-    <row r="185" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A185">
         <v>186</v>
       </c>
@@ -8512,7 +8524,7 @@
         <v/>
       </c>
     </row>
-    <row r="186" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A186">
         <v>187</v>
       </c>
@@ -8547,7 +8559,7 @@
         <v>![Navigating to the Synthetic generation tab](figures/ft/ss_syntheticdata_001_ann.png){#fig-2C04}</v>
       </c>
     </row>
-    <row r="187" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A187">
         <v>188</v>
       </c>
@@ -8579,7 +8591,7 @@
         <v/>
       </c>
     </row>
-    <row r="188" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A188">
         <v>189</v>
       </c>
@@ -8614,7 +8626,7 @@
         <v>![Adding cardiology documents for synthetic data generation](figures/ft/ss_syntheticdata_002_ann.png){#fig-DC10}</v>
       </c>
     </row>
-    <row r="189" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A189">
         <v>190</v>
       </c>
@@ -8646,7 +8658,7 @@
         <v/>
       </c>
     </row>
-    <row r="190" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A190">
         <v>191</v>
       </c>
@@ -8681,7 +8693,7 @@
         <v>![Monitoring the queued synthetic data job](figures/ft/ss_syntheticdata_003a_clean.png){#fig-2555}</v>
       </c>
     </row>
-    <row r="191" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A191">
         <v>192</v>
       </c>
@@ -8716,7 +8728,7 @@
         <v>![Viewing the synthetic data job results](figures/ft/ss_syntheticdata_003_ann.png){#fig-4C1D}</v>
       </c>
     </row>
-    <row r="192" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A192">
         <v>193</v>
       </c>
@@ -8748,7 +8760,7 @@
         <v/>
       </c>
     </row>
-    <row r="193" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A193">
         <v>194</v>
       </c>
@@ -8783,7 +8795,7 @@
         <v>![Continuing to fine-tune with the new cardiology synthetic data](figures/ft/ss_syntheticdata_004_ann.png){#fig-7C3B}</v>
       </c>
     </row>
-    <row r="194" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A194">
         <v>195</v>
       </c>
@@ -8815,7 +8827,7 @@
         <v/>
       </c>
     </row>
-    <row r="195" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A195">
         <v>196</v>
       </c>
@@ -8850,7 +8862,7 @@
         <v>![Initializing a fine-tuning job from the CLI](figures/ft/ss_cli_001_clean_neg.png){#fig-71F5}</v>
       </c>
     </row>
-    <row r="196" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A196">
         <v>197</v>
       </c>
@@ -8882,7 +8894,7 @@
         <v/>
       </c>
     </row>
-    <row r="197" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A197">
         <v>198</v>
       </c>
@@ -8917,7 +8929,7 @@
         <v>![Uploading training data and starting the fine-tuning job](figures/ft/ss_cli_002_clean_neg.png){#fig-70B6}</v>
       </c>
     </row>
-    <row r="198" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A198">
         <v>199</v>
       </c>
@@ -8949,7 +8961,7 @@
         <v/>
       </c>
     </row>
-    <row r="199" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A199">
         <v>200</v>
       </c>
@@ -8984,7 +8996,7 @@
         <v>![Listing fine-tuning jobs and showing job details](figures/ft/ss_cli_003_clean_neg.png){#fig-7077}</v>
       </c>
     </row>
-    <row r="200" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A200">
         <v>201</v>
       </c>
@@ -9019,7 +9031,7 @@
         <v>![Workflow template patterns](figures/wf/il_types_001_clean.png){#fig-965B}</v>
       </c>
     </row>
-    <row r="201" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A201">
         <v>202</v>
       </c>
@@ -9036,22 +9048,22 @@
         <v>0</v>
       </c>
       <c r="F201" t="s">
-        <v>100</v>
+        <v>517</v>
       </c>
       <c r="H201" s="1" t="str" cm="1">
         <f t="array" ref="H201">CRC16HASH(F201)</f>
-        <v>449C</v>
+        <v>3E52</v>
       </c>
       <c r="I201" t="str">
         <f t="shared" si="7"/>
-        <v>{#fig-449C}</v>
+        <v>{#fig-3E52}</v>
       </c>
       <c r="J201" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
     </row>
-    <row r="202" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A202">
         <v>203</v>
       </c>
@@ -9068,25 +9080,25 @@
         <v>1</v>
       </c>
       <c r="F202" t="s">
-        <v>99</v>
+        <v>518</v>
       </c>
       <c r="G202" t="s">
         <v>355</v>
       </c>
       <c r="H202" s="1" t="str" cm="1">
         <f t="array" ref="H202">CRC16HASH(F202)</f>
-        <v>693E</v>
+        <v>CFD6</v>
       </c>
       <c r="I202" t="str">
         <f t="shared" si="7"/>
-        <v>{#fig-693E}</v>
+        <v>{#fig-CFD6}</v>
       </c>
       <c r="J202" t="str">
         <f t="shared" si="6"/>
-        <v>![Locating Workflows from the Foundry UI](figures/wf/ss_portal_001_ann.png){#fig-693E}</v>
-      </c>
-    </row>
-    <row r="203" spans="1:10" x14ac:dyDescent="0.25">
+        <v>![Locating Workflows from the Foundry UI](figures/wf/ss_wfportal_001_ann.png){#fig-CFD6}</v>
+      </c>
+    </row>
+    <row r="203" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A203">
         <v>204</v>
       </c>
@@ -9103,22 +9115,22 @@
         <v>0</v>
       </c>
       <c r="F203" t="s">
-        <v>102</v>
+        <v>519</v>
       </c>
       <c r="H203" s="1" t="str" cm="1">
         <f t="array" ref="H203">CRC16HASH(F203)</f>
-        <v>93</v>
+        <v>7A5D</v>
       </c>
       <c r="I203" t="str">
         <f t="shared" si="7"/>
-        <v>{#fig-93}</v>
+        <v>{#fig-7A5D}</v>
       </c>
       <c r="J203" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
     </row>
-    <row r="204" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A204">
         <v>205</v>
       </c>
@@ -9135,25 +9147,25 @@
         <v>1</v>
       </c>
       <c r="F204" t="s">
-        <v>101</v>
+        <v>520</v>
       </c>
       <c r="G204" t="s">
         <v>357</v>
       </c>
       <c r="H204" s="1" t="str" cm="1">
         <f t="array" ref="H204">CRC16HASH(F204)</f>
-        <v>992A</v>
+        <v>3FC2</v>
       </c>
       <c r="I204" t="str">
         <f t="shared" si="7"/>
-        <v>{#fig-992A}</v>
+        <v>{#fig-3FC2}</v>
       </c>
       <c r="J204" t="str">
         <f t="shared" si="6"/>
-        <v>![Selecting the Human in Loop workflow template](figures/wf/ss_portal_002_ann.png){#fig-992A}</v>
-      </c>
-    </row>
-    <row r="205" spans="1:10" x14ac:dyDescent="0.25">
+        <v>![Selecting the Human in Loop workflow template](figures/wf/ss_wfportal_002_ann.png){#fig-3FC2}</v>
+      </c>
+    </row>
+    <row r="205" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A205">
         <v>206</v>
       </c>
@@ -9188,7 +9200,7 @@
         <v>![A blank Workflow canvas with only a start node](figures/wf/ss_canvas_001_clean.png){#fig-F349}</v>
       </c>
     </row>
-    <row r="206" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A206">
         <v>207</v>
       </c>
@@ -9220,7 +9232,7 @@
         <v/>
       </c>
     </row>
-    <row r="207" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A207">
         <v>208</v>
       </c>
@@ -9252,7 +9264,7 @@
         <v/>
       </c>
     </row>
-    <row r="208" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A208">
         <v>209</v>
       </c>
@@ -9287,7 +9299,7 @@
         <v>![Saving the Math Coder Workflow](figures/wf/ss_save_001_ann.png){#fig-C624}</v>
       </c>
     </row>
-    <row r="209" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A209">
         <v>210</v>
       </c>
@@ -9319,7 +9331,7 @@
         <v/>
       </c>
     </row>
-    <row r="210" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A210">
         <v>211</v>
       </c>
@@ -9354,7 +9366,7 @@
         <v>![The + New node panel](figures/wf/ss_nodes_001_ann.png){#fig-B84E}</v>
       </c>
     </row>
-    <row r="211" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A211">
         <v>212</v>
       </c>
@@ -9386,7 +9398,7 @@
         <v/>
       </c>
     </row>
-    <row r="212" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A212">
         <v>213</v>
       </c>
@@ -9421,7 +9433,7 @@
         <v>![Adding an Ask a question node](figures/wf/ss_canvas_002_ann.png){#fig-2C1A}</v>
       </c>
     </row>
-    <row r="213" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A213">
         <v>214</v>
       </c>
@@ -9453,7 +9465,7 @@
         <v/>
       </c>
     </row>
-    <row r="214" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A214">
         <v>215</v>
       </c>
@@ -9488,7 +9500,7 @@
         <v>![Configuring the Ask a question node to ask for a math problem](figures/wf/ss_canvas_003_ann.png){#fig-BC17}</v>
       </c>
     </row>
-    <row r="215" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A215">
         <v>216</v>
       </c>
@@ -9520,7 +9532,7 @@
         <v/>
       </c>
     </row>
-    <row r="216" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A216">
         <v>217</v>
       </c>
@@ -9555,7 +9567,7 @@
         <v>![Configuring the Latest Message variable](figures/wf/ss_canvas_004_ann.png){#fig-8C31}</v>
       </c>
     </row>
-    <row r="217" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A217">
         <v>218</v>
       </c>
@@ -9587,7 +9599,7 @@
         <v/>
       </c>
     </row>
-    <row r="218" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A218">
         <v>219</v>
       </c>
@@ -9622,7 +9634,7 @@
         <v>![Configuring the Turn Count variable](figures/wf/ss_canvas_005_ann.png){#fig-1C3C}</v>
       </c>
     </row>
-    <row r="219" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A219">
         <v>220</v>
       </c>
@@ -9654,7 +9666,7 @@
         <v/>
       </c>
     </row>
-    <row r="220" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A220">
         <v>221</v>
       </c>
@@ -9689,7 +9701,7 @@
         <v>![Configuring the Math Evaluator Agent node](figures/wf/ss_canvas_006_ann.png){#fig-EC28}</v>
       </c>
     </row>
-    <row r="221" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A221">
         <v>222</v>
       </c>
@@ -9721,7 +9733,7 @@
         <v/>
       </c>
     </row>
-    <row r="222" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A222">
         <v>223</v>
       </c>
@@ -9756,7 +9768,7 @@
         <v>![Configuring the Math Evaluator Agent's behavior](figures/wf/ss_canvas_007_ann.png){#fig-7C25}</v>
       </c>
     </row>
-    <row r="223" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A223">
         <v>224</v>
       </c>
@@ -9788,7 +9800,7 @@
         <v/>
       </c>
     </row>
-    <row r="224" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A224">
         <v>225</v>
       </c>
@@ -9823,7 +9835,7 @@
         <v>![Configuring the If/else logic to handle evaluation failures](figures/wf/ss_canvas_008_ann.png){#fig-8C64}</v>
       </c>
     </row>
-    <row r="225" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A225">
         <v>226</v>
       </c>
@@ -9855,7 +9867,7 @@
         <v/>
       </c>
     </row>
-    <row r="226" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A226">
         <v>227</v>
       </c>
@@ -9890,7 +9902,7 @@
         <v>![Configuring the message to the user if evaluation failed](figures/wf/ss_canvas_009_ann.png){#fig-1C69}</v>
       </c>
     </row>
-    <row r="227" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A227">
         <v>228</v>
       </c>
@@ -9922,7 +9934,7 @@
         <v/>
       </c>
     </row>
-    <row r="228" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A228">
         <v>229</v>
       </c>
@@ -9957,7 +9969,7 @@
         <v>![Configuring the message to the user if evaluation succeeded](figures/wf/ss_canvas_010_ann.png){#fig-8952}</v>
       </c>
     </row>
-    <row r="229" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A229">
         <v>230</v>
       </c>
@@ -9992,7 +10004,7 @@
         <v>![The first half of the Math Coder Workflow](figures/wf/ss_canvas_011_clean.png){#fig-30B4}</v>
       </c>
     </row>
-    <row r="230" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A230">
         <v>231</v>
       </c>
@@ -10024,7 +10036,7 @@
         <v/>
       </c>
     </row>
-    <row r="231" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A231">
         <v>232</v>
       </c>
@@ -10056,7 +10068,7 @@
         <v/>
       </c>
     </row>
-    <row r="232" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A232">
         <v>233</v>
       </c>
@@ -10091,7 +10103,7 @@
         <v>![Seeing the YAML version of what you've built](figures/wf/ss_canvas_012_ann.png){#fig-E94B}</v>
       </c>
     </row>
-    <row r="233" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A233">
         <v>234</v>
       </c>
@@ -10123,7 +10135,7 @@
         <v/>
       </c>
     </row>
-    <row r="234" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A234">
         <v>235</v>
       </c>
@@ -10158,7 +10170,7 @@
         <v>![Seeing the visual version of the full YAML pipeline](figures/wf/ss_canvas_013_ann.png){#fig-7946}</v>
       </c>
     </row>
-    <row r="235" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A235">
         <v>236</v>
       </c>
@@ -10190,7 +10202,7 @@
         <v/>
       </c>
     </row>
-    <row r="236" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A236">
         <v>237</v>
       </c>
@@ -10225,7 +10237,7 @@
         <v>![Configuring the Python Coder Agent's behavior](figures/wf/ss_canvas_014_ann.png){#fig-4960}</v>
       </c>
     </row>
-    <row r="237" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A237">
         <v>238</v>
       </c>
@@ -10260,7 +10272,7 @@
         <v>![The response node contained the problem's solution](figures/wf/ss_canvas_015_clean.png){#fig-A1}</v>
       </c>
     </row>
-    <row r="238" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A238">
         <v>239</v>
       </c>
@@ -10295,7 +10307,7 @@
         <v>![An example math problem input](figures/wf/ss_mathproblem_001_clean.png){#fig-8A6D}</v>
       </c>
     </row>
-    <row r="239" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A239">
         <v>240</v>
       </c>
@@ -10330,7 +10342,7 @@
         <v>![The evaluation of the math problem](figures/wf/ss_mathproblem_002_clean.png){#fig-CE62}</v>
       </c>
     </row>
-    <row r="240" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A240">
         <v>241</v>
       </c>
@@ -10365,7 +10377,7 @@
         <v>![The results and outputs of the math workflow](figures/wf/ss_mathproblem_003_clean.png){#fig-3266}</v>
       </c>
     </row>
-    <row r="241" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A241">
         <v>242</v>
       </c>
@@ -10400,7 +10412,7 @@
         <v>![Viewing the invocation logs for your chat session](figures/wf/ss_logs_001_clean.png){#fig-BBDE}</v>
       </c>
     </row>
-    <row r="242" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A242">
         <v>243</v>
       </c>
@@ -10432,7 +10444,7 @@
         <v/>
       </c>
     </row>
-    <row r="243" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A243">
         <v>244</v>
       </c>
@@ -10467,7 +10479,7 @@
         <v>![Locating Guardrails from the Foundry UI](figures/am/ss_guardrails_001_ann.png){#fig-D83D}</v>
       </c>
     </row>
-    <row r="244" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A244">
         <v>245</v>
       </c>
@@ -10499,7 +10511,7 @@
         <v/>
       </c>
     </row>
-    <row r="245" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A245">
         <v>246</v>
       </c>
@@ -10534,7 +10546,7 @@
         <v>![Selecting Risks in a new Guardrail](figures/am/ss_guardrails_002_ann.png){#fig-2829}</v>
       </c>
     </row>
-    <row r="246" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A246">
         <v>247</v>
       </c>
@@ -10566,7 +10578,7 @@
         <v/>
       </c>
     </row>
-    <row r="247" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A247">
         <v>248</v>
       </c>
@@ -10601,7 +10613,7 @@
         <v>![Selecting the intervention points and actions for the Risk](figures/am/ss_guardrails_003_ann.png){#fig-B824}</v>
       </c>
     </row>
-    <row r="248" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A248">
         <v>249</v>
       </c>
@@ -10636,7 +10648,7 @@
         <v>![Control intervention points in an Agent response flow](figures/am/il_controls_001_clean.png){#fig-515E}</v>
       </c>
     </row>
-    <row r="249" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A249">
         <v>250</v>
       </c>
@@ -10668,7 +10680,7 @@
         <v/>
       </c>
     </row>
-    <row r="250" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A250">
         <v>251</v>
       </c>
@@ -10703,7 +10715,7 @@
         <v>![Reviewing the Controls added to the Guardrail](figures/am/ss_guardrails_004_ann.png){#fig-8802}</v>
       </c>
     </row>
-    <row r="251" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A251">
         <v>252</v>
       </c>
@@ -10735,7 +10747,7 @@
         <v/>
       </c>
     </row>
-    <row r="252" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A252">
         <v>253</v>
       </c>
@@ -10770,7 +10782,7 @@
         <v>![Applying the Guardrail to Models and Agents](figures/am/ss_guardrails_005_ann.png){#fig-180F}</v>
       </c>
     </row>
-    <row r="253" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A253">
         <v>254</v>
       </c>
@@ -10805,7 +10817,7 @@
         <v>![Reviewing the Guardrail selections before saving](figures/am/ss_guardrails_006_clean.png){#fig-B446}</v>
       </c>
     </row>
-    <row r="254" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A254">
         <v>255</v>
       </c>
@@ -10837,7 +10849,7 @@
         <v/>
       </c>
     </row>
-    <row r="255" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A255">
         <v>256</v>
       </c>
@@ -10872,7 +10884,7 @@
         <v>![Locating Blocklists from the Foundry UI](figures/am/ss_blocklists_001_ann.png){#fig-9B6C}</v>
       </c>
     </row>
-    <row r="256" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A256">
         <v>257</v>
       </c>
@@ -10904,7 +10916,7 @@
         <v/>
       </c>
     </row>
-    <row r="257" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A257">
         <v>258</v>
       </c>
@@ -10939,7 +10951,7 @@
         <v>![Making a new Blocklist of competitor AI products](figures/am/ss_blocklists_002_ann.png){#fig-6B78}</v>
       </c>
     </row>
-    <row r="258" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A258">
         <v>259</v>
       </c>
@@ -10974,7 +10986,7 @@
         <v>![Adding the Blocklist in a Guardrail](figures/am/ss_blocklists_003_clean.png){#fig-192B}</v>
       </c>
     </row>
-    <row r="259" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A259">
         <v>260</v>
       </c>
@@ -11009,7 +11021,7 @@
         <v>![Exploring the available third-party integrations](figures/am/ss_integrations_001_clean.png){#fig-8807}</v>
       </c>
     </row>
-    <row r="260" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A260">
         <v>261</v>
       </c>
@@ -11041,7 +11053,7 @@
         <v/>
       </c>
     </row>
-    <row r="261" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A261">
         <v>262</v>
       </c>
@@ -11076,7 +11088,7 @@
         <v>![The Conrol Plane's Operate page of the Foundry UI](figures/am/ss_controlplane_001_ann.png){#fig-5103}</v>
       </c>
     </row>
-    <row r="262" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A262">
         <v>263</v>
       </c>
@@ -11108,7 +11120,7 @@
         <v/>
       </c>
     </row>
-    <row r="263" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A263">
         <v>264</v>
       </c>
@@ -11143,7 +11155,7 @@
         <v>![Viewing all your assets in the Control Plane](figures/am/ss_controlplane_002_ann.png){#fig-A117}</v>
       </c>
     </row>
-    <row r="264" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A264">
         <v>265</v>
       </c>
@@ -11178,7 +11190,7 @@
         <v>![Viewing the Monitor tab of an Agent](figures/am/ss_controlplane_002_clean.png){#fig-4282}</v>
       </c>
     </row>
-    <row r="265" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A265">
         <v>266</v>
       </c>
@@ -11210,7 +11222,7 @@
         <v/>
       </c>
     </row>
-    <row r="266" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A266">
         <v>267</v>
       </c>
@@ -11245,7 +11257,7 @@
         <v>![Viewing the Quotas table in the Control Plane](figures/am/ss_quotas_001_ann.png){#fig-34A7}</v>
       </c>
     </row>
-    <row r="267" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A267">
         <v>268</v>
       </c>
@@ -11277,7 +11289,7 @@
         <v/>
       </c>
     </row>
-    <row r="268" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A268">
         <v>269</v>
       </c>
@@ -11312,7 +11324,7 @@
         <v>![Editing the quota for a model](figures/am/ss_quotas_002_ann.png){#fig-C4B3}</v>
       </c>
     </row>
-    <row r="269" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A269">
         <v>270</v>
       </c>
@@ -11344,7 +11356,7 @@
         <v/>
       </c>
     </row>
-    <row r="270" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A270">
         <v>271</v>
       </c>
@@ -11379,7 +11391,7 @@
         <v>![Enabling Microsoft Purview monitoring of your Foundry Project](figures/am/ss_compliance_001_ann.png){#fig-AB2E}</v>
       </c>
     </row>
-    <row r="271" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A271">
         <v>272</v>
       </c>
@@ -11414,7 +11426,7 @@
         <v>![The Agent ID dashboard from the Azure Portal](figures/am/ss_agentid_001_clean.png){#fig-A73E}</v>
       </c>
     </row>
-    <row r="272" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A272">
         <v>273</v>
       </c>
@@ -11446,7 +11458,7 @@
         <v/>
       </c>
     </row>
-    <row r="273" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A273">
         <v>274</v>
       </c>
@@ -11481,7 +11493,7 @@
         <v>![Publishing an Agent to retrieve its Principal ID](figures/am/ss_entra_001_ann.png){#fig-D3C6}</v>
       </c>
     </row>
-    <row r="274" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A274">
         <v>275</v>
       </c>
@@ -11516,7 +11528,7 @@
         <v>![The general Application ID for the Foundry Project in Entra ID](figures/am/ss_entra_002_clean.png){#fig-7351}</v>
       </c>
     </row>
-    <row r="275" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A275">
         <v>276</v>
       </c>
@@ -11551,7 +11563,7 @@
         <v>![Key features of Foundry Local](figures/ed/il_local_001_clean.png){#fig-8639}</v>
       </c>
     </row>
-    <row r="276" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A276">
         <v>277</v>
       </c>
@@ -11586,7 +11598,7 @@
         <v>![Architecture components of Foundry Local](figures/ed/il_local_002_clean.png){#fig-C236}</v>
       </c>
     </row>
-    <row r="277" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A277">
         <v>278</v>
       </c>
@@ -11621,7 +11633,7 @@
         <v>![The Foundry Local website homepage](figures/ed/ss_localsite_001_clean.png){#fig-6A11}</v>
       </c>
     </row>
-    <row r="278" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A278">
         <v>279</v>
       </c>
@@ -11656,7 +11668,7 @@
         <v>![Chatting with a small Qwen 2.5 model using the Foundry Local CLI](figures/ed/ss_local_001_clean.png){#fig-9AEF}</v>
       </c>
     </row>
-    <row r="279" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A279">
         <v>280</v>
       </c>
@@ -11691,7 +11703,7 @@
         <v>![Chatting with a Phi-4 model with reasoning using the Foundry Local CLI](figures/ed/ss_local_002_clean.png){#fig-DEE0}</v>
       </c>
     </row>
-    <row r="280" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A280">
         <v>281</v>
       </c>
@@ -11726,7 +11738,7 @@
         <v>![Chatting with an LLM using the Foundry Local Python SDK](figures/ed/ss_local_003_clean.png){#fig-22E4}</v>
       </c>
     </row>
-    <row r="281" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A281">
         <v>282</v>
       </c>
@@ -11761,7 +11773,7 @@
         <v>![Audio transcription with a Whisper model using the Foundry Local Javascript app](figures/ed/ss_local_004_clean.png){#fig-56FE}</v>
       </c>
     </row>
-    <row r="282" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A282">
         <v>283</v>
       </c>
@@ -11796,7 +11808,7 @@
         <v>![Quantization example walkthrough from FP32 to INT4](figures/ed/il_quant_001_clean.png){#fig-6908}</v>
       </c>
     </row>
-    <row r="283" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A283">
         <v>284</v>
       </c>
@@ -11831,7 +11843,7 @@
         <v>![Quantization of Qwen 2.5 0.5B for CPU inference using Olive](figures/ed/ss_olive_001_clean.png){#fig-C0FB}</v>
       </c>
     </row>
-    <row r="284" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A284">
         <v>285</v>
       </c>
@@ -11866,7 +11878,7 @@
         <v>![How a memory store recalls previous context](figures/co/il_memory_001_clean.png){#fig-9BA0}</v>
       </c>
     </row>
-    <row r="285" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A285">
         <v>286</v>
       </c>
@@ -11898,7 +11910,7 @@
         <v/>
       </c>
     </row>
-    <row r="286" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A286">
         <v>287</v>
       </c>
@@ -11933,7 +11945,7 @@
         <v>![Locating the memory capability on an Agent](figures/co/ss_memory_001_ann.png){#fig-D4BD}</v>
       </c>
     </row>
-    <row r="287" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A287">
         <v>288</v>
       </c>
@@ -11968,7 +11980,7 @@
         <v>![Editing the memory store](figures/co/ss_memory_002_clean.png){#fig-4132}</v>
       </c>
     </row>
-    <row r="288" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A288">
         <v>289</v>
       </c>
@@ -12000,7 +12012,7 @@
         <v/>
       </c>
     </row>
-    <row r="289" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A289">
         <v>290</v>
       </c>
@@ -12035,7 +12047,7 @@
         <v>![Locating the Evaluations screen](figures/co/ss_evaluations_001_ann.png){#fig-AB12}</v>
       </c>
     </row>
-    <row r="290" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A290">
         <v>291</v>
       </c>
@@ -12070,7 +12082,7 @@
         <v>![Configuring the evaluation process for an agent using synthetic data](figures/co/ss_evaluations_002_clean.png){#fig-510E}</v>
       </c>
     </row>
-    <row r="291" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A291">
         <v>292</v>
       </c>
@@ -12102,7 +12114,7 @@
         <v/>
       </c>
     </row>
-    <row r="292" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A292">
         <v>293</v>
       </c>
@@ -12137,7 +12149,7 @@
         <v>![The Evaluator catalog show the details of a built-in evaluator](figures/co/ss_evaluations_003_ann.png){#fig-CB0B}</v>
       </c>
     </row>
-    <row r="293" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A293">
         <v>294</v>
       </c>
@@ -12169,7 +12181,7 @@
         <v/>
       </c>
     </row>
-    <row r="294" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A294">
         <v>295</v>
       </c>
@@ -12204,7 +12216,7 @@
         <v>![Locating the Batch jobs feature under Models](figures/co/ss_batchjobs_001_ann.png){#fig-17AA}</v>
       </c>
     </row>
-    <row r="295" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A295">
         <v>296</v>
       </c>
@@ -12239,7 +12251,7 @@
         <v>![Uploading .jsonl data to create a batch job](figures/co/ss_batchjobs_002_clean.png){#fig-E07D}</v>
       </c>
     </row>
-    <row r="296" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A296">
         <v>297</v>
       </c>
@@ -12271,7 +12283,7 @@
         <v/>
       </c>
     </row>
-    <row r="297" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A297">
         <v>298</v>
       </c>
@@ -12306,7 +12318,7 @@
         <v>![Locating the AI Services options under Models](figures/co/ss_aiservices_001_ann.png){#fig-2CED}</v>
       </c>
     </row>
-    <row r="298" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A298">
         <v>299</v>
       </c>
@@ -12341,7 +12353,7 @@
         <v>![Testing out the Voice Live AI service in a Playground](figures/co/ss_aiservices_002_clean.png){#fig-C30F}</v>
       </c>
     </row>
-    <row r="299" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A299">
         <v>300</v>
       </c>
@@ -12376,7 +12388,7 @@
         <v>![How GraphRAG forms an entity knowledge graph of communities](figures/co/il_graphrag_001_clean.png){#fig-331E}</v>
       </c>
     </row>
-    <row r="300" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A300">
         <v>301</v>
       </c>
@@ -12411,7 +12423,7 @@
         <v>![Governance workflow of the Microsoft Agent Governance Toolkit](figures/co/il_govframework_001_clean.png){#fig-1FED}</v>
       </c>
     </row>
-    <row r="301" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A301">
         <v>302</v>
       </c>
@@ -12446,7 +12458,7 @@
         <v>![The 4 privilege rings of zero-trust Agent identity](figures/co/il_govframework_002_clean.png){#fig-5BE2}</v>
       </c>
     </row>
-    <row r="302" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A302">
         <v>303</v>
       </c>
@@ -12481,7 +12493,7 @@
         <v>![Role-based access controls for Foundry resources](figures/co/ss_identity_001_clean.png){#fig-285E}</v>
       </c>
     </row>
-    <row r="303" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A303">
         <v>304</v>
       </c>
@@ -12513,7 +12525,7 @@
         <v/>
       </c>
     </row>
-    <row r="304" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A304">
         <v>305</v>
       </c>
@@ -12548,7 +12560,7 @@
         <v>![Viewing the Monitor tab of an Agent](figures/co/ss_monitor_001_ann.png){#fig-30D0}</v>
       </c>
     </row>
-    <row r="305" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A305">
         <v>306</v>
       </c>
@@ -12583,7 +12595,7 @@
         <v>![Viewing the Application Insights service for the Foundry Project](figures/co/ss_monitor_002_clean.png){#fig-9A1E}</v>
       </c>
     </row>
-    <row r="306" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A306">
         <v>307</v>
       </c>
@@ -12618,7 +12630,7 @@
         <v>![Viewing the Cost Management screen for the Foundry-related resources](figures/co/ss_costs_001_clean.png){#fig-DD24}</v>
       </c>
     </row>
-    <row r="307" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A307">
         <v>308</v>
       </c>
@@ -12653,7 +12665,7 @@
         <v>![A basic, mostly serverless architecture for AI](figures/co/il_architecture_001_clean.png){#fig-F9BA}</v>
       </c>
     </row>
-    <row r="308" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A308">
         <v>309</v>
       </c>
@@ -12680,11 +12692,11 @@
         <v>BDB5</v>
       </c>
       <c r="I308" t="str">
-        <f t="shared" ref="I308" si="39">_xlfn.CONCAT("{#fig-",H308,"}")</f>
+        <f>_xlfn.CONCAT("{#fig-",H308,"}")</f>
         <v>{#fig-BDB5}</v>
       </c>
       <c r="J308" t="str">
-        <f t="shared" ref="J308" si="40">IF(E308,_xlfn.CONCAT("![",G308,"](figures/",B308,"/",F308,")",I308),"")</f>
+        <f t="shared" ref="J308" si="39">IF(E308,_xlfn.CONCAT("![",G308,"](figures/",B308,"/",F308,")",I308),"")</f>
         <v>![A more sophisticated architecture with private networking](figures/co/il_architecture_002_clean.png){#fig-BDB5}</v>
       </c>
     </row>
@@ -12700,14 +12712,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F9AFBD1-7D36-4720-9798-1D6F918A5E59}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:C10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="54.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="54.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="12" t="s">
         <v>214</v>
       </c>
@@ -12718,7 +12730,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -12729,7 +12741,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -12740,7 +12752,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -12751,7 +12763,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -12762,7 +12774,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -12773,7 +12785,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -12784,7 +12796,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -12795,7 +12807,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -12806,7 +12818,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
         <v>9</v>
       </c>

</xml_diff>

<commit_message>
Rename figures for distinct hashes
</commit_message>
<xml_diff>
--- a/figures/figure_inventory.xlsx
+++ b/figures/figure_inventory.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/colbyford/Documents/GitHub/foundry-book/figures/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Colby\Documents\GitHub\foundry-book\figures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{917815D1-3703-9D46-AA37-55F05A8E38C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A60D9B89-A6BE-45B2-861C-A1D7030C2895}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="44800" windowHeight="22520" xr2:uid="{222F1F68-60B1-49B9-BFF7-2C9CF743DB25}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{222F1F68-60B1-49B9-BFF7-2C9CF743DB25}"/>
   </bookViews>
   <sheets>
     <sheet name="Figure Inventory" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Figure Inventory'!$A$1:$J$198</definedName>
   </definedNames>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1142" uniqueCount="521">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1150" uniqueCount="533">
   <si>
     <t>Type</t>
   </si>
@@ -1625,6 +1625,42 @@
   </si>
   <si>
     <t>ss_wfportal_002_ann.png</t>
+  </si>
+  <si>
+    <t>ss_vscode_001_clean.png</t>
+  </si>
+  <si>
+    <t>ss_vscode_002_clean.png</t>
+  </si>
+  <si>
+    <t>Locating the Foundry Toolkit extension in VS Code</t>
+  </si>
+  <si>
+    <t>Exploring models and creating agents in Foundry Toolkit</t>
+  </si>
+  <si>
+    <t>ss_kbagent_001_clean.png</t>
+  </si>
+  <si>
+    <t>ss_kbagent_001_ann.png</t>
+  </si>
+  <si>
+    <t>ss_kbagent_002_clean.png</t>
+  </si>
+  <si>
+    <t>ss_kbagent_003_clean.png</t>
+  </si>
+  <si>
+    <t>ss_kbagent_004_clean.png</t>
+  </si>
+  <si>
+    <t>ss_controlplane_003_clean.png</t>
+  </si>
+  <si>
+    <t>ss_earnings_001_clean.png</t>
+  </si>
+  <si>
+    <t>ss_storage_001_ann.png</t>
   </si>
 </sst>
 </file>
@@ -2259,22 +2295,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B464DFF5-94DA-41E0-B03E-143380050964}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:J308"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:J310"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="34.5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="73.83203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.1640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="34.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="73.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="118" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>29</v>
       </c>
@@ -2306,7 +2342,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2341,9 +2377,9 @@
         <v>![Parts of the Microsoft Foundry platform](figures/in/il_foundryplatform_001.png){#fig-4C72}</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>91</v>
@@ -2376,9 +2412,9 @@
         <v>![Foundry Resource and Project Organization](figures/in/il_portal_001.png){#fig-3498}</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>91</v>
@@ -2411,9 +2447,9 @@
         <v>![Azure Portal - Search Box](figures/in/ss_portal_001_ann.png){#fig-693E}</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>91</v>
@@ -2443,9 +2479,9 @@
         <v/>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>91</v>
@@ -2478,9 +2514,9 @@
         <v>![Azure Portal - Searching for "Microsoft Foundry"](figures/in/ss_portal_002_ann.png){#fig-992A}</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>91</v>
@@ -2510,9 +2546,9 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>91</v>
@@ -2545,9 +2581,9 @@
         <v>![Azure Portal - Creating a Foundry Resource](figures/in/ss_portal_003_ann.png){#fig-927}</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>91</v>
@@ -2577,9 +2613,9 @@
         <v/>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>91</v>
@@ -2612,9 +2648,9 @@
         <v>![Create a Foundry Resource - Basics tab](figures/in/ss_portal_004_ann.png){#fig-3901}</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>91</v>
@@ -2644,9 +2680,9 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>91</v>
@@ -2679,9 +2715,9 @@
         <v>![Create a Foundry Resource - Storage tab](figures/in/ss_portal_005_ann.png){#fig-A90C}</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>91</v>
@@ -2711,9 +2747,9 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>91</v>
@@ -2746,9 +2782,9 @@
         <v>![Create a Foundry Resource - Review + Create tab](figures/in/ss_portal_006_ann.png){#fig-5918}</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>91</v>
@@ -2778,9 +2814,9 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>91</v>
@@ -2813,9 +2849,9 @@
         <v>![Azure Portal - Deployment Overview](figures/in/ss_portal_007_clean.png){#fig-CC82}</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>91</v>
@@ -2848,9 +2884,9 @@
         <v>![Azure Portal - Resource Group of Foundry-related Resources](figures/in/ss_portal_008_ann.png){#fig-3954}</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>91</v>
@@ -2880,9 +2916,9 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>91</v>
@@ -2915,9 +2951,9 @@
         <v>![Azure Portal - Foundry Resource](figures/in/ss_portal_009_ann.png){#fig-A959}</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>91</v>
@@ -2947,9 +2983,9 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>91</v>
@@ -2982,9 +3018,9 @@
         <v>![Microsoft Foundry Project Homepage](figures/in/ss_portal_010_clean.png){#fig-7B65}</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>91</v>
@@ -3017,9 +3053,9 @@
         <v>![Example Azure CLI Login Subscription Selection](figures/in/cd_cli_001.png){#fig-360B}</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>91</v>
@@ -3052,9 +3088,9 @@
         <v>![Foundry Portal Header](figures/in/ss_portalheader_011_clean.png){#fig-B78E}</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>91</v>
@@ -3084,9 +3120,9 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>91</v>
@@ -3119,9 +3155,9 @@
         <v>![Copying the Project Endpoint URL](figures/in/ss_portal_012_ann.png){#fig-5C7B}</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B26" s="4" t="s">
         <v>93</v>
@@ -3151,9 +3187,9 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B27" s="4" t="s">
         <v>93</v>
@@ -3186,9 +3222,9 @@
         <v>![Locating the Discover tab](figures/md/ss_portal_013_ann.png){#fig-CC76}</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B28" s="4" t="s">
         <v>93</v>
@@ -3218,9 +3254,9 @@
         <v/>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B29" s="4" t="s">
         <v>93</v>
@@ -3253,9 +3289,9 @@
         <v>![Exploring featured models on the Discover page](figures/md/ss_discover_001_ann.png){#fig-BF54}</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B30" s="4" t="s">
         <v>93</v>
@@ -3288,9 +3324,9 @@
         <v>![Listing all available models in Foundry](figures/md/ss_discover_002_clean.png){#fig-3E3C}</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B31" s="4" t="s">
         <v>93</v>
@@ -3323,9 +3359,9 @@
         <v>![Locating the Compare models button](figures/md/ss_compare_001_ann.png){#fig-767C}</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B32" s="4" t="s">
         <v>93</v>
@@ -3358,9 +3394,9 @@
         <v>![Comparing models across benchmarks and capabilities](figures/md/ss_compare_002_clean.png){#fig-68E2}</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B33" s="4" t="s">
         <v>93</v>
@@ -3393,9 +3429,9 @@
         <v>![Locating the View leaderboard button](figures/md/ss_leaderboard_001_ann.png){#fig-4BC0}</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B34" s="4" t="s">
         <v>93</v>
@@ -3428,9 +3464,9 @@
         <v>![Exploring the model leaderboard](figures/md/ss_leaderboard_002_clean.png){#fig-7953}</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B35" s="4" t="s">
         <v>93</v>
@@ -3463,9 +3499,9 @@
         <v>![More details about a model's benchmark performance](figures/md/ss_leaderboard_003_ann.png){#fig-2BD9}</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B36" s="4" t="s">
         <v>93</v>
@@ -3498,9 +3534,9 @@
         <v>![Metric details across various model benchmarks](figures/md/ss_leaderboard_004_clean.png){#fig-F14D}</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B37" s="4" t="s">
         <v>93</v>
@@ -3530,9 +3566,9 @@
         <v/>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B38" s="4" t="s">
         <v>93</v>
@@ -3565,9 +3601,9 @@
         <v>![Searching for the Phi-4 model](figures/md/ss_deploy_001_ann.png){#fig-FF9}</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B39" s="4" t="s">
         <v>93</v>
@@ -3597,9 +3633,9 @@
         <v/>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B40" s="4" t="s">
         <v>93</v>
@@ -3632,9 +3668,9 @@
         <v>![Deploying Phi-4 with Default settings](figures/md/ss_deploy_002_ann.png){#fig-FFED}</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B41" s="4" t="s">
         <v>93</v>
@@ -3664,9 +3700,9 @@
         <v/>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B42" s="4" t="s">
         <v>93</v>
@@ -3699,9 +3735,9 @@
         <v>![Agreeing to the terms for deploying Phi-4](figures/md/ss_deploy_003_ann.png){#fig-6FE0}</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B43" s="4" t="s">
         <v>93</v>
@@ -3734,9 +3770,9 @@
         <v>![Playground UI for experimenting with a Phi-4 deployment](figures/md/ss_deploy_004_clean.png){#fig-925F}</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B44" s="4" t="s">
         <v>93</v>
@@ -3769,9 +3805,9 @@
         <v>![Learning to make intergalactic pizza](figures/md/ss_deploy_005_clean.png){#fig-6E5B}</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B45" s="4" t="s">
         <v>93</v>
@@ -3801,9 +3837,9 @@
         <v/>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B46" s="4" t="s">
         <v>93</v>
@@ -3836,9 +3872,9 @@
         <v>![Modifying model parameters](figures/md/ss_deploy_006_ann.png){#fig-3FDF}</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B47" s="4" t="s">
         <v>93</v>
@@ -3868,9 +3904,9 @@
         <v/>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B48" s="4" t="s">
         <v>93</v>
@@ -3903,9 +3939,9 @@
         <v>![A slightly more martian pizza recipe](figures/md/ss_deploy_008_clean.png){#fig-C260}</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B49" s="4" t="s">
         <v>93</v>
@@ -3938,9 +3974,9 @@
         <v>![Deployment endpoint and key on the Details tab](figures/md/ss_deploy_007_ann.png){#fig-AFD2}</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B50" s="5" t="s">
         <v>94</v>
@@ -3973,9 +4009,9 @@
         <v>![The agentic flow between inputs, the model, tools, and outputs](figures/ad/il_agent_001.png){#fig-2027}</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B51" s="5" t="s">
         <v>94</v>
@@ -4005,9 +4041,9 @@
         <v/>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B52" s="5" t="s">
         <v>94</v>
@@ -4040,9 +4076,9 @@
         <v>![Creating an agent from the Agents tab](figures/ad/ss_agent_001_ann.png){#fig-1BC}</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B53" s="5" t="s">
         <v>94</v>
@@ -4072,9 +4108,9 @@
         <v/>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B54" s="5" t="s">
         <v>94</v>
@@ -4107,9 +4143,9 @@
         <v>![Giving your new agent a name](figures/ad/ss_agent_002_ann.png){#fig-F1A8}</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B55" s="5" t="s">
         <v>94</v>
@@ -4139,9 +4175,9 @@
         <v/>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B56" s="5" t="s">
         <v>94</v>
@@ -4174,9 +4210,9 @@
         <v>![Listing all Agents in your Project](figures/ad/ss_agent_003_ann.png){#fig-61A5}</v>
       </c>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B57" s="5" t="s">
         <v>94</v>
@@ -4209,9 +4245,9 @@
         <v>![Your real estate Agent's Playground](figures/ad/ss_agent_004_clean.png){#fig-C6EC}</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B58" s="5" t="s">
         <v>94</v>
@@ -4241,9 +4277,9 @@
         <v/>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B59" s="5" t="s">
         <v>94</v>
@@ -4276,9 +4312,9 @@
         <v>![Giving the real estate Agent instructions](figures/ad/ss_agent_005_ann.png){#fig-C18E}</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B60" s="5" t="s">
         <v>94</v>
@@ -4308,9 +4344,9 @@
         <v/>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B61" s="5" t="s">
         <v>94</v>
@@ -4343,9 +4379,9 @@
         <v>![Previewing an Agent app](figures/ad/ss_agent_006_ann.png){#fig-319A}</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B62" s="5" t="s">
         <v>94</v>
@@ -4378,9 +4414,9 @@
         <v>![Your demo Agent app](figures/ad/ss_agent_007_clean.png){#fig-82E3}</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B63" s="5" t="s">
         <v>94</v>
@@ -4410,9 +4446,9 @@
         <v/>
       </c>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A64">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B64" s="5" t="s">
         <v>94</v>
@@ -4445,9 +4481,9 @@
         <v>![An example, yet beautiful home on Zillow](figures/ad/ss_agent_007b_cens_clean.png){#fig-AC5A}</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B65" s="5" t="s">
         <v>94</v>
@@ -4477,9 +4513,9 @@
         <v/>
       </c>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A66">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B66" s="5" t="s">
         <v>94</v>
@@ -4512,9 +4548,9 @@
         <v>![The Agent's Instagram post](figures/ad/ss_agent_008_cens_clean.png){#fig-1600}</v>
       </c>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A67">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B67" s="5" t="s">
         <v>94</v>
@@ -4544,9 +4580,9 @@
         <v/>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A68">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B68" s="5" t="s">
         <v>94</v>
@@ -4579,9 +4615,9 @@
         <v>![The Agent failing to read from the web](figures/ad/ss_agent_008b_cens_clean.png){#fig-5F6F}</v>
       </c>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A69">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B69" s="5" t="s">
         <v>94</v>
@@ -4611,9 +4647,9 @@
         <v/>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A70">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B70" s="5" t="s">
         <v>94</v>
@@ -4646,9 +4682,9 @@
         <v>![Publishing your Agent](figures/ad/ss_agent_009_ann.png){#fig-C1DB}</v>
       </c>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B71" s="5" t="s">
         <v>94</v>
@@ -4678,9 +4714,9 @@
         <v/>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A72">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B72" s="5" t="s">
         <v>94</v>
@@ -4713,9 +4749,9 @@
         <v>![Making your Agent production-ready](figures/ad/ss_agent_010_ann.png){#fig-54E0}</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A73">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B73" s="5" t="s">
         <v>94</v>
@@ -4748,9 +4784,9 @@
         <v>![Your Agent was published successfully](figures/ad/ss_agent_011_clean.png){#fig-C900}</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A74">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B74" s="5" t="s">
         <v>94</v>
@@ -4780,9 +4816,9 @@
         <v/>
       </c>
     </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A75">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B75" s="5" t="s">
         <v>94</v>
@@ -4815,9 +4851,9 @@
         <v>![Exploring Tools on the Discover page](figures/ad/ss_tools_001_ann.png){#fig-D127}</v>
       </c>
     </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A76">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B76" s="5" t="s">
         <v>94</v>
@@ -4847,9 +4883,9 @@
         <v/>
       </c>
     </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A77">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B77" s="5" t="s">
         <v>94</v>
@@ -4882,9 +4918,9 @@
         <v>![Locating your real estate Agent](figures/ad/ss_tools_002_ann.png){#fig-2133}</v>
       </c>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A78">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B78" s="5" t="s">
         <v>94</v>
@@ -4914,9 +4950,9 @@
         <v/>
       </c>
     </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A79">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B79" s="5" t="s">
         <v>94</v>
@@ -4949,9 +4985,9 @@
         <v>![Adding a Tool to your Agent](figures/ad/ss_tools_003_ann.png){#fig-B13E}</v>
       </c>
     </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A80">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B80" s="5" t="s">
         <v>94</v>
@@ -4981,9 +5017,9 @@
         <v/>
       </c>
     </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A81">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B81" s="5" t="s">
         <v>94</v>
@@ -5016,9 +5052,9 @@
         <v>![Selecting the Web search Tool](figures/ad/ss_tools_004_ann.png){#fig-8118}</v>
       </c>
     </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A82">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B82" s="5" t="s">
         <v>94</v>
@@ -5048,9 +5084,9 @@
         <v/>
       </c>
     </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A83">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B83" s="5" t="s">
         <v>94</v>
@@ -5083,9 +5119,9 @@
         <v>![Accepting the terms for Web Search](figures/ad/ss_tools_005_ann.png){#fig-1115}</v>
       </c>
     </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A84">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B84" s="5" t="s">
         <v>94</v>
@@ -5115,9 +5151,9 @@
         <v/>
       </c>
     </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A85">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B85" s="5" t="s">
         <v>94</v>
@@ -5150,9 +5186,9 @@
         <v>![Saving and previewing the Agent with Web Search connected](figures/ad/ss_tools_006_ann.png){#fig-E101}</v>
       </c>
     </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A86">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B86" s="5" t="s">
         <v>94</v>
@@ -5182,9 +5218,9 @@
         <v/>
       </c>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A87">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B87" s="5" t="s">
         <v>94</v>
@@ -5217,9 +5253,9 @@
         <v>![A much more functional real estate Agent](figures/ad/ss_tools_007_cens_clean.png){#fig-BB7C}</v>
       </c>
     </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A88">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B88" s="5" t="s">
         <v>94</v>
@@ -5252,9 +5288,9 @@
         <v>![Example MCP-based architecture](figures/ad/il_tools_001.png){#fig-4852}</v>
       </c>
     </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A89">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B89" s="5" t="s">
         <v>94</v>
@@ -5287,9 +5323,9 @@
         <v>![Foundry MCP client-server flow](figures/ad/il_mcp_001.png){#fig-3CBD}</v>
       </c>
     </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A90">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B90" s="5" t="s">
         <v>94</v>
@@ -5322,9 +5358,9 @@
         <v>![Configuring a general MCP tool](figures/ad/ss_tools_008_clean.png){#fig-3AB9}</v>
       </c>
     </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A91">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B91" s="5" t="s">
         <v>94</v>
@@ -5357,9 +5393,9 @@
         <v>![Selecting your Subscription and Resource Group in the azd prompt](figures/ad/ss_mcp_001_clean.png){#fig-C02E}</v>
       </c>
     </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A92">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B92" s="5" t="s">
         <v>94</v>
@@ -5392,9 +5428,9 @@
         <v>![azd has successfully deployed the resources](figures/ad/ss_mcp_002_clean.png){#fig-8421}</v>
       </c>
     </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A93">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B93" s="5" t="s">
         <v>94</v>
@@ -5424,9 +5460,9 @@
         <v/>
       </c>
     </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A94">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B94" s="5" t="s">
         <v>94</v>
@@ -5459,9 +5495,9 @@
         <v>![Successful deployment of the MCP Toolkit](figures/ad/ss_mcp_003_ann.png){#fig-B89C}</v>
       </c>
     </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A95">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B95" s="5" t="s">
         <v>94</v>
@@ -5491,9 +5527,9 @@
         <v/>
       </c>
     </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A96">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B96" s="5" t="s">
         <v>94</v>
@@ -5526,9 +5562,9 @@
         <v>![Authenticating the MCP Toolkit with your Tenant and Entra App IDs](figures/ad/ss_mcp_004_ann.png){#fig-88BA}</v>
       </c>
     </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A97">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B97" s="5" t="s">
         <v>94</v>
@@ -5558,9 +5594,9 @@
         <v/>
       </c>
     </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A98">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B98" s="5" t="s">
         <v>94</v>
@@ -5593,9 +5629,9 @@
         <v>![Granting permissions to the MCP Toolkit app](figures/ad/ss_mcp_005_ann.png){#fig-18B7}</v>
       </c>
     </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A99">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B99" s="5" t="s">
         <v>94</v>
@@ -5625,9 +5661,9 @@
         <v/>
       </c>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A100">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B100" s="5" t="s">
         <v>94</v>
@@ -5660,9 +5696,9 @@
         <v>![Successful authentication to the MCP Toolkit app](figures/ad/ss_mcp_006_ann.png){#fig-E8A3}</v>
       </c>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A101">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B101" s="5" t="s">
         <v>94</v>
@@ -5692,9 +5728,9 @@
         <v/>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A102">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B102" s="5" t="s">
         <v>94</v>
@@ -5727,9 +5763,9 @@
         <v>![The Cosmos DB screen in the Azure Portal](figures/ad/ss_cosmos_001_ann.png){#fig-23F7}</v>
       </c>
     </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A103">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B103" s="5" t="s">
         <v>94</v>
@@ -5759,9 +5795,9 @@
         <v/>
       </c>
     </row>
-    <row r="104" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A104">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B104" s="5" t="s">
         <v>94</v>
@@ -5794,9 +5830,9 @@
         <v>![Locating your Cosmos DB URI and Key](figures/ad/ss_cosmos_002_ann.png){#fig-D3E3}</v>
       </c>
     </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A105">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B105" s="5" t="s">
         <v>94</v>
@@ -5826,9 +5862,9 @@
         <v/>
       </c>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A106">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B106" s="5" t="s">
         <v>94</v>
@@ -5861,9 +5897,9 @@
         <v>![Adding another Tool to your Agent](figures/ad/ss_cosmos_003_ann.png){#fig-43EE}</v>
       </c>
     </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A107">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B107" s="5" t="s">
         <v>94</v>
@@ -5893,9 +5929,9 @@
         <v/>
       </c>
     </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A108">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B108" s="5" t="s">
         <v>94</v>
@@ -5928,9 +5964,9 @@
         <v>![Locating the Cosmos DB Tool in the Catalog](figures/ad/ss_cosmos_004_ann.png){#fig-73C8}</v>
       </c>
     </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A109">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B109" s="5" t="s">
         <v>94</v>
@@ -5960,9 +5996,9 @@
         <v/>
       </c>
     </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A110">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B110" s="5" t="s">
         <v>94</v>
@@ -5995,9 +6031,9 @@
         <v>![Information about hosting MCP servers](figures/ad/ss_cosmos_005_ann.png){#fig-E3C5}</v>
       </c>
     </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A111">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B111" s="5" t="s">
         <v>94</v>
@@ -6027,9 +6063,9 @@
         <v/>
       </c>
     </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A112">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B112" s="5" t="s">
         <v>94</v>
@@ -6062,9 +6098,9 @@
         <v>![Filling in the URI and authentication for the Cosmos DB Tool connection](figures/ad/ss_cosmos_006_ann.png){#fig-13D1}</v>
       </c>
     </row>
-    <row r="113" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A113">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B113" s="5" t="s">
         <v>94</v>
@@ -6094,9 +6130,9 @@
         <v/>
       </c>
     </row>
-    <row r="114" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A114">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B114" s="5" t="s">
         <v>94</v>
@@ -6129,9 +6165,9 @@
         <v>![Checking that your Cosmos DB Tool is connected](figures/ad/ss_cosmos_007_ann.png){#fig-83DC}</v>
       </c>
     </row>
-    <row r="115" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A115">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B115" s="5" t="s">
         <v>94</v>
@@ -6161,9 +6197,9 @@
         <v/>
       </c>
     </row>
-    <row r="116" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A116">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B116" s="5" t="s">
         <v>94</v>
@@ -6196,9 +6232,9 @@
         <v>![Checking the Cosmos DB Tool usage in the Agent response](figures/ad/ss_cosmos_008_ann.png){#fig-739D}</v>
       </c>
     </row>
-    <row r="117" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A117">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B117" s="5" t="s">
         <v>94</v>
@@ -6231,9 +6267,9 @@
         <v>![A successful Cosmos DB Tool call and augmented Agent response](figures/ad/ss_cosmos_009_clean.png){#fig-8361}</v>
       </c>
     </row>
-    <row r="118" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A118">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B118" s="5" t="s">
         <v>94</v>
@@ -6263,9 +6299,9 @@
         <v/>
       </c>
     </row>
-    <row r="119" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A119">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B119" s="5" t="s">
         <v>94</v>
@@ -6298,9 +6334,9 @@
         <v>![Creating a new Cosmos DB container](figures/ad/ss_database_001_ann.png){#fig-5117}</v>
       </c>
     </row>
-    <row r="120" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A120">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B120" s="5" t="s">
         <v>94</v>
@@ -6330,9 +6366,9 @@
         <v/>
       </c>
     </row>
-    <row r="121" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A121">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B121" s="5" t="s">
         <v>94</v>
@@ -6365,9 +6401,9 @@
         <v>![Creating a new Cosmos DB database](figures/ad/ss_database_002_ann.png){#fig-A103}</v>
       </c>
     </row>
-    <row r="122" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A122">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B122" s="5" t="s">
         <v>94</v>
@@ -6397,9 +6433,9 @@
         <v/>
       </c>
     </row>
-    <row r="123" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A123">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B123" s="5" t="s">
         <v>94</v>
@@ -6432,9 +6468,9 @@
         <v>![Uploading property records to your database](figures/ad/ss_database_003_ann.png){#fig-310E}</v>
       </c>
     </row>
-    <row r="124" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A124">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B124" s="5" t="s">
         <v>94</v>
@@ -6467,9 +6503,9 @@
         <v>![Listing your property records](figures/ad/ss_database_004_clean.png){#fig-CA93}</v>
       </c>
     </row>
-    <row r="125" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A125">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B125" s="6" t="s">
         <v>95</v>
@@ -6502,9 +6538,9 @@
         <v>![Orchestrating multi-source, complex RAG pipelines](figures/kb/il_layers_001.png){#fig-2B5B}</v>
       </c>
     </row>
-    <row r="126" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A126">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B126" s="6" t="s">
         <v>95</v>
@@ -6537,9 +6573,9 @@
         <v>![Building a multi-source Agent for financial insights](figures/kb/il_multisource_001.png){#fig-E787}</v>
       </c>
     </row>
-    <row r="127" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A127">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B127" s="6" t="s">
         <v>95</v>
@@ -6572,9 +6608,9 @@
         <v>![The basic RAG pattern](figures/kb/il_rag_001.png){#fig-D293}</v>
       </c>
     </row>
-    <row r="128" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A128">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B128" s="6" t="s">
         <v>95</v>
@@ -6607,9 +6643,9 @@
         <v>![Knowledge sources as part of the AI Search data retreival](figures/kb/il_knowledgesources_001.png){#fig-E63}</v>
       </c>
     </row>
-    <row r="129" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A129">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B129" s="6" t="s">
         <v>95</v>
@@ -6642,9 +6678,9 @@
         <v>![Enrichment tasks for documents](figures/kb/il_enrichment_001.png){#fig-3399}</v>
       </c>
     </row>
-    <row r="130" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A130">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B130" s="6" t="s">
         <v>95</v>
@@ -6656,30 +6692,30 @@
         <v>0</v>
       </c>
       <c r="E130" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F130" t="s">
-        <v>286</v>
+        <v>531</v>
       </c>
       <c r="G130" t="s">
         <v>290</v>
       </c>
       <c r="H130" s="1" t="str" cm="1">
         <f t="array" ref="H130">CRC16HASH(F130)</f>
-        <v>CB8E</v>
+        <v>6D53</v>
       </c>
       <c r="I130" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-CB8E}</v>
+        <v>{#fig-6D53}</v>
       </c>
       <c r="J130" t="str">
         <f t="shared" si="5"/>
-        <v>![Microsoft's public earnings release page](figures/kb/ss_storage_001_clean.png){#fig-CB8E}</v>
-      </c>
-    </row>
-    <row r="131" spans="1:10" x14ac:dyDescent="0.2">
+        <v/>
+      </c>
+    </row>
+    <row r="131" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A131">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B131" s="6" t="s">
         <v>95</v>
@@ -6694,24 +6730,24 @@
         <v>0</v>
       </c>
       <c r="F131" t="s">
-        <v>100</v>
+        <v>286</v>
       </c>
       <c r="H131" s="1" t="str" cm="1">
         <f t="array" ref="H131">CRC16HASH(F131)</f>
-        <v>449C</v>
+        <v>CB8E</v>
       </c>
       <c r="I131" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-449C}</v>
+        <v>{#fig-CB8E}</v>
       </c>
       <c r="J131" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
-    <row r="132" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A132">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B132" s="6" t="s">
         <v>95</v>
@@ -6726,27 +6762,27 @@
         <v>1</v>
       </c>
       <c r="F132" t="s">
-        <v>99</v>
+        <v>532</v>
       </c>
       <c r="G132" t="s">
         <v>291</v>
       </c>
       <c r="H132" s="1" t="str" cm="1">
         <f t="array" ref="H132">CRC16HASH(F132)</f>
-        <v>693E</v>
+        <v>82FA</v>
       </c>
       <c r="I132" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-693E}</v>
+        <v>{#fig-82FA}</v>
       </c>
       <c r="J132" t="str">
         <f t="shared" si="5"/>
-        <v>![Creating a new Container in Azure Storage](figures/kb/ss_portal_001_ann.png){#fig-693E}</v>
-      </c>
-    </row>
-    <row r="133" spans="1:10" x14ac:dyDescent="0.2">
+        <v>![Creating a new Container in Azure Storage](figures/kb/ss_storage_001_ann.png){#fig-82FA}</v>
+      </c>
+    </row>
+    <row r="133" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A133">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B133" s="6" t="s">
         <v>95</v>
@@ -6776,9 +6812,9 @@
         <v/>
       </c>
     </row>
-    <row r="134" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A134">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B134" s="6" t="s">
         <v>95</v>
@@ -6811,9 +6847,9 @@
         <v>![Uploading the financial reports to Azure Storage](figures/kb/ss_storage_002_ann.png){#fig-72EE}</v>
       </c>
     </row>
-    <row r="135" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A135">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B135" s="6" t="s">
         <v>95</v>
@@ -6843,9 +6879,9 @@
         <v/>
       </c>
     </row>
-    <row r="136" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A136">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B136" s="6" t="s">
         <v>95</v>
@@ -6878,9 +6914,9 @@
         <v>![Importing data into Azure AI Search](figures/kb/ss_search_001_ann.png){#fig-F62E}</v>
       </c>
     </row>
-    <row r="137" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A137">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B137" s="6" t="s">
         <v>95</v>
@@ -6910,9 +6946,9 @@
         <v/>
       </c>
     </row>
-    <row r="138" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A138">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B138" s="6" t="s">
         <v>95</v>
@@ -6945,9 +6981,9 @@
         <v>![Selecting the Azure Blob Storage built-in indexer](figures/kb/ss_search_002_ann.png){#fig-63A}</v>
       </c>
     </row>
-    <row r="139" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A139">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B139" s="6" t="s">
         <v>95</v>
@@ -6977,9 +7013,9 @@
         <v/>
       </c>
     </row>
-    <row r="140" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A140">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B140" s="6" t="s">
         <v>95</v>
@@ -7012,9 +7048,9 @@
         <v>![Selecting the Keyword search scenario](figures/kb/ss_search_003_ann.png){#fig-9637}</v>
       </c>
     </row>
-    <row r="141" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A141">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B141" s="6" t="s">
         <v>95</v>
@@ -7047,9 +7083,9 @@
         <v>![Connecting to data for the Keyword search](figures/kb/ss_search_004_clean.png){#fig-20C0}</v>
       </c>
     </row>
-    <row r="142" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A142">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B142" s="6" t="s">
         <v>95</v>
@@ -7079,9 +7115,9 @@
         <v/>
       </c>
     </row>
-    <row r="143" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A143">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B143" s="6" t="s">
         <v>95</v>
@@ -7114,9 +7150,9 @@
         <v>![Enrichments options for Keyword search](figures/kb/ss_enrichments_001_ann.png){#fig-6AFC}</v>
       </c>
     </row>
-    <row r="144" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A144">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B144" s="6" t="s">
         <v>95</v>
@@ -7146,9 +7182,9 @@
         <v/>
       </c>
     </row>
-    <row r="145" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A145">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B145" s="6" t="s">
         <v>95</v>
@@ -7181,9 +7217,9 @@
         <v>![Extract entities selection](figures/kb/ss_enrichments_002_ann.png){#fig-9AE8}</v>
       </c>
     </row>
-    <row r="146" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A146">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B146" s="6" t="s">
         <v>95</v>
@@ -7213,9 +7249,9 @@
         <v/>
       </c>
     </row>
-    <row r="147" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A147">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B147" s="6" t="s">
         <v>95</v>
@@ -7248,9 +7284,9 @@
         <v>![Extract text from images selection](figures/kb/ss_enrichments_003_ann.png){#fig-AE5}</v>
       </c>
     </row>
-    <row r="148" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A148">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B148" s="6" t="s">
         <v>95</v>
@@ -7283,9 +7319,9 @@
         <v>![Previewing the field mappings](figures/kb/ss_enrichments_004_clean.png){#fig-E99C}</v>
       </c>
     </row>
-    <row r="149" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A149">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B149" s="6" t="s">
         <v>95</v>
@@ -7315,9 +7351,9 @@
         <v/>
       </c>
     </row>
-    <row r="150" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A150">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B150" s="6" t="s">
         <v>95</v>
@@ -7350,9 +7386,9 @@
         <v>![Advanced settings for semantic search and re-indexing on a schedule](figures/kb/ss_enrichments_005_ann.png){#fig-AACE}</v>
       </c>
     </row>
-    <row r="151" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A151">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B151" s="6" t="s">
         <v>95</v>
@@ -7382,9 +7418,9 @@
         <v/>
       </c>
     </row>
-    <row r="152" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A152">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B152" s="6" t="s">
         <v>95</v>
@@ -7417,9 +7453,9 @@
         <v>![Reviewing the selections for Keyword search](figures/kb/ss_enrichments_006_ann.png){#fig-5ADA}</v>
       </c>
     </row>
-    <row r="153" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A153">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B153" s="6" t="s">
         <v>95</v>
@@ -7449,9 +7485,9 @@
         <v/>
       </c>
     </row>
-    <row r="154" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A154">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B154" s="6" t="s">
         <v>95</v>
@@ -7484,9 +7520,9 @@
         <v>![A successful indexing of the Microsoft financial documents from Azure Storage](figures/kb/ss_search_005_ann.png){#fig-361C}</v>
       </c>
     </row>
-    <row r="155" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A155">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B155" s="6" t="s">
         <v>95</v>
@@ -7516,9 +7552,9 @@
         <v/>
       </c>
     </row>
-    <row r="156" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A156">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B156" s="6" t="s">
         <v>95</v>
@@ -7551,9 +7587,9 @@
         <v>![Connecting to an Azure AI Search resource](figures/kb/ss_knowledge_001_ann.png){#fig-33E}</v>
       </c>
     </row>
-    <row r="157" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A157">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B157" s="6" t="s">
         <v>95</v>
@@ -7583,9 +7619,9 @@
         <v/>
       </c>
     </row>
-    <row r="158" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A158">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B158" s="6" t="s">
         <v>95</v>
@@ -7618,9 +7654,9 @@
         <v>![Creating a new Knowledge Base](figures/kb/ss_knowledge_002_ann.png){#fig-F32A}</v>
       </c>
     </row>
-    <row r="159" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A159">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B159" s="6" t="s">
         <v>95</v>
@@ -7650,9 +7686,9 @@
         <v/>
       </c>
     </row>
-    <row r="160" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A160">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B160" s="6" t="s">
         <v>95</v>
@@ -7685,9 +7721,9 @@
         <v>![Selecting a Knowledge Base type](figures/kb/ss_knowledge_003_ann.png){#fig-6327}</v>
       </c>
     </row>
-    <row r="161" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A161">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B161" s="6" t="s">
         <v>95</v>
@@ -7717,9 +7753,9 @@
         <v/>
       </c>
     </row>
-    <row r="162" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A162">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B162" s="6" t="s">
         <v>95</v>
@@ -7752,9 +7788,9 @@
         <v>![Connecting to the Search Index](figures/kb/ss_knowledge_004_ann.png){#fig-5301}</v>
       </c>
     </row>
-    <row r="163" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A163">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B163" s="6" t="s">
         <v>95</v>
@@ -7784,9 +7820,9 @@
         <v/>
       </c>
     </row>
-    <row r="164" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A164">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B164" s="6" t="s">
         <v>95</v>
@@ -7819,9 +7855,9 @@
         <v>![Final steps in creating the knowledge base](figures/kb/ss_knowledge_005_ann.png){#fig-C30C}</v>
       </c>
     </row>
-    <row r="165" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A165">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B165" s="6" t="s">
         <v>95</v>
@@ -7836,24 +7872,24 @@
         <v>0</v>
       </c>
       <c r="F165" t="s">
-        <v>145</v>
+        <v>525</v>
       </c>
       <c r="H165" s="1" t="str" cm="1">
         <f t="array" ref="H165">CRC16HASH(F165)</f>
-        <v>AFD</v>
+        <v>9D74</v>
       </c>
       <c r="I165" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-AFD}</v>
+        <v>{#fig-9D74}</v>
       </c>
       <c r="J165" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
-    <row r="166" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A166">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B166" s="6" t="s">
         <v>95</v>
@@ -7868,27 +7904,27 @@
         <v>1</v>
       </c>
       <c r="F166" t="s">
-        <v>146</v>
+        <v>526</v>
       </c>
       <c r="G166" t="s">
         <v>322</v>
       </c>
       <c r="H166" s="1" t="str" cm="1">
         <f t="array" ref="H166">CRC16HASH(F166)</f>
-        <v>1BC</v>
+        <v>8BA3</v>
       </c>
       <c r="I166" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-1BC}</v>
+        <v>{#fig-8BA3}</v>
       </c>
       <c r="J166" t="str">
         <f t="shared" si="5"/>
-        <v>![Connecting the Agent to the knowledge base](figures/kb/ss_agent_001_ann.png){#fig-1BC}</v>
-      </c>
-    </row>
-    <row r="167" spans="1:10" x14ac:dyDescent="0.2">
+        <v>![Connecting the Agent to the knowledge base](figures/kb/ss_kbagent_001_ann.png){#fig-8BA3}</v>
+      </c>
+    </row>
+    <row r="167" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A167">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B167" s="6" t="s">
         <v>95</v>
@@ -7903,27 +7939,27 @@
         <v>1</v>
       </c>
       <c r="F167" t="s">
-        <v>147</v>
+        <v>527</v>
       </c>
       <c r="G167" t="s">
         <v>321</v>
       </c>
       <c r="H167" s="1" t="str" cm="1">
         <f t="array" ref="H167">CRC16HASH(F167)</f>
-        <v>4EF2</v>
+        <v>D97B</v>
       </c>
       <c r="I167" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-4EF2}</v>
+        <v>{#fig-D97B}</v>
       </c>
       <c r="J167" t="str">
         <f t="shared" si="5"/>
-        <v>![Asking the Robo CFO Agent about year over year revenue](figures/kb/ss_agent_002_clean.png){#fig-4EF2}</v>
-      </c>
-    </row>
-    <row r="168" spans="1:10" x14ac:dyDescent="0.2">
+        <v>![Asking the Robo CFO Agent about year over year revenue](figures/kb/ss_kbagent_002_clean.png){#fig-D97B}</v>
+      </c>
+    </row>
+    <row r="168" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A168">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B168" s="6" t="s">
         <v>95</v>
@@ -7938,27 +7974,27 @@
         <v>1</v>
       </c>
       <c r="F168" t="s">
-        <v>149</v>
+        <v>528</v>
       </c>
       <c r="G168" t="s">
         <v>324</v>
       </c>
       <c r="H168" s="1" t="str" cm="1">
         <f t="array" ref="H168">CRC16HASH(F168)</f>
-        <v>B2F6</v>
+        <v>257F</v>
       </c>
       <c r="I168" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-B2F6}</v>
+        <v>{#fig-257F}</v>
       </c>
       <c r="J168" t="str">
         <f t="shared" si="5"/>
-        <v>![Asking about Microsoft's 2026 outlook](figures/kb/ss_agent_003_clean.png){#fig-B2F6}</v>
-      </c>
-    </row>
-    <row r="169" spans="1:10" x14ac:dyDescent="0.2">
+        <v>![Asking about Microsoft's 2026 outlook](figures/kb/ss_kbagent_003_clean.png){#fig-257F}</v>
+      </c>
+    </row>
+    <row r="169" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A169">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B169" s="6" t="s">
         <v>95</v>
@@ -7973,27 +8009,27 @@
         <v>1</v>
       </c>
       <c r="F169" t="s">
-        <v>151</v>
+        <v>529</v>
       </c>
       <c r="G169" t="s">
         <v>323</v>
       </c>
       <c r="H169" s="1" t="str" cm="1">
         <f t="array" ref="H169">CRC16HASH(F169)</f>
-        <v>C6EC</v>
+        <v>5165</v>
       </c>
       <c r="I169" t="str">
         <f t="shared" si="4"/>
-        <v>{#fig-C6EC}</v>
+        <v>{#fig-5165}</v>
       </c>
       <c r="J169" t="str">
         <f t="shared" si="5"/>
-        <v>![The "Microsoft FY26 Q2 Outlook" PowerPoint slide](figures/kb/ss_agent_004_clean.png){#fig-C6EC}</v>
-      </c>
-    </row>
-    <row r="170" spans="1:10" x14ac:dyDescent="0.2">
+        <v>![The "Microsoft FY26 Q2 Outlook" PowerPoint slide](figures/kb/ss_kbagent_004_clean.png){#fig-5165}</v>
+      </c>
+    </row>
+    <row r="170" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A170">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B170" s="7" t="s">
         <v>96</v>
@@ -8023,9 +8059,9 @@
         <v/>
       </c>
     </row>
-    <row r="171" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A171">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="B171" s="7" t="s">
         <v>96</v>
@@ -8058,9 +8094,9 @@
         <v>![Creating a new fine-tuning job](figures/ft/ss_finetune_001_ann.png){#fig-706E}</v>
       </c>
     </row>
-    <row r="172" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A172">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B172" s="7" t="s">
         <v>96</v>
@@ -8090,9 +8126,9 @@
         <v/>
       </c>
     </row>
-    <row r="173" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A173">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="B173" s="7" t="s">
         <v>96</v>
@@ -8125,9 +8161,9 @@
         <v>![Defining the fine-tuning job setting](figures/ft/ss_finetune_002_ann.png){#fig-807A}</v>
       </c>
     </row>
-    <row r="174" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A174">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B174" s="7" t="s">
         <v>96</v>
@@ -8157,9 +8193,9 @@
         <v/>
       </c>
     </row>
-    <row r="175" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A175">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B175" s="7" t="s">
         <v>96</v>
@@ -8189,9 +8225,9 @@
         <v/>
       </c>
     </row>
-    <row r="176" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A176">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B176" s="7" t="s">
         <v>96</v>
@@ -8224,9 +8260,9 @@
         <v>![Viewing the status of your new tuning job](figures/ft/ss_finetune_003_ann.png){#fig-1077}</v>
       </c>
     </row>
-    <row r="177" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A177">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B177" s="7" t="s">
         <v>96</v>
@@ -8256,9 +8292,9 @@
         <v/>
       </c>
     </row>
-    <row r="178" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A178">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B178" s="7" t="s">
         <v>96</v>
@@ -8288,9 +8324,9 @@
         <v/>
       </c>
     </row>
-    <row r="179" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A179">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B179" s="7" t="s">
         <v>96</v>
@@ -8323,9 +8359,9 @@
         <v>![The Monitor tab, showing fine-tuning metrics](figures/ft/ss_finetune_005_ann.png){#fig-B05C}</v>
       </c>
     </row>
-    <row r="180" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A180">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B180" s="7" t="s">
         <v>96</v>
@@ -8355,9 +8391,9 @@
         <v/>
       </c>
     </row>
-    <row r="181" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A181">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B181" s="7" t="s">
         <v>96</v>
@@ -8390,9 +8426,9 @@
         <v>![A completed fine-tuning status and metrics](figures/ft/ss_finetune_006_ann.png){#fig-4048}</v>
       </c>
     </row>
-    <row r="182" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A182">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B182" s="7" t="s">
         <v>96</v>
@@ -8422,9 +8458,9 @@
         <v/>
       </c>
     </row>
-    <row r="183" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A183">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B183" s="7" t="s">
         <v>96</v>
@@ -8457,9 +8493,9 @@
         <v>![Customizing the fine-tuned model deployment](figures/ft/ss_finetune_007_ann.png){#fig-D045}</v>
       </c>
     </row>
-    <row r="184" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A184">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B184" s="7" t="s">
         <v>96</v>
@@ -8492,9 +8528,9 @@
         <v>![Adding instructions and playing with your new medical assistant model](figures/ft/ss_finetune_008_clean.png){#fig-124F}</v>
       </c>
     </row>
-    <row r="185" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A185">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B185" s="7" t="s">
         <v>96</v>
@@ -8524,9 +8560,9 @@
         <v/>
       </c>
     </row>
-    <row r="186" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A186">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B186" s="7" t="s">
         <v>96</v>
@@ -8559,9 +8595,9 @@
         <v>![Navigating to the Synthetic generation tab](figures/ft/ss_syntheticdata_001_ann.png){#fig-2C04}</v>
       </c>
     </row>
-    <row r="187" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A187">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B187" s="7" t="s">
         <v>96</v>
@@ -8591,9 +8627,9 @@
         <v/>
       </c>
     </row>
-    <row r="188" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A188">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B188" s="7" t="s">
         <v>96</v>
@@ -8626,9 +8662,9 @@
         <v>![Adding cardiology documents for synthetic data generation](figures/ft/ss_syntheticdata_002_ann.png){#fig-DC10}</v>
       </c>
     </row>
-    <row r="189" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A189">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B189" s="7" t="s">
         <v>96</v>
@@ -8658,9 +8694,9 @@
         <v/>
       </c>
     </row>
-    <row r="190" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A190">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B190" s="7" t="s">
         <v>96</v>
@@ -8693,9 +8729,9 @@
         <v>![Monitoring the queued synthetic data job](figures/ft/ss_syntheticdata_003a_clean.png){#fig-2555}</v>
       </c>
     </row>
-    <row r="191" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A191">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B191" s="7" t="s">
         <v>96</v>
@@ -8728,9 +8764,9 @@
         <v>![Viewing the synthetic data job results](figures/ft/ss_syntheticdata_003_ann.png){#fig-4C1D}</v>
       </c>
     </row>
-    <row r="192" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A192">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B192" s="7" t="s">
         <v>96</v>
@@ -8760,9 +8796,9 @@
         <v/>
       </c>
     </row>
-    <row r="193" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A193">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B193" s="7" t="s">
         <v>96</v>
@@ -8795,9 +8831,9 @@
         <v>![Continuing to fine-tune with the new cardiology synthetic data](figures/ft/ss_syntheticdata_004_ann.png){#fig-7C3B}</v>
       </c>
     </row>
-    <row r="194" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A194">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B194" s="7" t="s">
         <v>96</v>
@@ -8827,9 +8863,9 @@
         <v/>
       </c>
     </row>
-    <row r="195" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A195">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B195" s="7" t="s">
         <v>96</v>
@@ -8862,9 +8898,9 @@
         <v>![Initializing a fine-tuning job from the CLI](figures/ft/ss_cli_001_clean_neg.png){#fig-71F5}</v>
       </c>
     </row>
-    <row r="196" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A196">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B196" s="7" t="s">
         <v>96</v>
@@ -8894,9 +8930,9 @@
         <v/>
       </c>
     </row>
-    <row r="197" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A197">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B197" s="7" t="s">
         <v>96</v>
@@ -8929,9 +8965,9 @@
         <v>![Uploading training data and starting the fine-tuning job](figures/ft/ss_cli_002_clean_neg.png){#fig-70B6}</v>
       </c>
     </row>
-    <row r="198" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A198">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B198" s="7" t="s">
         <v>96</v>
@@ -8961,9 +8997,9 @@
         <v/>
       </c>
     </row>
-    <row r="199" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A199">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B199" s="7" t="s">
         <v>96</v>
@@ -8996,9 +9032,9 @@
         <v>![Listing fine-tuning jobs and showing job details](figures/ft/ss_cli_003_clean_neg.png){#fig-7077}</v>
       </c>
     </row>
-    <row r="200" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A200">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="B200" s="9" t="s">
         <v>353</v>
@@ -9031,9 +9067,9 @@
         <v>![Workflow template patterns](figures/wf/il_types_001_clean.png){#fig-965B}</v>
       </c>
     </row>
-    <row r="201" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A201">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="B201" s="9" t="s">
         <v>353</v>
@@ -9063,9 +9099,9 @@
         <v/>
       </c>
     </row>
-    <row r="202" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A202">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B202" s="9" t="s">
         <v>353</v>
@@ -9098,9 +9134,9 @@
         <v>![Locating Workflows from the Foundry UI](figures/wf/ss_wfportal_001_ann.png){#fig-CFD6}</v>
       </c>
     </row>
-    <row r="203" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A203">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="B203" s="9" t="s">
         <v>353</v>
@@ -9130,9 +9166,9 @@
         <v/>
       </c>
     </row>
-    <row r="204" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A204">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B204" s="9" t="s">
         <v>353</v>
@@ -9165,9 +9201,9 @@
         <v>![Selecting the Human in Loop workflow template](figures/wf/ss_wfportal_002_ann.png){#fig-3FC2}</v>
       </c>
     </row>
-    <row r="205" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A205">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="B205" s="9" t="s">
         <v>353</v>
@@ -9200,9 +9236,9 @@
         <v>![A blank Workflow canvas with only a start node](figures/wf/ss_canvas_001_clean.png){#fig-F349}</v>
       </c>
     </row>
-    <row r="206" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A206">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B206" s="9" t="s">
         <v>353</v>
@@ -9232,9 +9268,9 @@
         <v/>
       </c>
     </row>
-    <row r="207" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A207">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B207" s="9" t="s">
         <v>353</v>
@@ -9264,9 +9300,9 @@
         <v/>
       </c>
     </row>
-    <row r="208" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A208">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B208" s="9" t="s">
         <v>353</v>
@@ -9299,9 +9335,9 @@
         <v>![Saving the Math Coder Workflow](figures/wf/ss_save_001_ann.png){#fig-C624}</v>
       </c>
     </row>
-    <row r="209" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A209">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B209" s="9" t="s">
         <v>353</v>
@@ -9331,9 +9367,9 @@
         <v/>
       </c>
     </row>
-    <row r="210" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A210">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B210" s="9" t="s">
         <v>353</v>
@@ -9366,9 +9402,9 @@
         <v>![The + New node panel](figures/wf/ss_nodes_001_ann.png){#fig-B84E}</v>
       </c>
     </row>
-    <row r="211" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A211">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B211" s="9" t="s">
         <v>353</v>
@@ -9398,9 +9434,9 @@
         <v/>
       </c>
     </row>
-    <row r="212" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A212">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="B212" s="9" t="s">
         <v>353</v>
@@ -9433,9 +9469,9 @@
         <v>![Adding an Ask a question node](figures/wf/ss_canvas_002_ann.png){#fig-2C1A}</v>
       </c>
     </row>
-    <row r="213" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A213">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="B213" s="9" t="s">
         <v>353</v>
@@ -9465,9 +9501,9 @@
         <v/>
       </c>
     </row>
-    <row r="214" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A214">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B214" s="9" t="s">
         <v>353</v>
@@ -9500,9 +9536,9 @@
         <v>![Configuring the Ask a question node to ask for a math problem](figures/wf/ss_canvas_003_ann.png){#fig-BC17}</v>
       </c>
     </row>
-    <row r="215" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="215" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A215">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B215" s="9" t="s">
         <v>353</v>
@@ -9532,9 +9568,9 @@
         <v/>
       </c>
     </row>
-    <row r="216" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="216" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A216">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B216" s="9" t="s">
         <v>353</v>
@@ -9567,9 +9603,9 @@
         <v>![Configuring the Latest Message variable](figures/wf/ss_canvas_004_ann.png){#fig-8C31}</v>
       </c>
     </row>
-    <row r="217" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="217" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A217">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B217" s="9" t="s">
         <v>353</v>
@@ -9599,9 +9635,9 @@
         <v/>
       </c>
     </row>
-    <row r="218" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="218" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A218">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B218" s="9" t="s">
         <v>353</v>
@@ -9634,9 +9670,9 @@
         <v>![Configuring the Turn Count variable](figures/wf/ss_canvas_005_ann.png){#fig-1C3C}</v>
       </c>
     </row>
-    <row r="219" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="219" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A219">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B219" s="9" t="s">
         <v>353</v>
@@ -9666,9 +9702,9 @@
         <v/>
       </c>
     </row>
-    <row r="220" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="220" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A220">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="B220" s="9" t="s">
         <v>353</v>
@@ -9701,9 +9737,9 @@
         <v>![Configuring the Math Evaluator Agent node](figures/wf/ss_canvas_006_ann.png){#fig-EC28}</v>
       </c>
     </row>
-    <row r="221" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="221" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A221">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B221" s="9" t="s">
         <v>353</v>
@@ -9733,9 +9769,9 @@
         <v/>
       </c>
     </row>
-    <row r="222" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A222">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B222" s="9" t="s">
         <v>353</v>
@@ -9768,9 +9804,9 @@
         <v>![Configuring the Math Evaluator Agent's behavior](figures/wf/ss_canvas_007_ann.png){#fig-7C25}</v>
       </c>
     </row>
-    <row r="223" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="223" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A223">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B223" s="9" t="s">
         <v>353</v>
@@ -9800,9 +9836,9 @@
         <v/>
       </c>
     </row>
-    <row r="224" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="224" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A224">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="B224" s="9" t="s">
         <v>353</v>
@@ -9835,9 +9871,9 @@
         <v>![Configuring the If/else logic to handle evaluation failures](figures/wf/ss_canvas_008_ann.png){#fig-8C64}</v>
       </c>
     </row>
-    <row r="225" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A225">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B225" s="9" t="s">
         <v>353</v>
@@ -9867,9 +9903,9 @@
         <v/>
       </c>
     </row>
-    <row r="226" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="226" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A226">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B226" s="9" t="s">
         <v>353</v>
@@ -9902,9 +9938,9 @@
         <v>![Configuring the message to the user if evaluation failed](figures/wf/ss_canvas_009_ann.png){#fig-1C69}</v>
       </c>
     </row>
-    <row r="227" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="227" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A227">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B227" s="9" t="s">
         <v>353</v>
@@ -9934,9 +9970,9 @@
         <v/>
       </c>
     </row>
-    <row r="228" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="228" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A228">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="B228" s="9" t="s">
         <v>353</v>
@@ -9969,9 +10005,9 @@
         <v>![Configuring the message to the user if evaluation succeeded](figures/wf/ss_canvas_010_ann.png){#fig-8952}</v>
       </c>
     </row>
-    <row r="229" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="229" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A229">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="B229" s="9" t="s">
         <v>353</v>
@@ -10004,9 +10040,9 @@
         <v>![The first half of the Math Coder Workflow](figures/wf/ss_canvas_011_clean.png){#fig-30B4}</v>
       </c>
     </row>
-    <row r="230" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A230">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="B230" s="9" t="s">
         <v>353</v>
@@ -10036,9 +10072,9 @@
         <v/>
       </c>
     </row>
-    <row r="231" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A231">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B231" s="9" t="s">
         <v>353</v>
@@ -10068,9 +10104,9 @@
         <v/>
       </c>
     </row>
-    <row r="232" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="232" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A232">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="B232" s="9" t="s">
         <v>353</v>
@@ -10103,9 +10139,9 @@
         <v>![Seeing the YAML version of what you've built](figures/wf/ss_canvas_012_ann.png){#fig-E94B}</v>
       </c>
     </row>
-    <row r="233" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="233" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A233">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B233" s="9" t="s">
         <v>353</v>
@@ -10135,9 +10171,9 @@
         <v/>
       </c>
     </row>
-    <row r="234" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A234">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="B234" s="9" t="s">
         <v>353</v>
@@ -10170,9 +10206,9 @@
         <v>![Seeing the visual version of the full YAML pipeline](figures/wf/ss_canvas_013_ann.png){#fig-7946}</v>
       </c>
     </row>
-    <row r="235" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="235" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A235">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B235" s="9" t="s">
         <v>353</v>
@@ -10202,9 +10238,9 @@
         <v/>
       </c>
     </row>
-    <row r="236" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="236" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A236">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="B236" s="9" t="s">
         <v>353</v>
@@ -10237,9 +10273,9 @@
         <v>![Configuring the Python Coder Agent's behavior](figures/wf/ss_canvas_014_ann.png){#fig-4960}</v>
       </c>
     </row>
-    <row r="237" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A237">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="B237" s="9" t="s">
         <v>353</v>
@@ -10272,9 +10308,9 @@
         <v>![The response node contained the problem's solution](figures/wf/ss_canvas_015_clean.png){#fig-A1}</v>
       </c>
     </row>
-    <row r="238" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="238" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A238">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B238" s="9" t="s">
         <v>353</v>
@@ -10307,9 +10343,9 @@
         <v>![An example math problem input](figures/wf/ss_mathproblem_001_clean.png){#fig-8A6D}</v>
       </c>
     </row>
-    <row r="239" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="239" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A239">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B239" s="9" t="s">
         <v>353</v>
@@ -10342,9 +10378,9 @@
         <v>![The evaluation of the math problem](figures/wf/ss_mathproblem_002_clean.png){#fig-CE62}</v>
       </c>
     </row>
-    <row r="240" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="240" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A240">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="B240" s="9" t="s">
         <v>353</v>
@@ -10377,9 +10413,9 @@
         <v>![The results and outputs of the math workflow](figures/wf/ss_mathproblem_003_clean.png){#fig-3266}</v>
       </c>
     </row>
-    <row r="241" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="241" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A241">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B241" s="9" t="s">
         <v>353</v>
@@ -10412,9 +10448,9 @@
         <v>![Viewing the invocation logs for your chat session](figures/wf/ss_logs_001_clean.png){#fig-BBDE}</v>
       </c>
     </row>
-    <row r="242" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="242" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A242">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="B242" s="10" t="s">
         <v>416</v>
@@ -10444,9 +10480,9 @@
         <v/>
       </c>
     </row>
-    <row r="243" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="243" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A243">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B243" s="10" t="s">
         <v>416</v>
@@ -10479,9 +10515,9 @@
         <v>![Locating Guardrails from the Foundry UI](figures/am/ss_guardrails_001_ann.png){#fig-D83D}</v>
       </c>
     </row>
-    <row r="244" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="244" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A244">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B244" s="10" t="s">
         <v>416</v>
@@ -10511,9 +10547,9 @@
         <v/>
       </c>
     </row>
-    <row r="245" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="245" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A245">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B245" s="10" t="s">
         <v>416</v>
@@ -10546,9 +10582,9 @@
         <v>![Selecting Risks in a new Guardrail](figures/am/ss_guardrails_002_ann.png){#fig-2829}</v>
       </c>
     </row>
-    <row r="246" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="246" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A246">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="B246" s="10" t="s">
         <v>416</v>
@@ -10578,9 +10614,9 @@
         <v/>
       </c>
     </row>
-    <row r="247" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="247" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A247">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B247" s="10" t="s">
         <v>416</v>
@@ -10613,9 +10649,9 @@
         <v>![Selecting the intervention points and actions for the Risk](figures/am/ss_guardrails_003_ann.png){#fig-B824}</v>
       </c>
     </row>
-    <row r="248" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="248" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A248">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B248" s="10" t="s">
         <v>416</v>
@@ -10648,9 +10684,9 @@
         <v>![Control intervention points in an Agent response flow](figures/am/il_controls_001_clean.png){#fig-515E}</v>
       </c>
     </row>
-    <row r="249" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="249" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A249">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B249" s="10" t="s">
         <v>416</v>
@@ -10680,9 +10716,9 @@
         <v/>
       </c>
     </row>
-    <row r="250" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="250" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A250">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="B250" s="10" t="s">
         <v>416</v>
@@ -10715,9 +10751,9 @@
         <v>![Reviewing the Controls added to the Guardrail](figures/am/ss_guardrails_004_ann.png){#fig-8802}</v>
       </c>
     </row>
-    <row r="251" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="251" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A251">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="B251" s="10" t="s">
         <v>416</v>
@@ -10747,9 +10783,9 @@
         <v/>
       </c>
     </row>
-    <row r="252" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="252" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A252">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="B252" s="10" t="s">
         <v>416</v>
@@ -10782,9 +10818,9 @@
         <v>![Applying the Guardrail to Models and Agents](figures/am/ss_guardrails_005_ann.png){#fig-180F}</v>
       </c>
     </row>
-    <row r="253" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="253" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A253">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B253" s="10" t="s">
         <v>416</v>
@@ -10817,9 +10853,9 @@
         <v>![Reviewing the Guardrail selections before saving](figures/am/ss_guardrails_006_clean.png){#fig-B446}</v>
       </c>
     </row>
-    <row r="254" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="254" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A254">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="B254" s="10" t="s">
         <v>416</v>
@@ -10849,9 +10885,9 @@
         <v/>
       </c>
     </row>
-    <row r="255" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="255" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A255">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="B255" s="10" t="s">
         <v>416</v>
@@ -10884,9 +10920,9 @@
         <v>![Locating Blocklists from the Foundry UI](figures/am/ss_blocklists_001_ann.png){#fig-9B6C}</v>
       </c>
     </row>
-    <row r="256" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="256" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A256">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="B256" s="10" t="s">
         <v>416</v>
@@ -10916,9 +10952,9 @@
         <v/>
       </c>
     </row>
-    <row r="257" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="257" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A257">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B257" s="10" t="s">
         <v>416</v>
@@ -10951,9 +10987,9 @@
         <v>![Making a new Blocklist of competitor AI products](figures/am/ss_blocklists_002_ann.png){#fig-6B78}</v>
       </c>
     </row>
-    <row r="258" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="258" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A258">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="B258" s="10" t="s">
         <v>416</v>
@@ -10986,9 +11022,9 @@
         <v>![Adding the Blocklist in a Guardrail](figures/am/ss_blocklists_003_clean.png){#fig-192B}</v>
       </c>
     </row>
-    <row r="259" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="259" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A259">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="B259" s="10" t="s">
         <v>416</v>
@@ -11021,9 +11057,9 @@
         <v>![Exploring the available third-party integrations](figures/am/ss_integrations_001_clean.png){#fig-8807}</v>
       </c>
     </row>
-    <row r="260" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="260" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A260">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="B260" s="10" t="s">
         <v>416</v>
@@ -11053,9 +11089,9 @@
         <v/>
       </c>
     </row>
-    <row r="261" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="261" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A261">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B261" s="10" t="s">
         <v>416</v>
@@ -11088,9 +11124,9 @@
         <v>![The Conrol Plane's Operate page of the Foundry UI](figures/am/ss_controlplane_001_ann.png){#fig-5103}</v>
       </c>
     </row>
-    <row r="262" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="262" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A262">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="B262" s="10" t="s">
         <v>416</v>
@@ -11120,9 +11156,9 @@
         <v/>
       </c>
     </row>
-    <row r="263" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="263" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A263">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="B263" s="10" t="s">
         <v>416</v>
@@ -11155,9 +11191,9 @@
         <v>![Viewing all your assets in the Control Plane](figures/am/ss_controlplane_002_ann.png){#fig-A117}</v>
       </c>
     </row>
-    <row r="264" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="264" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A264">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="B264" s="10" t="s">
         <v>416</v>
@@ -11172,27 +11208,27 @@
         <v>1</v>
       </c>
       <c r="F264" t="s">
-        <v>446</v>
+        <v>530</v>
       </c>
       <c r="G264" t="s">
         <v>450</v>
       </c>
       <c r="H264" s="1" t="str" cm="1">
         <f t="array" ref="H264">CRC16HASH(F264)</f>
-        <v>4282</v>
+        <v>BE86</v>
       </c>
       <c r="I264" t="str">
         <f t="shared" si="20"/>
-        <v>{#fig-4282}</v>
+        <v>{#fig-BE86}</v>
       </c>
       <c r="J264" t="str">
         <f t="shared" si="21"/>
-        <v>![Viewing the Monitor tab of an Agent](figures/am/ss_controlplane_002_clean.png){#fig-4282}</v>
-      </c>
-    </row>
-    <row r="265" spans="1:10" x14ac:dyDescent="0.2">
+        <v>![Viewing the Monitor tab of an Agent](figures/am/ss_controlplane_003_clean.png){#fig-BE86}</v>
+      </c>
+    </row>
+    <row r="265" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A265">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B265" s="10" t="s">
         <v>416</v>
@@ -11222,9 +11258,9 @@
         <v/>
       </c>
     </row>
-    <row r="266" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="266" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A266">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="B266" s="10" t="s">
         <v>416</v>
@@ -11257,9 +11293,9 @@
         <v>![Viewing the Quotas table in the Control Plane](figures/am/ss_quotas_001_ann.png){#fig-34A7}</v>
       </c>
     </row>
-    <row r="267" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="267" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A267">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B267" s="10" t="s">
         <v>416</v>
@@ -11289,9 +11325,9 @@
         <v/>
       </c>
     </row>
-    <row r="268" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="268" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A268">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="B268" s="10" t="s">
         <v>416</v>
@@ -11324,9 +11360,9 @@
         <v>![Editing the quota for a model](figures/am/ss_quotas_002_ann.png){#fig-C4B3}</v>
       </c>
     </row>
-    <row r="269" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="269" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A269">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B269" s="10" t="s">
         <v>416</v>
@@ -11356,9 +11392,9 @@
         <v/>
       </c>
     </row>
-    <row r="270" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="270" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A270">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="B270" s="10" t="s">
         <v>416</v>
@@ -11391,9 +11427,9 @@
         <v>![Enabling Microsoft Purview monitoring of your Foundry Project](figures/am/ss_compliance_001_ann.png){#fig-AB2E}</v>
       </c>
     </row>
-    <row r="271" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="271" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A271">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="B271" s="10" t="s">
         <v>416</v>
@@ -11426,9 +11462,9 @@
         <v>![The Agent ID dashboard from the Azure Portal](figures/am/ss_agentid_001_clean.png){#fig-A73E}</v>
       </c>
     </row>
-    <row r="272" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="272" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A272">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B272" s="10" t="s">
         <v>416</v>
@@ -11458,9 +11494,9 @@
         <v/>
       </c>
     </row>
-    <row r="273" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="273" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A273">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="B273" s="10" t="s">
         <v>416</v>
@@ -11493,9 +11529,9 @@
         <v>![Publishing an Agent to retrieve its Principal ID](figures/am/ss_entra_001_ann.png){#fig-D3C6}</v>
       </c>
     </row>
-    <row r="274" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="274" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A274">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="B274" s="10" t="s">
         <v>416</v>
@@ -11528,9 +11564,9 @@
         <v>![The general Application ID for the Foundry Project in Entra ID](figures/am/ss_entra_002_clean.png){#fig-7351}</v>
       </c>
     </row>
-    <row r="275" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="275" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A275">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="B275" s="8" t="s">
         <v>334</v>
@@ -11563,9 +11599,9 @@
         <v>![Key features of Foundry Local](figures/ed/il_local_001_clean.png){#fig-8639}</v>
       </c>
     </row>
-    <row r="276" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="276" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A276">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="B276" s="8" t="s">
         <v>334</v>
@@ -11598,9 +11634,9 @@
         <v>![Architecture components of Foundry Local](figures/ed/il_local_002_clean.png){#fig-C236}</v>
       </c>
     </row>
-    <row r="277" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="277" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A277">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="B277" s="8" t="s">
         <v>334</v>
@@ -11633,9 +11669,9 @@
         <v>![The Foundry Local website homepage](figures/ed/ss_localsite_001_clean.png){#fig-6A11}</v>
       </c>
     </row>
-    <row r="278" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="278" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A278">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B278" s="8" t="s">
         <v>334</v>
@@ -11668,9 +11704,9 @@
         <v>![Chatting with a small Qwen 2.5 model using the Foundry Local CLI](figures/ed/ss_local_001_clean.png){#fig-9AEF}</v>
       </c>
     </row>
-    <row r="279" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="279" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A279">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="B279" s="8" t="s">
         <v>334</v>
@@ -11703,9 +11739,9 @@
         <v>![Chatting with a Phi-4 model with reasoning using the Foundry Local CLI](figures/ed/ss_local_002_clean.png){#fig-DEE0}</v>
       </c>
     </row>
-    <row r="280" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="280" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A280">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="B280" s="8" t="s">
         <v>334</v>
@@ -11738,9 +11774,9 @@
         <v>![Chatting with an LLM using the Foundry Local Python SDK](figures/ed/ss_local_003_clean.png){#fig-22E4}</v>
       </c>
     </row>
-    <row r="281" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="281" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A281">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="B281" s="8" t="s">
         <v>334</v>
@@ -11773,9 +11809,9 @@
         <v>![Audio transcription with a Whisper model using the Foundry Local Javascript app](figures/ed/ss_local_004_clean.png){#fig-56FE}</v>
       </c>
     </row>
-    <row r="282" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="282" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A282">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="B282" s="8" t="s">
         <v>334</v>
@@ -11808,9 +11844,9 @@
         <v>![Quantization example walkthrough from FP32 to INT4](figures/ed/il_quant_001_clean.png){#fig-6908}</v>
       </c>
     </row>
-    <row r="283" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="283" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A283">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="B283" s="8" t="s">
         <v>334</v>
@@ -11835,17 +11871,17 @@
         <v>C0FB</v>
       </c>
       <c r="I283" t="str">
-        <f t="shared" ref="I283:I304" si="29">_xlfn.CONCAT("{#fig-",H283,"}")</f>
+        <f t="shared" ref="I283:I306" si="29">_xlfn.CONCAT("{#fig-",H283,"}")</f>
         <v>{#fig-C0FB}</v>
       </c>
       <c r="J283" t="str">
-        <f t="shared" ref="J283:J304" si="30">IF(E283,_xlfn.CONCAT("![",G283,"](figures/",B283,"/",F283,")",I283),"")</f>
+        <f t="shared" ref="J283:J306" si="30">IF(E283,_xlfn.CONCAT("![",G283,"](figures/",B283,"/",F283,")",I283),"")</f>
         <v>![Quantization of Qwen 2.5 0.5B for CPU inference using Olive](figures/ed/ss_olive_001_clean.png){#fig-C0FB}</v>
       </c>
     </row>
-    <row r="284" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="284" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A284">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="B284" s="11" t="s">
         <v>92</v>
@@ -11878,9 +11914,9 @@
         <v>![How a memory store recalls previous context](figures/co/il_memory_001_clean.png){#fig-9BA0}</v>
       </c>
     </row>
-    <row r="285" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="285" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A285">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="B285" s="11" t="s">
         <v>92</v>
@@ -11910,9 +11946,9 @@
         <v/>
       </c>
     </row>
-    <row r="286" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="286" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A286">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="B286" s="11" t="s">
         <v>92</v>
@@ -11945,9 +11981,9 @@
         <v>![Locating the memory capability on an Agent](figures/co/ss_memory_001_ann.png){#fig-D4BD}</v>
       </c>
     </row>
-    <row r="287" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="287" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A287">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="B287" s="11" t="s">
         <v>92</v>
@@ -11980,9 +12016,9 @@
         <v>![Editing the memory store](figures/co/ss_memory_002_clean.png){#fig-4132}</v>
       </c>
     </row>
-    <row r="288" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="288" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A288">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="B288" s="11" t="s">
         <v>92</v>
@@ -12012,9 +12048,9 @@
         <v/>
       </c>
     </row>
-    <row r="289" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="289" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A289">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="B289" s="11" t="s">
         <v>92</v>
@@ -12047,9 +12083,9 @@
         <v>![Locating the Evaluations screen](figures/co/ss_evaluations_001_ann.png){#fig-AB12}</v>
       </c>
     </row>
-    <row r="290" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="290" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A290">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="B290" s="11" t="s">
         <v>92</v>
@@ -12082,9 +12118,9 @@
         <v>![Configuring the evaluation process for an agent using synthetic data](figures/co/ss_evaluations_002_clean.png){#fig-510E}</v>
       </c>
     </row>
-    <row r="291" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="291" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A291">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="B291" s="11" t="s">
         <v>92</v>
@@ -12114,9 +12150,9 @@
         <v/>
       </c>
     </row>
-    <row r="292" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="292" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A292">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="B292" s="11" t="s">
         <v>92</v>
@@ -12149,9 +12185,9 @@
         <v>![The Evaluator catalog show the details of a built-in evaluator](figures/co/ss_evaluations_003_ann.png){#fig-CB0B}</v>
       </c>
     </row>
-    <row r="293" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="293" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A293">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B293" s="11" t="s">
         <v>92</v>
@@ -12181,9 +12217,9 @@
         <v/>
       </c>
     </row>
-    <row r="294" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="294" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A294">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="B294" s="11" t="s">
         <v>92</v>
@@ -12216,9 +12252,9 @@
         <v>![Locating the Batch jobs feature under Models](figures/co/ss_batchjobs_001_ann.png){#fig-17AA}</v>
       </c>
     </row>
-    <row r="295" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="295" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A295">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B295" s="11" t="s">
         <v>92</v>
@@ -12251,9 +12287,9 @@
         <v>![Uploading .jsonl data to create a batch job](figures/co/ss_batchjobs_002_clean.png){#fig-E07D}</v>
       </c>
     </row>
-    <row r="296" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="296" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A296">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="B296" s="11" t="s">
         <v>92</v>
@@ -12283,9 +12319,9 @@
         <v/>
       </c>
     </row>
-    <row r="297" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="297" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A297">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="B297" s="11" t="s">
         <v>92</v>
@@ -12318,9 +12354,9 @@
         <v>![Locating the AI Services options under Models](figures/co/ss_aiservices_001_ann.png){#fig-2CED}</v>
       </c>
     </row>
-    <row r="298" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="298" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A298">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="B298" s="11" t="s">
         <v>92</v>
@@ -12353,9 +12389,9 @@
         <v>![Testing out the Voice Live AI service in a Playground](figures/co/ss_aiservices_002_clean.png){#fig-C30F}</v>
       </c>
     </row>
-    <row r="299" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="299" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A299">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="B299" s="11" t="s">
         <v>92</v>
@@ -12380,23 +12416,23 @@
         <v>331E</v>
       </c>
       <c r="I299" t="str">
-        <f t="shared" ref="I299" si="31">_xlfn.CONCAT("{#fig-",H299,"}")</f>
+        <f t="shared" ref="I299:I301" si="31">_xlfn.CONCAT("{#fig-",H299,"}")</f>
         <v>{#fig-331E}</v>
       </c>
       <c r="J299" t="str">
-        <f t="shared" ref="J299" si="32">IF(E299,_xlfn.CONCAT("![",G299,"](figures/",B299,"/",F299,")",I299),"")</f>
+        <f t="shared" ref="J299:J301" si="32">IF(E299,_xlfn.CONCAT("![",G299,"](figures/",B299,"/",F299,")",I299),"")</f>
         <v>![How GraphRAG forms an entity knowledge graph of communities](figures/co/il_graphrag_001_clean.png){#fig-331E}</v>
       </c>
     </row>
-    <row r="300" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="300" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A300">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="B300" s="11" t="s">
         <v>92</v>
       </c>
       <c r="C300" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D300" t="b">
         <v>0</v>
@@ -12405,240 +12441,240 @@
         <v>1</v>
       </c>
       <c r="F300" t="s">
-        <v>473</v>
+        <v>521</v>
       </c>
       <c r="G300" t="s">
-        <v>474</v>
+        <v>523</v>
       </c>
       <c r="H300" s="1" t="str" cm="1">
         <f t="array" ref="H300">CRC16HASH(F300)</f>
+        <v>2BE6</v>
+      </c>
+      <c r="I300" t="str">
+        <f t="shared" si="31"/>
+        <v>{#fig-2BE6}</v>
+      </c>
+      <c r="J300" t="str">
+        <f t="shared" si="32"/>
+        <v>![Locating the Foundry Toolkit extension in VS Code](figures/co/ss_vscode_001_clean.png){#fig-2BE6}</v>
+      </c>
+    </row>
+    <row r="301" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A301">
+        <v>300</v>
+      </c>
+      <c r="B301" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="C301" t="s">
+        <v>4</v>
+      </c>
+      <c r="D301" t="b">
+        <v>0</v>
+      </c>
+      <c r="E301" t="b">
+        <v>1</v>
+      </c>
+      <c r="F301" t="s">
+        <v>522</v>
+      </c>
+      <c r="G301" t="s">
+        <v>524</v>
+      </c>
+      <c r="H301" s="1" t="str" cm="1">
+        <f t="array" ref="H301">CRC16HASH(F301)</f>
+        <v>6FE9</v>
+      </c>
+      <c r="I301" t="str">
+        <f t="shared" si="31"/>
+        <v>{#fig-6FE9}</v>
+      </c>
+      <c r="J301" t="str">
+        <f t="shared" si="32"/>
+        <v>![Exploring models and creating agents in Foundry Toolkit](figures/co/ss_vscode_002_clean.png){#fig-6FE9}</v>
+      </c>
+    </row>
+    <row r="302" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A302">
+        <v>301</v>
+      </c>
+      <c r="B302" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="C302" t="s">
+        <v>6</v>
+      </c>
+      <c r="D302" t="b">
+        <v>0</v>
+      </c>
+      <c r="E302" t="b">
+        <v>1</v>
+      </c>
+      <c r="F302" t="s">
+        <v>473</v>
+      </c>
+      <c r="G302" t="s">
+        <v>474</v>
+      </c>
+      <c r="H302" s="1" t="str" cm="1">
+        <f t="array" ref="H302">CRC16HASH(F302)</f>
         <v>1FED</v>
       </c>
-      <c r="I300" t="str">
+      <c r="I302" t="str">
         <f t="shared" si="29"/>
         <v>{#fig-1FED}</v>
       </c>
-      <c r="J300" t="str">
+      <c r="J302" t="str">
         <f t="shared" si="30"/>
         <v>![Governance workflow of the Microsoft Agent Governance Toolkit](figures/co/il_govframework_001_clean.png){#fig-1FED}</v>
       </c>
     </row>
-    <row r="301" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A301">
+    <row r="303" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A303">
         <v>302</v>
       </c>
-      <c r="B301" s="11" t="s">
+      <c r="B303" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="C301" t="s">
+      <c r="C303" t="s">
         <v>6</v>
       </c>
-      <c r="D301" t="b">
-        <v>0</v>
-      </c>
-      <c r="E301" t="b">
-        <v>1</v>
-      </c>
-      <c r="F301" t="s">
+      <c r="D303" t="b">
+        <v>0</v>
+      </c>
+      <c r="E303" t="b">
+        <v>1</v>
+      </c>
+      <c r="F303" t="s">
         <v>475</v>
       </c>
-      <c r="G301" t="s">
+      <c r="G303" t="s">
         <v>476</v>
       </c>
-      <c r="H301" s="1" t="str" cm="1">
-        <f t="array" ref="H301">CRC16HASH(F301)</f>
+      <c r="H303" s="1" t="str" cm="1">
+        <f t="array" ref="H303">CRC16HASH(F303)</f>
         <v>5BE2</v>
       </c>
-      <c r="I301" t="str">
+      <c r="I303" t="str">
         <f t="shared" si="29"/>
         <v>{#fig-5BE2}</v>
       </c>
-      <c r="J301" t="str">
+      <c r="J303" t="str">
         <f t="shared" si="30"/>
         <v>![The 4 privilege rings of zero-trust Agent identity](figures/co/il_govframework_002_clean.png){#fig-5BE2}</v>
       </c>
     </row>
-    <row r="302" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A302">
+    <row r="304" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A304">
         <v>303</v>
       </c>
-      <c r="B302" s="11" t="s">
+      <c r="B304" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="C302" t="s">
-        <v>4</v>
-      </c>
-      <c r="D302" t="b">
-        <v>0</v>
-      </c>
-      <c r="E302" t="b">
-        <v>1</v>
-      </c>
-      <c r="F302" t="s">
+      <c r="C304" t="s">
+        <v>4</v>
+      </c>
+      <c r="D304" t="b">
+        <v>0</v>
+      </c>
+      <c r="E304" t="b">
+        <v>1</v>
+      </c>
+      <c r="F304" t="s">
         <v>511</v>
       </c>
-      <c r="G302" t="s">
+      <c r="G304" t="s">
         <v>510</v>
       </c>
-      <c r="H302" s="1" t="str" cm="1">
-        <f t="array" ref="H302">CRC16HASH(F302)</f>
+      <c r="H304" s="1" t="str" cm="1">
+        <f t="array" ref="H304">CRC16HASH(F304)</f>
         <v>285E</v>
       </c>
-      <c r="I302" t="str">
+      <c r="I304" t="str">
         <f t="shared" si="29"/>
         <v>{#fig-285E}</v>
       </c>
-      <c r="J302" t="str">
+      <c r="J304" t="str">
         <f t="shared" si="30"/>
         <v>![Role-based access controls for Foundry resources](figures/co/ss_identity_001_clean.png){#fig-285E}</v>
       </c>
     </row>
-    <row r="303" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A303">
+    <row r="305" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A305">
         <v>304</v>
       </c>
-      <c r="B303" s="11" t="s">
+      <c r="B305" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="C303" t="s">
-        <v>4</v>
-      </c>
-      <c r="D303" t="b">
-        <v>0</v>
-      </c>
-      <c r="E303" t="b">
-        <v>0</v>
-      </c>
-      <c r="F303" t="s">
+      <c r="C305" t="s">
+        <v>4</v>
+      </c>
+      <c r="D305" t="b">
+        <v>0</v>
+      </c>
+      <c r="E305" t="b">
+        <v>0</v>
+      </c>
+      <c r="F305" t="s">
         <v>512</v>
       </c>
-      <c r="H303" s="1" t="str" cm="1">
-        <f t="array" ref="H303">CRC16HASH(F303)</f>
+      <c r="H305" s="1" t="str" cm="1">
+        <f t="array" ref="H305">CRC16HASH(F305)</f>
         <v>DE11</v>
       </c>
-      <c r="I303" t="str">
+      <c r="I305" t="str">
         <f t="shared" si="29"/>
         <v>{#fig-DE11}</v>
       </c>
-      <c r="J303" t="str">
+      <c r="J305" t="str">
         <f t="shared" si="30"/>
         <v/>
       </c>
     </row>
-    <row r="304" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A304">
+    <row r="306" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A306">
         <v>305</v>
       </c>
-      <c r="B304" s="11" t="s">
+      <c r="B306" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="C304" t="s">
-        <v>4</v>
-      </c>
-      <c r="D304" t="b">
-        <v>0</v>
-      </c>
-      <c r="E304" t="b">
-        <v>1</v>
-      </c>
-      <c r="F304" t="s">
+      <c r="C306" t="s">
+        <v>4</v>
+      </c>
+      <c r="D306" t="b">
+        <v>0</v>
+      </c>
+      <c r="E306" t="b">
+        <v>1</v>
+      </c>
+      <c r="F306" t="s">
         <v>513</v>
       </c>
-      <c r="G304" t="s">
+      <c r="G306" t="s">
         <v>450</v>
       </c>
-      <c r="H304" s="1" t="str" cm="1">
-        <f t="array" ref="H304">CRC16HASH(F304)</f>
+      <c r="H306" s="1" t="str" cm="1">
+        <f t="array" ref="H306">CRC16HASH(F306)</f>
         <v>30D0</v>
       </c>
-      <c r="I304" t="str">
+      <c r="I306" t="str">
         <f t="shared" si="29"/>
         <v>{#fig-30D0}</v>
       </c>
-      <c r="J304" t="str">
+      <c r="J306" t="str">
         <f t="shared" si="30"/>
         <v>![Viewing the Monitor tab of an Agent](figures/co/ss_monitor_001_ann.png){#fig-30D0}</v>
       </c>
     </row>
-    <row r="305" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A305">
+    <row r="307" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A307">
         <v>306</v>
-      </c>
-      <c r="B305" s="11" t="s">
-        <v>92</v>
-      </c>
-      <c r="C305" t="s">
-        <v>4</v>
-      </c>
-      <c r="D305" t="b">
-        <v>0</v>
-      </c>
-      <c r="E305" t="b">
-        <v>1</v>
-      </c>
-      <c r="F305" t="s">
-        <v>514</v>
-      </c>
-      <c r="G305" t="s">
-        <v>509</v>
-      </c>
-      <c r="H305" s="1" t="str" cm="1">
-        <f t="array" ref="H305">CRC16HASH(F305)</f>
-        <v>9A1E</v>
-      </c>
-      <c r="I305" t="str">
-        <f t="shared" ref="I305" si="33">_xlfn.CONCAT("{#fig-",H305,"}")</f>
-        <v>{#fig-9A1E}</v>
-      </c>
-      <c r="J305" t="str">
-        <f t="shared" ref="J305" si="34">IF(E305,_xlfn.CONCAT("![",G305,"](figures/",B305,"/",F305,")",I305),"")</f>
-        <v>![Viewing the Application Insights service for the Foundry Project](figures/co/ss_monitor_002_clean.png){#fig-9A1E}</v>
-      </c>
-    </row>
-    <row r="306" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A306">
-        <v>307</v>
-      </c>
-      <c r="B306" s="11" t="s">
-        <v>92</v>
-      </c>
-      <c r="C306" t="s">
-        <v>4</v>
-      </c>
-      <c r="D306" t="b">
-        <v>0</v>
-      </c>
-      <c r="E306" t="b">
-        <v>1</v>
-      </c>
-      <c r="F306" t="s">
-        <v>508</v>
-      </c>
-      <c r="G306" t="s">
-        <v>507</v>
-      </c>
-      <c r="H306" s="1" t="str" cm="1">
-        <f t="array" ref="H306">CRC16HASH(F306)</f>
-        <v>DD24</v>
-      </c>
-      <c r="I306" t="str">
-        <f t="shared" ref="I306" si="35">_xlfn.CONCAT("{#fig-",H306,"}")</f>
-        <v>{#fig-DD24}</v>
-      </c>
-      <c r="J306" t="str">
-        <f t="shared" ref="J306" si="36">IF(E306,_xlfn.CONCAT("![",G306,"](figures/",B306,"/",F306,")",I306),"")</f>
-        <v>![Viewing the Cost Management screen for the Foundry-related resources](figures/co/ss_costs_001_clean.png){#fig-DD24}</v>
-      </c>
-    </row>
-    <row r="307" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A307">
-        <v>308</v>
       </c>
       <c r="B307" s="11" t="s">
         <v>92</v>
       </c>
       <c r="C307" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D307" t="b">
         <v>0</v>
@@ -12647,33 +12683,33 @@
         <v>1</v>
       </c>
       <c r="F307" t="s">
-        <v>502</v>
+        <v>514</v>
       </c>
       <c r="G307" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="H307" s="1" t="str" cm="1">
         <f t="array" ref="H307">CRC16HASH(F307)</f>
-        <v>F9BA</v>
+        <v>9A1E</v>
       </c>
       <c r="I307" t="str">
-        <f t="shared" ref="I307" si="37">_xlfn.CONCAT("{#fig-",H307,"}")</f>
-        <v>{#fig-F9BA}</v>
+        <f t="shared" ref="I307" si="33">_xlfn.CONCAT("{#fig-",H307,"}")</f>
+        <v>{#fig-9A1E}</v>
       </c>
       <c r="J307" t="str">
-        <f t="shared" ref="J307" si="38">IF(E307,_xlfn.CONCAT("![",G307,"](figures/",B307,"/",F307,")",I307),"")</f>
-        <v>![A basic, mostly serverless architecture for AI](figures/co/il_architecture_001_clean.png){#fig-F9BA}</v>
-      </c>
-    </row>
-    <row r="308" spans="1:10" x14ac:dyDescent="0.2">
+        <f t="shared" ref="J307" si="34">IF(E307,_xlfn.CONCAT("![",G307,"](figures/",B307,"/",F307,")",I307),"")</f>
+        <v>![Viewing the Application Insights service for the Foundry Project](figures/co/ss_monitor_002_clean.png){#fig-9A1E}</v>
+      </c>
+    </row>
+    <row r="308" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A308">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="B308" s="11" t="s">
         <v>92</v>
       </c>
       <c r="C308" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D308" t="b">
         <v>0</v>
@@ -12682,21 +12718,91 @@
         <v>1</v>
       </c>
       <c r="F308" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="G308" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="H308" s="1" t="str" cm="1">
         <f t="array" ref="H308">CRC16HASH(F308)</f>
+        <v>DD24</v>
+      </c>
+      <c r="I308" t="str">
+        <f t="shared" ref="I308" si="35">_xlfn.CONCAT("{#fig-",H308,"}")</f>
+        <v>{#fig-DD24}</v>
+      </c>
+      <c r="J308" t="str">
+        <f t="shared" ref="J308" si="36">IF(E308,_xlfn.CONCAT("![",G308,"](figures/",B308,"/",F308,")",I308),"")</f>
+        <v>![Viewing the Cost Management screen for the Foundry-related resources](figures/co/ss_costs_001_clean.png){#fig-DD24}</v>
+      </c>
+    </row>
+    <row r="309" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A309">
+        <v>308</v>
+      </c>
+      <c r="B309" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="C309" t="s">
+        <v>6</v>
+      </c>
+      <c r="D309" t="b">
+        <v>0</v>
+      </c>
+      <c r="E309" t="b">
+        <v>1</v>
+      </c>
+      <c r="F309" t="s">
+        <v>502</v>
+      </c>
+      <c r="G309" t="s">
+        <v>503</v>
+      </c>
+      <c r="H309" s="1" t="str" cm="1">
+        <f t="array" ref="H309">CRC16HASH(F309)</f>
+        <v>F9BA</v>
+      </c>
+      <c r="I309" t="str">
+        <f t="shared" ref="I309" si="37">_xlfn.CONCAT("{#fig-",H309,"}")</f>
+        <v>{#fig-F9BA}</v>
+      </c>
+      <c r="J309" t="str">
+        <f t="shared" ref="J309" si="38">IF(E309,_xlfn.CONCAT("![",G309,"](figures/",B309,"/",F309,")",I309),"")</f>
+        <v>![A basic, mostly serverless architecture for AI](figures/co/il_architecture_001_clean.png){#fig-F9BA}</v>
+      </c>
+    </row>
+    <row r="310" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A310">
+        <v>309</v>
+      </c>
+      <c r="B310" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="C310" t="s">
+        <v>6</v>
+      </c>
+      <c r="D310" t="b">
+        <v>0</v>
+      </c>
+      <c r="E310" t="b">
+        <v>1</v>
+      </c>
+      <c r="F310" t="s">
+        <v>506</v>
+      </c>
+      <c r="G310" t="s">
+        <v>505</v>
+      </c>
+      <c r="H310" s="1" t="str" cm="1">
+        <f t="array" ref="H310">CRC16HASH(F310)</f>
         <v>BDB5</v>
       </c>
-      <c r="I308" t="str">
-        <f>_xlfn.CONCAT("{#fig-",H308,"}")</f>
+      <c r="I310" t="str">
+        <f>_xlfn.CONCAT("{#fig-",H310,"}")</f>
         <v>{#fig-BDB5}</v>
       </c>
-      <c r="J308" t="str">
-        <f t="shared" ref="J308" si="39">IF(E308,_xlfn.CONCAT("![",G308,"](figures/",B308,"/",F308,")",I308),"")</f>
+      <c r="J310" t="str">
+        <f t="shared" ref="J310" si="39">IF(E310,_xlfn.CONCAT("![",G310,"](figures/",B310,"/",F310,")",I310),"")</f>
         <v>![A more sophisticated architecture with private networking](figures/co/il_architecture_002_clean.png){#fig-BDB5}</v>
       </c>
     </row>
@@ -12712,14 +12818,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F9AFBD1-7D36-4720-9798-1D6F918A5E59}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:C10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="54.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="54.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>214</v>
       </c>
@@ -12730,7 +12836,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -12741,7 +12847,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -12752,7 +12858,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -12763,7 +12869,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -12774,7 +12880,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -12785,7 +12891,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -12796,7 +12902,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -12807,7 +12913,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -12818,7 +12924,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>9</v>
       </c>

</xml_diff>